<commit_message>
Reconstruit le chiffrier d'édition sur la version 3
Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015pjLsGPzf1MX1JC7QiKGGk
</commit_message>
<xml_diff>
--- a/communique-dragons/Lasclay_brouillons_a_editer.xlsx
+++ b/communique-dragons/Lasclay_brouillons_a_editer.xlsx
@@ -494,13 +494,13 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
-    <col width="104" customWidth="1" min="2" max="2"/>
+    <col width="106" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Version 3 — après ta remarque sur Victor Carré</t>
+          <t>Version 3 — tout corrigé</t>
         </is>
       </c>
       <c r="B1" s="2" t="inlineStr"/>
@@ -509,107 +509,107 @@
       <c r="A2" s="2" t="inlineStr"/>
       <c r="B2" s="2" t="inlineStr"/>
     </row>
-    <row r="3" ht="52" customHeight="1">
+    <row r="3" ht="54" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>Le reproche</t>
+          <t>Le registre</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>« Aucune présentation, mise en contexte. » Juste. Le courriel demandait à quelqu'un de s'intéresser à une entreprise dont il n'a jamais entendu parler et à une matière qu'il ne connaît pas.</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="52" customHeight="1">
+          <t>Plus d'excuses sur le virage manufacturier, plus de « un achat ne sauve pas un papillon », plus de « je ne peux pas dire comment ça s'est terminé ». Vérifié : zéro occurrence dans les 253 brouillons.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="54" customHeight="1">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>Ce que j'ai ajouté</t>
+          <t>La présentation</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Une vraie présentation en tête de tous les courriels froids : qui je suis, ce qu'est Lasclay, ce qu'est l'asclépiade — sous le nom de « petits cochons », que tout le monde reconnaît ici — ce que la fibre fait, ce qu'on en fabrique, et le lien avec le monarque.</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="52" customHeight="1">
+          <t>Les 217 courriels froids commencent par qui tu es, ce qu'est Lasclay et ce qu'est l'asclépiade — sous le nom de « petits cochons », que tout le monde reconnaît ici. Les 5 écrits à la main aussi, ils ne l'avaient pas.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="54" customHeight="1">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t>Et un « pourquoi vous »</t>
+          <t>Le « pourquoi vous »</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>Chaque courriel dit maintenant explicitement pourquoi je lui écris à lui. La raison vient de sa région quand l'asclépiade y a une histoire réelle (Saint-Tite, Granby, le Lac-Saint-Jean), de son sujet sinon.</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="52" customHeight="1">
+          <t>Chaque courriel froid dit explicitement pourquoi il s'adresse à cette personne-là : sa région quand l'asclépiade y a une histoire réelle, son sujet sinon.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="54" customHeight="1">
       <c r="A6" s="3" t="inlineStr">
         <is>
-          <t>Une accroche régionale retirée</t>
+          <t>Une fausse accroche retirée</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>« Notre atelier est dans Limoilou » n'est pas une accroche locale pour un journal de Charlevoix. La Capitale-Nationale passe au thématique.</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="52" customHeight="1">
+          <t>« Notre atelier est dans Limoilou » ne dit rien à un journal de Charlevoix. La Capitale-Nationale passe au thématique.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="54" customHeight="1">
       <c r="A7" s="3" t="inlineStr">
         <is>
-          <t>Les quatre de la liste chaude</t>
+          <t>Les quatre sans historique</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>Roberge, Laforest, Goubau et Dostie n'avaient aucun historique documenté et donc aucune présentation. Ils en ont une maintenant.</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="2" t="inlineStr"/>
-      <c r="B8" s="2" t="inlineStr"/>
+          <t>Roberge, Laforest, Goubau et Dostie n'avaient aucune présentation. Ils en ont une.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="54" customHeight="1">
+      <c r="A8" s="3" t="inlineStr">
+        <is>
+          <t>Les documents</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>04-gabarits-courriels.md est réécrit sur ton squelette. La matrice ne prescrit plus « nommer ce que le virage a coûté » ni la mise en garde sur les monarques.</t>
+        </is>
+      </c>
     </row>
     <row r="9">
-      <c r="A9" s="1" t="inlineStr">
-        <is>
-          <t>Ce qui n'a pas bougé</t>
-        </is>
-      </c>
+      <c r="A9" s="2" t="inlineStr"/>
       <c r="B9" s="2" t="inlineStr"/>
     </row>
     <row r="10">
-      <c r="A10" s="2" t="inlineStr"/>
+      <c r="A10" s="1" t="inlineStr">
+        <is>
+          <t>Ce qui vient de toi</t>
+        </is>
+      </c>
       <c r="B10" s="2" t="inlineStr"/>
     </row>
-    <row r="11" ht="52" customHeight="1">
-      <c r="A11" s="3" t="inlineStr">
-        <is>
-          <t>Ton squelette</t>
-        </is>
-      </c>
-      <c r="B11" s="2" t="inlineStr">
-        <is>
-          <t>Présentation, pourquoi vous, les 2 missions, l'annonce sur sa propre ligne, la rareté et la demande de suite, la chaîne ventes-cultivateurs-monarques, la clôture.</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="52" customHeight="1">
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr"/>
+      <c r="B11" s="2" t="inlineStr"/>
+    </row>
+    <row r="12" ht="54" customHeight="1">
       <c r="A12" s="3" t="inlineStr">
         <is>
-          <t>Larocque et Pouliot</t>
+          <t>Repris mot pour mot</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>Repris mot pour mot.</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="52" customHeight="1">
+          <t>Larocque et Pouliot.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="54" customHeight="1">
       <c r="A13" s="3" t="inlineStr">
         <is>
           <t>Registre</t>
@@ -637,7 +637,7 @@
       <c r="A16" s="2" t="inlineStr"/>
       <c r="B16" s="2" t="inlineStr"/>
     </row>
-    <row r="17" ht="52" customHeight="1">
+    <row r="17" ht="54" customHeight="1">
       <c r="A17" s="3" t="inlineStr">
         <is>
           <t>Diffusion</t>
@@ -649,7 +649,7 @@
         </is>
       </c>
     </row>
-    <row r="18" ht="52" customHeight="1">
+    <row r="18" ht="54" customHeight="1">
       <c r="A18" s="3" t="inlineStr">
         <is>
           <t>Ne pas envoyer</t>
@@ -661,7 +661,7 @@
         </is>
       </c>
     </row>
-    <row r="19" ht="52" customHeight="1">
+    <row r="19" ht="54" customHeight="1">
       <c r="A19" s="3" t="inlineStr">
         <is>
           <t>Courriels manquants</t>
@@ -673,7 +673,7 @@
         </is>
       </c>
     </row>
-    <row r="20" ht="52" customHeight="1">
+    <row r="20" ht="54" customHeight="1">
       <c r="A20" s="3" t="inlineStr">
         <is>
           <t>Salutations à vérifier</t>
@@ -681,7 +681,7 @@
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>Six fiches FPJQ mal formées, signalées dans la colonne Précaution du chiffrier de travail.</t>
+          <t>Six fiches FPJQ mal formées (nom en majuscules, prénoms multiples).</t>
         </is>
       </c>
     </row>
@@ -708,8 +708,8 @@
     <col width="32" customWidth="1" min="7" max="7"/>
     <col width="7" customWidth="1" min="8" max="8"/>
     <col width="10" customWidth="1" min="9" max="9"/>
-    <col width="84" customWidth="1" min="10" max="10"/>
-    <col width="84" customWidth="1" min="11" max="11"/>
+    <col width="88" customWidth="1" min="10" max="10"/>
+    <col width="88" customWidth="1" min="11" max="11"/>
     <col width="42" customWidth="1" min="12" max="12"/>
     <col width="14" customWidth="1" min="13" max="13"/>
   </cols>
@@ -781,7 +781,7 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="230" customHeight="1">
+    <row r="2" ht="270" customHeight="1">
       <c r="A2" s="5" t="inlineStr">
         <is>
           <t>chaude</t>
@@ -846,7 +846,7 @@
       <c r="L2" s="10" t="inlineStr"/>
       <c r="M2" s="10" t="inlineStr"/>
     </row>
-    <row r="3" ht="230" customHeight="1">
+    <row r="3" ht="270" customHeight="1">
       <c r="A3" s="5" t="inlineStr">
         <is>
           <t>chaude</t>
@@ -904,7 +904,7 @@
       <c r="L3" s="10" t="inlineStr"/>
       <c r="M3" s="10" t="inlineStr"/>
     </row>
-    <row r="4" ht="230" customHeight="1">
+    <row r="4" ht="270" customHeight="1">
       <c r="A4" s="5" t="inlineStr">
         <is>
           <t>chaude</t>
@@ -975,7 +975,7 @@
       <c r="L4" s="10" t="inlineStr"/>
       <c r="M4" s="10" t="inlineStr"/>
     </row>
-    <row r="5" ht="230" customHeight="1">
+    <row r="5" ht="270" customHeight="1">
       <c r="A5" s="5" t="inlineStr">
         <is>
           <t>chaude</t>
@@ -1032,7 +1032,7 @@
       <c r="L5" s="10" t="inlineStr"/>
       <c r="M5" s="10" t="inlineStr"/>
     </row>
-    <row r="6" ht="230" customHeight="1">
+    <row r="6" ht="270" customHeight="1">
       <c r="A6" s="5" t="inlineStr">
         <is>
           <t>chaude</t>
@@ -1090,7 +1090,7 @@
       <c r="L6" s="10" t="inlineStr"/>
       <c r="M6" s="10" t="inlineStr"/>
     </row>
-    <row r="7" ht="230" customHeight="1">
+    <row r="7" ht="270" customHeight="1">
       <c r="A7" s="5" t="inlineStr">
         <is>
           <t>chaude</t>
@@ -1148,7 +1148,7 @@
       <c r="L7" s="10" t="inlineStr"/>
       <c r="M7" s="10" t="inlineStr"/>
     </row>
-    <row r="8" ht="230" customHeight="1">
+    <row r="8" ht="270" customHeight="1">
       <c r="A8" s="5" t="inlineStr">
         <is>
           <t>chaude</t>
@@ -1206,7 +1206,7 @@
       <c r="L8" s="10" t="inlineStr"/>
       <c r="M8" s="10" t="inlineStr"/>
     </row>
-    <row r="9" ht="230" customHeight="1">
+    <row r="9" ht="270" customHeight="1">
       <c r="A9" s="5" t="inlineStr">
         <is>
           <t>chaude</t>
@@ -1264,7 +1264,7 @@
       <c r="L9" s="10" t="inlineStr"/>
       <c r="M9" s="10" t="inlineStr"/>
     </row>
-    <row r="10" ht="230" customHeight="1">
+    <row r="10" ht="270" customHeight="1">
       <c r="A10" s="5" t="inlineStr">
         <is>
           <t>chaude</t>
@@ -1322,7 +1322,7 @@
       <c r="L10" s="10" t="inlineStr"/>
       <c r="M10" s="10" t="inlineStr"/>
     </row>
-    <row r="11" ht="230" customHeight="1">
+    <row r="11" ht="270" customHeight="1">
       <c r="A11" s="5" t="inlineStr">
         <is>
           <t>chaude</t>
@@ -1380,7 +1380,7 @@
       <c r="L11" s="10" t="inlineStr"/>
       <c r="M11" s="10" t="inlineStr"/>
     </row>
-    <row r="12" ht="230" customHeight="1">
+    <row r="12" ht="270" customHeight="1">
       <c r="A12" s="5" t="inlineStr">
         <is>
           <t>chaude</t>
@@ -1438,7 +1438,7 @@
       <c r="L12" s="10" t="inlineStr"/>
       <c r="M12" s="10" t="inlineStr"/>
     </row>
-    <row r="13" ht="230" customHeight="1">
+    <row r="13" ht="270" customHeight="1">
       <c r="A13" s="5" t="inlineStr">
         <is>
           <t>chaude</t>
@@ -1496,7 +1496,7 @@
       <c r="L13" s="10" t="inlineStr"/>
       <c r="M13" s="10" t="inlineStr"/>
     </row>
-    <row r="14" ht="230" customHeight="1">
+    <row r="14" ht="270" customHeight="1">
       <c r="A14" s="5" t="inlineStr">
         <is>
           <t>chaude</t>
@@ -1554,7 +1554,7 @@
       <c r="L14" s="10" t="inlineStr"/>
       <c r="M14" s="10" t="inlineStr"/>
     </row>
-    <row r="15" ht="230" customHeight="1">
+    <row r="15" ht="270" customHeight="1">
       <c r="A15" s="5" t="inlineStr">
         <is>
           <t>chaude</t>
@@ -1612,7 +1612,7 @@
       <c r="L15" s="10" t="inlineStr"/>
       <c r="M15" s="10" t="inlineStr"/>
     </row>
-    <row r="16" ht="230" customHeight="1">
+    <row r="16" ht="270" customHeight="1">
       <c r="A16" s="5" t="inlineStr">
         <is>
           <t>chaude</t>
@@ -1669,7 +1669,7 @@
       <c r="L16" s="10" t="inlineStr"/>
       <c r="M16" s="10" t="inlineStr"/>
     </row>
-    <row r="17" ht="230" customHeight="1">
+    <row r="17" ht="270" customHeight="1">
       <c r="A17" s="5" t="inlineStr">
         <is>
           <t>chaude</t>
@@ -1727,7 +1727,7 @@
       <c r="L17" s="10" t="inlineStr"/>
       <c r="M17" s="10" t="inlineStr"/>
     </row>
-    <row r="18" ht="230" customHeight="1">
+    <row r="18" ht="270" customHeight="1">
       <c r="A18" s="5" t="inlineStr">
         <is>
           <t>chaude</t>
@@ -1785,7 +1785,7 @@
       <c r="L18" s="10" t="inlineStr"/>
       <c r="M18" s="10" t="inlineStr"/>
     </row>
-    <row r="19" ht="230" customHeight="1">
+    <row r="19" ht="270" customHeight="1">
       <c r="A19" s="5" t="inlineStr">
         <is>
           <t>chaude</t>
@@ -1843,7 +1843,7 @@
       <c r="L19" s="10" t="inlineStr"/>
       <c r="M19" s="10" t="inlineStr"/>
     </row>
-    <row r="20" ht="230" customHeight="1">
+    <row r="20" ht="270" customHeight="1">
       <c r="A20" s="5" t="inlineStr">
         <is>
           <t>chaude</t>
@@ -1901,7 +1901,7 @@
       <c r="L20" s="10" t="inlineStr"/>
       <c r="M20" s="10" t="inlineStr"/>
     </row>
-    <row r="21" ht="230" customHeight="1">
+    <row r="21" ht="270" customHeight="1">
       <c r="A21" s="5" t="inlineStr">
         <is>
           <t>chaude</t>
@@ -1959,7 +1959,7 @@
       <c r="L21" s="10" t="inlineStr"/>
       <c r="M21" s="10" t="inlineStr"/>
     </row>
-    <row r="22" ht="230" customHeight="1">
+    <row r="22" ht="270" customHeight="1">
       <c r="A22" s="5" t="inlineStr">
         <is>
           <t>chaude</t>
@@ -2017,7 +2017,7 @@
       <c r="L22" s="10" t="inlineStr"/>
       <c r="M22" s="10" t="inlineStr"/>
     </row>
-    <row r="23" ht="230" customHeight="1">
+    <row r="23" ht="270" customHeight="1">
       <c r="A23" s="5" t="inlineStr">
         <is>
           <t>chaude</t>
@@ -2075,7 +2075,7 @@
       <c r="L23" s="10" t="inlineStr"/>
       <c r="M23" s="10" t="inlineStr"/>
     </row>
-    <row r="24" ht="230" customHeight="1">
+    <row r="24" ht="270" customHeight="1">
       <c r="A24" s="5" t="inlineStr">
         <is>
           <t>chaude</t>
@@ -2133,7 +2133,7 @@
       <c r="L24" s="10" t="inlineStr"/>
       <c r="M24" s="10" t="inlineStr"/>
     </row>
-    <row r="25" ht="230" customHeight="1">
+    <row r="25" ht="270" customHeight="1">
       <c r="A25" s="5" t="inlineStr">
         <is>
           <t>chaude</t>
@@ -2191,7 +2191,7 @@
       <c r="L25" s="10" t="inlineStr"/>
       <c r="M25" s="10" t="inlineStr"/>
     </row>
-    <row r="26" ht="230" customHeight="1">
+    <row r="26" ht="270" customHeight="1">
       <c r="A26" s="5" t="inlineStr">
         <is>
           <t>chaude</t>
@@ -2242,7 +2242,7 @@
       <c r="L26" s="10" t="inlineStr"/>
       <c r="M26" s="10" t="inlineStr"/>
     </row>
-    <row r="27" ht="230" customHeight="1">
+    <row r="27" ht="270" customHeight="1">
       <c r="A27" s="5" t="inlineStr">
         <is>
           <t>chaude</t>
@@ -2300,7 +2300,7 @@
       <c r="L27" s="10" t="inlineStr"/>
       <c r="M27" s="10" t="inlineStr"/>
     </row>
-    <row r="28" ht="230" customHeight="1">
+    <row r="28" ht="270" customHeight="1">
       <c r="A28" s="5" t="inlineStr">
         <is>
           <t>chaude</t>
@@ -2350,7 +2350,7 @@
       <c r="L28" s="10" t="inlineStr"/>
       <c r="M28" s="10" t="inlineStr"/>
     </row>
-    <row r="29" ht="230" customHeight="1">
+    <row r="29" ht="270" customHeight="1">
       <c r="A29" s="5" t="inlineStr">
         <is>
           <t>chaude</t>
@@ -2400,7 +2400,7 @@
       <c r="L29" s="10" t="inlineStr"/>
       <c r="M29" s="10" t="inlineStr"/>
     </row>
-    <row r="30" ht="230" customHeight="1">
+    <row r="30" ht="270" customHeight="1">
       <c r="A30" s="5" t="inlineStr">
         <is>
           <t>chaude</t>
@@ -2450,7 +2450,7 @@
       <c r="L30" s="10" t="inlineStr"/>
       <c r="M30" s="10" t="inlineStr"/>
     </row>
-    <row r="31" ht="230" customHeight="1">
+    <row r="31" ht="270" customHeight="1">
       <c r="A31" s="5" t="inlineStr">
         <is>
           <t>chaude</t>
@@ -2508,7 +2508,7 @@
       <c r="L31" s="10" t="inlineStr"/>
       <c r="M31" s="10" t="inlineStr"/>
     </row>
-    <row r="32" ht="230" customHeight="1">
+    <row r="32" ht="270" customHeight="1">
       <c r="A32" s="5" t="inlineStr">
         <is>
           <t>chaude</t>
@@ -2558,7 +2558,7 @@
       <c r="L32" s="10" t="inlineStr"/>
       <c r="M32" s="10" t="inlineStr"/>
     </row>
-    <row r="33" ht="230" customHeight="1">
+    <row r="33" ht="270" customHeight="1">
       <c r="A33" s="5" t="inlineStr">
         <is>
           <t>chaude</t>
@@ -2608,7 +2608,7 @@
       <c r="L33" s="10" t="inlineStr"/>
       <c r="M33" s="10" t="inlineStr"/>
     </row>
-    <row r="34" ht="230" customHeight="1">
+    <row r="34" ht="270" customHeight="1">
       <c r="A34" s="5" t="inlineStr">
         <is>
           <t>chaude</t>
@@ -2658,7 +2658,7 @@
       <c r="L34" s="10" t="inlineStr"/>
       <c r="M34" s="10" t="inlineStr"/>
     </row>
-    <row r="35" ht="230" customHeight="1">
+    <row r="35" ht="270" customHeight="1">
       <c r="A35" s="5" t="inlineStr">
         <is>
           <t>chaude</t>
@@ -2708,7 +2708,7 @@
       <c r="L35" s="10" t="inlineStr"/>
       <c r="M35" s="10" t="inlineStr"/>
     </row>
-    <row r="36" ht="230" customHeight="1">
+    <row r="36" ht="270" customHeight="1">
       <c r="A36" s="5" t="inlineStr">
         <is>
           <t>chaude</t>
@@ -2762,7 +2762,7 @@
       <c r="L36" s="10" t="inlineStr"/>
       <c r="M36" s="10" t="inlineStr"/>
     </row>
-    <row r="37" ht="230" customHeight="1">
+    <row r="37" ht="270" customHeight="1">
       <c r="A37" s="5" t="inlineStr">
         <is>
           <t>chaude</t>
@@ -2816,7 +2816,7 @@
       <c r="L37" s="10" t="inlineStr"/>
       <c r="M37" s="10" t="inlineStr"/>
     </row>
-    <row r="38" ht="230" customHeight="1">
+    <row r="38" ht="270" customHeight="1">
       <c r="A38" s="5" t="inlineStr">
         <is>
           <t>chaude</t>
@@ -2870,7 +2870,7 @@
       <c r="L38" s="10" t="inlineStr"/>
       <c r="M38" s="10" t="inlineStr"/>
     </row>
-    <row r="39" ht="230" customHeight="1">
+    <row r="39" ht="270" customHeight="1">
       <c r="A39" s="6" t="inlineStr">
         <is>
           <t>froide A</t>
@@ -2919,6 +2919,8 @@
       <c r="J39" s="9" t="inlineStr">
         <is>
           <t>Bonjour Marie Allard,
+Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de
+Québec dont l'atelier est dans Limoilou.
 Il y a une belle histoire de sciences dans l'asclépiade. La soie attachée à ses graines n'est
 pas un poil : c'est un tube creux enduit d'une cire hydrophobe, et les fibres portent une
 charge qui les fait se repousser. C'est ce qui forme le parachute autour de la graine, et
@@ -2938,7 +2940,7 @@
       <c r="L39" s="10" t="inlineStr"/>
       <c r="M39" s="10" t="inlineStr"/>
     </row>
-    <row r="40" ht="230" customHeight="1">
+    <row r="40" ht="270" customHeight="1">
       <c r="A40" s="6" t="inlineStr">
         <is>
           <t>froide A</t>
@@ -3002,7 +3004,7 @@
       <c r="L40" s="10" t="inlineStr"/>
       <c r="M40" s="10" t="inlineStr"/>
     </row>
-    <row r="41" ht="230" customHeight="1">
+    <row r="41" ht="270" customHeight="1">
       <c r="A41" s="6" t="inlineStr">
         <is>
           <t>froide A</t>
@@ -3066,7 +3068,7 @@
       <c r="L41" s="10" t="inlineStr"/>
       <c r="M41" s="10" t="inlineStr"/>
     </row>
-    <row r="42" ht="230" customHeight="1">
+    <row r="42" ht="270" customHeight="1">
       <c r="A42" s="6" t="inlineStr">
         <is>
           <t>froide A</t>
@@ -3130,7 +3132,7 @@
       <c r="L42" s="10" t="inlineStr"/>
       <c r="M42" s="10" t="inlineStr"/>
     </row>
-    <row r="43" ht="230" customHeight="1">
+    <row r="43" ht="270" customHeight="1">
       <c r="A43" s="6" t="inlineStr">
         <is>
           <t>froide A</t>
@@ -3194,7 +3196,7 @@
       <c r="L43" s="10" t="inlineStr"/>
       <c r="M43" s="10" t="inlineStr"/>
     </row>
-    <row r="44" ht="230" customHeight="1">
+    <row r="44" ht="270" customHeight="1">
       <c r="A44" s="6" t="inlineStr">
         <is>
           <t>froide A</t>
@@ -3258,7 +3260,7 @@
       <c r="L44" s="10" t="inlineStr"/>
       <c r="M44" s="10" t="inlineStr"/>
     </row>
-    <row r="45" ht="230" customHeight="1">
+    <row r="45" ht="270" customHeight="1">
       <c r="A45" s="6" t="inlineStr">
         <is>
           <t>froide A</t>
@@ -3322,7 +3324,7 @@
       <c r="L45" s="10" t="inlineStr"/>
       <c r="M45" s="10" t="inlineStr"/>
     </row>
-    <row r="46" ht="230" customHeight="1">
+    <row r="46" ht="270" customHeight="1">
       <c r="A46" s="6" t="inlineStr">
         <is>
           <t>froide A</t>
@@ -3386,7 +3388,7 @@
       <c r="L46" s="10" t="inlineStr"/>
       <c r="M46" s="10" t="inlineStr"/>
     </row>
-    <row r="47" ht="230" customHeight="1">
+    <row r="47" ht="270" customHeight="1">
       <c r="A47" s="6" t="inlineStr">
         <is>
           <t>froide A</t>
@@ -3450,7 +3452,7 @@
       <c r="L47" s="10" t="inlineStr"/>
       <c r="M47" s="10" t="inlineStr"/>
     </row>
-    <row r="48" ht="230" customHeight="1">
+    <row r="48" ht="270" customHeight="1">
       <c r="A48" s="6" t="inlineStr">
         <is>
           <t>froide A</t>
@@ -3514,7 +3516,7 @@
       <c r="L48" s="10" t="inlineStr"/>
       <c r="M48" s="10" t="inlineStr"/>
     </row>
-    <row r="49" ht="230" customHeight="1">
+    <row r="49" ht="270" customHeight="1">
       <c r="A49" s="6" t="inlineStr">
         <is>
           <t>froide A</t>
@@ -3578,7 +3580,7 @@
       <c r="L49" s="10" t="inlineStr"/>
       <c r="M49" s="10" t="inlineStr"/>
     </row>
-    <row r="50" ht="230" customHeight="1">
+    <row r="50" ht="270" customHeight="1">
       <c r="A50" s="6" t="inlineStr">
         <is>
           <t>froide A</t>
@@ -3642,7 +3644,7 @@
       <c r="L50" s="10" t="inlineStr"/>
       <c r="M50" s="10" t="inlineStr"/>
     </row>
-    <row r="51" ht="230" customHeight="1">
+    <row r="51" ht="270" customHeight="1">
       <c r="A51" s="6" t="inlineStr">
         <is>
           <t>froide A</t>
@@ -3706,7 +3708,7 @@
       <c r="L51" s="10" t="inlineStr"/>
       <c r="M51" s="10" t="inlineStr"/>
     </row>
-    <row r="52" ht="230" customHeight="1">
+    <row r="52" ht="270" customHeight="1">
       <c r="A52" s="6" t="inlineStr">
         <is>
           <t>froide A</t>
@@ -3770,7 +3772,7 @@
       <c r="L52" s="10" t="inlineStr"/>
       <c r="M52" s="10" t="inlineStr"/>
     </row>
-    <row r="53" ht="230" customHeight="1">
+    <row r="53" ht="270" customHeight="1">
       <c r="A53" s="6" t="inlineStr">
         <is>
           <t>froide A</t>
@@ -3834,7 +3836,7 @@
       <c r="L53" s="10" t="inlineStr"/>
       <c r="M53" s="10" t="inlineStr"/>
     </row>
-    <row r="54" ht="230" customHeight="1">
+    <row r="54" ht="270" customHeight="1">
       <c r="A54" s="6" t="inlineStr">
         <is>
           <t>froide A</t>
@@ -3898,7 +3900,7 @@
       <c r="L54" s="10" t="inlineStr"/>
       <c r="M54" s="10" t="inlineStr"/>
     </row>
-    <row r="55" ht="230" customHeight="1">
+    <row r="55" ht="270" customHeight="1">
       <c r="A55" s="6" t="inlineStr">
         <is>
           <t>froide A</t>
@@ -3962,7 +3964,7 @@
       <c r="L55" s="10" t="inlineStr"/>
       <c r="M55" s="10" t="inlineStr"/>
     </row>
-    <row r="56" ht="230" customHeight="1">
+    <row r="56" ht="270" customHeight="1">
       <c r="A56" s="6" t="inlineStr">
         <is>
           <t>froide A</t>
@@ -4026,7 +4028,7 @@
       <c r="L56" s="10" t="inlineStr"/>
       <c r="M56" s="10" t="inlineStr"/>
     </row>
-    <row r="57" ht="230" customHeight="1">
+    <row r="57" ht="270" customHeight="1">
       <c r="A57" s="6" t="inlineStr">
         <is>
           <t>froide A</t>
@@ -4075,9 +4077,11 @@
       <c r="J57" s="9" t="inlineStr">
         <is>
           <t>Bonjour Gabriel Delisle,
+Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de
+Québec dont l'atelier est dans Limoilou.
 L'asclépiade a été une histoire mauricienne avant d'être la nôtre : l'usine de Saint-Tite
-achetait 90 % des récoltes du Québec. On est l'entreprise qui a démarré après la chute de
-cette filière, et six ans plus tard on achète encore de l'asclépiade québécoise et on la
+achetait 90 % des récoltes du Québec. On a démarré après la chute de cette filière, et six ans
+plus tard on achète encore de l'asclépiade québécoise et on la
 transforme nous-mêmes à Québec.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la
 culture de l'asclépiade.
@@ -4093,7 +4097,7 @@
       <c r="L57" s="10" t="inlineStr"/>
       <c r="M57" s="10" t="inlineStr"/>
     </row>
-    <row r="58" ht="230" customHeight="1">
+    <row r="58" ht="270" customHeight="1">
       <c r="A58" s="6" t="inlineStr">
         <is>
           <t>froide A</t>
@@ -4157,7 +4161,7 @@
       <c r="L58" s="10" t="inlineStr"/>
       <c r="M58" s="10" t="inlineStr"/>
     </row>
-    <row r="59" ht="230" customHeight="1">
+    <row r="59" ht="270" customHeight="1">
       <c r="A59" s="6" t="inlineStr">
         <is>
           <t>froide A</t>
@@ -4221,7 +4225,7 @@
       <c r="L59" s="10" t="inlineStr"/>
       <c r="M59" s="10" t="inlineStr"/>
     </row>
-    <row r="60" ht="230" customHeight="1">
+    <row r="60" ht="270" customHeight="1">
       <c r="A60" s="6" t="inlineStr">
         <is>
           <t>froide A</t>
@@ -4285,7 +4289,7 @@
       <c r="L60" s="10" t="inlineStr"/>
       <c r="M60" s="10" t="inlineStr"/>
     </row>
-    <row r="61" ht="230" customHeight="1">
+    <row r="61" ht="270" customHeight="1">
       <c r="A61" s="6" t="inlineStr">
         <is>
           <t>froide A</t>
@@ -4349,7 +4353,7 @@
       <c r="L61" s="10" t="inlineStr"/>
       <c r="M61" s="10" t="inlineStr"/>
     </row>
-    <row r="62" ht="230" customHeight="1">
+    <row r="62" ht="270" customHeight="1">
       <c r="A62" s="6" t="inlineStr">
         <is>
           <t>froide A</t>
@@ -4413,7 +4417,7 @@
       <c r="L62" s="10" t="inlineStr"/>
       <c r="M62" s="10" t="inlineStr"/>
     </row>
-    <row r="63" ht="230" customHeight="1">
+    <row r="63" ht="270" customHeight="1">
       <c r="A63" s="6" t="inlineStr">
         <is>
           <t>froide A</t>
@@ -4477,7 +4481,7 @@
       <c r="L63" s="10" t="inlineStr"/>
       <c r="M63" s="10" t="inlineStr"/>
     </row>
-    <row r="64" ht="230" customHeight="1">
+    <row r="64" ht="270" customHeight="1">
       <c r="A64" s="6" t="inlineStr">
         <is>
           <t>froide A</t>
@@ -4541,7 +4545,7 @@
       <c r="L64" s="10" t="inlineStr"/>
       <c r="M64" s="10" t="inlineStr"/>
     </row>
-    <row r="65" ht="230" customHeight="1">
+    <row r="65" ht="270" customHeight="1">
       <c r="A65" s="6" t="inlineStr">
         <is>
           <t>froide A</t>
@@ -4605,7 +4609,7 @@
       <c r="L65" s="10" t="inlineStr"/>
       <c r="M65" s="10" t="inlineStr"/>
     </row>
-    <row r="66" ht="230" customHeight="1">
+    <row r="66" ht="270" customHeight="1">
       <c r="A66" s="6" t="inlineStr">
         <is>
           <t>froide A</t>
@@ -4669,7 +4673,7 @@
       <c r="L66" s="10" t="inlineStr"/>
       <c r="M66" s="10" t="inlineStr"/>
     </row>
-    <row r="67" ht="230" customHeight="1">
+    <row r="67" ht="270" customHeight="1">
       <c r="A67" s="6" t="inlineStr">
         <is>
           <t>froide A</t>
@@ -4733,7 +4737,7 @@
       <c r="L67" s="10" t="inlineStr"/>
       <c r="M67" s="10" t="inlineStr"/>
     </row>
-    <row r="68" ht="230" customHeight="1">
+    <row r="68" ht="270" customHeight="1">
       <c r="A68" s="6" t="inlineStr">
         <is>
           <t>froide A</t>
@@ -4797,7 +4801,7 @@
       <c r="L68" s="10" t="inlineStr"/>
       <c r="M68" s="10" t="inlineStr"/>
     </row>
-    <row r="69" ht="230" customHeight="1">
+    <row r="69" ht="270" customHeight="1">
       <c r="A69" s="6" t="inlineStr">
         <is>
           <t>froide A</t>
@@ -4861,7 +4865,7 @@
       <c r="L69" s="10" t="inlineStr"/>
       <c r="M69" s="10" t="inlineStr"/>
     </row>
-    <row r="70" ht="230" customHeight="1">
+    <row r="70" ht="270" customHeight="1">
       <c r="A70" s="6" t="inlineStr">
         <is>
           <t>froide A</t>
@@ -4925,7 +4929,7 @@
       <c r="L70" s="10" t="inlineStr"/>
       <c r="M70" s="10" t="inlineStr"/>
     </row>
-    <row r="71" ht="230" customHeight="1">
+    <row r="71" ht="270" customHeight="1">
       <c r="A71" s="6" t="inlineStr">
         <is>
           <t>froide A</t>
@@ -4989,7 +4993,7 @@
       <c r="L71" s="10" t="inlineStr"/>
       <c r="M71" s="10" t="inlineStr"/>
     </row>
-    <row r="72" ht="230" customHeight="1">
+    <row r="72" ht="270" customHeight="1">
       <c r="A72" s="6" t="inlineStr">
         <is>
           <t>froide A</t>
@@ -5053,7 +5057,7 @@
       <c r="L72" s="10" t="inlineStr"/>
       <c r="M72" s="10" t="inlineStr"/>
     </row>
-    <row r="73" ht="230" customHeight="1">
+    <row r="73" ht="270" customHeight="1">
       <c r="A73" s="6" t="inlineStr">
         <is>
           <t>froide A</t>
@@ -5117,7 +5121,7 @@
       <c r="L73" s="10" t="inlineStr"/>
       <c r="M73" s="10" t="inlineStr"/>
     </row>
-    <row r="74" ht="230" customHeight="1">
+    <row r="74" ht="270" customHeight="1">
       <c r="A74" s="6" t="inlineStr">
         <is>
           <t>froide A</t>
@@ -5181,7 +5185,7 @@
       <c r="L74" s="10" t="inlineStr"/>
       <c r="M74" s="10" t="inlineStr"/>
     </row>
-    <row r="75" ht="230" customHeight="1">
+    <row r="75" ht="270" customHeight="1">
       <c r="A75" s="6" t="inlineStr">
         <is>
           <t>froide A</t>
@@ -5245,7 +5249,7 @@
       <c r="L75" s="10" t="inlineStr"/>
       <c r="M75" s="10" t="inlineStr"/>
     </row>
-    <row r="76" ht="230" customHeight="1">
+    <row r="76" ht="270" customHeight="1">
       <c r="A76" s="6" t="inlineStr">
         <is>
           <t>froide A</t>
@@ -5309,7 +5313,7 @@
       <c r="L76" s="10" t="inlineStr"/>
       <c r="M76" s="10" t="inlineStr"/>
     </row>
-    <row r="77" ht="230" customHeight="1">
+    <row r="77" ht="270" customHeight="1">
       <c r="A77" s="6" t="inlineStr">
         <is>
           <t>froide A</t>
@@ -5373,7 +5377,7 @@
       <c r="L77" s="10" t="inlineStr"/>
       <c r="M77" s="10" t="inlineStr"/>
     </row>
-    <row r="78" ht="230" customHeight="1">
+    <row r="78" ht="270" customHeight="1">
       <c r="A78" s="6" t="inlineStr">
         <is>
           <t>froide A</t>
@@ -5437,7 +5441,7 @@
       <c r="L78" s="10" t="inlineStr"/>
       <c r="M78" s="10" t="inlineStr"/>
     </row>
-    <row r="79" ht="230" customHeight="1">
+    <row r="79" ht="270" customHeight="1">
       <c r="A79" s="6" t="inlineStr">
         <is>
           <t>froide A</t>
@@ -5501,7 +5505,7 @@
       <c r="L79" s="10" t="inlineStr"/>
       <c r="M79" s="10" t="inlineStr"/>
     </row>
-    <row r="80" ht="230" customHeight="1">
+    <row r="80" ht="270" customHeight="1">
       <c r="A80" s="6" t="inlineStr">
         <is>
           <t>froide A</t>
@@ -5565,7 +5569,7 @@
       <c r="L80" s="10" t="inlineStr"/>
       <c r="M80" s="10" t="inlineStr"/>
     </row>
-    <row r="81" ht="230" customHeight="1">
+    <row r="81" ht="270" customHeight="1">
       <c r="A81" s="6" t="inlineStr">
         <is>
           <t>froide A</t>
@@ -5629,7 +5633,7 @@
       <c r="L81" s="10" t="inlineStr"/>
       <c r="M81" s="10" t="inlineStr"/>
     </row>
-    <row r="82" ht="230" customHeight="1">
+    <row r="82" ht="270" customHeight="1">
       <c r="A82" s="6" t="inlineStr">
         <is>
           <t>froide A</t>
@@ -5678,11 +5682,13 @@
       <c r="J82" s="9" t="inlineStr">
         <is>
           <t>Bonjour Réjean Martin,
+Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de
+Québec dont l'atelier est dans Limoilou.
 Vous couvrez Mékinac, donc Saint-Tite, donc l'endroit où l'asclépiade a eu son grand moment
 industriel au Québec. L'usine achetait 90 % des récoltes de la province avant que la filière
 se casse en 2018.
-On est l'entreprise qui a démarré après. Six ans plus tard, on achète encore de l'asclépiade
-québécoise et on la transforme nous-mêmes à Québec. Mes 2 grandes missions : faire connaître
+On a démarré après. Six ans plus tard, on achète encore de l'asclépiade québécoise et on la
+transforme nous-mêmes à Québec. Mes 2 grandes missions : faire connaître
 l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -5697,7 +5703,7 @@
       <c r="L82" s="10" t="inlineStr"/>
       <c r="M82" s="10" t="inlineStr"/>
     </row>
-    <row r="83" ht="230" customHeight="1">
+    <row r="83" ht="270" customHeight="1">
       <c r="A83" s="6" t="inlineStr">
         <is>
           <t>froide A</t>
@@ -5761,7 +5767,7 @@
       <c r="L83" s="10" t="inlineStr"/>
       <c r="M83" s="10" t="inlineStr"/>
     </row>
-    <row r="84" ht="230" customHeight="1">
+    <row r="84" ht="270" customHeight="1">
       <c r="A84" s="6" t="inlineStr">
         <is>
           <t>froide A</t>
@@ -5825,7 +5831,7 @@
       <c r="L84" s="10" t="inlineStr"/>
       <c r="M84" s="10" t="inlineStr"/>
     </row>
-    <row r="85" ht="230" customHeight="1">
+    <row r="85" ht="270" customHeight="1">
       <c r="A85" s="6" t="inlineStr">
         <is>
           <t>froide A</t>
@@ -5889,7 +5895,7 @@
       <c r="L85" s="10" t="inlineStr"/>
       <c r="M85" s="10" t="inlineStr"/>
     </row>
-    <row r="86" ht="230" customHeight="1">
+    <row r="86" ht="270" customHeight="1">
       <c r="A86" s="6" t="inlineStr">
         <is>
           <t>froide A</t>
@@ -5953,7 +5959,7 @@
       <c r="L86" s="10" t="inlineStr"/>
       <c r="M86" s="10" t="inlineStr"/>
     </row>
-    <row r="87" ht="230" customHeight="1">
+    <row r="87" ht="270" customHeight="1">
       <c r="A87" s="6" t="inlineStr">
         <is>
           <t>froide A</t>
@@ -6017,7 +6023,7 @@
       <c r="L87" s="10" t="inlineStr"/>
       <c r="M87" s="10" t="inlineStr"/>
     </row>
-    <row r="88" ht="230" customHeight="1">
+    <row r="88" ht="270" customHeight="1">
       <c r="A88" s="6" t="inlineStr">
         <is>
           <t>froide A</t>
@@ -6081,7 +6087,7 @@
       <c r="L88" s="10" t="inlineStr"/>
       <c r="M88" s="10" t="inlineStr"/>
     </row>
-    <row r="89" ht="230" customHeight="1">
+    <row r="89" ht="270" customHeight="1">
       <c r="A89" s="6" t="inlineStr">
         <is>
           <t>froide A</t>
@@ -6145,7 +6151,7 @@
       <c r="L89" s="10" t="inlineStr"/>
       <c r="M89" s="10" t="inlineStr"/>
     </row>
-    <row r="90" ht="230" customHeight="1">
+    <row r="90" ht="270" customHeight="1">
       <c r="A90" s="6" t="inlineStr">
         <is>
           <t>froide A</t>
@@ -6209,7 +6215,7 @@
       <c r="L90" s="10" t="inlineStr"/>
       <c r="M90" s="10" t="inlineStr"/>
     </row>
-    <row r="91" ht="230" customHeight="1">
+    <row r="91" ht="270" customHeight="1">
       <c r="A91" s="6" t="inlineStr">
         <is>
           <t>froide A</t>
@@ -6273,7 +6279,7 @@
       <c r="L91" s="10" t="inlineStr"/>
       <c r="M91" s="10" t="inlineStr"/>
     </row>
-    <row r="92" ht="230" customHeight="1">
+    <row r="92" ht="270" customHeight="1">
       <c r="A92" s="6" t="inlineStr">
         <is>
           <t>froide A</t>
@@ -6337,7 +6343,7 @@
       <c r="L92" s="10" t="inlineStr"/>
       <c r="M92" s="10" t="inlineStr"/>
     </row>
-    <row r="93" ht="230" customHeight="1">
+    <row r="93" ht="270" customHeight="1">
       <c r="A93" s="6" t="inlineStr">
         <is>
           <t>froide A</t>
@@ -6401,7 +6407,7 @@
       <c r="L93" s="10" t="inlineStr"/>
       <c r="M93" s="10" t="inlineStr"/>
     </row>
-    <row r="94" ht="230" customHeight="1">
+    <row r="94" ht="270" customHeight="1">
       <c r="A94" s="6" t="inlineStr">
         <is>
           <t>froide A</t>
@@ -6465,7 +6471,7 @@
       <c r="L94" s="10" t="inlineStr"/>
       <c r="M94" s="10" t="inlineStr"/>
     </row>
-    <row r="95" ht="230" customHeight="1">
+    <row r="95" ht="270" customHeight="1">
       <c r="A95" s="6" t="inlineStr">
         <is>
           <t>froide A</t>
@@ -6529,7 +6535,7 @@
       <c r="L95" s="10" t="inlineStr"/>
       <c r="M95" s="10" t="inlineStr"/>
     </row>
-    <row r="96" ht="230" customHeight="1">
+    <row r="96" ht="270" customHeight="1">
       <c r="A96" s="6" t="inlineStr">
         <is>
           <t>froide A</t>
@@ -6593,7 +6599,7 @@
       <c r="L96" s="10" t="inlineStr"/>
       <c r="M96" s="10" t="inlineStr"/>
     </row>
-    <row r="97" ht="230" customHeight="1">
+    <row r="97" ht="270" customHeight="1">
       <c r="A97" s="6" t="inlineStr">
         <is>
           <t>froide A</t>
@@ -6657,7 +6663,7 @@
       <c r="L97" s="10" t="inlineStr"/>
       <c r="M97" s="10" t="inlineStr"/>
     </row>
-    <row r="98" ht="230" customHeight="1">
+    <row r="98" ht="270" customHeight="1">
       <c r="A98" s="6" t="inlineStr">
         <is>
           <t>froide A</t>
@@ -6721,7 +6727,7 @@
       <c r="L98" s="10" t="inlineStr"/>
       <c r="M98" s="10" t="inlineStr"/>
     </row>
-    <row r="99" ht="230" customHeight="1">
+    <row r="99" ht="270" customHeight="1">
       <c r="A99" s="6" t="inlineStr">
         <is>
           <t>froide A</t>
@@ -6785,7 +6791,7 @@
       <c r="L99" s="10" t="inlineStr"/>
       <c r="M99" s="10" t="inlineStr"/>
     </row>
-    <row r="100" ht="230" customHeight="1">
+    <row r="100" ht="270" customHeight="1">
       <c r="A100" s="6" t="inlineStr">
         <is>
           <t>froide A</t>
@@ -6849,7 +6855,7 @@
       <c r="L100" s="10" t="inlineStr"/>
       <c r="M100" s="10" t="inlineStr"/>
     </row>
-    <row r="101" ht="230" customHeight="1">
+    <row r="101" ht="270" customHeight="1">
       <c r="A101" s="6" t="inlineStr">
         <is>
           <t>froide A</t>
@@ -6913,7 +6919,7 @@
       <c r="L101" s="10" t="inlineStr"/>
       <c r="M101" s="10" t="inlineStr"/>
     </row>
-    <row r="102" ht="230" customHeight="1">
+    <row r="102" ht="270" customHeight="1">
       <c r="A102" s="6" t="inlineStr">
         <is>
           <t>froide A</t>
@@ -6977,7 +6983,7 @@
       <c r="L102" s="10" t="inlineStr"/>
       <c r="M102" s="10" t="inlineStr"/>
     </row>
-    <row r="103" ht="230" customHeight="1">
+    <row r="103" ht="270" customHeight="1">
       <c r="A103" s="6" t="inlineStr">
         <is>
           <t>froide A</t>
@@ -7041,7 +7047,7 @@
       <c r="L103" s="10" t="inlineStr"/>
       <c r="M103" s="10" t="inlineStr"/>
     </row>
-    <row r="104" ht="230" customHeight="1">
+    <row r="104" ht="270" customHeight="1">
       <c r="A104" s="6" t="inlineStr">
         <is>
           <t>froide A</t>
@@ -7105,7 +7111,7 @@
       <c r="L104" s="10" t="inlineStr"/>
       <c r="M104" s="10" t="inlineStr"/>
     </row>
-    <row r="105" ht="230" customHeight="1">
+    <row r="105" ht="270" customHeight="1">
       <c r="A105" s="6" t="inlineStr">
         <is>
           <t>froide A</t>
@@ -7169,7 +7175,7 @@
       <c r="L105" s="10" t="inlineStr"/>
       <c r="M105" s="10" t="inlineStr"/>
     </row>
-    <row r="106" ht="230" customHeight="1">
+    <row r="106" ht="270" customHeight="1">
       <c r="A106" s="6" t="inlineStr">
         <is>
           <t>froide A</t>
@@ -7233,7 +7239,7 @@
       <c r="L106" s="10" t="inlineStr"/>
       <c r="M106" s="10" t="inlineStr"/>
     </row>
-    <row r="107" ht="230" customHeight="1">
+    <row r="107" ht="270" customHeight="1">
       <c r="A107" s="6" t="inlineStr">
         <is>
           <t>froide A</t>
@@ -7297,7 +7303,7 @@
       <c r="L107" s="10" t="inlineStr"/>
       <c r="M107" s="10" t="inlineStr"/>
     </row>
-    <row r="108" ht="230" customHeight="1">
+    <row r="108" ht="270" customHeight="1">
       <c r="A108" s="6" t="inlineStr">
         <is>
           <t>froide A</t>
@@ -7361,7 +7367,7 @@
       <c r="L108" s="10" t="inlineStr"/>
       <c r="M108" s="10" t="inlineStr"/>
     </row>
-    <row r="109" ht="230" customHeight="1">
+    <row r="109" ht="270" customHeight="1">
       <c r="A109" s="6" t="inlineStr">
         <is>
           <t>froide A</t>
@@ -7425,7 +7431,7 @@
       <c r="L109" s="10" t="inlineStr"/>
       <c r="M109" s="10" t="inlineStr"/>
     </row>
-    <row r="110" ht="230" customHeight="1">
+    <row r="110" ht="270" customHeight="1">
       <c r="A110" s="6" t="inlineStr">
         <is>
           <t>froide B</t>
@@ -7489,7 +7495,7 @@
       <c r="L110" s="10" t="inlineStr"/>
       <c r="M110" s="10" t="inlineStr"/>
     </row>
-    <row r="111" ht="230" customHeight="1">
+    <row r="111" ht="270" customHeight="1">
       <c r="A111" s="6" t="inlineStr">
         <is>
           <t>froide B</t>
@@ -7553,7 +7559,7 @@
       <c r="L111" s="10" t="inlineStr"/>
       <c r="M111" s="10" t="inlineStr"/>
     </row>
-    <row r="112" ht="230" customHeight="1">
+    <row r="112" ht="270" customHeight="1">
       <c r="A112" s="6" t="inlineStr">
         <is>
           <t>froide B</t>
@@ -7617,7 +7623,7 @@
       <c r="L112" s="10" t="inlineStr"/>
       <c r="M112" s="10" t="inlineStr"/>
     </row>
-    <row r="113" ht="230" customHeight="1">
+    <row r="113" ht="270" customHeight="1">
       <c r="A113" s="6" t="inlineStr">
         <is>
           <t>froide B</t>
@@ -7681,7 +7687,7 @@
       <c r="L113" s="10" t="inlineStr"/>
       <c r="M113" s="10" t="inlineStr"/>
     </row>
-    <row r="114" ht="230" customHeight="1">
+    <row r="114" ht="270" customHeight="1">
       <c r="A114" s="6" t="inlineStr">
         <is>
           <t>froide B</t>
@@ -7745,7 +7751,7 @@
       <c r="L114" s="10" t="inlineStr"/>
       <c r="M114" s="10" t="inlineStr"/>
     </row>
-    <row r="115" ht="230" customHeight="1">
+    <row r="115" ht="270" customHeight="1">
       <c r="A115" s="6" t="inlineStr">
         <is>
           <t>froide B</t>
@@ -7809,7 +7815,7 @@
       <c r="L115" s="10" t="inlineStr"/>
       <c r="M115" s="10" t="inlineStr"/>
     </row>
-    <row r="116" ht="230" customHeight="1">
+    <row r="116" ht="270" customHeight="1">
       <c r="A116" s="6" t="inlineStr">
         <is>
           <t>froide B</t>
@@ -7873,7 +7879,7 @@
       <c r="L116" s="10" t="inlineStr"/>
       <c r="M116" s="10" t="inlineStr"/>
     </row>
-    <row r="117" ht="230" customHeight="1">
+    <row r="117" ht="270" customHeight="1">
       <c r="A117" s="6" t="inlineStr">
         <is>
           <t>froide B</t>
@@ -7937,7 +7943,7 @@
       <c r="L117" s="10" t="inlineStr"/>
       <c r="M117" s="10" t="inlineStr"/>
     </row>
-    <row r="118" ht="230" customHeight="1">
+    <row r="118" ht="270" customHeight="1">
       <c r="A118" s="6" t="inlineStr">
         <is>
           <t>froide B</t>
@@ -8001,7 +8007,7 @@
       <c r="L118" s="10" t="inlineStr"/>
       <c r="M118" s="10" t="inlineStr"/>
     </row>
-    <row r="119" ht="230" customHeight="1">
+    <row r="119" ht="270" customHeight="1">
       <c r="A119" s="6" t="inlineStr">
         <is>
           <t>froide B</t>
@@ -8065,7 +8071,7 @@
       <c r="L119" s="10" t="inlineStr"/>
       <c r="M119" s="10" t="inlineStr"/>
     </row>
-    <row r="120" ht="230" customHeight="1">
+    <row r="120" ht="270" customHeight="1">
       <c r="A120" s="6" t="inlineStr">
         <is>
           <t>froide B</t>
@@ -8129,7 +8135,7 @@
       <c r="L120" s="10" t="inlineStr"/>
       <c r="M120" s="10" t="inlineStr"/>
     </row>
-    <row r="121" ht="230" customHeight="1">
+    <row r="121" ht="270" customHeight="1">
       <c r="A121" s="6" t="inlineStr">
         <is>
           <t>froide B</t>
@@ -8193,7 +8199,7 @@
       <c r="L121" s="10" t="inlineStr"/>
       <c r="M121" s="10" t="inlineStr"/>
     </row>
-    <row r="122" ht="230" customHeight="1">
+    <row r="122" ht="270" customHeight="1">
       <c r="A122" s="6" t="inlineStr">
         <is>
           <t>froide B</t>
@@ -8257,7 +8263,7 @@
       <c r="L122" s="10" t="inlineStr"/>
       <c r="M122" s="10" t="inlineStr"/>
     </row>
-    <row r="123" ht="230" customHeight="1">
+    <row r="123" ht="270" customHeight="1">
       <c r="A123" s="6" t="inlineStr">
         <is>
           <t>froide B</t>
@@ -8321,7 +8327,7 @@
       <c r="L123" s="10" t="inlineStr"/>
       <c r="M123" s="10" t="inlineStr"/>
     </row>
-    <row r="124" ht="230" customHeight="1">
+    <row r="124" ht="270" customHeight="1">
       <c r="A124" s="6" t="inlineStr">
         <is>
           <t>froide B</t>
@@ -8385,7 +8391,7 @@
       <c r="L124" s="10" t="inlineStr"/>
       <c r="M124" s="10" t="inlineStr"/>
     </row>
-    <row r="125" ht="230" customHeight="1">
+    <row r="125" ht="270" customHeight="1">
       <c r="A125" s="6" t="inlineStr">
         <is>
           <t>froide B</t>
@@ -8449,7 +8455,7 @@
       <c r="L125" s="10" t="inlineStr"/>
       <c r="M125" s="10" t="inlineStr"/>
     </row>
-    <row r="126" ht="230" customHeight="1">
+    <row r="126" ht="270" customHeight="1">
       <c r="A126" s="6" t="inlineStr">
         <is>
           <t>froide B</t>
@@ -8513,7 +8519,7 @@
       <c r="L126" s="10" t="inlineStr"/>
       <c r="M126" s="10" t="inlineStr"/>
     </row>
-    <row r="127" ht="230" customHeight="1">
+    <row r="127" ht="270" customHeight="1">
       <c r="A127" s="6" t="inlineStr">
         <is>
           <t>froide B</t>
@@ -8577,7 +8583,7 @@
       <c r="L127" s="10" t="inlineStr"/>
       <c r="M127" s="10" t="inlineStr"/>
     </row>
-    <row r="128" ht="230" customHeight="1">
+    <row r="128" ht="270" customHeight="1">
       <c r="A128" s="6" t="inlineStr">
         <is>
           <t>froide B</t>
@@ -8641,7 +8647,7 @@
       <c r="L128" s="10" t="inlineStr"/>
       <c r="M128" s="10" t="inlineStr"/>
     </row>
-    <row r="129" ht="230" customHeight="1">
+    <row r="129" ht="270" customHeight="1">
       <c r="A129" s="6" t="inlineStr">
         <is>
           <t>froide B</t>
@@ -8705,7 +8711,7 @@
       <c r="L129" s="10" t="inlineStr"/>
       <c r="M129" s="10" t="inlineStr"/>
     </row>
-    <row r="130" ht="230" customHeight="1">
+    <row r="130" ht="270" customHeight="1">
       <c r="A130" s="6" t="inlineStr">
         <is>
           <t>froide B</t>
@@ -8769,7 +8775,7 @@
       <c r="L130" s="10" t="inlineStr"/>
       <c r="M130" s="10" t="inlineStr"/>
     </row>
-    <row r="131" ht="230" customHeight="1">
+    <row r="131" ht="270" customHeight="1">
       <c r="A131" s="6" t="inlineStr">
         <is>
           <t>froide B</t>
@@ -8833,7 +8839,7 @@
       <c r="L131" s="10" t="inlineStr"/>
       <c r="M131" s="10" t="inlineStr"/>
     </row>
-    <row r="132" ht="230" customHeight="1">
+    <row r="132" ht="270" customHeight="1">
       <c r="A132" s="6" t="inlineStr">
         <is>
           <t>froide B</t>
@@ -8897,7 +8903,7 @@
       <c r="L132" s="10" t="inlineStr"/>
       <c r="M132" s="10" t="inlineStr"/>
     </row>
-    <row r="133" ht="230" customHeight="1">
+    <row r="133" ht="270" customHeight="1">
       <c r="A133" s="6" t="inlineStr">
         <is>
           <t>froide B</t>
@@ -8961,7 +8967,7 @@
       <c r="L133" s="10" t="inlineStr"/>
       <c r="M133" s="10" t="inlineStr"/>
     </row>
-    <row r="134" ht="230" customHeight="1">
+    <row r="134" ht="270" customHeight="1">
       <c r="A134" s="6" t="inlineStr">
         <is>
           <t>froide B</t>
@@ -9025,7 +9031,7 @@
       <c r="L134" s="10" t="inlineStr"/>
       <c r="M134" s="10" t="inlineStr"/>
     </row>
-    <row r="135" ht="230" customHeight="1">
+    <row r="135" ht="270" customHeight="1">
       <c r="A135" s="6" t="inlineStr">
         <is>
           <t>froide B</t>
@@ -9089,7 +9095,7 @@
       <c r="L135" s="10" t="inlineStr"/>
       <c r="M135" s="10" t="inlineStr"/>
     </row>
-    <row r="136" ht="230" customHeight="1">
+    <row r="136" ht="270" customHeight="1">
       <c r="A136" s="6" t="inlineStr">
         <is>
           <t>froide B</t>
@@ -9153,7 +9159,7 @@
       <c r="L136" s="10" t="inlineStr"/>
       <c r="M136" s="10" t="inlineStr"/>
     </row>
-    <row r="137" ht="230" customHeight="1">
+    <row r="137" ht="270" customHeight="1">
       <c r="A137" s="6" t="inlineStr">
         <is>
           <t>froide B</t>
@@ -9217,7 +9223,7 @@
       <c r="L137" s="10" t="inlineStr"/>
       <c r="M137" s="10" t="inlineStr"/>
     </row>
-    <row r="138" ht="230" customHeight="1">
+    <row r="138" ht="270" customHeight="1">
       <c r="A138" s="6" t="inlineStr">
         <is>
           <t>froide B</t>
@@ -9281,7 +9287,7 @@
       <c r="L138" s="10" t="inlineStr"/>
       <c r="M138" s="10" t="inlineStr"/>
     </row>
-    <row r="139" ht="230" customHeight="1">
+    <row r="139" ht="270" customHeight="1">
       <c r="A139" s="6" t="inlineStr">
         <is>
           <t>froide B</t>
@@ -9345,7 +9351,7 @@
       <c r="L139" s="10" t="inlineStr"/>
       <c r="M139" s="10" t="inlineStr"/>
     </row>
-    <row r="140" ht="230" customHeight="1">
+    <row r="140" ht="270" customHeight="1">
       <c r="A140" s="6" t="inlineStr">
         <is>
           <t>froide B</t>
@@ -9409,7 +9415,7 @@
       <c r="L140" s="10" t="inlineStr"/>
       <c r="M140" s="10" t="inlineStr"/>
     </row>
-    <row r="141" ht="230" customHeight="1">
+    <row r="141" ht="270" customHeight="1">
       <c r="A141" s="6" t="inlineStr">
         <is>
           <t>froide B</t>
@@ -9473,7 +9479,7 @@
       <c r="L141" s="10" t="inlineStr"/>
       <c r="M141" s="10" t="inlineStr"/>
     </row>
-    <row r="142" ht="230" customHeight="1">
+    <row r="142" ht="270" customHeight="1">
       <c r="A142" s="6" t="inlineStr">
         <is>
           <t>froide B</t>
@@ -9537,7 +9543,7 @@
       <c r="L142" s="10" t="inlineStr"/>
       <c r="M142" s="10" t="inlineStr"/>
     </row>
-    <row r="143" ht="230" customHeight="1">
+    <row r="143" ht="270" customHeight="1">
       <c r="A143" s="6" t="inlineStr">
         <is>
           <t>froide B</t>
@@ -9601,7 +9607,7 @@
       <c r="L143" s="10" t="inlineStr"/>
       <c r="M143" s="10" t="inlineStr"/>
     </row>
-    <row r="144" ht="230" customHeight="1">
+    <row r="144" ht="270" customHeight="1">
       <c r="A144" s="6" t="inlineStr">
         <is>
           <t>froide B</t>
@@ -9665,7 +9671,7 @@
       <c r="L144" s="10" t="inlineStr"/>
       <c r="M144" s="10" t="inlineStr"/>
     </row>
-    <row r="145" ht="230" customHeight="1">
+    <row r="145" ht="270" customHeight="1">
       <c r="A145" s="6" t="inlineStr">
         <is>
           <t>froide B</t>
@@ -9729,7 +9735,7 @@
       <c r="L145" s="10" t="inlineStr"/>
       <c r="M145" s="10" t="inlineStr"/>
     </row>
-    <row r="146" ht="230" customHeight="1">
+    <row r="146" ht="270" customHeight="1">
       <c r="A146" s="6" t="inlineStr">
         <is>
           <t>froide B</t>
@@ -9793,7 +9799,7 @@
       <c r="L146" s="10" t="inlineStr"/>
       <c r="M146" s="10" t="inlineStr"/>
     </row>
-    <row r="147" ht="230" customHeight="1">
+    <row r="147" ht="270" customHeight="1">
       <c r="A147" s="6" t="inlineStr">
         <is>
           <t>froide B</t>
@@ -9857,7 +9863,7 @@
       <c r="L147" s="10" t="inlineStr"/>
       <c r="M147" s="10" t="inlineStr"/>
     </row>
-    <row r="148" ht="230" customHeight="1">
+    <row r="148" ht="270" customHeight="1">
       <c r="A148" s="6" t="inlineStr">
         <is>
           <t>froide B</t>
@@ -9921,7 +9927,7 @@
       <c r="L148" s="10" t="inlineStr"/>
       <c r="M148" s="10" t="inlineStr"/>
     </row>
-    <row r="149" ht="230" customHeight="1">
+    <row r="149" ht="270" customHeight="1">
       <c r="A149" s="6" t="inlineStr">
         <is>
           <t>froide B</t>
@@ -9985,7 +9991,7 @@
       <c r="L149" s="10" t="inlineStr"/>
       <c r="M149" s="10" t="inlineStr"/>
     </row>
-    <row r="150" ht="230" customHeight="1">
+    <row r="150" ht="270" customHeight="1">
       <c r="A150" s="6" t="inlineStr">
         <is>
           <t>froide B</t>
@@ -10049,7 +10055,7 @@
       <c r="L150" s="10" t="inlineStr"/>
       <c r="M150" s="10" t="inlineStr"/>
     </row>
-    <row r="151" ht="230" customHeight="1">
+    <row r="151" ht="270" customHeight="1">
       <c r="A151" s="6" t="inlineStr">
         <is>
           <t>froide B</t>
@@ -10113,7 +10119,7 @@
       <c r="L151" s="10" t="inlineStr"/>
       <c r="M151" s="10" t="inlineStr"/>
     </row>
-    <row r="152" ht="230" customHeight="1">
+    <row r="152" ht="270" customHeight="1">
       <c r="A152" s="6" t="inlineStr">
         <is>
           <t>froide B</t>
@@ -10177,7 +10183,7 @@
       <c r="L152" s="10" t="inlineStr"/>
       <c r="M152" s="10" t="inlineStr"/>
     </row>
-    <row r="153" ht="230" customHeight="1">
+    <row r="153" ht="270" customHeight="1">
       <c r="A153" s="6" t="inlineStr">
         <is>
           <t>froide B</t>
@@ -10241,7 +10247,7 @@
       <c r="L153" s="10" t="inlineStr"/>
       <c r="M153" s="10" t="inlineStr"/>
     </row>
-    <row r="154" ht="230" customHeight="1">
+    <row r="154" ht="270" customHeight="1">
       <c r="A154" s="6" t="inlineStr">
         <is>
           <t>froide B</t>
@@ -10305,7 +10311,7 @@
       <c r="L154" s="10" t="inlineStr"/>
       <c r="M154" s="10" t="inlineStr"/>
     </row>
-    <row r="155" ht="230" customHeight="1">
+    <row r="155" ht="270" customHeight="1">
       <c r="A155" s="6" t="inlineStr">
         <is>
           <t>froide B</t>
@@ -10369,7 +10375,7 @@
       <c r="L155" s="10" t="inlineStr"/>
       <c r="M155" s="10" t="inlineStr"/>
     </row>
-    <row r="156" ht="230" customHeight="1">
+    <row r="156" ht="270" customHeight="1">
       <c r="A156" s="6" t="inlineStr">
         <is>
           <t>froide B</t>
@@ -10433,7 +10439,7 @@
       <c r="L156" s="10" t="inlineStr"/>
       <c r="M156" s="10" t="inlineStr"/>
     </row>
-    <row r="157" ht="230" customHeight="1">
+    <row r="157" ht="270" customHeight="1">
       <c r="A157" s="6" t="inlineStr">
         <is>
           <t>froide B</t>
@@ -10497,7 +10503,7 @@
       <c r="L157" s="10" t="inlineStr"/>
       <c r="M157" s="10" t="inlineStr"/>
     </row>
-    <row r="158" ht="230" customHeight="1">
+    <row r="158" ht="270" customHeight="1">
       <c r="A158" s="6" t="inlineStr">
         <is>
           <t>froide B</t>
@@ -10561,7 +10567,7 @@
       <c r="L158" s="10" t="inlineStr"/>
       <c r="M158" s="10" t="inlineStr"/>
     </row>
-    <row r="159" ht="230" customHeight="1">
+    <row r="159" ht="270" customHeight="1">
       <c r="A159" s="6" t="inlineStr">
         <is>
           <t>froide B</t>
@@ -10625,7 +10631,7 @@
       <c r="L159" s="10" t="inlineStr"/>
       <c r="M159" s="10" t="inlineStr"/>
     </row>
-    <row r="160" ht="230" customHeight="1">
+    <row r="160" ht="270" customHeight="1">
       <c r="A160" s="6" t="inlineStr">
         <is>
           <t>froide B</t>
@@ -10689,7 +10695,7 @@
       <c r="L160" s="10" t="inlineStr"/>
       <c r="M160" s="10" t="inlineStr"/>
     </row>
-    <row r="161" ht="230" customHeight="1">
+    <row r="161" ht="270" customHeight="1">
       <c r="A161" s="6" t="inlineStr">
         <is>
           <t>froide B</t>
@@ -10753,7 +10759,7 @@
       <c r="L161" s="10" t="inlineStr"/>
       <c r="M161" s="10" t="inlineStr"/>
     </row>
-    <row r="162" ht="230" customHeight="1">
+    <row r="162" ht="270" customHeight="1">
       <c r="A162" s="6" t="inlineStr">
         <is>
           <t>froide B</t>
@@ -10817,7 +10823,7 @@
       <c r="L162" s="10" t="inlineStr"/>
       <c r="M162" s="10" t="inlineStr"/>
     </row>
-    <row r="163" ht="230" customHeight="1">
+    <row r="163" ht="270" customHeight="1">
       <c r="A163" s="6" t="inlineStr">
         <is>
           <t>froide C</t>
@@ -10881,7 +10887,7 @@
       <c r="L163" s="10" t="inlineStr"/>
       <c r="M163" s="10" t="inlineStr"/>
     </row>
-    <row r="164" ht="230" customHeight="1">
+    <row r="164" ht="270" customHeight="1">
       <c r="A164" s="6" t="inlineStr">
         <is>
           <t>froide C</t>
@@ -10945,7 +10951,7 @@
       <c r="L164" s="10" t="inlineStr"/>
       <c r="M164" s="10" t="inlineStr"/>
     </row>
-    <row r="165" ht="230" customHeight="1">
+    <row r="165" ht="270" customHeight="1">
       <c r="A165" s="6" t="inlineStr">
         <is>
           <t>froide C</t>
@@ -11009,7 +11015,7 @@
       <c r="L165" s="10" t="inlineStr"/>
       <c r="M165" s="10" t="inlineStr"/>
     </row>
-    <row r="166" ht="230" customHeight="1">
+    <row r="166" ht="270" customHeight="1">
       <c r="A166" s="6" t="inlineStr">
         <is>
           <t>froide C</t>
@@ -11073,7 +11079,7 @@
       <c r="L166" s="10" t="inlineStr"/>
       <c r="M166" s="10" t="inlineStr"/>
     </row>
-    <row r="167" ht="230" customHeight="1">
+    <row r="167" ht="270" customHeight="1">
       <c r="A167" s="6" t="inlineStr">
         <is>
           <t>froide C</t>
@@ -11137,7 +11143,7 @@
       <c r="L167" s="10" t="inlineStr"/>
       <c r="M167" s="10" t="inlineStr"/>
     </row>
-    <row r="168" ht="230" customHeight="1">
+    <row r="168" ht="270" customHeight="1">
       <c r="A168" s="6" t="inlineStr">
         <is>
           <t>froide C</t>
@@ -11201,7 +11207,7 @@
       <c r="L168" s="10" t="inlineStr"/>
       <c r="M168" s="10" t="inlineStr"/>
     </row>
-    <row r="169" ht="230" customHeight="1">
+    <row r="169" ht="270" customHeight="1">
       <c r="A169" s="6" t="inlineStr">
         <is>
           <t>froide C</t>
@@ -11265,7 +11271,7 @@
       <c r="L169" s="10" t="inlineStr"/>
       <c r="M169" s="10" t="inlineStr"/>
     </row>
-    <row r="170" ht="230" customHeight="1">
+    <row r="170" ht="270" customHeight="1">
       <c r="A170" s="6" t="inlineStr">
         <is>
           <t>froide C</t>
@@ -11329,7 +11335,7 @@
       <c r="L170" s="10" t="inlineStr"/>
       <c r="M170" s="10" t="inlineStr"/>
     </row>
-    <row r="171" ht="230" customHeight="1">
+    <row r="171" ht="270" customHeight="1">
       <c r="A171" s="6" t="inlineStr">
         <is>
           <t>froide C</t>
@@ -11393,7 +11399,7 @@
       <c r="L171" s="10" t="inlineStr"/>
       <c r="M171" s="10" t="inlineStr"/>
     </row>
-    <row r="172" ht="230" customHeight="1">
+    <row r="172" ht="270" customHeight="1">
       <c r="A172" s="6" t="inlineStr">
         <is>
           <t>froide C</t>
@@ -11457,7 +11463,7 @@
       <c r="L172" s="10" t="inlineStr"/>
       <c r="M172" s="10" t="inlineStr"/>
     </row>
-    <row r="173" ht="230" customHeight="1">
+    <row r="173" ht="270" customHeight="1">
       <c r="A173" s="6" t="inlineStr">
         <is>
           <t>froide C</t>
@@ -11521,7 +11527,7 @@
       <c r="L173" s="10" t="inlineStr"/>
       <c r="M173" s="10" t="inlineStr"/>
     </row>
-    <row r="174" ht="230" customHeight="1">
+    <row r="174" ht="270" customHeight="1">
       <c r="A174" s="6" t="inlineStr">
         <is>
           <t>froide C</t>
@@ -11585,7 +11591,7 @@
       <c r="L174" s="10" t="inlineStr"/>
       <c r="M174" s="10" t="inlineStr"/>
     </row>
-    <row r="175" ht="230" customHeight="1">
+    <row r="175" ht="270" customHeight="1">
       <c r="A175" s="6" t="inlineStr">
         <is>
           <t>froide C</t>
@@ -11649,7 +11655,7 @@
       <c r="L175" s="10" t="inlineStr"/>
       <c r="M175" s="10" t="inlineStr"/>
     </row>
-    <row r="176" ht="230" customHeight="1">
+    <row r="176" ht="270" customHeight="1">
       <c r="A176" s="6" t="inlineStr">
         <is>
           <t>froide C</t>
@@ -11713,7 +11719,7 @@
       <c r="L176" s="10" t="inlineStr"/>
       <c r="M176" s="10" t="inlineStr"/>
     </row>
-    <row r="177" ht="230" customHeight="1">
+    <row r="177" ht="270" customHeight="1">
       <c r="A177" s="6" t="inlineStr">
         <is>
           <t>froide C</t>
@@ -11777,7 +11783,7 @@
       <c r="L177" s="10" t="inlineStr"/>
       <c r="M177" s="10" t="inlineStr"/>
     </row>
-    <row r="178" ht="230" customHeight="1">
+    <row r="178" ht="270" customHeight="1">
       <c r="A178" s="6" t="inlineStr">
         <is>
           <t>froide C</t>
@@ -11841,7 +11847,7 @@
       <c r="L178" s="10" t="inlineStr"/>
       <c r="M178" s="10" t="inlineStr"/>
     </row>
-    <row r="179" ht="230" customHeight="1">
+    <row r="179" ht="270" customHeight="1">
       <c r="A179" s="6" t="inlineStr">
         <is>
           <t>froide C</t>
@@ -11905,7 +11911,7 @@
       <c r="L179" s="10" t="inlineStr"/>
       <c r="M179" s="10" t="inlineStr"/>
     </row>
-    <row r="180" ht="230" customHeight="1">
+    <row r="180" ht="270" customHeight="1">
       <c r="A180" s="6" t="inlineStr">
         <is>
           <t>froide C</t>
@@ -11969,7 +11975,7 @@
       <c r="L180" s="10" t="inlineStr"/>
       <c r="M180" s="10" t="inlineStr"/>
     </row>
-    <row r="181" ht="230" customHeight="1">
+    <row r="181" ht="270" customHeight="1">
       <c r="A181" s="6" t="inlineStr">
         <is>
           <t>froide C</t>
@@ -12033,7 +12039,7 @@
       <c r="L181" s="10" t="inlineStr"/>
       <c r="M181" s="10" t="inlineStr"/>
     </row>
-    <row r="182" ht="230" customHeight="1">
+    <row r="182" ht="270" customHeight="1">
       <c r="A182" s="6" t="inlineStr">
         <is>
           <t>froide C</t>
@@ -12097,7 +12103,7 @@
       <c r="L182" s="10" t="inlineStr"/>
       <c r="M182" s="10" t="inlineStr"/>
     </row>
-    <row r="183" ht="230" customHeight="1">
+    <row r="183" ht="270" customHeight="1">
       <c r="A183" s="6" t="inlineStr">
         <is>
           <t>froide C</t>
@@ -12161,7 +12167,7 @@
       <c r="L183" s="10" t="inlineStr"/>
       <c r="M183" s="10" t="inlineStr"/>
     </row>
-    <row r="184" ht="230" customHeight="1">
+    <row r="184" ht="270" customHeight="1">
       <c r="A184" s="6" t="inlineStr">
         <is>
           <t>froide C</t>
@@ -12225,7 +12231,7 @@
       <c r="L184" s="10" t="inlineStr"/>
       <c r="M184" s="10" t="inlineStr"/>
     </row>
-    <row r="185" ht="230" customHeight="1">
+    <row r="185" ht="270" customHeight="1">
       <c r="A185" s="6" t="inlineStr">
         <is>
           <t>froide C</t>
@@ -12289,7 +12295,7 @@
       <c r="L185" s="10" t="inlineStr"/>
       <c r="M185" s="10" t="inlineStr"/>
     </row>
-    <row r="186" ht="230" customHeight="1">
+    <row r="186" ht="270" customHeight="1">
       <c r="A186" s="6" t="inlineStr">
         <is>
           <t>froide C</t>
@@ -12353,7 +12359,7 @@
       <c r="L186" s="10" t="inlineStr"/>
       <c r="M186" s="10" t="inlineStr"/>
     </row>
-    <row r="187" ht="230" customHeight="1">
+    <row r="187" ht="270" customHeight="1">
       <c r="A187" s="6" t="inlineStr">
         <is>
           <t>froide C</t>
@@ -12417,7 +12423,7 @@
       <c r="L187" s="10" t="inlineStr"/>
       <c r="M187" s="10" t="inlineStr"/>
     </row>
-    <row r="188" ht="230" customHeight="1">
+    <row r="188" ht="270" customHeight="1">
       <c r="A188" s="6" t="inlineStr">
         <is>
           <t>froide C</t>
@@ -12481,7 +12487,7 @@
       <c r="L188" s="10" t="inlineStr"/>
       <c r="M188" s="10" t="inlineStr"/>
     </row>
-    <row r="189" ht="230" customHeight="1">
+    <row r="189" ht="270" customHeight="1">
       <c r="A189" s="6" t="inlineStr">
         <is>
           <t>froide C</t>
@@ -12545,7 +12551,7 @@
       <c r="L189" s="10" t="inlineStr"/>
       <c r="M189" s="10" t="inlineStr"/>
     </row>
-    <row r="190" ht="230" customHeight="1">
+    <row r="190" ht="270" customHeight="1">
       <c r="A190" s="6" t="inlineStr">
         <is>
           <t>froide C</t>
@@ -12609,7 +12615,7 @@
       <c r="L190" s="10" t="inlineStr"/>
       <c r="M190" s="10" t="inlineStr"/>
     </row>
-    <row r="191" ht="230" customHeight="1">
+    <row r="191" ht="270" customHeight="1">
       <c r="A191" s="6" t="inlineStr">
         <is>
           <t>froide C</t>
@@ -12673,7 +12679,7 @@
       <c r="L191" s="10" t="inlineStr"/>
       <c r="M191" s="10" t="inlineStr"/>
     </row>
-    <row r="192" ht="230" customHeight="1">
+    <row r="192" ht="270" customHeight="1">
       <c r="A192" s="6" t="inlineStr">
         <is>
           <t>froide C</t>
@@ -12737,7 +12743,7 @@
       <c r="L192" s="10" t="inlineStr"/>
       <c r="M192" s="10" t="inlineStr"/>
     </row>
-    <row r="193" ht="230" customHeight="1">
+    <row r="193" ht="270" customHeight="1">
       <c r="A193" s="6" t="inlineStr">
         <is>
           <t>froide C</t>
@@ -12801,7 +12807,7 @@
       <c r="L193" s="10" t="inlineStr"/>
       <c r="M193" s="10" t="inlineStr"/>
     </row>
-    <row r="194" ht="230" customHeight="1">
+    <row r="194" ht="270" customHeight="1">
       <c r="A194" s="6" t="inlineStr">
         <is>
           <t>froide C</t>
@@ -12865,7 +12871,7 @@
       <c r="L194" s="10" t="inlineStr"/>
       <c r="M194" s="10" t="inlineStr"/>
     </row>
-    <row r="195" ht="230" customHeight="1">
+    <row r="195" ht="270" customHeight="1">
       <c r="A195" s="6" t="inlineStr">
         <is>
           <t>froide C</t>
@@ -12929,7 +12935,7 @@
       <c r="L195" s="10" t="inlineStr"/>
       <c r="M195" s="10" t="inlineStr"/>
     </row>
-    <row r="196" ht="230" customHeight="1">
+    <row r="196" ht="270" customHeight="1">
       <c r="A196" s="6" t="inlineStr">
         <is>
           <t>froide C</t>
@@ -12993,7 +12999,7 @@
       <c r="L196" s="10" t="inlineStr"/>
       <c r="M196" s="10" t="inlineStr"/>
     </row>
-    <row r="197" ht="230" customHeight="1">
+    <row r="197" ht="270" customHeight="1">
       <c r="A197" s="6" t="inlineStr">
         <is>
           <t>froide C</t>
@@ -13057,7 +13063,7 @@
       <c r="L197" s="10" t="inlineStr"/>
       <c r="M197" s="10" t="inlineStr"/>
     </row>
-    <row r="198" ht="230" customHeight="1">
+    <row r="198" ht="270" customHeight="1">
       <c r="A198" s="6" t="inlineStr">
         <is>
           <t>froide C</t>
@@ -13121,7 +13127,7 @@
       <c r="L198" s="10" t="inlineStr"/>
       <c r="M198" s="10" t="inlineStr"/>
     </row>
-    <row r="199" ht="230" customHeight="1">
+    <row r="199" ht="270" customHeight="1">
       <c r="A199" s="6" t="inlineStr">
         <is>
           <t>froide C</t>
@@ -13185,7 +13191,7 @@
       <c r="L199" s="10" t="inlineStr"/>
       <c r="M199" s="10" t="inlineStr"/>
     </row>
-    <row r="200" ht="230" customHeight="1">
+    <row r="200" ht="270" customHeight="1">
       <c r="A200" s="6" t="inlineStr">
         <is>
           <t>froide C</t>
@@ -13249,7 +13255,7 @@
       <c r="L200" s="10" t="inlineStr"/>
       <c r="M200" s="10" t="inlineStr"/>
     </row>
-    <row r="201" ht="230" customHeight="1">
+    <row r="201" ht="270" customHeight="1">
       <c r="A201" s="6" t="inlineStr">
         <is>
           <t>froide C</t>
@@ -13313,7 +13319,7 @@
       <c r="L201" s="10" t="inlineStr"/>
       <c r="M201" s="10" t="inlineStr"/>
     </row>
-    <row r="202" ht="230" customHeight="1">
+    <row r="202" ht="270" customHeight="1">
       <c r="A202" s="6" t="inlineStr">
         <is>
           <t>froide C</t>
@@ -13377,7 +13383,7 @@
       <c r="L202" s="10" t="inlineStr"/>
       <c r="M202" s="10" t="inlineStr"/>
     </row>
-    <row r="203" ht="230" customHeight="1">
+    <row r="203" ht="270" customHeight="1">
       <c r="A203" s="6" t="inlineStr">
         <is>
           <t>froide C</t>
@@ -13441,7 +13447,7 @@
       <c r="L203" s="10" t="inlineStr"/>
       <c r="M203" s="10" t="inlineStr"/>
     </row>
-    <row r="204" ht="230" customHeight="1">
+    <row r="204" ht="270" customHeight="1">
       <c r="A204" s="6" t="inlineStr">
         <is>
           <t>froide C</t>
@@ -13496,7 +13502,7 @@
       <c r="L204" s="10" t="inlineStr"/>
       <c r="M204" s="10" t="inlineStr"/>
     </row>
-    <row r="205" ht="230" customHeight="1">
+    <row r="205" ht="270" customHeight="1">
       <c r="A205" s="6" t="inlineStr">
         <is>
           <t>froide C</t>
@@ -13560,7 +13566,7 @@
       <c r="L205" s="10" t="inlineStr"/>
       <c r="M205" s="10" t="inlineStr"/>
     </row>
-    <row r="206" ht="230" customHeight="1">
+    <row r="206" ht="270" customHeight="1">
       <c r="A206" s="6" t="inlineStr">
         <is>
           <t>froide C</t>
@@ -13624,7 +13630,7 @@
       <c r="L206" s="10" t="inlineStr"/>
       <c r="M206" s="10" t="inlineStr"/>
     </row>
-    <row r="207" ht="230" customHeight="1">
+    <row r="207" ht="270" customHeight="1">
       <c r="A207" s="6" t="inlineStr">
         <is>
           <t>froide C</t>
@@ -13688,7 +13694,7 @@
       <c r="L207" s="10" t="inlineStr"/>
       <c r="M207" s="10" t="inlineStr"/>
     </row>
-    <row r="208" ht="230" customHeight="1">
+    <row r="208" ht="270" customHeight="1">
       <c r="A208" s="6" t="inlineStr">
         <is>
           <t>froide C</t>
@@ -13752,7 +13758,7 @@
       <c r="L208" s="10" t="inlineStr"/>
       <c r="M208" s="10" t="inlineStr"/>
     </row>
-    <row r="209" ht="230" customHeight="1">
+    <row r="209" ht="270" customHeight="1">
       <c r="A209" s="6" t="inlineStr">
         <is>
           <t>froide C</t>
@@ -13816,7 +13822,7 @@
       <c r="L209" s="10" t="inlineStr"/>
       <c r="M209" s="10" t="inlineStr"/>
     </row>
-    <row r="210" ht="230" customHeight="1">
+    <row r="210" ht="270" customHeight="1">
       <c r="A210" s="6" t="inlineStr">
         <is>
           <t>froide C</t>
@@ -13871,7 +13877,7 @@
       <c r="L210" s="10" t="inlineStr"/>
       <c r="M210" s="10" t="inlineStr"/>
     </row>
-    <row r="211" ht="230" customHeight="1">
+    <row r="211" ht="270" customHeight="1">
       <c r="A211" s="6" t="inlineStr">
         <is>
           <t>froide C</t>
@@ -13935,7 +13941,7 @@
       <c r="L211" s="10" t="inlineStr"/>
       <c r="M211" s="10" t="inlineStr"/>
     </row>
-    <row r="212" ht="230" customHeight="1">
+    <row r="212" ht="270" customHeight="1">
       <c r="A212" s="6" t="inlineStr">
         <is>
           <t>froide C</t>
@@ -13999,7 +14005,7 @@
       <c r="L212" s="10" t="inlineStr"/>
       <c r="M212" s="10" t="inlineStr"/>
     </row>
-    <row r="213" ht="230" customHeight="1">
+    <row r="213" ht="270" customHeight="1">
       <c r="A213" s="6" t="inlineStr">
         <is>
           <t>froide C</t>
@@ -14063,7 +14069,7 @@
       <c r="L213" s="10" t="inlineStr"/>
       <c r="M213" s="10" t="inlineStr"/>
     </row>
-    <row r="214" ht="230" customHeight="1">
+    <row r="214" ht="270" customHeight="1">
       <c r="A214" s="6" t="inlineStr">
         <is>
           <t>froide C</t>
@@ -14127,7 +14133,7 @@
       <c r="L214" s="10" t="inlineStr"/>
       <c r="M214" s="10" t="inlineStr"/>
     </row>
-    <row r="215" ht="230" customHeight="1">
+    <row r="215" ht="270" customHeight="1">
       <c r="A215" s="6" t="inlineStr">
         <is>
           <t>froide C</t>
@@ -14191,7 +14197,7 @@
       <c r="L215" s="10" t="inlineStr"/>
       <c r="M215" s="10" t="inlineStr"/>
     </row>
-    <row r="216" ht="230" customHeight="1">
+    <row r="216" ht="270" customHeight="1">
       <c r="A216" s="6" t="inlineStr">
         <is>
           <t>froide C</t>
@@ -14255,7 +14261,7 @@
       <c r="L216" s="10" t="inlineStr"/>
       <c r="M216" s="10" t="inlineStr"/>
     </row>
-    <row r="217" ht="230" customHeight="1">
+    <row r="217" ht="270" customHeight="1">
       <c r="A217" s="6" t="inlineStr">
         <is>
           <t>froide C</t>
@@ -14319,7 +14325,7 @@
       <c r="L217" s="10" t="inlineStr"/>
       <c r="M217" s="10" t="inlineStr"/>
     </row>
-    <row r="218" ht="230" customHeight="1">
+    <row r="218" ht="270" customHeight="1">
       <c r="A218" s="6" t="inlineStr">
         <is>
           <t>froide C</t>
@@ -14383,7 +14389,7 @@
       <c r="L218" s="10" t="inlineStr"/>
       <c r="M218" s="10" t="inlineStr"/>
     </row>
-    <row r="219" ht="230" customHeight="1">
+    <row r="219" ht="270" customHeight="1">
       <c r="A219" s="6" t="inlineStr">
         <is>
           <t>froide C</t>
@@ -14447,7 +14453,7 @@
       <c r="L219" s="10" t="inlineStr"/>
       <c r="M219" s="10" t="inlineStr"/>
     </row>
-    <row r="220" ht="230" customHeight="1">
+    <row r="220" ht="270" customHeight="1">
       <c r="A220" s="6" t="inlineStr">
         <is>
           <t>froide C</t>
@@ -14511,7 +14517,7 @@
       <c r="L220" s="10" t="inlineStr"/>
       <c r="M220" s="10" t="inlineStr"/>
     </row>
-    <row r="221" ht="230" customHeight="1">
+    <row r="221" ht="270" customHeight="1">
       <c r="A221" s="6" t="inlineStr">
         <is>
           <t>froide C</t>
@@ -14575,7 +14581,7 @@
       <c r="L221" s="10" t="inlineStr"/>
       <c r="M221" s="10" t="inlineStr"/>
     </row>
-    <row r="222" ht="230" customHeight="1">
+    <row r="222" ht="270" customHeight="1">
       <c r="A222" s="6" t="inlineStr">
         <is>
           <t>froide C</t>
@@ -14639,7 +14645,7 @@
       <c r="L222" s="10" t="inlineStr"/>
       <c r="M222" s="10" t="inlineStr"/>
     </row>
-    <row r="223" ht="230" customHeight="1">
+    <row r="223" ht="270" customHeight="1">
       <c r="A223" s="6" t="inlineStr">
         <is>
           <t>froide C</t>
@@ -14703,7 +14709,7 @@
       <c r="L223" s="10" t="inlineStr"/>
       <c r="M223" s="10" t="inlineStr"/>
     </row>
-    <row r="224" ht="230" customHeight="1">
+    <row r="224" ht="270" customHeight="1">
       <c r="A224" s="6" t="inlineStr">
         <is>
           <t>froide C</t>
@@ -14767,7 +14773,7 @@
       <c r="L224" s="10" t="inlineStr"/>
       <c r="M224" s="10" t="inlineStr"/>
     </row>
-    <row r="225" ht="230" customHeight="1">
+    <row r="225" ht="270" customHeight="1">
       <c r="A225" s="6" t="inlineStr">
         <is>
           <t>froide C</t>
@@ -14831,7 +14837,7 @@
       <c r="L225" s="10" t="inlineStr"/>
       <c r="M225" s="10" t="inlineStr"/>
     </row>
-    <row r="226" ht="230" customHeight="1">
+    <row r="226" ht="270" customHeight="1">
       <c r="A226" s="6" t="inlineStr">
         <is>
           <t>froide C</t>
@@ -14895,7 +14901,7 @@
       <c r="L226" s="10" t="inlineStr"/>
       <c r="M226" s="10" t="inlineStr"/>
     </row>
-    <row r="227" ht="230" customHeight="1">
+    <row r="227" ht="270" customHeight="1">
       <c r="A227" s="6" t="inlineStr">
         <is>
           <t>froide C</t>
@@ -14959,7 +14965,7 @@
       <c r="L227" s="10" t="inlineStr"/>
       <c r="M227" s="10" t="inlineStr"/>
     </row>
-    <row r="228" ht="230" customHeight="1">
+    <row r="228" ht="270" customHeight="1">
       <c r="A228" s="6" t="inlineStr">
         <is>
           <t>froide C</t>
@@ -15023,7 +15029,7 @@
       <c r="L228" s="10" t="inlineStr"/>
       <c r="M228" s="10" t="inlineStr"/>
     </row>
-    <row r="229" ht="230" customHeight="1">
+    <row r="229" ht="270" customHeight="1">
       <c r="A229" s="6" t="inlineStr">
         <is>
           <t>froide C</t>
@@ -15087,7 +15093,7 @@
       <c r="L229" s="10" t="inlineStr"/>
       <c r="M229" s="10" t="inlineStr"/>
     </row>
-    <row r="230" ht="230" customHeight="1">
+    <row r="230" ht="270" customHeight="1">
       <c r="A230" s="6" t="inlineStr">
         <is>
           <t>froide C</t>
@@ -15151,7 +15157,7 @@
       <c r="L230" s="10" t="inlineStr"/>
       <c r="M230" s="10" t="inlineStr"/>
     </row>
-    <row r="231" ht="230" customHeight="1">
+    <row r="231" ht="270" customHeight="1">
       <c r="A231" s="6" t="inlineStr">
         <is>
           <t>froide C</t>
@@ -15215,7 +15221,7 @@
       <c r="L231" s="10" t="inlineStr"/>
       <c r="M231" s="10" t="inlineStr"/>
     </row>
-    <row r="232" ht="230" customHeight="1">
+    <row r="232" ht="270" customHeight="1">
       <c r="A232" s="6" t="inlineStr">
         <is>
           <t>froide C</t>
@@ -15279,7 +15285,7 @@
       <c r="L232" s="10" t="inlineStr"/>
       <c r="M232" s="10" t="inlineStr"/>
     </row>
-    <row r="233" ht="230" customHeight="1">
+    <row r="233" ht="270" customHeight="1">
       <c r="A233" s="6" t="inlineStr">
         <is>
           <t>froide C</t>
@@ -15343,7 +15349,7 @@
       <c r="L233" s="10" t="inlineStr"/>
       <c r="M233" s="10" t="inlineStr"/>
     </row>
-    <row r="234" ht="230" customHeight="1">
+    <row r="234" ht="270" customHeight="1">
       <c r="A234" s="6" t="inlineStr">
         <is>
           <t>froide C</t>
@@ -15407,7 +15413,7 @@
       <c r="L234" s="10" t="inlineStr"/>
       <c r="M234" s="10" t="inlineStr"/>
     </row>
-    <row r="235" ht="230" customHeight="1">
+    <row r="235" ht="270" customHeight="1">
       <c r="A235" s="6" t="inlineStr">
         <is>
           <t>froide C</t>
@@ -15471,7 +15477,7 @@
       <c r="L235" s="10" t="inlineStr"/>
       <c r="M235" s="10" t="inlineStr"/>
     </row>
-    <row r="236" ht="230" customHeight="1">
+    <row r="236" ht="270" customHeight="1">
       <c r="A236" s="6" t="inlineStr">
         <is>
           <t>froide C</t>
@@ -15535,7 +15541,7 @@
       <c r="L236" s="10" t="inlineStr"/>
       <c r="M236" s="10" t="inlineStr"/>
     </row>
-    <row r="237" ht="230" customHeight="1">
+    <row r="237" ht="270" customHeight="1">
       <c r="A237" s="6" t="inlineStr">
         <is>
           <t>froide C</t>
@@ -15599,7 +15605,7 @@
       <c r="L237" s="10" t="inlineStr"/>
       <c r="M237" s="10" t="inlineStr"/>
     </row>
-    <row r="238" ht="230" customHeight="1">
+    <row r="238" ht="270" customHeight="1">
       <c r="A238" s="6" t="inlineStr">
         <is>
           <t>froide C</t>
@@ -15663,7 +15669,7 @@
       <c r="L238" s="10" t="inlineStr"/>
       <c r="M238" s="10" t="inlineStr"/>
     </row>
-    <row r="239" ht="230" customHeight="1">
+    <row r="239" ht="270" customHeight="1">
       <c r="A239" s="6" t="inlineStr">
         <is>
           <t>froide C</t>
@@ -15727,7 +15733,7 @@
       <c r="L239" s="10" t="inlineStr"/>
       <c r="M239" s="10" t="inlineStr"/>
     </row>
-    <row r="240" ht="230" customHeight="1">
+    <row r="240" ht="270" customHeight="1">
       <c r="A240" s="6" t="inlineStr">
         <is>
           <t>froide C</t>
@@ -15791,7 +15797,7 @@
       <c r="L240" s="10" t="inlineStr"/>
       <c r="M240" s="10" t="inlineStr"/>
     </row>
-    <row r="241" ht="230" customHeight="1">
+    <row r="241" ht="270" customHeight="1">
       <c r="A241" s="6" t="inlineStr">
         <is>
           <t>froide C</t>
@@ -15855,7 +15861,7 @@
       <c r="L241" s="10" t="inlineStr"/>
       <c r="M241" s="10" t="inlineStr"/>
     </row>
-    <row r="242" ht="230" customHeight="1">
+    <row r="242" ht="270" customHeight="1">
       <c r="A242" s="6" t="inlineStr">
         <is>
           <t>froide C</t>
@@ -15919,7 +15925,7 @@
       <c r="L242" s="10" t="inlineStr"/>
       <c r="M242" s="10" t="inlineStr"/>
     </row>
-    <row r="243" ht="230" customHeight="1">
+    <row r="243" ht="270" customHeight="1">
       <c r="A243" s="6" t="inlineStr">
         <is>
           <t>froide C</t>
@@ -15983,7 +15989,7 @@
       <c r="L243" s="10" t="inlineStr"/>
       <c r="M243" s="10" t="inlineStr"/>
     </row>
-    <row r="244" ht="230" customHeight="1">
+    <row r="244" ht="270" customHeight="1">
       <c r="A244" s="6" t="inlineStr">
         <is>
           <t>froide C</t>
@@ -16047,7 +16053,7 @@
       <c r="L244" s="10" t="inlineStr"/>
       <c r="M244" s="10" t="inlineStr"/>
     </row>
-    <row r="245" ht="230" customHeight="1">
+    <row r="245" ht="270" customHeight="1">
       <c r="A245" s="6" t="inlineStr">
         <is>
           <t>froide C</t>
@@ -16111,7 +16117,7 @@
       <c r="L245" s="10" t="inlineStr"/>
       <c r="M245" s="10" t="inlineStr"/>
     </row>
-    <row r="246" ht="230" customHeight="1">
+    <row r="246" ht="270" customHeight="1">
       <c r="A246" s="6" t="inlineStr">
         <is>
           <t>froide C</t>
@@ -16175,7 +16181,7 @@
       <c r="L246" s="10" t="inlineStr"/>
       <c r="M246" s="10" t="inlineStr"/>
     </row>
-    <row r="247" ht="230" customHeight="1">
+    <row r="247" ht="270" customHeight="1">
       <c r="A247" s="6" t="inlineStr">
         <is>
           <t>froide C</t>
@@ -16239,7 +16245,7 @@
       <c r="L247" s="10" t="inlineStr"/>
       <c r="M247" s="10" t="inlineStr"/>
     </row>
-    <row r="248" ht="230" customHeight="1">
+    <row r="248" ht="270" customHeight="1">
       <c r="A248" s="6" t="inlineStr">
         <is>
           <t>froide C</t>
@@ -16303,7 +16309,7 @@
       <c r="L248" s="10" t="inlineStr"/>
       <c r="M248" s="10" t="inlineStr"/>
     </row>
-    <row r="249" ht="230" customHeight="1">
+    <row r="249" ht="270" customHeight="1">
       <c r="A249" s="6" t="inlineStr">
         <is>
           <t>froide C</t>
@@ -16367,7 +16373,7 @@
       <c r="L249" s="10" t="inlineStr"/>
       <c r="M249" s="10" t="inlineStr"/>
     </row>
-    <row r="250" ht="230" customHeight="1">
+    <row r="250" ht="270" customHeight="1">
       <c r="A250" s="6" t="inlineStr">
         <is>
           <t>froide C</t>
@@ -16431,7 +16437,7 @@
       <c r="L250" s="10" t="inlineStr"/>
       <c r="M250" s="10" t="inlineStr"/>
     </row>
-    <row r="251" ht="230" customHeight="1">
+    <row r="251" ht="270" customHeight="1">
       <c r="A251" s="6" t="inlineStr">
         <is>
           <t>froide C</t>
@@ -16495,7 +16501,7 @@
       <c r="L251" s="10" t="inlineStr"/>
       <c r="M251" s="10" t="inlineStr"/>
     </row>
-    <row r="252" ht="230" customHeight="1">
+    <row r="252" ht="270" customHeight="1">
       <c r="A252" s="6" t="inlineStr">
         <is>
           <t>froide C</t>
@@ -16559,7 +16565,7 @@
       <c r="L252" s="10" t="inlineStr"/>
       <c r="M252" s="10" t="inlineStr"/>
     </row>
-    <row r="253" ht="230" customHeight="1">
+    <row r="253" ht="270" customHeight="1">
       <c r="A253" s="6" t="inlineStr">
         <is>
           <t>froide C</t>
@@ -16623,7 +16629,7 @@
       <c r="L253" s="10" t="inlineStr"/>
       <c r="M253" s="10" t="inlineStr"/>
     </row>
-    <row r="254" ht="230" customHeight="1">
+    <row r="254" ht="270" customHeight="1">
       <c r="A254" s="6" t="inlineStr">
         <is>
           <t>froide C</t>
@@ -16687,7 +16693,7 @@
       <c r="L254" s="10" t="inlineStr"/>
       <c r="M254" s="10" t="inlineStr"/>
     </row>
-    <row r="255" ht="230" customHeight="1">
+    <row r="255" ht="270" customHeight="1">
       <c r="A255" s="6" t="inlineStr">
         <is>
           <t>froide C</t>
@@ -16751,7 +16757,7 @@
       <c r="L255" s="10" t="inlineStr"/>
       <c r="M255" s="10" t="inlineStr"/>
     </row>
-    <row r="256" ht="230" customHeight="1">
+    <row r="256" ht="270" customHeight="1">
       <c r="A256" s="6" t="inlineStr">
         <is>
           <t>froide A</t>
@@ -16800,12 +16806,13 @@
       <c r="J256" s="9" t="inlineStr">
         <is>
           <t>Bonjour Jean-Michel Leprince,
+Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de
+Québec dont l'atelier est dans Limoilou.
 Vous couvrez l'asclépiade depuis au moins 2014 : le Téléjournal, la soie d'Amérique partie
 sur l'Everest, le pouvoir absorbant de la fibre sur les hydrocarbures, le lien avec le
 monarque. Vous avez suivi cette histoire plus longtemps que la plupart des entreprises qui
 s'y sont essayées.
-On est l'entreprise qui a démarré après la chute de la première filière. Six ans plus tard,
-on achète encore de l'asclépiade québécoise et on transforme l'isolant nous-mêmes à
+On a démarré après la chute de la première filière. Six ans plus tard, on achète encore de l'asclépiade québécoise et on transforme l'isolant nous-mêmes à
 Limoilou. Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques
 par la culture de l'asclépiade.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
@@ -16821,7 +16828,7 @@
       <c r="L256" s="10" t="inlineStr"/>
       <c r="M256" s="10" t="inlineStr"/>
     </row>
-    <row r="257" ht="230" customHeight="1">
+    <row r="257" ht="270" customHeight="1">
       <c r="A257" s="6" t="inlineStr">
         <is>
           <t>froide B</t>
@@ -16866,10 +16873,11 @@
       <c r="J257" s="9" t="inlineStr">
         <is>
           <t>Bonjour Antoine Stab,
+Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de
+Québec dont l'atelier est dans Limoilou.
 Vous aviez écrit sur le soyer du Québec dans Espaces en février 2015, à l'époque où la fibre
 devait remplacer le duvet.
-On est l'entreprise qui a démarré après la chute de cette première filière. Six ans plus
-tard, on achète encore de l'asclépiade québécoise, on transforme l'isolant nous-mêmes, et il
+On a démarré après la chute de cette première filière. Six ans plus tard, on achète encore de l'asclépiade québécoise, on transforme l'isolant nous-mêmes, et il
 existe maintenant un manteau à inserts d'asclépiade amovibles autour de 300 $.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.

</xml_diff>

<commit_message>
Retire « invité disponible » et met l'asclépiade en tête des objets
Gabriel a retenu la formule « L'asclépiade s'en va à Dragons' Den le
17 septembre! », qui passe de 54 à 149 contacts.

La ligne de partage n'est plus l'angle mais ce que la personne sait déjà:
« nous serons diffusés » suppose qu'elle sait qui est « nous », ce qui n'est
vrai que pour la liste chaude et les journalistes d'affaires. Partout ailleurs,
c'est la plante qui accroche.

Le suffixe « — invité disponible » disparaît des objets de radio et télé; la
disponibilité reste dans le corps du courriel, où elle a sa place.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015pjLsGPzf1MX1JC7QiKGGk
</commit_message>
<xml_diff>
--- a/communique-dragons/Lasclay_brouillons_a_editer.xlsx
+++ b/communique-dragons/Lasclay_brouillons_a_editer.xlsx
@@ -508,7 +508,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Version 4 — les objets</t>
+          <t>Version 5 — les objets, suite</t>
         </is>
       </c>
       <c r="B1" s="2" t="inlineStr"/>
@@ -520,66 +520,66 @@
     <row r="3" ht="56" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>Le modèle</t>
+          <t>« Invité disponible »</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>« Nous serons diffusés à Dragons' Den le 17 septembre! » L'objet annonce la nouvelle, avec la date, et il a le droit d'être content.</t>
+          <t>Retiré. Zéro occurrence.</t>
         </is>
       </c>
     </row>
     <row r="4" ht="56" customHeight="1">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>Ce qu'ils étaient</t>
+          <t>L'asclépiade en tête</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>« Le monarque, l'asclépiade, et l'idée qu'il faut la rendre payante ». Un titre d'essai, pas un objet de courriel. Et sans accents.</t>
+          <t>Tu as aimé la formule, alors elle passe de 54 à 149 contacts. « Nous serons diffusés » suppose que la personne sait déjà qui est « nous » : ça ne vaut que pour ceux qui nous connaissent, la liste chaude et les journalistes d'affaires.</t>
         </is>
       </c>
     </row>
     <row r="5" ht="56" customHeight="1">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t>Quatre variantes</t>
+          <t>Les trois objets</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>A, B, E, G : Nous serons diffusés à Dragons' Den le 17 septembre!  |  C, F, J : L'asclépiade s'en va à Dragons' Den le 17 septembre!  |  D : L'asclépiade et les monarques à Dragons' Den le 17 septembre!  |  I : … — invité disponible.</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="56" customHeight="1">
-      <c r="A6" s="3" t="inlineStr">
-        <is>
-          <t>Pourquoi pas un seul</t>
-        </is>
-      </c>
-      <c r="B6" s="2" t="inlineStr">
-        <is>
-          <t>253 courriels avec exactement la même ligne d'objet se comportent comme du publipostage aux yeux des filtres, et « l'asclépiade s'en va » parle plus à un journaliste agricole qu'à un chroniqueur d'affaires.</t>
-        </is>
-      </c>
+          <t>149 : L'asclépiade s'en va à Dragons' Den le 17 septembre!  |  59 : Nous serons diffusés à Dragons' Den le 17 septembre!  |  45 : L'asclépiade et les monarques à Dragons' Den le 17 septembre!</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr"/>
+      <c r="B6" s="2" t="inlineStr"/>
     </row>
     <row r="7">
-      <c r="A7" s="2" t="inlineStr"/>
+      <c r="A7" s="1" t="inlineStr">
+        <is>
+          <t>Les versions précédentes</t>
+        </is>
+      </c>
       <c r="B7" s="2" t="inlineStr"/>
     </row>
     <row r="8">
-      <c r="A8" s="1" t="inlineStr">
-        <is>
-          <t>Rappel des versions précédentes</t>
-        </is>
-      </c>
+      <c r="A8" s="2" t="inlineStr"/>
       <c r="B8" s="2" t="inlineStr"/>
     </row>
-    <row r="9">
-      <c r="A9" s="2" t="inlineStr"/>
-      <c r="B9" s="2" t="inlineStr"/>
+    <row r="9" ht="56" customHeight="1">
+      <c r="A9" s="3" t="inlineStr">
+        <is>
+          <t>v4</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>Objets refaits : de « titre d'essai » à annonce datée.</t>
+        </is>
+      </c>
     </row>
     <row r="10" ht="56" customHeight="1">
       <c r="A10" s="3" t="inlineStr">
@@ -589,7 +589,7 @@
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>Présentation complète en tête des courriels froids, « pourquoi vous » explicite, fausse accroche régionale retirée.</t>
+          <t>Présentation complète en tête des courriels froids, « pourquoi vous » explicite.</t>
         </is>
       </c>
     </row>
@@ -601,7 +601,7 @@
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>Registre de Gabriel : plus d'excuses sur le virage, plus de mise en garde sur les monarques, plus de rappel de confidentialité.</t>
+          <t>Registre de Gabriel : plus d'excuses, plus de mise en garde, plus de rappel de confidentialité.</t>
         </is>
       </c>
     </row>
@@ -752,7 +752,7 @@
       </c>
       <c r="K1" s="4" t="inlineStr">
         <is>
-          <t>Brouillon v4</t>
+          <t>Brouillon v5</t>
         </is>
       </c>
       <c r="L1" s="4" t="inlineStr">
@@ -1024,7 +1024,7 @@
       </c>
       <c r="J5" s="9" t="inlineStr">
         <is>
-          <t>Nous serons diffusés à Dragons' Den le 17 septembre — invité disponible</t>
+          <t>L'asclépiade s'en va à Dragons' Den le 17 septembre!</t>
         </is>
       </c>
       <c r="K5" s="10" t="inlineStr">
@@ -1275,7 +1275,7 @@
       </c>
       <c r="J9" s="9" t="inlineStr">
         <is>
-          <t>Nous serons diffusés à Dragons' Den le 17 septembre — invité disponible</t>
+          <t>L'asclépiade s'en va à Dragons' Den le 17 septembre!</t>
         </is>
       </c>
       <c r="K9" s="10" t="inlineStr">
@@ -1716,7 +1716,7 @@
       </c>
       <c r="J16" s="9" t="inlineStr">
         <is>
-          <t>Nous serons diffusés à Dragons' Den le 17 septembre — invité disponible</t>
+          <t>L'asclépiade s'en va à Dragons' Den le 17 septembre!</t>
         </is>
       </c>
       <c r="K16" s="10" t="inlineStr">
@@ -3237,7 +3237,7 @@
       </c>
       <c r="J41" s="9" t="inlineStr">
         <is>
-          <t>Nous serons diffusés à Dragons' Den le 17 septembre!</t>
+          <t>L'asclépiade s'en va à Dragons' Den le 17 septembre!</t>
         </is>
       </c>
       <c r="K41" s="10" t="inlineStr">
@@ -3306,7 +3306,7 @@
       </c>
       <c r="J42" s="9" t="inlineStr">
         <is>
-          <t>Nous serons diffusés à Dragons' Den le 17 septembre!</t>
+          <t>L'asclépiade s'en va à Dragons' Den le 17 septembre!</t>
         </is>
       </c>
       <c r="K42" s="10" t="inlineStr">
@@ -3444,7 +3444,7 @@
       </c>
       <c r="J44" s="9" t="inlineStr">
         <is>
-          <t>Nous serons diffusés à Dragons' Den le 17 septembre!</t>
+          <t>L'asclépiade s'en va à Dragons' Den le 17 septembre!</t>
         </is>
       </c>
       <c r="K44" s="10" t="inlineStr">
@@ -3651,7 +3651,7 @@
       </c>
       <c r="J47" s="9" t="inlineStr">
         <is>
-          <t>Nous serons diffusés à Dragons' Den le 17 septembre!</t>
+          <t>L'asclépiade s'en va à Dragons' Den le 17 septembre!</t>
         </is>
       </c>
       <c r="K47" s="10" t="inlineStr">
@@ -3720,7 +3720,7 @@
       </c>
       <c r="J48" s="9" t="inlineStr">
         <is>
-          <t>Nous serons diffusés à Dragons' Den le 17 septembre — invité disponible</t>
+          <t>L'asclépiade s'en va à Dragons' Den le 17 septembre!</t>
         </is>
       </c>
       <c r="K48" s="10" t="inlineStr">
@@ -3789,7 +3789,7 @@
       </c>
       <c r="J49" s="9" t="inlineStr">
         <is>
-          <t>Nous serons diffusés à Dragons' Den le 17 septembre!</t>
+          <t>L'asclépiade s'en va à Dragons' Den le 17 septembre!</t>
         </is>
       </c>
       <c r="K49" s="10" t="inlineStr">
@@ -3927,7 +3927,7 @@
       </c>
       <c r="J51" s="9" t="inlineStr">
         <is>
-          <t>Nous serons diffusés à Dragons' Den le 17 septembre!</t>
+          <t>L'asclépiade s'en va à Dragons' Den le 17 septembre!</t>
         </is>
       </c>
       <c r="K51" s="10" t="inlineStr">
@@ -4134,7 +4134,7 @@
       </c>
       <c r="J54" s="9" t="inlineStr">
         <is>
-          <t>Nous serons diffusés à Dragons' Den le 17 septembre!</t>
+          <t>L'asclépiade s'en va à Dragons' Den le 17 septembre!</t>
         </is>
       </c>
       <c r="K54" s="10" t="inlineStr">
@@ -4341,7 +4341,7 @@
       </c>
       <c r="J57" s="9" t="inlineStr">
         <is>
-          <t>Nous serons diffusés à Dragons' Den le 17 septembre!</t>
+          <t>L'asclépiade s'en va à Dragons' Den le 17 septembre!</t>
         </is>
       </c>
       <c r="K57" s="10" t="inlineStr">
@@ -4553,7 +4553,7 @@
       </c>
       <c r="J60" s="9" t="inlineStr">
         <is>
-          <t>Nous serons diffusés à Dragons' Den le 17 septembre — invité disponible</t>
+          <t>L'asclépiade s'en va à Dragons' Den le 17 septembre!</t>
         </is>
       </c>
       <c r="K60" s="10" t="inlineStr">
@@ -4622,7 +4622,7 @@
       </c>
       <c r="J61" s="9" t="inlineStr">
         <is>
-          <t>Nous serons diffusés à Dragons' Den le 17 septembre!</t>
+          <t>L'asclépiade s'en va à Dragons' Den le 17 septembre!</t>
         </is>
       </c>
       <c r="K61" s="10" t="inlineStr">
@@ -4760,7 +4760,7 @@
       </c>
       <c r="J63" s="9" t="inlineStr">
         <is>
-          <t>Nous serons diffusés à Dragons' Den le 17 septembre — invité disponible</t>
+          <t>L'asclépiade s'en va à Dragons' Den le 17 septembre!</t>
         </is>
       </c>
       <c r="K63" s="10" t="inlineStr">
@@ -4829,7 +4829,7 @@
       </c>
       <c r="J64" s="9" t="inlineStr">
         <is>
-          <t>Nous serons diffusés à Dragons' Den le 17 septembre!</t>
+          <t>L'asclépiade s'en va à Dragons' Den le 17 septembre!</t>
         </is>
       </c>
       <c r="K64" s="10" t="inlineStr">
@@ -4967,7 +4967,7 @@
       </c>
       <c r="J66" s="9" t="inlineStr">
         <is>
-          <t>Nous serons diffusés à Dragons' Den le 17 septembre — invité disponible</t>
+          <t>L'asclépiade s'en va à Dragons' Den le 17 septembre!</t>
         </is>
       </c>
       <c r="K66" s="10" t="inlineStr">
@@ -5243,7 +5243,7 @@
       </c>
       <c r="J70" s="9" t="inlineStr">
         <is>
-          <t>Nous serons diffusés à Dragons' Den le 17 septembre — invité disponible</t>
+          <t>L'asclépiade s'en va à Dragons' Den le 17 septembre!</t>
         </is>
       </c>
       <c r="K70" s="10" t="inlineStr">
@@ -5519,7 +5519,7 @@
       </c>
       <c r="J74" s="9" t="inlineStr">
         <is>
-          <t>Nous serons diffusés à Dragons' Den le 17 septembre — invité disponible</t>
+          <t>L'asclépiade s'en va à Dragons' Den le 17 septembre!</t>
         </is>
       </c>
       <c r="K74" s="10" t="inlineStr">
@@ -5657,7 +5657,7 @@
       </c>
       <c r="J76" s="9" t="inlineStr">
         <is>
-          <t>Nous serons diffusés à Dragons' Den le 17 septembre — invité disponible</t>
+          <t>L'asclépiade s'en va à Dragons' Den le 17 septembre!</t>
         </is>
       </c>
       <c r="K76" s="10" t="inlineStr">
@@ -5726,7 +5726,7 @@
       </c>
       <c r="J77" s="9" t="inlineStr">
         <is>
-          <t>Nous serons diffusés à Dragons' Den le 17 septembre!</t>
+          <t>L'asclépiade s'en va à Dragons' Den le 17 septembre!</t>
         </is>
       </c>
       <c r="K77" s="10" t="inlineStr">
@@ -6353,7 +6353,7 @@
       </c>
       <c r="J86" s="9" t="inlineStr">
         <is>
-          <t>Nous serons diffusés à Dragons' Den le 17 septembre — invité disponible</t>
+          <t>L'asclépiade s'en va à Dragons' Den le 17 septembre!</t>
         </is>
       </c>
       <c r="K86" s="10" t="inlineStr">
@@ -6629,7 +6629,7 @@
       </c>
       <c r="J90" s="9" t="inlineStr">
         <is>
-          <t>Nous serons diffusés à Dragons' Den le 17 septembre — invité disponible</t>
+          <t>L'asclépiade s'en va à Dragons' Den le 17 septembre!</t>
         </is>
       </c>
       <c r="K90" s="10" t="inlineStr">
@@ -6698,7 +6698,7 @@
       </c>
       <c r="J91" s="9" t="inlineStr">
         <is>
-          <t>Nous serons diffusés à Dragons' Den le 17 septembre!</t>
+          <t>L'asclépiade s'en va à Dragons' Den le 17 septembre!</t>
         </is>
       </c>
       <c r="K91" s="10" t="inlineStr">
@@ -7319,7 +7319,7 @@
       </c>
       <c r="J100" s="9" t="inlineStr">
         <is>
-          <t>Nous serons diffusés à Dragons' Den le 17 septembre!</t>
+          <t>L'asclépiade s'en va à Dragons' Den le 17 septembre!</t>
         </is>
       </c>
       <c r="K100" s="10" t="inlineStr">
@@ -7388,7 +7388,7 @@
       </c>
       <c r="J101" s="9" t="inlineStr">
         <is>
-          <t>Nous serons diffusés à Dragons' Den le 17 septembre!</t>
+          <t>L'asclépiade s'en va à Dragons' Den le 17 septembre!</t>
         </is>
       </c>
       <c r="K101" s="10" t="inlineStr">
@@ -7733,7 +7733,7 @@
       </c>
       <c r="J106" s="9" t="inlineStr">
         <is>
-          <t>Nous serons diffusés à Dragons' Den le 17 septembre — invité disponible</t>
+          <t>L'asclépiade s'en va à Dragons' Den le 17 septembre!</t>
         </is>
       </c>
       <c r="K106" s="10" t="inlineStr">
@@ -7802,7 +7802,7 @@
       </c>
       <c r="J107" s="9" t="inlineStr">
         <is>
-          <t>Nous serons diffusés à Dragons' Den le 17 septembre!</t>
+          <t>L'asclépiade s'en va à Dragons' Den le 17 septembre!</t>
         </is>
       </c>
       <c r="K107" s="10" t="inlineStr">
@@ -8009,7 +8009,7 @@
       </c>
       <c r="J110" s="9" t="inlineStr">
         <is>
-          <t>Nous serons diffusés à Dragons' Den le 17 septembre!</t>
+          <t>L'asclépiade s'en va à Dragons' Den le 17 septembre!</t>
         </is>
       </c>
       <c r="K110" s="10" t="inlineStr">
@@ -8423,7 +8423,7 @@
       </c>
       <c r="J116" s="9" t="inlineStr">
         <is>
-          <t>Nous serons diffusés à Dragons' Den le 17 septembre — invité disponible</t>
+          <t>L'asclépiade s'en va à Dragons' Den le 17 septembre!</t>
         </is>
       </c>
       <c r="K116" s="10" t="inlineStr">
@@ -8492,7 +8492,7 @@
       </c>
       <c r="J117" s="9" t="inlineStr">
         <is>
-          <t>Nous serons diffusés à Dragons' Den le 17 septembre — invité disponible</t>
+          <t>L'asclépiade s'en va à Dragons' Den le 17 septembre!</t>
         </is>
       </c>
       <c r="K117" s="10" t="inlineStr">
@@ -8699,7 +8699,7 @@
       </c>
       <c r="J120" s="9" t="inlineStr">
         <is>
-          <t>Nous serons diffusés à Dragons' Den le 17 septembre!</t>
+          <t>L'asclépiade s'en va à Dragons' Den le 17 septembre!</t>
         </is>
       </c>
       <c r="K120" s="10" t="inlineStr">
@@ -9113,7 +9113,7 @@
       </c>
       <c r="J126" s="9" t="inlineStr">
         <is>
-          <t>Nous serons diffusés à Dragons' Den le 17 septembre!</t>
+          <t>L'asclépiade s'en va à Dragons' Den le 17 septembre!</t>
         </is>
       </c>
       <c r="K126" s="10" t="inlineStr">
@@ -9251,7 +9251,7 @@
       </c>
       <c r="J128" s="9" t="inlineStr">
         <is>
-          <t>Nous serons diffusés à Dragons' Den le 17 septembre!</t>
+          <t>L'asclépiade s'en va à Dragons' Den le 17 septembre!</t>
         </is>
       </c>
       <c r="K128" s="10" t="inlineStr">
@@ -9458,7 +9458,7 @@
       </c>
       <c r="J131" s="9" t="inlineStr">
         <is>
-          <t>Nous serons diffusés à Dragons' Den le 17 septembre!</t>
+          <t>L'asclépiade s'en va à Dragons' Den le 17 septembre!</t>
         </is>
       </c>
       <c r="K131" s="10" t="inlineStr">
@@ -9596,7 +9596,7 @@
       </c>
       <c r="J133" s="9" t="inlineStr">
         <is>
-          <t>Nous serons diffusés à Dragons' Den le 17 septembre!</t>
+          <t>L'asclépiade s'en va à Dragons' Den le 17 septembre!</t>
         </is>
       </c>
       <c r="K133" s="10" t="inlineStr">
@@ -9734,7 +9734,7 @@
       </c>
       <c r="J135" s="9" t="inlineStr">
         <is>
-          <t>Nous serons diffusés à Dragons' Den le 17 septembre — invité disponible</t>
+          <t>L'asclépiade s'en va à Dragons' Den le 17 septembre!</t>
         </is>
       </c>
       <c r="K135" s="10" t="inlineStr">
@@ -10148,7 +10148,7 @@
       </c>
       <c r="J141" s="9" t="inlineStr">
         <is>
-          <t>Nous serons diffusés à Dragons' Den le 17 septembre!</t>
+          <t>L'asclépiade s'en va à Dragons' Den le 17 septembre!</t>
         </is>
       </c>
       <c r="K141" s="10" t="inlineStr">
@@ -10493,7 +10493,7 @@
       </c>
       <c r="J146" s="9" t="inlineStr">
         <is>
-          <t>Nous serons diffusés à Dragons' Den le 17 septembre!</t>
+          <t>L'asclépiade s'en va à Dragons' Den le 17 septembre!</t>
         </is>
       </c>
       <c r="K146" s="10" t="inlineStr">
@@ -10562,7 +10562,7 @@
       </c>
       <c r="J147" s="9" t="inlineStr">
         <is>
-          <t>Nous serons diffusés à Dragons' Den le 17 septembre — invité disponible</t>
+          <t>L'asclépiade s'en va à Dragons' Den le 17 septembre!</t>
         </is>
       </c>
       <c r="K147" s="10" t="inlineStr">
@@ -10700,7 +10700,7 @@
       </c>
       <c r="J149" s="9" t="inlineStr">
         <is>
-          <t>Nous serons diffusés à Dragons' Den le 17 septembre!</t>
+          <t>L'asclépiade s'en va à Dragons' Den le 17 septembre!</t>
         </is>
       </c>
       <c r="K149" s="10" t="inlineStr">
@@ -10838,7 +10838,7 @@
       </c>
       <c r="J151" s="9" t="inlineStr">
         <is>
-          <t>Nous serons diffusés à Dragons' Den le 17 septembre!</t>
+          <t>L'asclépiade s'en va à Dragons' Den le 17 septembre!</t>
         </is>
       </c>
       <c r="K151" s="10" t="inlineStr">
@@ -10907,7 +10907,7 @@
       </c>
       <c r="J152" s="9" t="inlineStr">
         <is>
-          <t>Nous serons diffusés à Dragons' Den le 17 septembre!</t>
+          <t>L'asclépiade s'en va à Dragons' Den le 17 septembre!</t>
         </is>
       </c>
       <c r="K152" s="10" t="inlineStr">
@@ -10976,7 +10976,7 @@
       </c>
       <c r="J153" s="9" t="inlineStr">
         <is>
-          <t>Nous serons diffusés à Dragons' Den le 17 septembre — invité disponible</t>
+          <t>L'asclépiade s'en va à Dragons' Den le 17 septembre!</t>
         </is>
       </c>
       <c r="K153" s="10" t="inlineStr">
@@ -11942,7 +11942,7 @@
       </c>
       <c r="J167" s="9" t="inlineStr">
         <is>
-          <t>Nous serons diffusés à Dragons' Den le 17 septembre!</t>
+          <t>L'asclépiade s'en va à Dragons' Den le 17 septembre!</t>
         </is>
       </c>
       <c r="K167" s="10" t="inlineStr">
@@ -12080,7 +12080,7 @@
       </c>
       <c r="J169" s="9" t="inlineStr">
         <is>
-          <t>Nous serons diffusés à Dragons' Den le 17 septembre — invité disponible</t>
+          <t>L'asclépiade s'en va à Dragons' Den le 17 septembre!</t>
         </is>
       </c>
       <c r="K169" s="10" t="inlineStr">
@@ -12149,7 +12149,7 @@
       </c>
       <c r="J170" s="9" t="inlineStr">
         <is>
-          <t>Nous serons diffusés à Dragons' Den le 17 septembre!</t>
+          <t>L'asclépiade s'en va à Dragons' Den le 17 septembre!</t>
         </is>
       </c>
       <c r="K170" s="10" t="inlineStr">
@@ -12218,7 +12218,7 @@
       </c>
       <c r="J171" s="9" t="inlineStr">
         <is>
-          <t>Nous serons diffusés à Dragons' Den le 17 septembre!</t>
+          <t>L'asclépiade s'en va à Dragons' Den le 17 septembre!</t>
         </is>
       </c>
       <c r="K171" s="10" t="inlineStr">
@@ -12425,7 +12425,7 @@
       </c>
       <c r="J174" s="9" t="inlineStr">
         <is>
-          <t>Nous serons diffusés à Dragons' Den le 17 septembre — invité disponible</t>
+          <t>L'asclépiade s'en va à Dragons' Den le 17 septembre!</t>
         </is>
       </c>
       <c r="K174" s="10" t="inlineStr">
@@ -12494,7 +12494,7 @@
       </c>
       <c r="J175" s="9" t="inlineStr">
         <is>
-          <t>Nous serons diffusés à Dragons' Den le 17 septembre — invité disponible</t>
+          <t>L'asclépiade s'en va à Dragons' Den le 17 septembre!</t>
         </is>
       </c>
       <c r="K175" s="10" t="inlineStr">
@@ -12563,7 +12563,7 @@
       </c>
       <c r="J176" s="9" t="inlineStr">
         <is>
-          <t>Nous serons diffusés à Dragons' Den le 17 septembre!</t>
+          <t>L'asclépiade s'en va à Dragons' Den le 17 septembre!</t>
         </is>
       </c>
       <c r="K176" s="10" t="inlineStr">
@@ -12770,7 +12770,7 @@
       </c>
       <c r="J179" s="9" t="inlineStr">
         <is>
-          <t>Nous serons diffusés à Dragons' Den le 17 septembre — invité disponible</t>
+          <t>L'asclépiade s'en va à Dragons' Den le 17 septembre!</t>
         </is>
       </c>
       <c r="K179" s="10" t="inlineStr">
@@ -12839,7 +12839,7 @@
       </c>
       <c r="J180" s="9" t="inlineStr">
         <is>
-          <t>Nous serons diffusés à Dragons' Den le 17 septembre — invité disponible</t>
+          <t>L'asclépiade s'en va à Dragons' Den le 17 septembre!</t>
         </is>
       </c>
       <c r="K180" s="10" t="inlineStr">
@@ -12908,7 +12908,7 @@
       </c>
       <c r="J181" s="9" t="inlineStr">
         <is>
-          <t>Nous serons diffusés à Dragons' Den le 17 septembre — invité disponible</t>
+          <t>L'asclépiade s'en va à Dragons' Den le 17 septembre!</t>
         </is>
       </c>
       <c r="K181" s="10" t="inlineStr">
@@ -13046,7 +13046,7 @@
       </c>
       <c r="J183" s="9" t="inlineStr">
         <is>
-          <t>Nous serons diffusés à Dragons' Den le 17 septembre!</t>
+          <t>L'asclépiade s'en va à Dragons' Den le 17 septembre!</t>
         </is>
       </c>
       <c r="K183" s="10" t="inlineStr">
@@ -13115,7 +13115,7 @@
       </c>
       <c r="J184" s="9" t="inlineStr">
         <is>
-          <t>Nous serons diffusés à Dragons' Den le 17 septembre!</t>
+          <t>L'asclépiade s'en va à Dragons' Den le 17 septembre!</t>
         </is>
       </c>
       <c r="K184" s="10" t="inlineStr">
@@ -13184,7 +13184,7 @@
       </c>
       <c r="J185" s="9" t="inlineStr">
         <is>
-          <t>Nous serons diffusés à Dragons' Den le 17 septembre!</t>
+          <t>L'asclépiade s'en va à Dragons' Den le 17 septembre!</t>
         </is>
       </c>
       <c r="K185" s="10" t="inlineStr">
@@ -13460,7 +13460,7 @@
       </c>
       <c r="J189" s="9" t="inlineStr">
         <is>
-          <t>Nous serons diffusés à Dragons' Den le 17 septembre!</t>
+          <t>L'asclépiade s'en va à Dragons' Den le 17 septembre!</t>
         </is>
       </c>
       <c r="K189" s="10" t="inlineStr">
@@ -13529,7 +13529,7 @@
       </c>
       <c r="J190" s="9" t="inlineStr">
         <is>
-          <t>Nous serons diffusés à Dragons' Den le 17 septembre!</t>
+          <t>L'asclépiade s'en va à Dragons' Den le 17 septembre!</t>
         </is>
       </c>
       <c r="K190" s="10" t="inlineStr">
@@ -13736,7 +13736,7 @@
       </c>
       <c r="J193" s="9" t="inlineStr">
         <is>
-          <t>Nous serons diffusés à Dragons' Den le 17 septembre!</t>
+          <t>L'asclépiade s'en va à Dragons' Den le 17 septembre!</t>
         </is>
       </c>
       <c r="K193" s="10" t="inlineStr">
@@ -13805,7 +13805,7 @@
       </c>
       <c r="J194" s="9" t="inlineStr">
         <is>
-          <t>Nous serons diffusés à Dragons' Den le 17 septembre — invité disponible</t>
+          <t>L'asclépiade s'en va à Dragons' Den le 17 septembre!</t>
         </is>
       </c>
       <c r="K194" s="10" t="inlineStr">
@@ -13943,7 +13943,7 @@
       </c>
       <c r="J196" s="9" t="inlineStr">
         <is>
-          <t>Nous serons diffusés à Dragons' Den le 17 septembre!</t>
+          <t>L'asclépiade s'en va à Dragons' Den le 17 septembre!</t>
         </is>
       </c>
       <c r="K196" s="10" t="inlineStr">
@@ -14081,7 +14081,7 @@
       </c>
       <c r="J198" s="9" t="inlineStr">
         <is>
-          <t>Nous serons diffusés à Dragons' Den le 17 septembre — invité disponible</t>
+          <t>L'asclépiade s'en va à Dragons' Den le 17 septembre!</t>
         </is>
       </c>
       <c r="K198" s="10" t="inlineStr">
@@ -14288,7 +14288,7 @@
       </c>
       <c r="J201" s="9" t="inlineStr">
         <is>
-          <t>Nous serons diffusés à Dragons' Den le 17 septembre!</t>
+          <t>L'asclépiade s'en va à Dragons' Den le 17 septembre!</t>
         </is>
       </c>
       <c r="K201" s="10" t="inlineStr">
@@ -14357,7 +14357,7 @@
       </c>
       <c r="J202" s="9" t="inlineStr">
         <is>
-          <t>Nous serons diffusés à Dragons' Den le 17 septembre!</t>
+          <t>L'asclépiade s'en va à Dragons' Den le 17 septembre!</t>
         </is>
       </c>
       <c r="K202" s="10" t="inlineStr">
@@ -14620,7 +14620,7 @@
       </c>
       <c r="J206" s="9" t="inlineStr">
         <is>
-          <t>Nous serons diffusés à Dragons' Den le 17 septembre!</t>
+          <t>L'asclépiade s'en va à Dragons' Den le 17 septembre!</t>
         </is>
       </c>
       <c r="K206" s="10" t="inlineStr">
@@ -14758,7 +14758,7 @@
       </c>
       <c r="J208" s="9" t="inlineStr">
         <is>
-          <t>Nous serons diffusés à Dragons' Den le 17 septembre — invité disponible</t>
+          <t>L'asclépiade s'en va à Dragons' Den le 17 septembre!</t>
         </is>
       </c>
       <c r="K208" s="10" t="inlineStr">
@@ -14827,7 +14827,7 @@
       </c>
       <c r="J209" s="9" t="inlineStr">
         <is>
-          <t>Nous serons diffusés à Dragons' Den le 17 septembre — invité disponible</t>
+          <t>L'asclépiade s'en va à Dragons' Den le 17 septembre!</t>
         </is>
       </c>
       <c r="K209" s="10" t="inlineStr">
@@ -14952,7 +14952,7 @@
       </c>
       <c r="J211" s="9" t="inlineStr">
         <is>
-          <t>Nous serons diffusés à Dragons' Den le 17 septembre!</t>
+          <t>L'asclépiade s'en va à Dragons' Den le 17 septembre!</t>
         </is>
       </c>
       <c r="K211" s="10" t="inlineStr">
@@ -15159,7 +15159,7 @@
       </c>
       <c r="J214" s="9" t="inlineStr">
         <is>
-          <t>Nous serons diffusés à Dragons' Den le 17 septembre — invité disponible</t>
+          <t>L'asclépiade s'en va à Dragons' Den le 17 septembre!</t>
         </is>
       </c>
       <c r="K214" s="10" t="inlineStr">
@@ -15297,7 +15297,7 @@
       </c>
       <c r="J216" s="9" t="inlineStr">
         <is>
-          <t>Nous serons diffusés à Dragons' Den le 17 septembre!</t>
+          <t>L'asclépiade s'en va à Dragons' Den le 17 septembre!</t>
         </is>
       </c>
       <c r="K216" s="10" t="inlineStr">
@@ -15504,7 +15504,7 @@
       </c>
       <c r="J219" s="9" t="inlineStr">
         <is>
-          <t>Nous serons diffusés à Dragons' Den le 17 septembre — invité disponible</t>
+          <t>L'asclépiade s'en va à Dragons' Den le 17 septembre!</t>
         </is>
       </c>
       <c r="K219" s="10" t="inlineStr">
@@ -15573,7 +15573,7 @@
       </c>
       <c r="J220" s="9" t="inlineStr">
         <is>
-          <t>Nous serons diffusés à Dragons' Den le 17 septembre — invité disponible</t>
+          <t>L'asclépiade s'en va à Dragons' Den le 17 septembre!</t>
         </is>
       </c>
       <c r="K220" s="10" t="inlineStr">
@@ -15711,7 +15711,7 @@
       </c>
       <c r="J222" s="9" t="inlineStr">
         <is>
-          <t>Nous serons diffusés à Dragons' Den le 17 septembre!</t>
+          <t>L'asclépiade s'en va à Dragons' Den le 17 septembre!</t>
         </is>
       </c>
       <c r="K222" s="10" t="inlineStr">
@@ -15849,7 +15849,7 @@
       </c>
       <c r="J224" s="9" t="inlineStr">
         <is>
-          <t>Nous serons diffusés à Dragons' Den le 17 septembre!</t>
+          <t>L'asclépiade s'en va à Dragons' Den le 17 septembre!</t>
         </is>
       </c>
       <c r="K224" s="10" t="inlineStr">
@@ -15918,7 +15918,7 @@
       </c>
       <c r="J225" s="9" t="inlineStr">
         <is>
-          <t>Nous serons diffusés à Dragons' Den le 17 septembre — invité disponible</t>
+          <t>L'asclépiade s'en va à Dragons' Den le 17 septembre!</t>
         </is>
       </c>
       <c r="K225" s="10" t="inlineStr">
@@ -15987,7 +15987,7 @@
       </c>
       <c r="J226" s="9" t="inlineStr">
         <is>
-          <t>Nous serons diffusés à Dragons' Den le 17 septembre!</t>
+          <t>L'asclépiade s'en va à Dragons' Den le 17 septembre!</t>
         </is>
       </c>
       <c r="K226" s="10" t="inlineStr">
@@ -16056,7 +16056,7 @@
       </c>
       <c r="J227" s="9" t="inlineStr">
         <is>
-          <t>Nous serons diffusés à Dragons' Den le 17 septembre!</t>
+          <t>L'asclépiade s'en va à Dragons' Den le 17 septembre!</t>
         </is>
       </c>
       <c r="K227" s="10" t="inlineStr">
@@ -16125,7 +16125,7 @@
       </c>
       <c r="J228" s="9" t="inlineStr">
         <is>
-          <t>Nous serons diffusés à Dragons' Den le 17 septembre!</t>
+          <t>L'asclépiade s'en va à Dragons' Den le 17 septembre!</t>
         </is>
       </c>
       <c r="K228" s="10" t="inlineStr">
@@ -16194,7 +16194,7 @@
       </c>
       <c r="J229" s="9" t="inlineStr">
         <is>
-          <t>Nous serons diffusés à Dragons' Den le 17 septembre — invité disponible</t>
+          <t>L'asclépiade s'en va à Dragons' Den le 17 septembre!</t>
         </is>
       </c>
       <c r="K229" s="10" t="inlineStr">
@@ -16263,7 +16263,7 @@
       </c>
       <c r="J230" s="9" t="inlineStr">
         <is>
-          <t>Nous serons diffusés à Dragons' Den le 17 septembre!</t>
+          <t>L'asclépiade s'en va à Dragons' Den le 17 septembre!</t>
         </is>
       </c>
       <c r="K230" s="10" t="inlineStr">
@@ -16332,7 +16332,7 @@
       </c>
       <c r="J231" s="9" t="inlineStr">
         <is>
-          <t>Nous serons diffusés à Dragons' Den le 17 septembre — invité disponible</t>
+          <t>L'asclépiade s'en va à Dragons' Den le 17 septembre!</t>
         </is>
       </c>
       <c r="K231" s="10" t="inlineStr">
@@ -16401,7 +16401,7 @@
       </c>
       <c r="J232" s="9" t="inlineStr">
         <is>
-          <t>Nous serons diffusés à Dragons' Den le 17 septembre!</t>
+          <t>L'asclépiade s'en va à Dragons' Den le 17 septembre!</t>
         </is>
       </c>
       <c r="K232" s="10" t="inlineStr">
@@ -16470,7 +16470,7 @@
       </c>
       <c r="J233" s="9" t="inlineStr">
         <is>
-          <t>Nous serons diffusés à Dragons' Den le 17 septembre!</t>
+          <t>L'asclépiade s'en va à Dragons' Den le 17 septembre!</t>
         </is>
       </c>
       <c r="K233" s="10" t="inlineStr">
@@ -16539,7 +16539,7 @@
       </c>
       <c r="J234" s="9" t="inlineStr">
         <is>
-          <t>Nous serons diffusés à Dragons' Den le 17 septembre!</t>
+          <t>L'asclépiade s'en va à Dragons' Den le 17 septembre!</t>
         </is>
       </c>
       <c r="K234" s="10" t="inlineStr">
@@ -16677,7 +16677,7 @@
       </c>
       <c r="J236" s="9" t="inlineStr">
         <is>
-          <t>Nous serons diffusés à Dragons' Den le 17 septembre — invité disponible</t>
+          <t>L'asclépiade s'en va à Dragons' Den le 17 septembre!</t>
         </is>
       </c>
       <c r="K236" s="10" t="inlineStr">
@@ -16746,7 +16746,7 @@
       </c>
       <c r="J237" s="9" t="inlineStr">
         <is>
-          <t>Nous serons diffusés à Dragons' Den le 17 septembre!</t>
+          <t>L'asclépiade s'en va à Dragons' Den le 17 septembre!</t>
         </is>
       </c>
       <c r="K237" s="10" t="inlineStr">
@@ -16815,7 +16815,7 @@
       </c>
       <c r="J238" s="9" t="inlineStr">
         <is>
-          <t>Nous serons diffusés à Dragons' Den le 17 septembre!</t>
+          <t>L'asclépiade s'en va à Dragons' Den le 17 septembre!</t>
         </is>
       </c>
       <c r="K238" s="10" t="inlineStr">
@@ -16953,7 +16953,7 @@
       </c>
       <c r="J240" s="9" t="inlineStr">
         <is>
-          <t>Nous serons diffusés à Dragons' Den le 17 septembre!</t>
+          <t>L'asclépiade s'en va à Dragons' Den le 17 septembre!</t>
         </is>
       </c>
       <c r="K240" s="10" t="inlineStr">
@@ -17160,7 +17160,7 @@
       </c>
       <c r="J243" s="9" t="inlineStr">
         <is>
-          <t>Nous serons diffusés à Dragons' Den le 17 septembre — invité disponible</t>
+          <t>L'asclépiade s'en va à Dragons' Den le 17 septembre!</t>
         </is>
       </c>
       <c r="K243" s="10" t="inlineStr">
@@ -17436,7 +17436,7 @@
       </c>
       <c r="J247" s="9" t="inlineStr">
         <is>
-          <t>Nous serons diffusés à Dragons' Den le 17 septembre — invité disponible</t>
+          <t>L'asclépiade s'en va à Dragons' Den le 17 septembre!</t>
         </is>
       </c>
       <c r="K247" s="10" t="inlineStr">
@@ -17574,7 +17574,7 @@
       </c>
       <c r="J249" s="9" t="inlineStr">
         <is>
-          <t>Nous serons diffusés à Dragons' Den le 17 septembre — invité disponible</t>
+          <t>L'asclépiade s'en va à Dragons' Den le 17 septembre!</t>
         </is>
       </c>
       <c r="K249" s="10" t="inlineStr">
@@ -17643,7 +17643,7 @@
       </c>
       <c r="J250" s="9" t="inlineStr">
         <is>
-          <t>Nous serons diffusés à Dragons' Den le 17 septembre!</t>
+          <t>L'asclépiade s'en va à Dragons' Den le 17 septembre!</t>
         </is>
       </c>
       <c r="K250" s="10" t="inlineStr">
@@ -17712,7 +17712,7 @@
       </c>
       <c r="J251" s="9" t="inlineStr">
         <is>
-          <t>Nous serons diffusés à Dragons' Den le 17 septembre — invité disponible</t>
+          <t>L'asclépiade s'en va à Dragons' Den le 17 septembre!</t>
         </is>
       </c>
       <c r="K251" s="10" t="inlineStr">
@@ -17850,7 +17850,7 @@
       </c>
       <c r="J253" s="9" t="inlineStr">
         <is>
-          <t>Nous serons diffusés à Dragons' Den le 17 septembre!</t>
+          <t>L'asclépiade s'en va à Dragons' Den le 17 septembre!</t>
         </is>
       </c>
       <c r="K253" s="10" t="inlineStr">

</xml_diff>

<commit_message>
Remplace l'ouverture par ce que l'entreprise fait, pas par où elle loge
« Une entreprise de Québec dont l'atelier est dans Limoilou » ne dit rien à
quelqu'un qui ne nous connaît pas, et brûlait la seule ligne qu'un journaliste
lit à coup sûr. L'ouverture devient « On isole des manteaux avec une mauvaise
herbe. »

Le paragraphe suivant est resserré: l'asclépiade et les « petits cochons »
arrivent en tête de phrase au lieu d'être annoncés, et « on la transforme en
isolant à Québec » garde le lieu là où il compte, sans le quartier.

Limoilou reste là où c'est une invitation à venir voir l'atelier, et dans les
courriels aux journalistes de Québec, qui savent où c'est.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015pjLsGPzf1MX1JC7QiKGGk
</commit_message>
<xml_diff>
--- a/communique-dragons/Lasclay_brouillons_a_editer.xlsx
+++ b/communique-dragons/Lasclay_brouillons_a_editer.xlsx
@@ -498,7 +498,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B18"/>
+  <dimension ref="A1:B21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -508,7 +508,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Version 5 — les objets, suite</t>
+          <t>Version 6 — la première ligne</t>
         </is>
       </c>
       <c r="B1" s="2" t="inlineStr"/>
@@ -520,150 +520,186 @@
     <row r="3" ht="56" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>« Invité disponible »</t>
+          <t>Le reproche</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Retiré. Zéro occurrence.</t>
+          <t>Limoilou est impertinent pour décrire l'entreprise. Un quartier ne dit rien à quelqu'un qui ne nous connaît pas, et ça brûlait la seule ligne qu'un journaliste lit à coup sûr.</t>
         </is>
       </c>
     </row>
     <row r="4" ht="56" customHeight="1">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>L'asclépiade en tête</t>
+          <t>Avant</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Tu as aimé la formule, alors elle passe de 54 à 149 contacts. « Nous serons diffusés » suppose que la personne sait déjà qui est « nous » : ça ne vaut que pour ceux qui nous connaissent, la liste chaude et les journalistes d'affaires.</t>
+          <t>« Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou. »</t>
         </is>
       </c>
     </row>
     <row r="5" ht="56" customHeight="1">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t>Les trois objets</t>
+          <t>Maintenant</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>149 : L'asclépiade s'en va à Dragons' Den le 17 septembre!  |  59 : Nous serons diffusés à Dragons' Den le 17 septembre!  |  45 : L'asclépiade et les monarques à Dragons' Den le 17 septembre!</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="2" t="inlineStr"/>
-      <c r="B6" s="2" t="inlineStr"/>
-    </row>
-    <row r="7">
-      <c r="A7" s="1" t="inlineStr">
-        <is>
-          <t>Les versions précédentes</t>
-        </is>
-      </c>
-      <c r="B7" s="2" t="inlineStr"/>
+          <t>« Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe. »</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="56" customHeight="1">
+      <c r="A6" s="3" t="inlineStr">
+        <is>
+          <t>Le paragraphe suivant</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>Resserré aussi : l'asclépiade et les « petits cochons » arrivent en tête de phrase au lieu d'être annoncés. « On la transforme en isolant à Québec » garde le lieu là où il compte, sans le quartier.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="56" customHeight="1">
+      <c r="A7" s="3" t="inlineStr">
+        <is>
+          <t>Limoilou reste</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>Là où c'est une invitation — « l'atelier de Limoilou est ouvert si vous voulez voir la matière » — et dans les courriels aux journalistes de Québec, qui savent où c'est.</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr"/>
       <c r="B8" s="2" t="inlineStr"/>
     </row>
-    <row r="9" ht="56" customHeight="1">
-      <c r="A9" s="3" t="inlineStr">
-        <is>
-          <t>v4</t>
-        </is>
-      </c>
-      <c r="B9" s="2" t="inlineStr">
-        <is>
-          <t>Objets refaits : de « titre d'essai » à annonce datée.</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="56" customHeight="1">
-      <c r="A10" s="3" t="inlineStr">
-        <is>
-          <t>v3</t>
-        </is>
-      </c>
-      <c r="B10" s="2" t="inlineStr">
-        <is>
-          <t>Présentation complète en tête des courriels froids, « pourquoi vous » explicite.</t>
-        </is>
-      </c>
+    <row r="9">
+      <c r="A9" s="1" t="inlineStr">
+        <is>
+          <t>Les versions précédentes</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr"/>
+      <c r="B10" s="2" t="inlineStr"/>
     </row>
     <row r="11" ht="56" customHeight="1">
       <c r="A11" s="3" t="inlineStr">
         <is>
-          <t>v2</t>
+          <t>v5</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>Registre de Gabriel : plus d'excuses, plus de mise en garde, plus de rappel de confidentialité.</t>
+          <t>« Invité disponible » retiré, l'asclépiade en tête des objets pour 149 contacts.</t>
         </is>
       </c>
     </row>
     <row r="12" ht="56" customHeight="1">
       <c r="A12" s="3" t="inlineStr">
         <is>
+          <t>v4</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>Objets refaits : de titre d'essai à annonce datée.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="56" customHeight="1">
+      <c r="A13" s="3" t="inlineStr">
+        <is>
+          <t>v3</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>Présentation et « pourquoi vous » dans les courriels froids.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="56" customHeight="1">
+      <c r="A14" s="3" t="inlineStr">
+        <is>
+          <t>v2</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>Registre de Gabriel : plus d'excuses, plus de mise en garde, plus de confidentialité.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="56" customHeight="1">
+      <c r="A15" s="3" t="inlineStr">
+        <is>
           <t>Repris mot pour mot</t>
         </is>
       </c>
-      <c r="B12" s="2" t="inlineStr">
+      <c r="B15" s="2" t="inlineStr">
         <is>
           <t>Larocque et Pouliot.</t>
         </is>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" s="2" t="inlineStr"/>
-      <c r="B13" s="2" t="inlineStr"/>
-    </row>
-    <row r="14">
-      <c r="A14" s="1" t="inlineStr">
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr"/>
+      <c r="B16" s="2" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="1" t="inlineStr">
         <is>
           <t>Rappels</t>
         </is>
       </c>
-      <c r="B14" s="2" t="inlineStr"/>
-    </row>
-    <row r="15">
-      <c r="A15" s="2" t="inlineStr"/>
-      <c r="B15" s="2" t="inlineStr"/>
-    </row>
-    <row r="16" ht="56" customHeight="1">
-      <c r="A16" s="3" t="inlineStr">
+      <c r="B17" s="2" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr"/>
+      <c r="B18" s="2" t="inlineStr"/>
+    </row>
+    <row r="19" ht="56" customHeight="1">
+      <c r="A19" s="3" t="inlineStr">
         <is>
           <t>Diffusion</t>
         </is>
       </c>
-      <c r="B16" s="2" t="inlineStr">
+      <c r="B19" s="2" t="inlineStr">
         <is>
           <t>Jeudi 17 septembre 2026, 20 h (20 h 30 NT), CBC et CBC Gem. Prévente le samedi 12 septembre à 9 h.</t>
         </is>
       </c>
     </row>
-    <row r="17" ht="56" customHeight="1">
-      <c r="A17" s="3" t="inlineStr">
+    <row r="20" ht="56" customHeight="1">
+      <c r="A20" s="3" t="inlineStr">
         <is>
           <t>Ne pas envoyer</t>
         </is>
       </c>
-      <c r="B17" s="2" t="inlineStr">
+      <c r="B20" s="2" t="inlineStr">
         <is>
           <t>Anne-Sophie Roy à l'adresse Québecor. Annie Lafrance et Francis Higgins en liste froide.</t>
         </is>
       </c>
     </row>
-    <row r="18" ht="56" customHeight="1">
-      <c r="A18" s="3" t="inlineStr">
+    <row r="21" ht="56" customHeight="1">
+      <c r="A21" s="3" t="inlineStr">
         <is>
           <t>Courriels manquants</t>
         </is>
       </c>
-      <c r="B18" s="2" t="inlineStr">
+      <c r="B21" s="2" t="inlineStr">
         <is>
           <t>Sophie Poisson, Caroline Bertrand, Karine Benoist, Antoine Stab.</t>
         </is>
@@ -752,7 +788,7 @@
       </c>
       <c r="K1" s="4" t="inlineStr">
         <is>
-          <t>Brouillon v5</t>
+          <t>Brouillon v6</t>
         </is>
       </c>
       <c r="L1" s="4" t="inlineStr">
@@ -2517,7 +2553,7 @@
       <c r="K29" s="10" t="inlineStr">
         <is>
           <t>Bonjour Mme Roberge,
-Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou. On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe : l'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -2572,7 +2608,7 @@
       <c r="K30" s="10" t="inlineStr">
         <is>
           <t>Bonjour Mme Laforest,
-Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou. On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe : l'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -2800,7 +2836,7 @@
       <c r="K34" s="10" t="inlineStr">
         <is>
           <t>Bonjour Mme Goubau,
-Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou. Vous couvrez le textile et la mode, alors voici une matière que peu de gens ont vue de près : la soie d'asclépiade, une fibre creuse et naturellement hydrophobe attachée aux graines d'une plante que les agriculteurs arrachent de leurs champs depuis 50 ans. On la transforme en isolant, et on en fait des manteaux, des mitaines et des tuques.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe. Vous couvrez le textile et la mode, alors voici une matière que peu de gens ont vue de près : la soie d'asclépiade, une fibre creuse et naturellement hydrophobe attachée aux graines d'une plante que les agriculteurs arrachent de leurs champs depuis 50 ans. On la transforme en isolant, et on en fait des manteaux, des mitaines et des tuques.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -2855,7 +2891,7 @@
       <c r="K35" s="10" t="inlineStr">
         <is>
           <t>Bonjour Mme Dostie,
-Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou. On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe : l'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -3099,8 +3135,8 @@
       <c r="K39" s="10" t="inlineStr">
         <is>
           <t>Bonjour Marie Allard,
-Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de
-Québec dont l'atelier est dans Limoilou.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une
+mauvaise herbe.
 Il y a une belle histoire de sciences dans l'asclépiade. La soie attachée à ses graines n'est
 pas un poil : c'est un tube creux enduit d'une cire hydrophobe, et les fibres portent une
 charge qui les fait se repousser. C'est ce qui forme le parachute autour de la graine, et
@@ -3174,8 +3210,8 @@
       <c r="K40" s="10" t="inlineStr">
         <is>
           <t>Bonjour Zoé Allemand,
-Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
-On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
+L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
 Je vous écris parce que vous couvrez l'agriculture. La question qui compte pour les producteurs n'a pas changé depuis l'effondrement de la filière en 2018 : est-ce qu'il y a un acheteur stable au bout du champ. On achète encore la récolte de producteurs d'ici et on la transforme nous-mêmes.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
@@ -3243,8 +3279,8 @@
       <c r="K41" s="10" t="inlineStr">
         <is>
           <t>Bonjour Victoria Bakos,
-Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
-On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
+L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
 Je vous écris parce que vous couvrez l'art de vivre et la consommation. Le contraste se photographie bien : la gousse dans le champ, la soie blanche dans la main, le manteau porté en ville.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
@@ -3312,8 +3348,8 @@
       <c r="K42" s="10" t="inlineStr">
         <is>
           <t>Bonjour Marie-Émélie Bernier,
-Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
-On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
+L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
 Je vous écris parce que c'est une nouvelle de chez nous qui passe au national.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
@@ -3381,8 +3417,8 @@
       <c r="K43" s="10" t="inlineStr">
         <is>
           <t>Bonjour Normand Blouin,
-Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
-On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
+L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
 Je vous écris parce que vous couvrez l'agriculture. La question qui compte pour les producteurs n'a pas changé depuis l'effondrement de la filière en 2018 : est-ce qu'il y a un acheteur stable au bout du champ. On achète encore la récolte de producteurs d'ici et on la transforme nous-mêmes.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
@@ -3450,8 +3486,8 @@
       <c r="K44" s="10" t="inlineStr">
         <is>
           <t>Bonjour Louise Bourbonnais,
-Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
-On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
+L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
 Je vous écris parce que c'est une nouvelle de chez nous qui passe au national.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
@@ -3519,8 +3555,8 @@
       <c r="K45" s="10" t="inlineStr">
         <is>
           <t>Bonjour Francois Bourque,
-Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
-On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
+L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
 Je vous écris parce que vous couvrez l'économie. On a bâti nos propres procédés de transformation parce qu'aucun sous-traitant ne voulait toucher à l'asclépiade, puis on a changé de modèle manufacturier l'an dernier pour rendre un manteau accessible à 300 $. J'en ai fait une vidéo ici : https://www.youtube.com/watch?v=GKyHh-Ok9JU.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
@@ -3588,8 +3624,8 @@
       <c r="K46" s="10" t="inlineStr">
         <is>
           <t>Bonjour Ariane Boyer,
-Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
-On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
+L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
 Je vous écris parce que vous couvrez l'environnement. Notre pari est économique avant d'être militant : si l'asclépiade devient payante, les agriculteurs la gardent dans leurs champs, et les monarques retrouvent de l'habitat de reproduction.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
@@ -3657,8 +3693,8 @@
       <c r="K47" s="10" t="inlineStr">
         <is>
           <t>Bonjour Gilbert Bégin,
-Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
-On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
+L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
 Je vous écris parce que c'est une nouvelle de chez nous qui passe au national.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
@@ -3726,8 +3762,8 @@
       <c r="K48" s="10" t="inlineStr">
         <is>
           <t>Bonjour Papa Moussa Camara,
-Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
-On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
+L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
 Je vous écris parce que le sujet se raconte bien en ondes : une entreprise de Québec qui va expliquer à un auditoire pancanadien pourquoi la mauvaise herbe des champs de maïs peut isoler un manteau.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
@@ -3795,8 +3831,8 @@
       <c r="K49" s="10" t="inlineStr">
         <is>
           <t>Bonjour Victor Carré,
-Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
-On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
+L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
 Je vous écris parce que c'est une nouvelle de chez nous qui passe au national.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
@@ -3864,8 +3900,8 @@
       <c r="K50" s="10" t="inlineStr">
         <is>
           <t>Bonjour Eric Chabot,
-Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
-On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
+L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
 Je vous écris parce que vous couvrez le plein air. À poids égal, la littérature donne la soie d'asclépiade pour environ 10 % plus isolante que le duvet. C'est un repère de laboratoire, pas une promesse de manteau, et c'est exactement pour ça que je préfère qu'on la teste.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
@@ -3933,8 +3969,8 @@
       <c r="K51" s="10" t="inlineStr">
         <is>
           <t>Bonjour Tristan Champagne-Lessard,
-Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
-On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
+L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
 Je vous écris entre autres parce que la Montérégie est une des régions où l'asclépiade se cultive encore, et que c'est de champs comme ceux-là que vient la fibre qu'on transforme.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
@@ -4002,8 +4038,8 @@
       <c r="K52" s="10" t="inlineStr">
         <is>
           <t>Bonjour Jean-Marc Chevalier,
-Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
-On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
+L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
 Je vous écris entre autres parce que la Montérégie est une des régions où l'asclépiade se cultive encore, et que c'est de champs comme ceux-là que vient la fibre qu'on transforme.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
@@ -4071,8 +4107,8 @@
       <c r="K53" s="10" t="inlineStr">
         <is>
           <t>Bonjour Simon Chrétien,
-Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
-On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
+L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
 Je vous écris parce que vous couvrez l'agriculture. La question qui compte pour les producteurs n'a pas changé depuis l'effondrement de la filière en 2018 : est-ce qu'il y a un acheteur stable au bout du champ. On achète encore la récolte de producteurs d'ici et on la transforme nous-mêmes.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
@@ -4140,8 +4176,8 @@
       <c r="K54" s="10" t="inlineStr">
         <is>
           <t>Bonjour Maxime Corneau,
-Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
-On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
+L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
 Je vous écris entre autres parce qu'un de nos fournisseurs d'asclépiade cultive au Lac-Saint-Jean depuis nos tout débuts, et qu'il l'est encore aujourd'hui. La fibre de chez vous se retrouve dans nos produits.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
@@ -4209,8 +4245,8 @@
       <c r="K55" s="10" t="inlineStr">
         <is>
           <t>Bonjour Aurélia Crémoux,
-Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
-On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
+L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
 Je vous écris parce que vous couvrez le plein air. À poids égal, la littérature donne la soie d'asclépiade pour environ 10 % plus isolante que le duvet. C'est un repère de laboratoire, pas une promesse de manteau, et c'est exactement pour ça que je préfère qu'on la teste.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
@@ -4278,8 +4314,8 @@
       <c r="K56" s="10" t="inlineStr">
         <is>
           <t>Bonjour Catherine Dallaire,
-Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
-On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
+L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
 Je vous écris entre autres parce qu'une des premières usines de transformation de la fibre était à Granby, et que l'Estrie compte encore des producteurs d'asclépiade.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
@@ -4347,8 +4383,8 @@
       <c r="K57" s="10" t="inlineStr">
         <is>
           <t>Bonjour Gabriel Delisle,
-Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de
-Québec dont l'atelier est dans Limoilou.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une
+mauvaise herbe.
 L'asclépiade a été une histoire mauricienne avant d'être la nôtre : l'usine de Saint-Tite
 achetait 90 % des récoltes du Québec. On a démarré après la chute de cette filière, et six ans
 plus tard on achète encore de l'asclépiade québécoise et on la
@@ -4421,8 +4457,8 @@
       <c r="K58" s="10" t="inlineStr">
         <is>
           <t>Bonjour Anaïs Desjardins,
-Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
-On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
+L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
 Je vous écris parce que vous couvrez l'environnement. Notre pari est économique avant d'être militant : si l'asclépiade devient payante, les agriculteurs la gardent dans leurs champs, et les monarques retrouvent de l'habitat de reproduction.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
@@ -4490,8 +4526,8 @@
       <c r="K59" s="10" t="inlineStr">
         <is>
           <t>Bonjour Simon Dominé,
-Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
-On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
+L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
 Je vous écris parce que vous couvrez l'agriculture. La question qui compte pour les producteurs n'a pas changé depuis l'effondrement de la filière en 2018 : est-ce qu'il y a un acheteur stable au bout du champ. On achète encore la récolte de producteurs d'ici et on la transforme nous-mêmes.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
@@ -4559,8 +4595,8 @@
       <c r="K60" s="10" t="inlineStr">
         <is>
           <t>Bonjour Karl-Ivann Dubé,
-Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
-On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
+L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
 Je vous écris parce que le sujet se raconte bien en ondes : une entreprise de Québec qui va expliquer à un auditoire pancanadien pourquoi la mauvaise herbe des champs de maïs peut isoler un manteau.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
@@ -4628,8 +4664,8 @@
       <c r="K61" s="10" t="inlineStr">
         <is>
           <t>Bonjour André Fauteux,
-Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
-On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
+L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
 Je vous écris parce que c'est une nouvelle de chez nous qui passe au national.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
@@ -4697,8 +4733,8 @@
       <c r="K62" s="10" t="inlineStr">
         <is>
           <t>Bonjour Myriam Fimbry,
-Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
-On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
+L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
 Je vous écris parce que vous couvrez l'agriculture. La question qui compte pour les producteurs n'a pas changé depuis l'effondrement de la filière en 2018 : est-ce qu'il y a un acheteur stable au bout du champ. On achète encore la récolte de producteurs d'ici et on la transforme nous-mêmes.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
@@ -4766,8 +4802,8 @@
       <c r="K63" s="10" t="inlineStr">
         <is>
           <t>Bonjour Étienne Fortin-Gauthier,
-Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
-On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
+L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
 Je vous écris parce que le sujet se raconte bien en ondes : une entreprise de Québec qui va expliquer à un auditoire pancanadien pourquoi la mauvaise herbe des champs de maïs peut isoler un manteau.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
@@ -4835,8 +4871,8 @@
       <c r="K64" s="10" t="inlineStr">
         <is>
           <t>Bonjour Johanne Fournier,
-Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
-On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
+L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
 Je vous écris parce que c'est une nouvelle de chez nous qui passe au national.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
@@ -4904,8 +4940,8 @@
       <c r="K65" s="10" t="inlineStr">
         <is>
           <t>Bonjour Jean Garon,
-Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
-On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
+L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
 Je vous écris parce que vous couvrez l'environnement. Notre pari est économique avant d'être militant : si l'asclépiade devient payante, les agriculteurs la gardent dans leurs champs, et les monarques retrouvent de l'habitat de reproduction.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
@@ -4973,8 +5009,8 @@
       <c r="K66" s="10" t="inlineStr">
         <is>
           <t>Bonjour Cécile Gladel,
-Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
-On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
+L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
 Je vous écris parce que le sujet se raconte bien en ondes : une entreprise de Québec qui va expliquer à un auditoire pancanadien pourquoi la mauvaise herbe des champs de maïs peut isoler un manteau.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
@@ -5042,8 +5078,8 @@
       <c r="K67" s="10" t="inlineStr">
         <is>
           <t>Bonjour Marieke Glorieux-Stryckman,
-Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
-On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
+L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
 Je vous écris parce que vous couvrez le plein air. À poids égal, la littérature donne la soie d'asclépiade pour environ 10 % plus isolante que le duvet. C'est un repère de laboratoire, pas une promesse de manteau, et c'est exactement pour ça que je préfère qu'on la teste.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
@@ -5111,8 +5147,8 @@
       <c r="K68" s="10" t="inlineStr">
         <is>
           <t>Bonjour Maude Goyer,
-Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
-On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
+L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
 Je vous écris parce que vous couvrez le plein air. À poids égal, la littérature donne la soie d'asclépiade pour environ 10 % plus isolante que le duvet. C'est un repère de laboratoire, pas une promesse de manteau, et c'est exactement pour ça que je préfère qu'on la teste.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
@@ -5180,8 +5216,8 @@
       <c r="K69" s="10" t="inlineStr">
         <is>
           <t>Bonjour Pauline Gravel,
-Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
-On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
+L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
 Je vous écris parce que vous couvrez l'agriculture. La question qui compte pour les producteurs n'a pas changé depuis l'effondrement de la filière en 2018 : est-ce qu'il y a un acheteur stable au bout du champ. On achète encore la récolte de producteurs d'ici et on la transforme nous-mêmes.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
@@ -5249,8 +5285,8 @@
       <c r="K70" s="10" t="inlineStr">
         <is>
           <t>Bonjour Bernard Hervieux,
-Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
-On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
+L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
 Je vous écris parce que le sujet se raconte bien en ondes : une entreprise de Québec qui va expliquer à un auditoire pancanadien pourquoi la mauvaise herbe des champs de maïs peut isoler un manteau.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
@@ -5318,8 +5354,8 @@
       <c r="K71" s="10" t="inlineStr">
         <is>
           <t>Bonjour Leïla Jolin-Dahel,
-Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
-On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
+L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
 Je vous écris parce que vous couvrez l'agriculture. La question qui compte pour les producteurs n'a pas changé depuis l'effondrement de la filière en 2018 : est-ce qu'il y a un acheteur stable au bout du champ. On achète encore la récolte de producteurs d'ici et on la transforme nous-mêmes.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
@@ -5387,8 +5423,8 @@
       <c r="K72" s="10" t="inlineStr">
         <is>
           <t>Bonjour Kodjo Edjinam Nulagnon LOGO,
-Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
-On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
+L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
 Je vous écris parce que vous couvrez l'environnement. Notre pari est économique avant d'être militant : si l'asclépiade devient payante, les agriculteurs la gardent dans leurs champs, et les monarques retrouvent de l'habitat de reproduction.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
@@ -5456,8 +5492,8 @@
       <c r="K73" s="10" t="inlineStr">
         <is>
           <t>Bonjour Annie Labrecque,
-Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
-On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
+L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
 Je vous écris parce que vous couvrez l'agriculture. La question qui compte pour les producteurs n'a pas changé depuis l'effondrement de la filière en 2018 : est-ce qu'il y a un acheteur stable au bout du champ. On achète encore la récolte de producteurs d'ici et on la transforme nous-mêmes.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
@@ -5525,8 +5561,8 @@
       <c r="K74" s="10" t="inlineStr">
         <is>
           <t>Bonjour Marianne Lachapelle,
-Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
-On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
+L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
 Je vous écris entre autres parce qu'une des premières usines de transformation de la fibre était à Granby, et que l'Estrie compte encore des producteurs d'asclépiade.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
@@ -5594,8 +5630,8 @@
       <c r="K75" s="10" t="inlineStr">
         <is>
           <t>Bonjour Sophie Lachapelle,
-Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
-On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
+L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
 Je vous écris parce que vous couvrez l'agriculture. La question qui compte pour les producteurs n'a pas changé depuis l'effondrement de la filière en 2018 : est-ce qu'il y a un acheteur stable au bout du champ. On achète encore la récolte de producteurs d'ici et on la transforme nous-mêmes.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
@@ -5663,8 +5699,8 @@
       <c r="K76" s="10" t="inlineStr">
         <is>
           <t>Bonjour Alain Laforest,
-Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
-On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
+L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
 Je vous écris parce que le sujet se raconte bien en ondes : une entreprise de Québec qui va expliquer à un auditoire pancanadien pourquoi la mauvaise herbe des champs de maïs peut isoler un manteau.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
@@ -5732,8 +5768,8 @@
       <c r="K77" s="10" t="inlineStr">
         <is>
           <t>Bonjour Mikaël Lalancette,
-Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
-On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
+L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
 Je vous écris parce que c'est une nouvelle de chez nous qui passe au national.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
@@ -5801,8 +5837,8 @@
       <c r="K78" s="10" t="inlineStr">
         <is>
           <t>Bonjour Jean-Luc Lavallée,
-Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
-On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
+L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
 Je vous écris parce que vous couvrez l'économie. On a bâti nos propres procédés de transformation parce qu'aucun sous-traitant ne voulait toucher à l'asclépiade, puis on a changé de modèle manufacturier l'an dernier pour rendre un manteau accessible à 300 $. J'en ai fait une vidéo ici : https://www.youtube.com/watch?v=GKyHh-Ok9JU.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
@@ -5870,8 +5906,8 @@
       <c r="K79" s="10" t="inlineStr">
         <is>
           <t>Bonjour Jean-Francois Leblanc,
-Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
-On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
+L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
 Je vous écris parce que vous couvrez le plein air. À poids égal, la littérature donne la soie d'asclépiade pour environ 10 % plus isolante que le duvet. C'est un repère de laboratoire, pas une promesse de manteau, et c'est exactement pour ça que je préfère qu'on la teste.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
@@ -5939,8 +5975,8 @@
       <c r="K80" s="10" t="inlineStr">
         <is>
           <t>Bonjour Julie Leduc,
-Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
-On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
+L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
 Je vous écris parce que vous couvrez le plein air. À poids égal, la littérature donne la soie d'asclépiade pour environ 10 % plus isolante que le duvet. C'est un repère de laboratoire, pas une promesse de manteau, et c'est exactement pour ça que je préfère qu'on la teste.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
@@ -6008,8 +6044,8 @@
       <c r="K81" s="10" t="inlineStr">
         <is>
           <t>Bonjour Annie Martin,
-Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
-On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
+L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
 Je vous écris parce que vous couvrez l'agriculture. La question qui compte pour les producteurs n'a pas changé depuis l'effondrement de la filière en 2018 : est-ce qu'il y a un acheteur stable au bout du champ. On achète encore la récolte de producteurs d'ici et on la transforme nous-mêmes.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
@@ -6077,8 +6113,8 @@
       <c r="K82" s="10" t="inlineStr">
         <is>
           <t>Bonjour Réjean Martin,
-Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de
-Québec dont l'atelier est dans Limoilou.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une
+mauvaise herbe.
 Vous couvrez Mékinac, donc Saint-Tite, donc l'endroit où l'asclépiade a eu son grand moment
 industriel au Québec. L'usine achetait 90 % des récoltes de la province avant que la filière
 se casse en 2018.
@@ -6152,8 +6188,8 @@
       <c r="K83" s="10" t="inlineStr">
         <is>
           <t>Bonjour Charles Mathieu,
-Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
-On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
+L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
 Je vous écris parce que vous couvrez l'environnement. Notre pari est économique avant d'être militant : si l'asclépiade devient payante, les agriculteurs la gardent dans leurs champs, et les monarques retrouvent de l'habitat de reproduction.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
@@ -6221,8 +6257,8 @@
       <c r="K84" s="10" t="inlineStr">
         <is>
           <t>Bonjour Clara Matthey-Jonais,
-Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
-On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
+L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
 Je vous écris parce que vous couvrez l'agriculture. La question qui compte pour les producteurs n'a pas changé depuis l'effondrement de la filière en 2018 : est-ce qu'il y a un acheteur stable au bout du champ. On achète encore la récolte de producteurs d'ici et on la transforme nous-mêmes.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
@@ -6290,8 +6326,8 @@
       <c r="K85" s="10" t="inlineStr">
         <is>
           <t>Bonjour Valérian Mazataud,
-Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
-On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
+L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
 Je vous écris parce que vous couvrez l'agriculture. La question qui compte pour les producteurs n'a pas changé depuis l'effondrement de la filière en 2018 : est-ce qu'il y a un acheteur stable au bout du champ. On achète encore la récolte de producteurs d'ici et on la transforme nous-mêmes.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
@@ -6359,8 +6395,8 @@
       <c r="K86" s="10" t="inlineStr">
         <is>
           <t>Bonjour Lili Mercure,
-Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
-On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
+L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
 Je vous écris parce que le sujet se raconte bien en ondes : une entreprise de Québec qui va expliquer à un auditoire pancanadien pourquoi la mauvaise herbe des champs de maïs peut isoler un manteau.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
@@ -6428,8 +6464,8 @@
       <c r="K87" s="10" t="inlineStr">
         <is>
           <t>Bonjour Nicolas Mesly,
-Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
-On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
+L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
 Je vous écris parce que vous couvrez l'agriculture. La question qui compte pour les producteurs n'a pas changé depuis l'effondrement de la filière en 2018 : est-ce qu'il y a un acheteur stable au bout du champ. On achète encore la récolte de producteurs d'ici et on la transforme nous-mêmes.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
@@ -6497,8 +6533,8 @@
       <c r="K88" s="10" t="inlineStr">
         <is>
           <t>Bonjour Nicolas Michaud,
-Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
-On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
+L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
 Je vous écris parce que vous couvrez l'agriculture. La question qui compte pour les producteurs n'a pas changé depuis l'effondrement de la filière en 2018 : est-ce qu'il y a un acheteur stable au bout du champ. On achète encore la récolte de producteurs d'ici et on la transforme nous-mêmes.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
@@ -6566,8 +6602,8 @@
       <c r="K89" s="10" t="inlineStr">
         <is>
           <t>Bonjour Véronique Morin,
-Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
-On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
+L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
 Je vous écris parce que vous couvrez l'agriculture. La question qui compte pour les producteurs n'a pas changé depuis l'effondrement de la filière en 2018 : est-ce qu'il y a un acheteur stable au bout du champ. On achète encore la récolte de producteurs d'ici et on la transforme nous-mêmes.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
@@ -6635,8 +6671,8 @@
       <c r="K90" s="10" t="inlineStr">
         <is>
           <t>Bonjour Lila Mouch,
-Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
-On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
+L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
 Je vous écris parce que le sujet se raconte bien en ondes : une entreprise de Québec qui va expliquer à un auditoire pancanadien pourquoi la mauvaise herbe des champs de maïs peut isoler un manteau.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
@@ -6704,8 +6740,8 @@
       <c r="K91" s="10" t="inlineStr">
         <is>
           <t>Bonjour Olivier Mougeot,
-Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
-On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
+L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
 Je vous écris parce que c'est une nouvelle de chez nous qui passe au national.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
@@ -6773,8 +6809,8 @@
       <c r="K92" s="10" t="inlineStr">
         <is>
           <t>Bonjour Emmanuelle Mozayan-Verschaeve,
-Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
-On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
+L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
 Je vous écris parce que vous couvrez le plein air. À poids égal, la littérature donne la soie d'asclépiade pour environ 10 % plus isolante que le duvet. C'est un repère de laboratoire, pas une promesse de manteau, et c'est exactement pour ça que je préfère qu'on la teste.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
@@ -6842,8 +6878,8 @@
       <c r="K93" s="10" t="inlineStr">
         <is>
           <t>Bonjour Jean-Benoît Nadeau,
-Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
-On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
+L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
 Je vous écris parce que vous couvrez le plein air. À poids égal, la littérature donne la soie d'asclépiade pour environ 10 % plus isolante que le duvet. C'est un repère de laboratoire, pas une promesse de manteau, et c'est exactement pour ça que je préfère qu'on la teste.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
@@ -6911,8 +6947,8 @@
       <c r="K94" s="10" t="inlineStr">
         <is>
           <t>Bonjour Yves Ouellet,
-Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
-On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
+L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
 Je vous écris parce que vous couvrez le plein air. À poids égal, la littérature donne la soie d'asclépiade pour environ 10 % plus isolante que le duvet. C'est un repère de laboratoire, pas une promesse de manteau, et c'est exactement pour ça que je préfère qu'on la teste.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
@@ -6980,8 +7016,8 @@
       <c r="K95" s="10" t="inlineStr">
         <is>
           <t>Bonjour Josée Panet-Raymond,
-Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
-On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
+L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
 Je vous écris parce que vous couvrez l'agriculture. La question qui compte pour les producteurs n'a pas changé depuis l'effondrement de la filière en 2018 : est-ce qu'il y a un acheteur stable au bout du champ. On achète encore la récolte de producteurs d'ici et on la transforme nous-mêmes.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
@@ -7049,8 +7085,8 @@
       <c r="K96" s="10" t="inlineStr">
         <is>
           <t>Bonjour Yannick Patelli,
-Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
-On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
+L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
 Je vous écris parce que vous couvrez l'agriculture. La question qui compte pour les producteurs n'a pas changé depuis l'effondrement de la filière en 2018 : est-ce qu'il y a un acheteur stable au bout du champ. On achète encore la récolte de producteurs d'ici et on la transforme nous-mêmes.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
@@ -7118,8 +7154,8 @@
       <c r="K97" s="10" t="inlineStr">
         <is>
           <t>Bonjour Félix Pedneault,
-Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
-On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
+L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
 Je vous écris parce que vous couvrez l'environnement. Notre pari est économique avant d'être militant : si l'asclépiade devient payante, les agriculteurs la gardent dans leurs champs, et les monarques retrouvent de l'habitat de reproduction.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
@@ -7187,8 +7223,8 @@
       <c r="K98" s="10" t="inlineStr">
         <is>
           <t>Bonjour Marie-Eve Poulin,
-Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
-On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
+L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
 Je vous écris parce que vous couvrez le plein air. À poids égal, la littérature donne la soie d'asclépiade pour environ 10 % plus isolante que le duvet. C'est un repère de laboratoire, pas une promesse de manteau, et c'est exactement pour ça que je préfère qu'on la teste.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
@@ -7256,8 +7292,8 @@
       <c r="K99" s="10" t="inlineStr">
         <is>
           <t>Bonjour Marie-Hélène Proulx,
-Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
-On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
+L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
 Je vous écris parce que vous couvrez l'agriculture. La question qui compte pour les producteurs n'a pas changé depuis l'effondrement de la filière en 2018 : est-ce qu'il y a un acheteur stable au bout du champ. On achète encore la récolte de producteurs d'ici et on la transforme nous-mêmes.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
@@ -7325,8 +7361,8 @@
       <c r="K100" s="10" t="inlineStr">
         <is>
           <t>Bonjour Jean-Hugues Roy,
-Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
-On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
+L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
 Je vous écris parce que c'est une nouvelle de chez nous qui passe au national.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
@@ -7394,8 +7430,8 @@
       <c r="K101" s="10" t="inlineStr">
         <is>
           <t>Bonjour Martin Roy,
-Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
-On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
+L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
 Je vous écris parce que c'est une nouvelle de chez nous qui passe au national.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
@@ -7463,8 +7499,8 @@
       <c r="K102" s="10" t="inlineStr">
         <is>
           <t>Bonjour Sylvain Sarrazin,
-Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
-On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
+L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
 Je vous écris parce que vous couvrez le plein air. À poids égal, la littérature donne la soie d'asclépiade pour environ 10 % plus isolante que le duvet. C'est un repère de laboratoire, pas une promesse de manteau, et c'est exactement pour ça que je préfère qu'on la teste.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
@@ -7532,8 +7568,8 @@
       <c r="K103" s="10" t="inlineStr">
         <is>
           <t>Bonjour Pierre Sormany,
-Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
-On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
+L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
 Je vous écris parce que vous couvrez le plein air. À poids égal, la littérature donne la soie d'asclépiade pour environ 10 % plus isolante que le duvet. C'est un repère de laboratoire, pas une promesse de manteau, et c'est exactement pour ça que je préfère qu'on la teste.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
@@ -7601,8 +7637,8 @@
       <c r="K104" s="10" t="inlineStr">
         <is>
           <t>Bonjour Scott Stevenson,
-Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
-On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
+L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
 Je vous écris entre autres parce qu'une des premières usines de transformation de la fibre était à Granby, et que l'Estrie compte encore des producteurs d'asclépiade.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
@@ -7670,8 +7706,8 @@
       <c r="K105" s="10" t="inlineStr">
         <is>
           <t>Bonjour Michèle Tanganika,
-Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
-On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
+L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
 Je vous écris parce que vous couvrez l'agriculture. La question qui compte pour les producteurs n'a pas changé depuis l'effondrement de la filière en 2018 : est-ce qu'il y a un acheteur stable au bout du champ. On achète encore la récolte de producteurs d'ici et on la transforme nous-mêmes.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
@@ -7739,8 +7775,8 @@
       <c r="K106" s="10" t="inlineStr">
         <is>
           <t>Bonjour Stephane Tellier,
-Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
-On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
+L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
 Je vous écris parce que le sujet se raconte bien en ondes : une entreprise de Québec qui va expliquer à un auditoire pancanadien pourquoi la mauvaise herbe des champs de maïs peut isoler un manteau.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
@@ -7808,8 +7844,8 @@
       <c r="K107" s="10" t="inlineStr">
         <is>
           <t>Bonjour Karine Tremblay,
-Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
-On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
+L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
 Je vous écris entre autres parce qu'une des premières usines de transformation de la fibre était à Granby, et que l'Estrie compte encore des producteurs d'asclépiade.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
@@ -7877,8 +7913,8 @@
       <c r="K108" s="10" t="inlineStr">
         <is>
           <t>Bonjour Jean-Francois Venne,
-Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
-On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
+L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
 Je vous écris parce que vous couvrez l'environnement. Notre pari est économique avant d'être militant : si l'asclépiade devient payante, les agriculteurs la gardent dans leurs champs, et les monarques retrouvent de l'habitat de reproduction.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
@@ -7946,8 +7982,8 @@
       <c r="K109" s="10" t="inlineStr">
         <is>
           <t>Bonjour Shahram Yazdanpanah,
-Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
-On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
+L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
 Je vous écris parce que vous couvrez le plein air. À poids égal, la littérature donne la soie d'asclépiade pour environ 10 % plus isolante que le duvet. C'est un repère de laboratoire, pas une promesse de manteau, et c'est exactement pour ça que je préfère qu'on la teste.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
@@ -8015,8 +8051,8 @@
       <c r="K110" s="10" t="inlineStr">
         <is>
           <t>Bonjour Malika Alaoui,
-Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
-On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
+L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
 Je vous écris parce que vous couvrez l'art de vivre et la consommation. Le contraste se photographie bien : la gousse dans le champ, la soie blanche dans la main, le manteau porté en ville.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
@@ -8084,8 +8120,8 @@
       <c r="K111" s="10" t="inlineStr">
         <is>
           <t>Bonjour Yahia Arkat,
-Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
-On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
+L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
 Je vous écris parce que vous couvrez l'environnement. Notre pari est économique avant d'être militant : si l'asclépiade devient payante, les agriculteurs la gardent dans leurs champs, et les monarques retrouvent de l'habitat de reproduction.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
@@ -8153,8 +8189,8 @@
       <c r="K112" s="10" t="inlineStr">
         <is>
           <t>Bonjour MARC-OLIVIER BISSON,
-Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
-On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
+L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
 Je vous écris parce que vous couvrez l'agriculture. La question qui compte pour les producteurs n'a pas changé depuis l'effondrement de la filière en 2018 : est-ce qu'il y a un acheteur stable au bout du champ. On achète encore la récolte de producteurs d'ici et on la transforme nous-mêmes.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
@@ -8222,8 +8258,8 @@
       <c r="K113" s="10" t="inlineStr">
         <is>
           <t>Bonjour Maïté Belmir,
-Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
-On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
+L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
 Je vous écris parce que vous couvrez l'environnement. Notre pari est économique avant d'être militant : si l'asclépiade devient payante, les agriculteurs la gardent dans leurs champs, et les monarques retrouvent de l'habitat de reproduction.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
@@ -8291,8 +8327,8 @@
       <c r="K114" s="10" t="inlineStr">
         <is>
           <t>Bonjour André Bernard,
-Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
-On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
+L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
 Je vous écris parce que vous couvrez l'environnement. Notre pari est économique avant d'être militant : si l'asclépiade devient payante, les agriculteurs la gardent dans leurs champs, et les monarques retrouvent de l'habitat de reproduction.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
@@ -8360,8 +8396,8 @@
       <c r="K115" s="10" t="inlineStr">
         <is>
           <t>Bonjour Didier Bert,
-Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
-On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
+L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
 Je vous écris parce que vous couvrez l'environnement. Notre pari est économique avant d'être militant : si l'asclépiade devient payante, les agriculteurs la gardent dans leurs champs, et les monarques retrouvent de l'habitat de reproduction.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
@@ -8429,8 +8465,8 @@
       <c r="K116" s="10" t="inlineStr">
         <is>
           <t>Bonjour Sophie-Andrée Blondin,
-Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
-On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
+L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
 Je vous écris parce que le sujet se raconte bien en ondes : une entreprise de Québec qui va expliquer à un auditoire pancanadien pourquoi la mauvaise herbe des champs de maïs peut isoler un manteau.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
@@ -8498,8 +8534,8 @@
       <c r="K117" s="10" t="inlineStr">
         <is>
           <t>Bonjour Pierre Brochu,
-Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
-On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
+L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
 Je vous écris entre autres parce qu'une des premières usines de transformation de la fibre était à Granby, et que l'Estrie compte encore des producteurs d'asclépiade.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
@@ -8567,8 +8603,8 @@
       <c r="K118" s="10" t="inlineStr">
         <is>
           <t>Bonjour Gilles Bérubé,
-Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
-On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
+L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
 Je vous écris entre autres parce que la Montérégie est une des régions où l'asclépiade se cultive encore, et que c'est de champs comme ceux-là que vient la fibre qu'on transforme.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
@@ -8636,8 +8672,8 @@
       <c r="K119" s="10" t="inlineStr">
         <is>
           <t>Bonjour Daphné Cameron,
-Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
-On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
+L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
 Je vous écris parce que vous couvrez l'agriculture. La question qui compte pour les producteurs n'a pas changé depuis l'effondrement de la filière en 2018 : est-ce qu'il y a un acheteur stable au bout du champ. On achète encore la récolte de producteurs d'ici et on la transforme nous-mêmes.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
@@ -8705,8 +8741,8 @@
       <c r="K120" s="10" t="inlineStr">
         <is>
           <t>Bonjour Godefroy Macaire Chabi,
-Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
-On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
+L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
 Je vous écris parce que c'est une nouvelle de chez nous qui passe au national.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
@@ -8774,8 +8810,8 @@
       <c r="K121" s="10" t="inlineStr">
         <is>
           <t>Bonjour Sara Champagne,
-Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
-On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
+L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
 Je vous écris parce que vous couvrez l'environnement. Notre pari est économique avant d'être militant : si l'asclépiade devient payante, les agriculteurs la gardent dans leurs champs, et les monarques retrouvent de l'habitat de reproduction.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
@@ -8843,8 +8879,8 @@
       <c r="K122" s="10" t="inlineStr">
         <is>
           <t>Bonjour Sarah Champagne,
-Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
-On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
+L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
 Je vous écris parce que vous couvrez l'agriculture. La question qui compte pour les producteurs n'a pas changé depuis l'effondrement de la filière en 2018 : est-ce qu'il y a un acheteur stable au bout du champ. On achète encore la récolte de producteurs d'ici et on la transforme nous-mêmes.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
@@ -8912,8 +8948,8 @@
       <c r="K123" s="10" t="inlineStr">
         <is>
           <t>Bonjour Éric-Pierre Champagne,
-Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
-On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
+L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
 Je vous écris parce que vous couvrez l'environnement. Notre pari est économique avant d'être militant : si l'asclépiade devient payante, les agriculteurs la gardent dans leurs champs, et les monarques retrouvent de l'habitat de reproduction.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
@@ -8981,8 +9017,8 @@
       <c r="K124" s="10" t="inlineStr">
         <is>
           <t>Bonjour Marine Corniou,
-Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
-On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
+L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
 Je vous écris parce que vous couvrez l'environnement. Notre pari est économique avant d'être militant : si l'asclépiade devient payante, les agriculteurs la gardent dans leurs champs, et les monarques retrouvent de l'habitat de reproduction.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
@@ -9050,8 +9086,8 @@
       <c r="K125" s="10" t="inlineStr">
         <is>
           <t>Bonjour Catherine Crépeau,
-Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
-On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
+L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
 Je vous écris parce que vous couvrez l'environnement. Notre pari est économique avant d'être militant : si l'asclépiade devient payante, les agriculteurs la gardent dans leurs champs, et les monarques retrouvent de l'habitat de reproduction.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
@@ -9119,8 +9155,8 @@
       <c r="K126" s="10" t="inlineStr">
         <is>
           <t>Bonjour Laurence Dami-Houle,
-Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
-On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
+L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
 Je vous écris parce que c'est une nouvelle de chez nous qui passe au national.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
@@ -9188,8 +9224,8 @@
       <c r="K127" s="10" t="inlineStr">
         <is>
           <t>Bonjour Amélie Daoust-Boisvert,
-Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
-On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
+L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
 Je vous écris entre autres parce que la Montérégie est une des régions où l'asclépiade se cultive encore, et que c'est de champs comme ceux-là que vient la fibre qu'on transforme.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
@@ -9257,8 +9293,8 @@
       <c r="K128" s="10" t="inlineStr">
         <is>
           <t>Bonjour Dominique Degré,
-Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
-On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
+L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
 Je vous écris entre autres parce que la Montérégie est une des régions où l'asclépiade se cultive encore, et que c'est de champs comme ceux-là que vient la fibre qu'on transforme.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
@@ -9326,8 +9362,8 @@
       <c r="K129" s="10" t="inlineStr">
         <is>
           <t>Bonjour Quentin Dufranne,
-Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
-On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
+L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
 Je vous écris parce que vous couvrez l'environnement. Notre pari est économique avant d'être militant : si l'asclépiade devient payante, les agriculteurs la gardent dans leurs champs, et les monarques retrouvent de l'habitat de reproduction.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
@@ -9395,8 +9431,8 @@
       <c r="K130" s="10" t="inlineStr">
         <is>
           <t>Bonjour Ève Dumas,
-Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
-On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
+L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
 Je vous écris parce que vous couvrez l'agriculture. La question qui compte pour les producteurs n'a pas changé depuis l'effondrement de la filière en 2018 : est-ce qu'il y a un acheteur stable au bout du champ. On achète encore la récolte de producteurs d'ici et on la transforme nous-mêmes.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
@@ -9464,8 +9500,8 @@
       <c r="K131" s="10" t="inlineStr">
         <is>
           <t>Bonjour Michel Fortier,
-Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
-On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
+L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
 Je vous écris parce que c'est une nouvelle de chez nous qui passe au national.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
@@ -9533,8 +9569,8 @@
       <c r="K132" s="10" t="inlineStr">
         <is>
           <t>Bonjour Marie-Eve Fournier,
-Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
-On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
+L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
 Je vous écris parce que vous couvrez l'économie. On a bâti nos propres procédés de transformation parce qu'aucun sous-traitant ne voulait toucher à l'asclépiade, puis on a changé de modèle manufacturier l'an dernier pour rendre un manteau accessible à 300 $. J'en ai fait une vidéo ici : https://www.youtube.com/watch?v=GKyHh-Ok9JU.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
@@ -9602,8 +9638,8 @@
       <c r="K133" s="10" t="inlineStr">
         <is>
           <t>Bonjour Raymond Fournier,
-Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
-On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
+L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
 Je vous écris entre autres parce que la Montérégie est une des régions où l'asclépiade se cultive encore, et que c'est de champs comme ceux-là que vient la fibre qu'on transforme.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
@@ -9671,8 +9707,8 @@
       <c r="K134" s="10" t="inlineStr">
         <is>
           <t>Bonjour Marie-Pier Frappier,
-Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
-On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
+L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
 Je vous écris parce que vous couvrez l'économie. On a bâti nos propres procédés de transformation parce qu'aucun sous-traitant ne voulait toucher à l'asclépiade, puis on a changé de modèle manufacturier l'an dernier pour rendre un manteau accessible à 300 $. J'en ai fait une vidéo ici : https://www.youtube.com/watch?v=GKyHh-Ok9JU.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
@@ -9740,8 +9776,8 @@
       <c r="K135" s="10" t="inlineStr">
         <is>
           <t>Bonjour Marie-Julie Gagnon,
-Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
-On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
+L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
 Je vous écris entre autres parce que la Montérégie est une des régions où l'asclépiade se cultive encore, et que c'est de champs comme ceux-là que vient la fibre qu'on transforme.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
@@ -9809,8 +9845,8 @@
       <c r="K136" s="10" t="inlineStr">
         <is>
           <t>Bonjour Chloé Germain-Thérien,
-Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
-On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
+L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
 Je vous écris entre autres parce que l'asclépiade a eu son grand moment industriel chez vous : l'usine de Saint-Tite achetait 90 % des récoltes du Québec avant que la filière se casse en 2018. Des producteurs de la Mauricie cultivent encore, et on continue d'acheter leur récolte.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
@@ -9878,8 +9914,8 @@
       <c r="K137" s="10" t="inlineStr">
         <is>
           <t>Bonjour Charlotte Glorieux,
-Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
-On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
+L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
 Je vous écris parce que vous couvrez le plein air. À poids égal, la littérature donne la soie d'asclépiade pour environ 10 % plus isolante que le duvet. C'est un repère de laboratoire, pas une promesse de manteau, et c'est exactement pour ça que je préfère qu'on la teste.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
@@ -9947,8 +9983,8 @@
       <c r="K138" s="10" t="inlineStr">
         <is>
           <t>Bonjour Annie Hudon,
-Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
-On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
+L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
 Je vous écris parce que vous couvrez l'économie. On a bâti nos propres procédés de transformation parce qu'aucun sous-traitant ne voulait toucher à l'asclépiade, puis on a changé de modèle manufacturier l'an dernier pour rendre un manteau accessible à 300 $. J'en ai fait une vidéo ici : https://www.youtube.com/watch?v=GKyHh-Ok9JU.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
@@ -10016,8 +10052,8 @@
       <c r="K139" s="10" t="inlineStr">
         <is>
           <t>Bonjour Ahmed Kouaou,
-Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
-On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
+L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
 Je vous écris parce que vous couvrez l'environnement. Notre pari est économique avant d'être militant : si l'asclépiade devient payante, les agriculteurs la gardent dans leurs champs, et les monarques retrouvent de l'habitat de reproduction.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
@@ -10085,8 +10121,8 @@
       <c r="K140" s="10" t="inlineStr">
         <is>
           <t>Bonjour Tania Krywiak,
-Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
-On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
+L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
 Je vous écris parce que vous couvrez l'environnement. Notre pari est économique avant d'être militant : si l'asclépiade devient payante, les agriculteurs la gardent dans leurs champs, et les monarques retrouvent de l'habitat de reproduction.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
@@ -10154,8 +10190,8 @@
       <c r="K141" s="10" t="inlineStr">
         <is>
           <t>Bonjour Jacinthe Lafrance,
-Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
-On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
+L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
 Je vous écris entre autres parce que l'asclépiade a eu son grand moment industriel chez vous : l'usine de Saint-Tite achetait 90 % des récoltes du Québec avant que la filière se casse en 2018. Des producteurs de la Mauricie cultivent encore, et on continue d'acheter leur récolte.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
@@ -10223,8 +10259,8 @@
       <c r="K142" s="10" t="inlineStr">
         <is>
           <t>Bonjour Bruno Lamolet,
-Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
-On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
+L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
 Je vous écris entre autres parce que la Montérégie est une des régions où l'asclépiade se cultive encore, et que c'est de champs comme ceux-là que vient la fibre qu'on transforme.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
@@ -10292,8 +10328,8 @@
       <c r="K143" s="10" t="inlineStr">
         <is>
           <t>Bonjour Yvan Lamontagne,
-Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
-On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
+L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
 Je vous écris entre autres parce qu'une des premières usines de transformation de la fibre était à Granby, et que l'Estrie compte encore des producteurs d'asclépiade.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
@@ -10361,8 +10397,8 @@
       <c r="K144" s="10" t="inlineStr">
         <is>
           <t>Bonjour Yves Langlois,
-Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
-On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
+L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
 Je vous écris entre autres parce qu'une des premières usines de transformation de la fibre était à Granby, et que l'Estrie compte encore des producteurs d'asclépiade.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
@@ -10430,8 +10466,8 @@
       <c r="K145" s="10" t="inlineStr">
         <is>
           <t>Bonjour Anne Marie Lecomte,
-Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
-On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
+L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
 Je vous écris parce que vous couvrez l'économie. On a bâti nos propres procédés de transformation parce qu'aucun sous-traitant ne voulait toucher à l'asclépiade, puis on a changé de modèle manufacturier l'an dernier pour rendre un manteau accessible à 300 $. J'en ai fait une vidéo ici : https://www.youtube.com/watch?v=GKyHh-Ok9JU.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
@@ -10499,8 +10535,8 @@
       <c r="K146" s="10" t="inlineStr">
         <is>
           <t>Bonjour Stéphanie Mac Farlane,
-Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
-On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
+L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
 Je vous écris entre autres parce que la Montérégie est une des régions où l'asclépiade se cultive encore, et que c'est de champs comme ceux-là que vient la fibre qu'on transforme.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
@@ -10568,8 +10604,8 @@
       <c r="K147" s="10" t="inlineStr">
         <is>
           <t>Bonjour Philippe Marois,
-Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
-On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
+L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
 Je vous écris entre autres parce que la Montérégie est une des régions où l'asclépiade se cultive encore, et que c'est de champs comme ceux-là que vient la fibre qu'on transforme.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
@@ -10637,8 +10673,8 @@
       <c r="K148" s="10" t="inlineStr">
         <is>
           <t>Bonjour Gildas Meneu,
-Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
-On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
+L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
 Je vous écris parce que vous couvrez l'agriculture. La question qui compte pour les producteurs n'a pas changé depuis l'effondrement de la filière en 2018 : est-ce qu'il y a un acheteur stable au bout du champ. On achète encore la récolte de producteurs d'ici et on la transforme nous-mêmes.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
@@ -10706,8 +10742,8 @@
       <c r="K149" s="10" t="inlineStr">
         <is>
           <t>Bonjour Louis-Xavier Michaud,
-Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
-On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
+L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
 Je vous écris parce que c'est une nouvelle de chez nous qui passe au national.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
@@ -10775,8 +10811,8 @@
       <c r="K150" s="10" t="inlineStr">
         <is>
           <t>Bonjour Anne Montplaisir,
-Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
-On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
+L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
 Je vous écris parce que vous couvrez le plein air. À poids égal, la littérature donne la soie d'asclépiade pour environ 10 % plus isolante que le duvet. C'est un repère de laboratoire, pas une promesse de manteau, et c'est exactement pour ça que je préfère qu'on la teste.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
@@ -10844,8 +10880,8 @@
       <c r="K151" s="10" t="inlineStr">
         <is>
           <t>Bonjour Karianne Nepton-Philippe,
-Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
-On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
+L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
 Je vous écris parce que c'est une nouvelle de chez nous qui passe au national.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
@@ -10913,8 +10949,8 @@
       <c r="K152" s="10" t="inlineStr">
         <is>
           <t>Bonjour Geneviève Normand,
-Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
-On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
+L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
 Je vous écris entre autres parce que la Montérégie est une des régions où l'asclépiade se cultive encore, et que c'est de champs comme ceux-là que vient la fibre qu'on transforme.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
@@ -10982,8 +11018,8 @@
       <c r="K153" s="10" t="inlineStr">
         <is>
           <t>Bonjour Carole Payer,
-Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
-On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
+L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
 Je vous écris entre autres parce que l'asclépiade se cultive dans votre région depuis la première vague de 2013, et que plusieurs des producteurs qui ont tenu bon nous vendent encore leur récolte.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
@@ -11051,8 +11087,8 @@
       <c r="K154" s="10" t="inlineStr">
         <is>
           <t>Bonjour Boris Proulx,
-Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
-On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
+L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
 Je vous écris parce que vous couvrez l'environnement. Notre pari est économique avant d'être militant : si l'asclépiade devient payante, les agriculteurs la gardent dans leurs champs, et les monarques retrouvent de l'habitat de reproduction.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
@@ -11120,8 +11156,8 @@
       <c r="K155" s="10" t="inlineStr">
         <is>
           <t>Bonjour Philippe Robitaille-Grou,
-Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
-On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
+L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
 Je vous écris parce que vous couvrez l'environnement. Notre pari est économique avant d'être militant : si l'asclépiade devient payante, les agriculteurs la gardent dans leurs champs, et les monarques retrouvent de l'habitat de reproduction.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
@@ -11189,8 +11225,8 @@
       <c r="K156" s="10" t="inlineStr">
         <is>
           <t>Bonjour Gwen Roley,
-Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
-On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
+L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
 Je vous écris parce que vous couvrez l'environnement. Notre pari est économique avant d'être militant : si l'asclépiade devient payante, les agriculteurs la gardent dans leurs champs, et les monarques retrouvent de l'habitat de reproduction.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
@@ -11258,8 +11294,8 @@
       <c r="K157" s="10" t="inlineStr">
         <is>
           <t>Bonjour Mathieu-Robert Sauvé,
-Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
-On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
+L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
 Je vous écris parce que vous couvrez l'environnement. Notre pari est économique avant d'être militant : si l'asclépiade devient payante, les agriculteurs la gardent dans leurs champs, et les monarques retrouvent de l'habitat de reproduction.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
@@ -11327,8 +11363,8 @@
       <c r="K158" s="10" t="inlineStr">
         <is>
           <t>Bonjour Pierre St-Arnaud,
-Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
-On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
+L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
 Je vous écris parce que vous couvrez l'agriculture. La question qui compte pour les producteurs n'a pas changé depuis l'effondrement de la filière en 2018 : est-ce qu'il y a un acheteur stable au bout du champ. On achète encore la récolte de producteurs d'ici et on la transforme nous-mêmes.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
@@ -11396,8 +11432,8 @@
       <c r="K159" s="10" t="inlineStr">
         <is>
           <t>Bonjour Katherine Tremblay,
-Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
-On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
+L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
 Je vous écris entre autres parce que la Montérégie est une des régions où l'asclépiade se cultive encore, et que c'est de champs comme ceux-là que vient la fibre qu'on transforme.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
@@ -11465,8 +11501,8 @@
       <c r="K160" s="10" t="inlineStr">
         <is>
           <t>Bonjour Michel Tremblay,
-Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
-On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
+L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
 Je vous écris entre autres parce que l'asclépiade se cultive dans votre région depuis la première vague de 2013, et que plusieurs des producteurs qui ont tenu bon nous vendent encore leur récolte.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
@@ -11534,8 +11570,8 @@
       <c r="K161" s="10" t="inlineStr">
         <is>
           <t>Bonjour Martin Vallières,
-Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
-On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
+L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
 Je vous écris parce que vous couvrez l'économie. On a bâti nos propres procédés de transformation parce qu'aucun sous-traitant ne voulait toucher à l'asclépiade, puis on a changé de modèle manufacturier l'an dernier pour rendre un manteau accessible à 300 $. J'en ai fait une vidéo ici : https://www.youtube.com/watch?v=GKyHh-Ok9JU.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
@@ -11603,8 +11639,8 @@
       <c r="K162" s="10" t="inlineStr">
         <is>
           <t>Bonjour Yanick Villedieu,
-Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
-On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
+L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
 Je vous écris parce que vous couvrez l'environnement. Notre pari est économique avant d'être militant : si l'asclépiade devient payante, les agriculteurs la gardent dans leurs champs, et les monarques retrouvent de l'habitat de reproduction.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
@@ -11672,8 +11708,8 @@
       <c r="K163" s="10" t="inlineStr">
         <is>
           <t>Bonjour Jonathan Allard,
-Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
-On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
+L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
 Je vous écris parce que vous couvrez l'environnement. Notre pari est économique avant d'être militant : si l'asclépiade devient payante, les agriculteurs la gardent dans leurs champs, et les monarques retrouvent de l'habitat de reproduction.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
@@ -11741,8 +11777,8 @@
       <c r="K164" s="10" t="inlineStr">
         <is>
           <t>Bonjour Anick Baribeau,
-Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
-On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
+L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
 Je vous écris entre autres parce que l'asclépiade a eu son grand moment industriel chez vous : l'usine de Saint-Tite achetait 90 % des récoltes du Québec avant que la filière se casse en 2018. Des producteurs de la Mauricie cultivent encore, et on continue d'acheter leur récolte.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
@@ -11810,8 +11846,8 @@
       <c r="K165" s="10" t="inlineStr">
         <is>
           <t>Bonjour Félix-Antoine Beauchemin,
-Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
-On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
+L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
 Je vous écris entre autres parce que la Montérégie est une des régions où l'asclépiade se cultive encore, et que c'est de champs comme ceux-là que vient la fibre qu'on transforme.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
@@ -11879,8 +11915,8 @@
       <c r="K166" s="10" t="inlineStr">
         <is>
           <t>Bonjour Karim Benessaieh,
-Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
-On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
+L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
 Je vous écris parce que vous couvrez l'environnement. Notre pari est économique avant d'être militant : si l'asclépiade devient payante, les agriculteurs la gardent dans leurs champs, et les monarques retrouvent de l'habitat de reproduction.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
@@ -11948,8 +11984,8 @@
       <c r="K167" s="10" t="inlineStr">
         <is>
           <t>Bonjour Julia Bernier,
-Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
-On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
+L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
 Je vous écris entre autres parce que l'asclépiade se cultive dans votre région depuis la première vague de 2013, et que plusieurs des producteurs qui ont tenu bon nous vendent encore leur récolte.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
@@ -12017,8 +12053,8 @@
       <c r="K168" s="10" t="inlineStr">
         <is>
           <t>Bonjour Karine Boivin Forcier,
-Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
-On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
+L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
 Je vous écris entre autres parce qu'un de nos fournisseurs d'asclépiade cultive au Lac-Saint-Jean depuis nos tout débuts, et qu'il l'est encore aujourd'hui. La fibre de chez vous se retrouve dans nos produits.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
@@ -12086,8 +12122,8 @@
       <c r="K169" s="10" t="inlineStr">
         <is>
           <t>Bonjour Audrey Bonaque,
-Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
-On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
+L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
 Je vous écris parce que le sujet se raconte bien en ondes : une entreprise de Québec qui va expliquer à un auditoire pancanadien pourquoi la mauvaise herbe des champs de maïs peut isoler un manteau.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
@@ -12155,8 +12191,8 @@
       <c r="K170" s="10" t="inlineStr">
         <is>
           <t>Bonjour Luc Boulanger,
-Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
-On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
+L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
 Je vous écris parce que vous couvrez l'art de vivre et la consommation. Le contraste se photographie bien : la gousse dans le champ, la soie blanche dans la main, le manteau porté en ville.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
@@ -12224,8 +12260,8 @@
       <c r="K171" s="10" t="inlineStr">
         <is>
           <t>Bonjour Mario Boulianne,
-Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
-On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
+L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
 Je vous écris parce que c'est une nouvelle de chez nous qui passe au national.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
@@ -12293,8 +12329,8 @@
       <c r="K172" s="10" t="inlineStr">
         <is>
           <t>Bonjour Bernard Brault,
-Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
-On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
+L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
 Je vous écris entre autres parce que la Montérégie est une des régions où l'asclépiade se cultive encore, et que c'est de champs comme ceux-là que vient la fibre qu'on transforme.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
@@ -12362,8 +12398,8 @@
       <c r="K173" s="10" t="inlineStr">
         <is>
           <t>Bonjour Pierre Brisson,
-Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
-On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
+L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
 Je vous écris parce que vous couvrez l'économie. On a bâti nos propres procédés de transformation parce qu'aucun sous-traitant ne voulait toucher à l'asclépiade, puis on a changé de modèle manufacturier l'an dernier pour rendre un manteau accessible à 300 $. J'en ai fait une vidéo ici : https://www.youtube.com/watch?v=GKyHh-Ok9JU.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
@@ -12431,8 +12467,8 @@
       <c r="K174" s="10" t="inlineStr">
         <is>
           <t>Bonjour Laurence Brisson Dubreuil,
-Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
-On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
+L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
 Je vous écris parce que le sujet se raconte bien en ondes : une entreprise de Québec qui va expliquer à un auditoire pancanadien pourquoi la mauvaise herbe des champs de maïs peut isoler un manteau.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
@@ -12500,8 +12536,8 @@
       <c r="K175" s="10" t="inlineStr">
         <is>
           <t>Bonjour Nathaniel Bronner,
-Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
-On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
+L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
 Je vous écris parce que le sujet se raconte bien en ondes : une entreprise de Québec qui va expliquer à un auditoire pancanadien pourquoi la mauvaise herbe des champs de maïs peut isoler un manteau.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
@@ -12569,8 +12605,8 @@
       <c r="K176" s="10" t="inlineStr">
         <is>
           <t>Bonjour Marie-France Bélanger,
-Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
-On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
+L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
 Je vous écris parce que vous couvrez l'art de vivre et la consommation. Le contraste se photographie bien : la gousse dans le champ, la soie blanche dans la main, le manteau porté en ville.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
@@ -12638,8 +12674,8 @@
       <c r="K177" s="10" t="inlineStr">
         <is>
           <t>Bonjour Diane Bérard,
-Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
-On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
+L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
 Je vous écris parce que vous couvrez l'économie. On a bâti nos propres procédés de transformation parce qu'aucun sous-traitant ne voulait toucher à l'asclépiade, puis on a changé de modèle manufacturier l'an dernier pour rendre un manteau accessible à 300 $. J'en ai fait une vidéo ici : https://www.youtube.com/watch?v=GKyHh-Ok9JU.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
@@ -12707,8 +12743,8 @@
       <c r="K178" s="10" t="inlineStr">
         <is>
           <t>Bonjour Julien Cayouette,
-Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
-On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
+L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
 Je vous écris parce que vous couvrez l'environnement. Notre pari est économique avant d'être militant : si l'asclépiade devient payante, les agriculteurs la gardent dans leurs champs, et les monarques retrouvent de l'habitat de reproduction.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
@@ -12776,8 +12812,8 @@
       <c r="K179" s="10" t="inlineStr">
         <is>
           <t>Bonjour Rudy Chabannes,
-Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
-On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
+L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
 Je vous écris parce que le sujet se raconte bien en ondes : une entreprise de Québec qui va expliquer à un auditoire pancanadien pourquoi la mauvaise herbe des champs de maïs peut isoler un manteau.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
@@ -12845,8 +12881,8 @@
       <c r="K180" s="10" t="inlineStr">
         <is>
           <t>Bonjour Denis-Martin Chabot,
-Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
-On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
+L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
 Je vous écris parce que le sujet se raconte bien en ondes : une entreprise de Québec qui va expliquer à un auditoire pancanadien pourquoi la mauvaise herbe des champs de maïs peut isoler un manteau.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
@@ -12914,8 +12950,8 @@
       <c r="K181" s="10" t="inlineStr">
         <is>
           <t>Bonjour Loubna Majda Chourouk,
-Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
-On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
+L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
 Je vous écris parce que le sujet se raconte bien en ondes : une entreprise de Québec qui va expliquer à un auditoire pancanadien pourquoi la mauvaise herbe des champs de maïs peut isoler un manteau.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
@@ -12983,8 +13019,8 @@
       <c r="K182" s="10" t="inlineStr">
         <is>
           <t>Bonjour Sarah Collardey,
-Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
-On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
+L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
 Je vous écris parce que vous couvrez l'environnement. Notre pari est économique avant d'être militant : si l'asclépiade devient payante, les agriculteurs la gardent dans leurs champs, et les monarques retrouvent de l'habitat de reproduction.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
@@ -13052,8 +13088,8 @@
       <c r="K183" s="10" t="inlineStr">
         <is>
           <t>Bonjour Kathleen Couillard,
-Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
-On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
+L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
 Je vous écris entre autres parce que la Montérégie est une des régions où l'asclépiade se cultive encore, et que c'est de champs comme ceux-là que vient la fibre qu'on transforme.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
@@ -13121,8 +13157,8 @@
       <c r="K184" s="10" t="inlineStr">
         <is>
           <t>Bonjour Oumou DIAKITÉ,
-Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
-On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
+L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
 Je vous écris parce que vous couvrez l'art de vivre et la consommation. Le contraste se photographie bien : la gousse dans le champ, la soie blanche dans la main, le manteau porté en ville.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
@@ -13190,8 +13226,8 @@
       <c r="K185" s="10" t="inlineStr">
         <is>
           <t>Bonjour Agnès Delavault,
-Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
-On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
+L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
 Je vous écris parce que vous couvrez l'art de vivre et la consommation. Le contraste se photographie bien : la gousse dans le champ, la soie blanche dans la main, le manteau porté en ville.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
@@ -13259,8 +13295,8 @@
       <c r="K186" s="10" t="inlineStr">
         <is>
           <t>Bonjour Marcelin Delice,
-Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
-On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
+L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
 Je vous écris parce que vous couvrez l'environnement. Notre pari est économique avant d'être militant : si l'asclépiade devient payante, les agriculteurs la gardent dans leurs champs, et les monarques retrouvent de l'habitat de reproduction.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
@@ -13328,8 +13364,8 @@
       <c r="K187" s="10" t="inlineStr">
         <is>
           <t>Bonjour Alain Demers,
-Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
-On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
+L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
 Je vous écris parce que vous couvrez le plein air. À poids égal, la littérature donne la soie d'asclépiade pour environ 10 % plus isolante que le duvet. C'est un repère de laboratoire, pas une promesse de manteau, et c'est exactement pour ça que je préfère qu'on la teste.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
@@ -13397,8 +13433,8 @@
       <c r="K188" s="10" t="inlineStr">
         <is>
           <t>Bonjour Ivanoh Demers,
-Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
-On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
+L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
 Je vous écris parce que vous couvrez l'économie. On a bâti nos propres procédés de transformation parce qu'aucun sous-traitant ne voulait toucher à l'asclépiade, puis on a changé de modèle manufacturier l'an dernier pour rendre un manteau accessible à 300 $. J'en ai fait une vidéo ici : https://www.youtube.com/watch?v=GKyHh-Ok9JU.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
@@ -13466,8 +13502,8 @@
       <c r="K189" s="10" t="inlineStr">
         <is>
           <t>Bonjour Claude Deschênes,
-Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
-On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
+L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
 Je vous écris parce que vous couvrez l'art de vivre et la consommation. Le contraste se photographie bien : la gousse dans le champ, la soie blanche dans la main, le manteau porté en ville.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
@@ -13535,8 +13571,8 @@
       <c r="K190" s="10" t="inlineStr">
         <is>
           <t>Bonjour Thomas Deshaies,
-Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
-On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
+L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
 Je vous écris entre autres parce qu'une des premières usines de transformation de la fibre était à Granby, et que l'Estrie compte encore des producteurs d'asclépiade.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
@@ -13604,8 +13640,8 @@
       <c r="K191" s="10" t="inlineStr">
         <is>
           <t>Bonjour Claude Desjardins,
-Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
-On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
+L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
 Je vous écris parce que vous couvrez l'économie. On a bâti nos propres procédés de transformation parce qu'aucun sous-traitant ne voulait toucher à l'asclépiade, puis on a changé de modèle manufacturier l'an dernier pour rendre un manteau accessible à 300 $. J'en ai fait une vidéo ici : https://www.youtube.com/watch?v=GKyHh-Ok9JU.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
@@ -13673,8 +13709,8 @@
       <c r="K192" s="10" t="inlineStr">
         <is>
           <t>Bonjour Martine Deslauriers,
-Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
-On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
+L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
 Je vous écris parce que vous couvrez l'environnement. Notre pari est économique avant d'être militant : si l'asclépiade devient payante, les agriculteurs la gardent dans leurs champs, et les monarques retrouvent de l'habitat de reproduction.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
@@ -13742,8 +13778,8 @@
       <c r="K193" s="10" t="inlineStr">
         <is>
           <t>Bonjour Marie-Claude Di Lillo,
-Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
-On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
+L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
 Je vous écris parce que c'est une nouvelle de chez nous qui passe au national.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
@@ -13811,8 +13847,8 @@
       <c r="K194" s="10" t="inlineStr">
         <is>
           <t>Bonjour Jean-René Dufort,
-Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
-On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
+L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
 Je vous écris parce que le sujet se raconte bien en ondes : une entreprise de Québec qui va expliquer à un auditoire pancanadien pourquoi la mauvaise herbe des champs de maïs peut isoler un manteau.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
@@ -13880,8 +13916,8 @@
       <c r="K195" s="10" t="inlineStr">
         <is>
           <t>Bonjour Richard Dupaul,
-Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
-On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
+L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
 Je vous écris parce que vous couvrez l'économie. On a bâti nos propres procédés de transformation parce qu'aucun sous-traitant ne voulait toucher à l'asclépiade, puis on a changé de modèle manufacturier l'an dernier pour rendre un manteau accessible à 300 $. J'en ai fait une vidéo ici : https://www.youtube.com/watch?v=GKyHh-Ok9JU.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
@@ -13949,8 +13985,8 @@
       <c r="K196" s="10" t="inlineStr">
         <is>
           <t>Bonjour Stéphanie Dupuis,
-Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
-On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
+L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
 Je vous écris parce que vous couvrez l'art de vivre et la consommation. Le contraste se photographie bien : la gousse dans le champ, la soie blanche dans la main, le manteau porté en ville.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
@@ -14018,8 +14054,8 @@
       <c r="K197" s="10" t="inlineStr">
         <is>
           <t>Bonjour Maxim Fauteux,
-Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
-On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
+L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
 Je vous écris entre autres parce qu'un de nos fournisseurs d'asclépiade cultive au Lac-Saint-Jean depuis nos tout débuts, et qu'il l'est encore aujourd'hui. La fibre de chez vous se retrouve dans nos produits.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
@@ -14087,8 +14123,8 @@
       <c r="K198" s="10" t="inlineStr">
         <is>
           <t>Bonjour Ronald Georges,
-Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
-On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
+L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
 Je vous écris parce que le sujet se raconte bien en ondes : une entreprise de Québec qui va expliquer à un auditoire pancanadien pourquoi la mauvaise herbe des champs de maïs peut isoler un manteau.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
@@ -14156,8 +14192,8 @@
       <c r="K199" s="10" t="inlineStr">
         <is>
           <t>Bonjour Stéphane Giroux,
-Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
-On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
+L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
 Je vous écris parce que vous couvrez l'économie. On a bâti nos propres procédés de transformation parce qu'aucun sous-traitant ne voulait toucher à l'asclépiade, puis on a changé de modèle manufacturier l'an dernier pour rendre un manteau accessible à 300 $. J'en ai fait une vidéo ici : https://www.youtube.com/watch?v=GKyHh-Ok9JU.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
@@ -14225,8 +14261,8 @@
       <c r="K200" s="10" t="inlineStr">
         <is>
           <t>Bonjour Zacharie Goudreault,
-Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
-On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
+L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
 Je vous écris parce que vous couvrez l'environnement. Notre pari est économique avant d'être militant : si l'asclépiade devient payante, les agriculteurs la gardent dans leurs champs, et les monarques retrouvent de l'habitat de reproduction.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
@@ -14294,8 +14330,8 @@
       <c r="K201" s="10" t="inlineStr">
         <is>
           <t>Bonjour Isabelle Grégoire,
-Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
-On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
+L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
 Je vous écris parce que vous couvrez l'art de vivre et la consommation. Le contraste se photographie bien : la gousse dans le champ, la soie blanche dans la main, le manteau porté en ville.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
@@ -14363,8 +14399,8 @@
       <c r="K202" s="10" t="inlineStr">
         <is>
           <t>Bonjour Chantal Guy,
-Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
-On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
+L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
 Je vous écris parce que vous couvrez l'art de vivre et la consommation. Le contraste se photographie bien : la gousse dans le champ, la soie blanche dans la main, le manteau porté en ville.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
@@ -14432,8 +14468,8 @@
       <c r="K203" s="10" t="inlineStr">
         <is>
           <t>Bonjour Matthieu Hains,
-Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
-On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
+L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
 Je vous écris parce que vous couvrez l'économie. On a bâti nos propres procédés de transformation parce qu'aucun sous-traitant ne voulait toucher à l'asclépiade, puis on a changé de modèle manufacturier l'an dernier pour rendre un manteau accessible à 300 $. J'en ai fait une vidéo ici : https://www.youtube.com/watch?v=GKyHh-Ok9JU.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
@@ -14557,8 +14593,8 @@
       <c r="K205" s="10" t="inlineStr">
         <is>
           <t>Bonjour ANGELO JEAN-BAPTISTE,
-Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
-On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
+L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
 Je vous écris parce que vous couvrez l'environnement. Notre pari est économique avant d'être militant : si l'asclépiade devient payante, les agriculteurs la gardent dans leurs champs, et les monarques retrouvent de l'habitat de reproduction.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
@@ -14626,8 +14662,8 @@
       <c r="K206" s="10" t="inlineStr">
         <is>
           <t>Bonjour Andréanne Joly,
-Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
-On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
+L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
 Je vous écris parce que vous couvrez l'art de vivre et la consommation. Le contraste se photographie bien : la gousse dans le champ, la soie blanche dans la main, le manteau porté en ville.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
@@ -14695,8 +14731,8 @@
       <c r="K207" s="10" t="inlineStr">
         <is>
           <t>Bonjour Hugo Joncas,
-Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
-On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
+L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
 Je vous écris parce que vous couvrez l'économie. On a bâti nos propres procédés de transformation parce qu'aucun sous-traitant ne voulait toucher à l'asclépiade, puis on a changé de modèle manufacturier l'an dernier pour rendre un manteau accessible à 300 $. J'en ai fait une vidéo ici : https://www.youtube.com/watch?v=GKyHh-Ok9JU.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
@@ -14764,8 +14800,8 @@
       <c r="K208" s="10" t="inlineStr">
         <is>
           <t>Bonjour Philémon La Frenière-Prémont,
-Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
-On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
+L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
 Je vous écris parce que le sujet se raconte bien en ondes : une entreprise de Québec qui va expliquer à un auditoire pancanadien pourquoi la mauvaise herbe des champs de maïs peut isoler un manteau.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
@@ -14833,8 +14869,8 @@
       <c r="K209" s="10" t="inlineStr">
         <is>
           <t>Bonjour Henri Laban,
-Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
-On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
+L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
 Je vous écris parce que le sujet se raconte bien en ondes : une entreprise de Québec qui va expliquer à un auditoire pancanadien pourquoi la mauvaise herbe des champs de maïs peut isoler un manteau.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
@@ -14958,8 +14994,8 @@
       <c r="K211" s="10" t="inlineStr">
         <is>
           <t>Bonjour Joannie Lafrenière,
-Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
-On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
+L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
 Je vous écris parce que vous couvrez l'art de vivre et la consommation. Le contraste se photographie bien : la gousse dans le champ, la soie blanche dans la main, le manteau porté en ville.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
@@ -15027,8 +15063,8 @@
       <c r="K212" s="10" t="inlineStr">
         <is>
           <t>Bonjour Angie Landry,
-Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
-On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
+L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
 Je vous écris parce que vous couvrez l'environnement. Notre pari est économique avant d'être militant : si l'asclépiade devient payante, les agriculteurs la gardent dans leurs champs, et les monarques retrouvent de l'habitat de reproduction.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
@@ -15096,8 +15132,8 @@
       <c r="K213" s="10" t="inlineStr">
         <is>
           <t>Bonjour Camille Langlade,
-Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
-On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
+L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
 Je vous écris parce que vous couvrez l'environnement. Notre pari est économique avant d'être militant : si l'asclépiade devient payante, les agriculteurs la gardent dans leurs champs, et les monarques retrouvent de l'habitat de reproduction.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
@@ -15165,8 +15201,8 @@
       <c r="K214" s="10" t="inlineStr">
         <is>
           <t>Bonjour Claudia Larochelle,
-Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
-On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
+L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
 Je vous écris parce que le sujet se raconte bien en ondes : une entreprise de Québec qui va expliquer à un auditoire pancanadien pourquoi la mauvaise herbe des champs de maïs peut isoler un manteau.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
@@ -15234,8 +15270,8 @@
       <c r="K215" s="10" t="inlineStr">
         <is>
           <t>Bonjour Étienne Leblanc,
-Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
-On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
+L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
 Je vous écris parce que vous couvrez l'environnement. Notre pari est économique avant d'être militant : si l'asclépiade devient payante, les agriculteurs la gardent dans leurs champs, et les monarques retrouvent de l'habitat de reproduction.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
@@ -15303,8 +15339,8 @@
       <c r="K216" s="10" t="inlineStr">
         <is>
           <t>Bonjour Louise Leduc,
-Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
-On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
+L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
 Je vous écris parce que vous couvrez l'art de vivre et la consommation. Le contraste se photographie bien : la gousse dans le champ, la soie blanche dans la main, le manteau porté en ville.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
@@ -15372,8 +15408,8 @@
       <c r="K217" s="10" t="inlineStr">
         <is>
           <t>Bonjour Guillaume Longuépée,
-Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
-On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
+L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
 Je vous écris parce que vous couvrez l'économie. On a bâti nos propres procédés de transformation parce qu'aucun sous-traitant ne voulait toucher à l'asclépiade, puis on a changé de modèle manufacturier l'an dernier pour rendre un manteau accessible à 300 $. J'en ai fait une vidéo ici : https://www.youtube.com/watch?v=GKyHh-Ok9JU.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
@@ -15441,8 +15477,8 @@
       <c r="K218" s="10" t="inlineStr">
         <is>
           <t>Bonjour Roxane Léouzon,
-Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
-On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
+L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
 Je vous écris parce que vous couvrez l'économie. On a bâti nos propres procédés de transformation parce qu'aucun sous-traitant ne voulait toucher à l'asclépiade, puis on a changé de modèle manufacturier l'an dernier pour rendre un manteau accessible à 300 $. J'en ai fait une vidéo ici : https://www.youtube.com/watch?v=GKyHh-Ok9JU.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
@@ -15510,8 +15546,8 @@
       <c r="K219" s="10" t="inlineStr">
         <is>
           <t>Bonjour Ève Lévesque,
-Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
-On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
+L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
 Je vous écris parce que le sujet se raconte bien en ondes : une entreprise de Québec qui va expliquer à un auditoire pancanadien pourquoi la mauvaise herbe des champs de maïs peut isoler un manteau.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
@@ -15579,8 +15615,8 @@
       <c r="K220" s="10" t="inlineStr">
         <is>
           <t>Bonjour Sophie Mangado,
-Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
-On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
+L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
 Je vous écris parce que le sujet se raconte bien en ondes : une entreprise de Québec qui va expliquer à un auditoire pancanadien pourquoi la mauvaise herbe des champs de maïs peut isoler un manteau.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
@@ -15648,8 +15684,8 @@
       <c r="K221" s="10" t="inlineStr">
         <is>
           <t>Bonjour Colin McGregor,
-Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
-On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
+L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
 Je vous écris parce que vous couvrez l'environnement. Notre pari est économique avant d'être militant : si l'asclépiade devient payante, les agriculteurs la gardent dans leurs champs, et les monarques retrouvent de l'habitat de reproduction.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
@@ -15717,8 +15753,8 @@
       <c r="K222" s="10" t="inlineStr">
         <is>
           <t>Bonjour Isabelle Morin,
-Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
-On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
+L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
 Je vous écris parce que vous couvrez l'art de vivre et la consommation. Le contraste se photographie bien : la gousse dans le champ, la soie blanche dans la main, le manteau porté en ville.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
@@ -15786,8 +15822,8 @@
       <c r="K223" s="10" t="inlineStr">
         <is>
           <t>Bonjour Timothy Morson,
-Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
-On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
+L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
 Je vous écris entre autres parce que l'asclépiade se cultive dans votre région depuis la première vague de 2013, et que plusieurs des producteurs qui ont tenu bon nous vendent encore leur récolte.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
@@ -15855,8 +15891,8 @@
       <c r="K224" s="10" t="inlineStr">
         <is>
           <t>Bonjour Rachid Najahi,
-Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
-On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
+L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
 Je vous écris parce que vous couvrez l'art de vivre et la consommation. Le contraste se photographie bien : la gousse dans le champ, la soie blanche dans la main, le manteau porté en ville.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
@@ -15924,8 +15960,8 @@
       <c r="K225" s="10" t="inlineStr">
         <is>
           <t>Bonjour Richard Olivier,
-Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
-On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
+L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
 Je vous écris parce que le sujet se raconte bien en ondes : une entreprise de Québec qui va expliquer à un auditoire pancanadien pourquoi la mauvaise herbe des champs de maïs peut isoler un manteau.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
@@ -15993,8 +16029,8 @@
       <c r="K226" s="10" t="inlineStr">
         <is>
           <t>Bonjour MELISSA PELLETIER,
-Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
-On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
+L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
 Je vous écris entre autres parce que la Montérégie est une des régions où l'asclépiade se cultive encore, et que c'est de champs comme ceux-là que vient la fibre qu'on transforme.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
@@ -16062,8 +16098,8 @@
       <c r="K227" s="10" t="inlineStr">
         <is>
           <t>Bonjour Isaac Peltz,
-Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
-On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
+L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
 Je vous écris entre autres parce que l'asclépiade se cultive dans votre région depuis la première vague de 2013, et que plusieurs des producteurs qui ont tenu bon nous vendent encore leur récolte.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
@@ -16131,8 +16167,8 @@
       <c r="K228" s="10" t="inlineStr">
         <is>
           <t>Bonjour Frédéric Perron,
-Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
-On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
+L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
 Je vous écris parce que vous couvrez l'art de vivre et la consommation. Le contraste se photographie bien : la gousse dans le champ, la soie blanche dans la main, le manteau porté en ville.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
@@ -16200,8 +16236,8 @@
       <c r="K229" s="10" t="inlineStr">
         <is>
           <t>Bonjour Nathalie Petrowski,
-Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
-On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
+L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
 Je vous écris parce que le sujet se raconte bien en ondes : une entreprise de Québec qui va expliquer à un auditoire pancanadien pourquoi la mauvaise herbe des champs de maïs peut isoler un manteau.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
@@ -16269,8 +16305,8 @@
       <c r="K230" s="10" t="inlineStr">
         <is>
           <t>Bonjour Francis Plourde,
-Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
-On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
+L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
 Je vous écris parce que c'est une nouvelle de chez nous qui passe au national.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
@@ -16338,8 +16374,8 @@
       <c r="K231" s="10" t="inlineStr">
         <is>
           <t>Bonjour Raymonde Provencher,
-Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
-On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
+L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
 Je vous écris parce que le sujet se raconte bien en ondes : une entreprise de Québec qui va expliquer à un auditoire pancanadien pourquoi la mauvaise herbe des champs de maïs peut isoler un manteau.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
@@ -16407,8 +16443,8 @@
       <c r="K232" s="10" t="inlineStr">
         <is>
           <t>Bonjour Richard Prudhomme,
-Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
-On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
+L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
 Je vous écris parce que vous couvrez l'art de vivre et la consommation. Le contraste se photographie bien : la gousse dans le champ, la soie blanche dans la main, le manteau porté en ville.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
@@ -16476,8 +16512,8 @@
       <c r="K233" s="10" t="inlineStr">
         <is>
           <t>Bonjour Pascale Renaud,
-Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
-On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
+L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
 Je vous écris parce que vous couvrez l'art de vivre et la consommation. Le contraste se photographie bien : la gousse dans le champ, la soie blanche dans la main, le manteau porté en ville.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
@@ -16545,8 +16581,8 @@
       <c r="K234" s="10" t="inlineStr">
         <is>
           <t>Bonjour Marc Sony Ricot,
-Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
-On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
+L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
 Je vous écris parce que vous couvrez l'art de vivre et la consommation. Le contraste se photographie bien : la gousse dans le champ, la soie blanche dans la main, le manteau porté en ville.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
@@ -16614,8 +16650,8 @@
       <c r="K235" s="10" t="inlineStr">
         <is>
           <t>Bonjour Marie-Paul Rouleau,
-Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
-On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
+L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
 Je vous écris parce que vous couvrez l'environnement. Notre pari est économique avant d'être militant : si l'asclépiade devient payante, les agriculteurs la gardent dans leurs champs, et les monarques retrouvent de l'habitat de reproduction.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
@@ -16683,8 +16719,8 @@
       <c r="K236" s="10" t="inlineStr">
         <is>
           <t>Bonjour Emmalie Ruest,
-Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
-On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
+L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
 Je vous écris parce que le sujet se raconte bien en ondes : une entreprise de Québec qui va expliquer à un auditoire pancanadien pourquoi la mauvaise herbe des champs de maïs peut isoler un manteau.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
@@ -16752,8 +16788,8 @@
       <c r="K237" s="10" t="inlineStr">
         <is>
           <t>Bonjour Louis-Philippe Samson,
-Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
-On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
+L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
 Je vous écris entre autres parce que l'asclépiade se cultive dans votre région depuis la première vague de 2013, et que plusieurs des producteurs qui ont tenu bon nous vendent encore leur récolte.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
@@ -16821,8 +16857,8 @@
       <c r="K238" s="10" t="inlineStr">
         <is>
           <t>Bonjour Catherine Schlager,
-Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
-On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
+L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
 Je vous écris parce que vous couvrez l'art de vivre et la consommation. Le contraste se photographie bien : la gousse dans le champ, la soie blanche dans la main, le manteau porté en ville.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
@@ -16890,8 +16926,8 @@
       <c r="K239" s="10" t="inlineStr">
         <is>
           <t>Bonjour Olivier Schmouker,
-Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
-On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
+L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
 Je vous écris parce que vous couvrez l'économie. On a bâti nos propres procédés de transformation parce qu'aucun sous-traitant ne voulait toucher à l'asclépiade, puis on a changé de modèle manufacturier l'an dernier pour rendre un manteau accessible à 300 $. J'en ai fait une vidéo ici : https://www.youtube.com/watch?v=GKyHh-Ok9JU.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
@@ -16959,8 +16995,8 @@
       <c r="K240" s="10" t="inlineStr">
         <is>
           <t>Bonjour Jacques Sennechael,
-Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
-On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
+L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
 Je vous écris parce que c'est une nouvelle de chez nous qui passe au national.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
@@ -17028,8 +17064,8 @@
       <c r="K241" s="10" t="inlineStr">
         <is>
           <t>Bonjour Alexandre Shields,
-Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
-On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
+L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
 Je vous écris parce que vous couvrez l'environnement. Notre pari est économique avant d'être militant : si l'asclépiade devient payante, les agriculteurs la gardent dans leurs champs, et les monarques retrouvent de l'habitat de reproduction.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
@@ -17097,8 +17133,8 @@
       <c r="K242" s="10" t="inlineStr">
         <is>
           <t>Bonjour Chloé Sondervorst,
-Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
-On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
+L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
 Je vous écris parce que vous couvrez l'environnement. Notre pari est économique avant d'être militant : si l'asclépiade devient payante, les agriculteurs la gardent dans leurs champs, et les monarques retrouvent de l'habitat de reproduction.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
@@ -17166,8 +17202,8 @@
       <c r="K243" s="10" t="inlineStr">
         <is>
           <t>Bonjour Kimberley Sullivan,
-Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
-On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
+L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
 Je vous écris entre autres parce que la Montérégie est une des régions où l'asclépiade se cultive encore, et que c'est de champs comme ceux-là que vient la fibre qu'on transforme.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
@@ -17235,8 +17271,8 @@
       <c r="K244" s="10" t="inlineStr">
         <is>
           <t>Bonjour William Thériault,
-Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
-On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
+L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
 Je vous écris entre autres parce que la Montérégie est une des régions où l'asclépiade se cultive encore, et que c'est de champs comme ceux-là que vient la fibre qu'on transforme.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
@@ -17304,8 +17340,8 @@
       <c r="K245" s="10" t="inlineStr">
         <is>
           <t>Bonjour Katia Tobar,
-Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
-On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
+L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
 Je vous écris parce que vous couvrez l'économie. On a bâti nos propres procédés de transformation parce qu'aucun sous-traitant ne voulait toucher à l'asclépiade, puis on a changé de modèle manufacturier l'an dernier pour rendre un manteau accessible à 300 $. J'en ai fait une vidéo ici : https://www.youtube.com/watch?v=GKyHh-Ok9JU.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
@@ -17373,8 +17409,8 @@
       <c r="K246" s="10" t="inlineStr">
         <is>
           <t>Bonjour Martin Tremblay,
-Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
-On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
+L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
 Je vous écris parce que vous couvrez l'environnement. Notre pari est économique avant d'être militant : si l'asclépiade devient payante, les agriculteurs la gardent dans leurs champs, et les monarques retrouvent de l'habitat de reproduction.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
@@ -17442,8 +17478,8 @@
       <c r="K247" s="10" t="inlineStr">
         <is>
           <t>Bonjour Marie-Christine Trottier,
-Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
-On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
+L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
 Je vous écris parce que le sujet se raconte bien en ondes : une entreprise de Québec qui va expliquer à un auditoire pancanadien pourquoi la mauvaise herbe des champs de maïs peut isoler un manteau.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
@@ -17511,8 +17547,8 @@
       <c r="K248" s="10" t="inlineStr">
         <is>
           <t>Bonjour Pierre-Luc Trudel,
-Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
-On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
+L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
 Je vous écris parce que vous couvrez l'économie. On a bâti nos propres procédés de transformation parce qu'aucun sous-traitant ne voulait toucher à l'asclépiade, puis on a changé de modèle manufacturier l'an dernier pour rendre un manteau accessible à 300 $. J'en ai fait une vidéo ici : https://www.youtube.com/watch?v=GKyHh-Ok9JU.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
@@ -17580,8 +17616,8 @@
       <c r="K249" s="10" t="inlineStr">
         <is>
           <t>Bonjour David Turbis,
-Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
-On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
+L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
 Je vous écris parce que le sujet se raconte bien en ondes : une entreprise de Québec qui va expliquer à un auditoire pancanadien pourquoi la mauvaise herbe des champs de maïs peut isoler un manteau.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
@@ -17649,8 +17685,8 @@
       <c r="K250" s="10" t="inlineStr">
         <is>
           <t>Bonjour Paule Vermot-Desroches,
-Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
-On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
+L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
 Je vous écris entre autres parce que l'asclépiade a eu son grand moment industriel chez vous : l'usine de Saint-Tite achetait 90 % des récoltes du Québec avant que la filière se casse en 2018. Des producteurs de la Mauricie cultivent encore, et on continue d'acheter leur récolte.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
@@ -17718,8 +17754,8 @@
       <c r="K251" s="10" t="inlineStr">
         <is>
           <t>Bonjour Alexandra Viau,
-Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
-On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
+L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
 Je vous écris parce que le sujet se raconte bien en ondes : une entreprise de Québec qui va expliquer à un auditoire pancanadien pourquoi la mauvaise herbe des champs de maïs peut isoler un manteau.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
@@ -17787,8 +17823,8 @@
       <c r="K252" s="10" t="inlineStr">
         <is>
           <t>Bonjour Raymond Viger,
-Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
-On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
+L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
 Je vous écris parce que vous couvrez l'environnement. Notre pari est économique avant d'être militant : si l'asclépiade devient payante, les agriculteurs la gardent dans leurs champs, et les monarques retrouvent de l'habitat de reproduction.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
@@ -17856,8 +17892,8 @@
       <c r="K253" s="10" t="inlineStr">
         <is>
           <t>Bonjour Paul Émile d'Entremont,
-Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
-On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
+L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
 Je vous écris parce que c'est une nouvelle de chez nous qui passe au national.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
@@ -17925,8 +17961,8 @@
       <c r="K254" s="10" t="inlineStr">
         <is>
           <t>Bonjour Augustin de Baudinière,
-Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
-On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
+L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
 Je vous écris parce que vous couvrez l'environnement. Notre pari est économique avant d'être militant : si l'asclépiade devient payante, les agriculteurs la gardent dans leurs champs, et les monarques retrouvent de l'habitat de reproduction.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
@@ -17994,8 +18030,8 @@
       <c r="K255" s="10" t="inlineStr">
         <is>
           <t>Bonjour Ivan de Jacquelin-Dulphe,
-Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
-On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
+L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
 Je vous écris parce que vous couvrez l'environnement. Notre pari est économique avant d'être militant : si l'asclépiade devient payante, les agriculteurs la gardent dans leurs champs, et les monarques retrouvent de l'habitat de reproduction.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
@@ -18063,8 +18099,8 @@
       <c r="K256" s="10" t="inlineStr">
         <is>
           <t>Bonjour Jean-Michel Leprince,
-Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de
-Québec dont l'atelier est dans Limoilou.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une
+mauvaise herbe.
 Vous couvrez l'asclépiade depuis au moins 2014 : le Téléjournal, la soie d'Amérique partie
 sur l'Everest, le pouvoir absorbant de la fibre sur les hydrocarbures, le lien avec le
 monarque. Vous avez suivi cette histoire plus longtemps que la plupart des entreprises qui
@@ -18135,8 +18171,8 @@
       <c r="K257" s="10" t="inlineStr">
         <is>
           <t>Bonjour Antoine Stab,
-Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de
-Québec dont l'atelier est dans Limoilou.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une
+mauvaise herbe.
 Vous aviez écrit sur le soyer du Québec dans Espaces en février 2015, à l'époque où la fibre
 devait remplacer le duvet.
 On a démarré après la chute de cette première filière. Six ans plus tard, on achète encore de l'asclépiade québécoise, on transforme l'isolant nous-mêmes, et il

</xml_diff>

<commit_message>
Retire les « petits cochons »
Le nom populaire est retiré des 253 brouillons et des documents. L'ouverture
enchaîne directement sur la matière: « Ses gousses sont remplies d'une soie
creuse, très légère et naturellement hydrophobe. »

« Mauvaise herbe » est déjà dans la phrase d'ouverture, donc la mention des
agriculteurs qui l'arrachent depuis 50 ans n'ajoutait plus rien et rattachait
mal sa relative.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015pjLsGPzf1MX1JC7QiKGGk
</commit_message>
<xml_diff>
--- a/communique-dragons/Lasclay_brouillons_a_editer.xlsx
+++ b/communique-dragons/Lasclay_brouillons_a_editer.xlsx
@@ -508,7 +508,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Version 7 — ta phrase d'ouverture</t>
+          <t>Version 8</t>
         </is>
       </c>
       <c r="B1" s="2" t="inlineStr"/>
@@ -520,54 +520,54 @@
     <row r="3" ht="58" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>L'ouverture</t>
+          <t>Les « petits cochons »</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>« On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque. » Elle porte le produit, la plante et la mission d'un seul coup.</t>
+          <t>Retirés partout. Zéro occurrence dans les 253 brouillons et dans les documents.</t>
         </is>
       </c>
     </row>
     <row r="4" ht="58" customHeight="1">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>Le courriel raccourcit</t>
+          <t>L'ouverture</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Comme l'ouverture dit déjà la mission, le paragraphe « Mes 2 grandes missions » saute de toute la liste froide et des quatre contacts chauds sans historique. Zéro répétition.</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="58" customHeight="1">
-      <c r="A5" s="3" t="inlineStr">
-        <is>
-          <t>Un détail corrigé</t>
-        </is>
-      </c>
-      <c r="B5" s="2" t="inlineStr">
-        <is>
-          <t>Les « petits cochons » sont les gousses, pas la soie. La phrase le dit maintenant dans le bon ordre : « Ses gousses, les petits cochons…, sont remplies d'une soie creuse. »</t>
-        </is>
-      </c>
+          <t>« On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque. » Puis, directement : « Ses gousses sont remplies d'une soie creuse, très légère et naturellement hydrophobe. »</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr"/>
+      <c r="B5" s="2" t="inlineStr"/>
     </row>
     <row r="6">
-      <c r="A6" s="2" t="inlineStr"/>
+      <c r="A6" s="1" t="inlineStr">
+        <is>
+          <t>Les versions précédentes</t>
+        </is>
+      </c>
       <c r="B6" s="2" t="inlineStr"/>
     </row>
     <row r="7">
-      <c r="A7" s="1" t="inlineStr">
-        <is>
-          <t>Les versions précédentes</t>
-        </is>
-      </c>
+      <c r="A7" s="2" t="inlineStr"/>
       <c r="B7" s="2" t="inlineStr"/>
     </row>
-    <row r="8">
-      <c r="A8" s="2" t="inlineStr"/>
-      <c r="B8" s="2" t="inlineStr"/>
+    <row r="8" ht="58" customHeight="1">
+      <c r="A8" s="3" t="inlineStr">
+        <is>
+          <t>v7</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>Ton ouverture adoptée, paragraphe des missions retiré.</t>
+        </is>
+      </c>
     </row>
     <row r="9" ht="58" customHeight="1">
       <c r="A9" s="3" t="inlineStr">
@@ -776,7 +776,7 @@
       </c>
       <c r="K1" s="4" t="inlineStr">
         <is>
-          <t>Brouillon v7</t>
+          <t>Brouillon v8</t>
         </is>
       </c>
       <c r="L1" s="4" t="inlineStr">
@@ -795,7 +795,7 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="250" customHeight="1">
+    <row r="2" ht="240" customHeight="1">
       <c r="A2" s="5" t="inlineStr">
         <is>
           <t>chaude</t>
@@ -865,7 +865,7 @@
       <c r="M2" s="11" t="inlineStr"/>
       <c r="N2" s="11" t="inlineStr"/>
     </row>
-    <row r="3" ht="250" customHeight="1">
+    <row r="3" ht="240" customHeight="1">
       <c r="A3" s="5" t="inlineStr">
         <is>
           <t>chaude</t>
@@ -928,7 +928,7 @@
       <c r="M3" s="11" t="inlineStr"/>
       <c r="N3" s="11" t="inlineStr"/>
     </row>
-    <row r="4" ht="250" customHeight="1">
+    <row r="4" ht="240" customHeight="1">
       <c r="A4" s="5" t="inlineStr">
         <is>
           <t>chaude</t>
@@ -1004,7 +1004,7 @@
       <c r="M4" s="11" t="inlineStr"/>
       <c r="N4" s="11" t="inlineStr"/>
     </row>
-    <row r="5" ht="250" customHeight="1">
+    <row r="5" ht="240" customHeight="1">
       <c r="A5" s="5" t="inlineStr">
         <is>
           <t>chaude</t>
@@ -1066,7 +1066,7 @@
       <c r="M5" s="11" t="inlineStr"/>
       <c r="N5" s="11" t="inlineStr"/>
     </row>
-    <row r="6" ht="250" customHeight="1">
+    <row r="6" ht="240" customHeight="1">
       <c r="A6" s="5" t="inlineStr">
         <is>
           <t>chaude</t>
@@ -1129,7 +1129,7 @@
       <c r="M6" s="11" t="inlineStr"/>
       <c r="N6" s="11" t="inlineStr"/>
     </row>
-    <row r="7" ht="250" customHeight="1">
+    <row r="7" ht="240" customHeight="1">
       <c r="A7" s="5" t="inlineStr">
         <is>
           <t>chaude</t>
@@ -1192,7 +1192,7 @@
       <c r="M7" s="11" t="inlineStr"/>
       <c r="N7" s="11" t="inlineStr"/>
     </row>
-    <row r="8" ht="250" customHeight="1">
+    <row r="8" ht="240" customHeight="1">
       <c r="A8" s="5" t="inlineStr">
         <is>
           <t>chaude</t>
@@ -1255,7 +1255,7 @@
       <c r="M8" s="11" t="inlineStr"/>
       <c r="N8" s="11" t="inlineStr"/>
     </row>
-    <row r="9" ht="250" customHeight="1">
+    <row r="9" ht="240" customHeight="1">
       <c r="A9" s="5" t="inlineStr">
         <is>
           <t>chaude</t>
@@ -1318,7 +1318,7 @@
       <c r="M9" s="11" t="inlineStr"/>
       <c r="N9" s="11" t="inlineStr"/>
     </row>
-    <row r="10" ht="250" customHeight="1">
+    <row r="10" ht="240" customHeight="1">
       <c r="A10" s="5" t="inlineStr">
         <is>
           <t>chaude</t>
@@ -1381,7 +1381,7 @@
       <c r="M10" s="11" t="inlineStr"/>
       <c r="N10" s="11" t="inlineStr"/>
     </row>
-    <row r="11" ht="250" customHeight="1">
+    <row r="11" ht="240" customHeight="1">
       <c r="A11" s="5" t="inlineStr">
         <is>
           <t>chaude</t>
@@ -1444,7 +1444,7 @@
       <c r="M11" s="11" t="inlineStr"/>
       <c r="N11" s="11" t="inlineStr"/>
     </row>
-    <row r="12" ht="250" customHeight="1">
+    <row r="12" ht="240" customHeight="1">
       <c r="A12" s="5" t="inlineStr">
         <is>
           <t>chaude</t>
@@ -1507,7 +1507,7 @@
       <c r="M12" s="11" t="inlineStr"/>
       <c r="N12" s="11" t="inlineStr"/>
     </row>
-    <row r="13" ht="250" customHeight="1">
+    <row r="13" ht="240" customHeight="1">
       <c r="A13" s="5" t="inlineStr">
         <is>
           <t>chaude</t>
@@ -1570,7 +1570,7 @@
       <c r="M13" s="11" t="inlineStr"/>
       <c r="N13" s="11" t="inlineStr"/>
     </row>
-    <row r="14" ht="250" customHeight="1">
+    <row r="14" ht="240" customHeight="1">
       <c r="A14" s="5" t="inlineStr">
         <is>
           <t>chaude</t>
@@ -1633,7 +1633,7 @@
       <c r="M14" s="11" t="inlineStr"/>
       <c r="N14" s="11" t="inlineStr"/>
     </row>
-    <row r="15" ht="250" customHeight="1">
+    <row r="15" ht="240" customHeight="1">
       <c r="A15" s="5" t="inlineStr">
         <is>
           <t>chaude</t>
@@ -1696,7 +1696,7 @@
       <c r="M15" s="11" t="inlineStr"/>
       <c r="N15" s="11" t="inlineStr"/>
     </row>
-    <row r="16" ht="250" customHeight="1">
+    <row r="16" ht="240" customHeight="1">
       <c r="A16" s="5" t="inlineStr">
         <is>
           <t>chaude</t>
@@ -1758,7 +1758,7 @@
       <c r="M16" s="11" t="inlineStr"/>
       <c r="N16" s="11" t="inlineStr"/>
     </row>
-    <row r="17" ht="250" customHeight="1">
+    <row r="17" ht="240" customHeight="1">
       <c r="A17" s="5" t="inlineStr">
         <is>
           <t>chaude</t>
@@ -1821,7 +1821,7 @@
       <c r="M17" s="11" t="inlineStr"/>
       <c r="N17" s="11" t="inlineStr"/>
     </row>
-    <row r="18" ht="250" customHeight="1">
+    <row r="18" ht="240" customHeight="1">
       <c r="A18" s="5" t="inlineStr">
         <is>
           <t>chaude</t>
@@ -1884,7 +1884,7 @@
       <c r="M18" s="11" t="inlineStr"/>
       <c r="N18" s="11" t="inlineStr"/>
     </row>
-    <row r="19" ht="250" customHeight="1">
+    <row r="19" ht="240" customHeight="1">
       <c r="A19" s="5" t="inlineStr">
         <is>
           <t>chaude</t>
@@ -1947,7 +1947,7 @@
       <c r="M19" s="11" t="inlineStr"/>
       <c r="N19" s="11" t="inlineStr"/>
     </row>
-    <row r="20" ht="250" customHeight="1">
+    <row r="20" ht="240" customHeight="1">
       <c r="A20" s="5" t="inlineStr">
         <is>
           <t>chaude</t>
@@ -2010,7 +2010,7 @@
       <c r="M20" s="11" t="inlineStr"/>
       <c r="N20" s="11" t="inlineStr"/>
     </row>
-    <row r="21" ht="250" customHeight="1">
+    <row r="21" ht="240" customHeight="1">
       <c r="A21" s="5" t="inlineStr">
         <is>
           <t>chaude</t>
@@ -2073,7 +2073,7 @@
       <c r="M21" s="11" t="inlineStr"/>
       <c r="N21" s="11" t="inlineStr"/>
     </row>
-    <row r="22" ht="250" customHeight="1">
+    <row r="22" ht="240" customHeight="1">
       <c r="A22" s="5" t="inlineStr">
         <is>
           <t>chaude</t>
@@ -2136,7 +2136,7 @@
       <c r="M22" s="11" t="inlineStr"/>
       <c r="N22" s="11" t="inlineStr"/>
     </row>
-    <row r="23" ht="250" customHeight="1">
+    <row r="23" ht="240" customHeight="1">
       <c r="A23" s="5" t="inlineStr">
         <is>
           <t>chaude</t>
@@ -2199,7 +2199,7 @@
       <c r="M23" s="11" t="inlineStr"/>
       <c r="N23" s="11" t="inlineStr"/>
     </row>
-    <row r="24" ht="250" customHeight="1">
+    <row r="24" ht="240" customHeight="1">
       <c r="A24" s="5" t="inlineStr">
         <is>
           <t>chaude</t>
@@ -2262,7 +2262,7 @@
       <c r="M24" s="11" t="inlineStr"/>
       <c r="N24" s="11" t="inlineStr"/>
     </row>
-    <row r="25" ht="250" customHeight="1">
+    <row r="25" ht="240" customHeight="1">
       <c r="A25" s="5" t="inlineStr">
         <is>
           <t>chaude</t>
@@ -2325,7 +2325,7 @@
       <c r="M25" s="11" t="inlineStr"/>
       <c r="N25" s="11" t="inlineStr"/>
     </row>
-    <row r="26" ht="250" customHeight="1">
+    <row r="26" ht="240" customHeight="1">
       <c r="A26" s="5" t="inlineStr">
         <is>
           <t>chaude</t>
@@ -2381,7 +2381,7 @@
       <c r="M26" s="11" t="inlineStr"/>
       <c r="N26" s="11" t="inlineStr"/>
     </row>
-    <row r="27" ht="250" customHeight="1">
+    <row r="27" ht="240" customHeight="1">
       <c r="A27" s="5" t="inlineStr">
         <is>
           <t>chaude</t>
@@ -2444,7 +2444,7 @@
       <c r="M27" s="11" t="inlineStr"/>
       <c r="N27" s="11" t="inlineStr"/>
     </row>
-    <row r="28" ht="250" customHeight="1">
+    <row r="28" ht="240" customHeight="1">
       <c r="A28" s="5" t="inlineStr">
         <is>
           <t>chaude</t>
@@ -2499,7 +2499,7 @@
       <c r="M28" s="11" t="inlineStr"/>
       <c r="N28" s="11" t="inlineStr"/>
     </row>
-    <row r="29" ht="250" customHeight="1">
+    <row r="29" ht="240" customHeight="1">
       <c r="A29" s="5" t="inlineStr">
         <is>
           <t>chaude</t>
@@ -2541,7 +2541,7 @@
       <c r="K29" s="10" t="inlineStr">
         <is>
           <t>Bonjour Mme Roberge,
-Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque. Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe, qu'on transforme en isolant à Québec.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque. Ses gousses sont remplies d'une soie creuse, très légère et naturellement hydrophobe, qu'on transforme en isolant à Québec.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part : je suis disponible pour une entrevue la semaine du 14 septembre et le vendredi 18 au matin.
@@ -2553,7 +2553,7 @@
       <c r="M29" s="11" t="inlineStr"/>
       <c r="N29" s="11" t="inlineStr"/>
     </row>
-    <row r="30" ht="250" customHeight="1">
+    <row r="30" ht="240" customHeight="1">
       <c r="A30" s="5" t="inlineStr">
         <is>
           <t>chaude</t>
@@ -2595,7 +2595,7 @@
       <c r="K30" s="10" t="inlineStr">
         <is>
           <t>Bonjour Mme Laforest,
-Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque. Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe, qu'on transforme en isolant à Québec.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque. Ses gousses sont remplies d'une soie creuse, très légère et naturellement hydrophobe, qu'on transforme en isolant à Québec.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part : je suis disponible pour une entrevue la semaine du 14 septembre et le vendredi 18 au matin.
@@ -2607,7 +2607,7 @@
       <c r="M30" s="11" t="inlineStr"/>
       <c r="N30" s="11" t="inlineStr"/>
     </row>
-    <row r="31" ht="250" customHeight="1">
+    <row r="31" ht="240" customHeight="1">
       <c r="A31" s="5" t="inlineStr">
         <is>
           <t>chaude</t>
@@ -2670,7 +2670,7 @@
       <c r="M31" s="11" t="inlineStr"/>
       <c r="N31" s="11" t="inlineStr"/>
     </row>
-    <row r="32" ht="250" customHeight="1">
+    <row r="32" ht="240" customHeight="1">
       <c r="A32" s="5" t="inlineStr">
         <is>
           <t>chaude</t>
@@ -2725,7 +2725,7 @@
       <c r="M32" s="11" t="inlineStr"/>
       <c r="N32" s="11" t="inlineStr"/>
     </row>
-    <row r="33" ht="250" customHeight="1">
+    <row r="33" ht="240" customHeight="1">
       <c r="A33" s="5" t="inlineStr">
         <is>
           <t>chaude</t>
@@ -2780,7 +2780,7 @@
       <c r="M33" s="11" t="inlineStr"/>
       <c r="N33" s="11" t="inlineStr"/>
     </row>
-    <row r="34" ht="250" customHeight="1">
+    <row r="34" ht="240" customHeight="1">
       <c r="A34" s="5" t="inlineStr">
         <is>
           <t>chaude</t>
@@ -2834,7 +2834,7 @@
       <c r="M34" s="11" t="inlineStr"/>
       <c r="N34" s="11" t="inlineStr"/>
     </row>
-    <row r="35" ht="250" customHeight="1">
+    <row r="35" ht="240" customHeight="1">
       <c r="A35" s="5" t="inlineStr">
         <is>
           <t>chaude</t>
@@ -2876,7 +2876,7 @@
       <c r="K35" s="10" t="inlineStr">
         <is>
           <t>Bonjour Mme Dostie,
-Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque. Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe, qu'on transforme en isolant à Québec.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque. Ses gousses sont remplies d'une soie creuse, très légère et naturellement hydrophobe, qu'on transforme en isolant à Québec.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet.
@@ -2888,7 +2888,7 @@
       <c r="M35" s="11" t="inlineStr"/>
       <c r="N35" s="11" t="inlineStr"/>
     </row>
-    <row r="36" ht="250" customHeight="1">
+    <row r="36" ht="240" customHeight="1">
       <c r="A36" s="5" t="inlineStr">
         <is>
           <t>chaude</t>
@@ -2947,7 +2947,7 @@
       <c r="M36" s="11" t="inlineStr"/>
       <c r="N36" s="11" t="inlineStr"/>
     </row>
-    <row r="37" ht="250" customHeight="1">
+    <row r="37" ht="240" customHeight="1">
       <c r="A37" s="5" t="inlineStr">
         <is>
           <t>chaude</t>
@@ -3006,7 +3006,7 @@
       <c r="M37" s="11" t="inlineStr"/>
       <c r="N37" s="11" t="inlineStr"/>
     </row>
-    <row r="38" ht="250" customHeight="1">
+    <row r="38" ht="240" customHeight="1">
       <c r="A38" s="5" t="inlineStr">
         <is>
           <t>chaude</t>
@@ -3065,7 +3065,7 @@
       <c r="M38" s="11" t="inlineStr"/>
       <c r="N38" s="11" t="inlineStr"/>
     </row>
-    <row r="39" ht="250" customHeight="1">
+    <row r="39" ht="240" customHeight="1">
       <c r="A39" s="6" t="inlineStr">
         <is>
           <t>froide A</t>
@@ -3140,7 +3140,7 @@
       <c r="M39" s="11" t="inlineStr"/>
       <c r="N39" s="11" t="inlineStr"/>
     </row>
-    <row r="40" ht="250" customHeight="1">
+    <row r="40" ht="240" customHeight="1">
       <c r="A40" s="6" t="inlineStr">
         <is>
           <t>froide A</t>
@@ -3195,7 +3195,7 @@
         <is>
           <t>Bonjour Zoé Allemand,
 Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
-Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
+Ses gousses sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris parce que vous couvrez l'agriculture. La question qui compte pour les producteurs n'a pas changé depuis l'effondrement de la filière en 2018 : est-ce qu'il y a un acheteur stable au bout du champ. On achète encore la récolte de producteurs d'ici et on la transforme nous-mêmes.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -3208,7 +3208,7 @@
       <c r="M40" s="11" t="inlineStr"/>
       <c r="N40" s="11" t="inlineStr"/>
     </row>
-    <row r="41" ht="250" customHeight="1">
+    <row r="41" ht="240" customHeight="1">
       <c r="A41" s="6" t="inlineStr">
         <is>
           <t>froide A</t>
@@ -3263,7 +3263,7 @@
         <is>
           <t>Bonjour Victoria Bakos,
 Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
-Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
+Ses gousses sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris parce que vous couvrez l'art de vivre et la consommation. Le contraste se photographie bien : la gousse dans le champ, la soie blanche dans la main, le manteau porté en ville.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -3276,7 +3276,7 @@
       <c r="M41" s="11" t="inlineStr"/>
       <c r="N41" s="11" t="inlineStr"/>
     </row>
-    <row r="42" ht="250" customHeight="1">
+    <row r="42" ht="240" customHeight="1">
       <c r="A42" s="6" t="inlineStr">
         <is>
           <t>froide A</t>
@@ -3331,7 +3331,7 @@
         <is>
           <t>Bonjour Marie-Émélie Bernier,
 Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
-Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
+Ses gousses sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris parce que c'est une nouvelle de chez nous qui passe au national.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -3344,7 +3344,7 @@
       <c r="M42" s="11" t="inlineStr"/>
       <c r="N42" s="11" t="inlineStr"/>
     </row>
-    <row r="43" ht="250" customHeight="1">
+    <row r="43" ht="240" customHeight="1">
       <c r="A43" s="6" t="inlineStr">
         <is>
           <t>froide A</t>
@@ -3399,7 +3399,7 @@
         <is>
           <t>Bonjour Normand Blouin,
 Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
-Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
+Ses gousses sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris parce que vous couvrez l'agriculture. La question qui compte pour les producteurs n'a pas changé depuis l'effondrement de la filière en 2018 : est-ce qu'il y a un acheteur stable au bout du champ. On achète encore la récolte de producteurs d'ici et on la transforme nous-mêmes.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -3412,7 +3412,7 @@
       <c r="M43" s="11" t="inlineStr"/>
       <c r="N43" s="11" t="inlineStr"/>
     </row>
-    <row r="44" ht="250" customHeight="1">
+    <row r="44" ht="240" customHeight="1">
       <c r="A44" s="6" t="inlineStr">
         <is>
           <t>froide A</t>
@@ -3467,7 +3467,7 @@
         <is>
           <t>Bonjour Louise Bourbonnais,
 Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
-Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
+Ses gousses sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris parce que c'est une nouvelle de chez nous qui passe au national.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -3480,7 +3480,7 @@
       <c r="M44" s="11" t="inlineStr"/>
       <c r="N44" s="11" t="inlineStr"/>
     </row>
-    <row r="45" ht="250" customHeight="1">
+    <row r="45" ht="240" customHeight="1">
       <c r="A45" s="6" t="inlineStr">
         <is>
           <t>froide A</t>
@@ -3535,7 +3535,7 @@
         <is>
           <t>Bonjour Francois Bourque,
 Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
-Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
+Ses gousses sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris parce que vous couvrez l'économie. On a bâti nos propres procédés de transformation parce qu'aucun sous-traitant ne voulait toucher à l'asclépiade, puis on a changé de modèle manufacturier l'an dernier pour rendre un manteau accessible à 300 $. J'en ai fait une vidéo ici : https://www.youtube.com/watch?v=GKyHh-Ok9JU.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -3548,7 +3548,7 @@
       <c r="M45" s="11" t="inlineStr"/>
       <c r="N45" s="11" t="inlineStr"/>
     </row>
-    <row r="46" ht="250" customHeight="1">
+    <row r="46" ht="240" customHeight="1">
       <c r="A46" s="6" t="inlineStr">
         <is>
           <t>froide A</t>
@@ -3603,7 +3603,7 @@
         <is>
           <t>Bonjour Ariane Boyer,
 Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
-Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
+Ses gousses sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris parce que vous couvrez l'environnement. Notre pari est économique avant d'être militant : si l'asclépiade devient payante, les agriculteurs la gardent dans leurs champs, et les monarques retrouvent de l'habitat de reproduction.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -3616,7 +3616,7 @@
       <c r="M46" s="11" t="inlineStr"/>
       <c r="N46" s="11" t="inlineStr"/>
     </row>
-    <row r="47" ht="250" customHeight="1">
+    <row r="47" ht="240" customHeight="1">
       <c r="A47" s="6" t="inlineStr">
         <is>
           <t>froide A</t>
@@ -3671,7 +3671,7 @@
         <is>
           <t>Bonjour Gilbert Bégin,
 Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
-Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
+Ses gousses sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris parce que c'est une nouvelle de chez nous qui passe au national.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -3684,7 +3684,7 @@
       <c r="M47" s="11" t="inlineStr"/>
       <c r="N47" s="11" t="inlineStr"/>
     </row>
-    <row r="48" ht="250" customHeight="1">
+    <row r="48" ht="240" customHeight="1">
       <c r="A48" s="6" t="inlineStr">
         <is>
           <t>froide A</t>
@@ -3739,7 +3739,7 @@
         <is>
           <t>Bonjour Papa Moussa Camara,
 Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
-Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
+Ses gousses sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris parce que le sujet se raconte bien en ondes : une entreprise de Québec qui va expliquer à un auditoire pancanadien pourquoi la mauvaise herbe des champs de maïs peut isoler un manteau.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -3752,7 +3752,7 @@
       <c r="M48" s="11" t="inlineStr"/>
       <c r="N48" s="11" t="inlineStr"/>
     </row>
-    <row r="49" ht="250" customHeight="1">
+    <row r="49" ht="240" customHeight="1">
       <c r="A49" s="6" t="inlineStr">
         <is>
           <t>froide A</t>
@@ -3807,7 +3807,7 @@
         <is>
           <t>Bonjour Victor Carré,
 Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
-Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
+Ses gousses sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris parce que c'est une nouvelle de chez nous qui passe au national.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -3820,7 +3820,7 @@
       <c r="M49" s="11" t="inlineStr"/>
       <c r="N49" s="11" t="inlineStr"/>
     </row>
-    <row r="50" ht="250" customHeight="1">
+    <row r="50" ht="240" customHeight="1">
       <c r="A50" s="6" t="inlineStr">
         <is>
           <t>froide A</t>
@@ -3875,7 +3875,7 @@
         <is>
           <t>Bonjour Eric Chabot,
 Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
-Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
+Ses gousses sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris parce que vous couvrez le plein air. À poids égal, la littérature donne la soie d'asclépiade pour environ 10 % plus isolante que le duvet. C'est un repère de laboratoire, pas une promesse de manteau, et c'est exactement pour ça que je préfère qu'on la teste.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -3888,7 +3888,7 @@
       <c r="M50" s="11" t="inlineStr"/>
       <c r="N50" s="11" t="inlineStr"/>
     </row>
-    <row r="51" ht="250" customHeight="1">
+    <row r="51" ht="240" customHeight="1">
       <c r="A51" s="6" t="inlineStr">
         <is>
           <t>froide A</t>
@@ -3943,7 +3943,7 @@
         <is>
           <t>Bonjour Tristan Champagne-Lessard,
 Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
-Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
+Ses gousses sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris entre autres parce que la Montérégie est une des régions où l'asclépiade se cultive encore, et que c'est de champs comme ceux-là que vient la fibre qu'on transforme.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -3956,7 +3956,7 @@
       <c r="M51" s="11" t="inlineStr"/>
       <c r="N51" s="11" t="inlineStr"/>
     </row>
-    <row r="52" ht="250" customHeight="1">
+    <row r="52" ht="240" customHeight="1">
       <c r="A52" s="6" t="inlineStr">
         <is>
           <t>froide A</t>
@@ -4011,7 +4011,7 @@
         <is>
           <t>Bonjour Jean-Marc Chevalier,
 Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
-Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
+Ses gousses sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris entre autres parce que la Montérégie est une des régions où l'asclépiade se cultive encore, et que c'est de champs comme ceux-là que vient la fibre qu'on transforme.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -4024,7 +4024,7 @@
       <c r="M52" s="11" t="inlineStr"/>
       <c r="N52" s="11" t="inlineStr"/>
     </row>
-    <row r="53" ht="250" customHeight="1">
+    <row r="53" ht="240" customHeight="1">
       <c r="A53" s="6" t="inlineStr">
         <is>
           <t>froide A</t>
@@ -4079,7 +4079,7 @@
         <is>
           <t>Bonjour Simon Chrétien,
 Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
-Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
+Ses gousses sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris parce que vous couvrez l'agriculture. La question qui compte pour les producteurs n'a pas changé depuis l'effondrement de la filière en 2018 : est-ce qu'il y a un acheteur stable au bout du champ. On achète encore la récolte de producteurs d'ici et on la transforme nous-mêmes.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -4092,7 +4092,7 @@
       <c r="M53" s="11" t="inlineStr"/>
       <c r="N53" s="11" t="inlineStr"/>
     </row>
-    <row r="54" ht="250" customHeight="1">
+    <row r="54" ht="240" customHeight="1">
       <c r="A54" s="6" t="inlineStr">
         <is>
           <t>froide A</t>
@@ -4147,7 +4147,7 @@
         <is>
           <t>Bonjour Maxime Corneau,
 Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
-Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
+Ses gousses sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris entre autres parce qu'un de nos fournisseurs d'asclépiade cultive au Lac-Saint-Jean depuis nos tout débuts, et qu'il l'est encore aujourd'hui. La fibre de chez vous se retrouve dans nos produits.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -4160,7 +4160,7 @@
       <c r="M54" s="11" t="inlineStr"/>
       <c r="N54" s="11" t="inlineStr"/>
     </row>
-    <row r="55" ht="250" customHeight="1">
+    <row r="55" ht="240" customHeight="1">
       <c r="A55" s="6" t="inlineStr">
         <is>
           <t>froide A</t>
@@ -4215,7 +4215,7 @@
         <is>
           <t>Bonjour Aurélia Crémoux,
 Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
-Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
+Ses gousses sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris parce que vous couvrez le plein air. À poids égal, la littérature donne la soie d'asclépiade pour environ 10 % plus isolante que le duvet. C'est un repère de laboratoire, pas une promesse de manteau, et c'est exactement pour ça que je préfère qu'on la teste.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -4228,7 +4228,7 @@
       <c r="M55" s="11" t="inlineStr"/>
       <c r="N55" s="11" t="inlineStr"/>
     </row>
-    <row r="56" ht="250" customHeight="1">
+    <row r="56" ht="240" customHeight="1">
       <c r="A56" s="6" t="inlineStr">
         <is>
           <t>froide A</t>
@@ -4283,7 +4283,7 @@
         <is>
           <t>Bonjour Catherine Dallaire,
 Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
-Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
+Ses gousses sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris entre autres parce qu'une des premières usines de transformation de la fibre était à Granby, et que l'Estrie compte encore des producteurs d'asclépiade.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -4296,7 +4296,7 @@
       <c r="M56" s="11" t="inlineStr"/>
       <c r="N56" s="11" t="inlineStr"/>
     </row>
-    <row r="57" ht="250" customHeight="1">
+    <row r="57" ht="240" customHeight="1">
       <c r="A57" s="6" t="inlineStr">
         <is>
           <t>froide A</t>
@@ -4369,7 +4369,7 @@
       <c r="M57" s="11" t="inlineStr"/>
       <c r="N57" s="11" t="inlineStr"/>
     </row>
-    <row r="58" ht="250" customHeight="1">
+    <row r="58" ht="240" customHeight="1">
       <c r="A58" s="6" t="inlineStr">
         <is>
           <t>froide A</t>
@@ -4424,7 +4424,7 @@
         <is>
           <t>Bonjour Anaïs Desjardins,
 Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
-Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
+Ses gousses sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris parce que vous couvrez l'environnement. Notre pari est économique avant d'être militant : si l'asclépiade devient payante, les agriculteurs la gardent dans leurs champs, et les monarques retrouvent de l'habitat de reproduction.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -4437,7 +4437,7 @@
       <c r="M58" s="11" t="inlineStr"/>
       <c r="N58" s="11" t="inlineStr"/>
     </row>
-    <row r="59" ht="250" customHeight="1">
+    <row r="59" ht="240" customHeight="1">
       <c r="A59" s="6" t="inlineStr">
         <is>
           <t>froide A</t>
@@ -4492,7 +4492,7 @@
         <is>
           <t>Bonjour Simon Dominé,
 Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
-Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
+Ses gousses sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris parce que vous couvrez l'agriculture. La question qui compte pour les producteurs n'a pas changé depuis l'effondrement de la filière en 2018 : est-ce qu'il y a un acheteur stable au bout du champ. On achète encore la récolte de producteurs d'ici et on la transforme nous-mêmes.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -4505,7 +4505,7 @@
       <c r="M59" s="11" t="inlineStr"/>
       <c r="N59" s="11" t="inlineStr"/>
     </row>
-    <row r="60" ht="250" customHeight="1">
+    <row r="60" ht="240" customHeight="1">
       <c r="A60" s="6" t="inlineStr">
         <is>
           <t>froide A</t>
@@ -4560,7 +4560,7 @@
         <is>
           <t>Bonjour Karl-Ivann Dubé,
 Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
-Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
+Ses gousses sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris parce que le sujet se raconte bien en ondes : une entreprise de Québec qui va expliquer à un auditoire pancanadien pourquoi la mauvaise herbe des champs de maïs peut isoler un manteau.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -4573,7 +4573,7 @@
       <c r="M60" s="11" t="inlineStr"/>
       <c r="N60" s="11" t="inlineStr"/>
     </row>
-    <row r="61" ht="250" customHeight="1">
+    <row r="61" ht="240" customHeight="1">
       <c r="A61" s="6" t="inlineStr">
         <is>
           <t>froide A</t>
@@ -4628,7 +4628,7 @@
         <is>
           <t>Bonjour André Fauteux,
 Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
-Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
+Ses gousses sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris parce que c'est une nouvelle de chez nous qui passe au national.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -4641,7 +4641,7 @@
       <c r="M61" s="11" t="inlineStr"/>
       <c r="N61" s="11" t="inlineStr"/>
     </row>
-    <row r="62" ht="250" customHeight="1">
+    <row r="62" ht="240" customHeight="1">
       <c r="A62" s="6" t="inlineStr">
         <is>
           <t>froide A</t>
@@ -4696,7 +4696,7 @@
         <is>
           <t>Bonjour Myriam Fimbry,
 Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
-Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
+Ses gousses sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris parce que vous couvrez l'agriculture. La question qui compte pour les producteurs n'a pas changé depuis l'effondrement de la filière en 2018 : est-ce qu'il y a un acheteur stable au bout du champ. On achète encore la récolte de producteurs d'ici et on la transforme nous-mêmes.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -4709,7 +4709,7 @@
       <c r="M62" s="11" t="inlineStr"/>
       <c r="N62" s="11" t="inlineStr"/>
     </row>
-    <row r="63" ht="250" customHeight="1">
+    <row r="63" ht="240" customHeight="1">
       <c r="A63" s="6" t="inlineStr">
         <is>
           <t>froide A</t>
@@ -4764,7 +4764,7 @@
         <is>
           <t>Bonjour Étienne Fortin-Gauthier,
 Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
-Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
+Ses gousses sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris parce que le sujet se raconte bien en ondes : une entreprise de Québec qui va expliquer à un auditoire pancanadien pourquoi la mauvaise herbe des champs de maïs peut isoler un manteau.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -4777,7 +4777,7 @@
       <c r="M63" s="11" t="inlineStr"/>
       <c r="N63" s="11" t="inlineStr"/>
     </row>
-    <row r="64" ht="250" customHeight="1">
+    <row r="64" ht="240" customHeight="1">
       <c r="A64" s="6" t="inlineStr">
         <is>
           <t>froide A</t>
@@ -4832,7 +4832,7 @@
         <is>
           <t>Bonjour Johanne Fournier,
 Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
-Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
+Ses gousses sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris parce que c'est une nouvelle de chez nous qui passe au national.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -4845,7 +4845,7 @@
       <c r="M64" s="11" t="inlineStr"/>
       <c r="N64" s="11" t="inlineStr"/>
     </row>
-    <row r="65" ht="250" customHeight="1">
+    <row r="65" ht="240" customHeight="1">
       <c r="A65" s="6" t="inlineStr">
         <is>
           <t>froide A</t>
@@ -4900,7 +4900,7 @@
         <is>
           <t>Bonjour Jean Garon,
 Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
-Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
+Ses gousses sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris parce que vous couvrez l'environnement. Notre pari est économique avant d'être militant : si l'asclépiade devient payante, les agriculteurs la gardent dans leurs champs, et les monarques retrouvent de l'habitat de reproduction.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -4913,7 +4913,7 @@
       <c r="M65" s="11" t="inlineStr"/>
       <c r="N65" s="11" t="inlineStr"/>
     </row>
-    <row r="66" ht="250" customHeight="1">
+    <row r="66" ht="240" customHeight="1">
       <c r="A66" s="6" t="inlineStr">
         <is>
           <t>froide A</t>
@@ -4968,7 +4968,7 @@
         <is>
           <t>Bonjour Cécile Gladel,
 Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
-Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
+Ses gousses sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris parce que le sujet se raconte bien en ondes : une entreprise de Québec qui va expliquer à un auditoire pancanadien pourquoi la mauvaise herbe des champs de maïs peut isoler un manteau.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -4981,7 +4981,7 @@
       <c r="M66" s="11" t="inlineStr"/>
       <c r="N66" s="11" t="inlineStr"/>
     </row>
-    <row r="67" ht="250" customHeight="1">
+    <row r="67" ht="240" customHeight="1">
       <c r="A67" s="6" t="inlineStr">
         <is>
           <t>froide A</t>
@@ -5036,7 +5036,7 @@
         <is>
           <t>Bonjour Marieke Glorieux-Stryckman,
 Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
-Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
+Ses gousses sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris parce que vous couvrez le plein air. À poids égal, la littérature donne la soie d'asclépiade pour environ 10 % plus isolante que le duvet. C'est un repère de laboratoire, pas une promesse de manteau, et c'est exactement pour ça que je préfère qu'on la teste.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -5049,7 +5049,7 @@
       <c r="M67" s="11" t="inlineStr"/>
       <c r="N67" s="11" t="inlineStr"/>
     </row>
-    <row r="68" ht="250" customHeight="1">
+    <row r="68" ht="240" customHeight="1">
       <c r="A68" s="6" t="inlineStr">
         <is>
           <t>froide A</t>
@@ -5104,7 +5104,7 @@
         <is>
           <t>Bonjour Maude Goyer,
 Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
-Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
+Ses gousses sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris parce que vous couvrez le plein air. À poids égal, la littérature donne la soie d'asclépiade pour environ 10 % plus isolante que le duvet. C'est un repère de laboratoire, pas une promesse de manteau, et c'est exactement pour ça que je préfère qu'on la teste.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -5117,7 +5117,7 @@
       <c r="M68" s="11" t="inlineStr"/>
       <c r="N68" s="11" t="inlineStr"/>
     </row>
-    <row r="69" ht="250" customHeight="1">
+    <row r="69" ht="240" customHeight="1">
       <c r="A69" s="6" t="inlineStr">
         <is>
           <t>froide A</t>
@@ -5172,7 +5172,7 @@
         <is>
           <t>Bonjour Pauline Gravel,
 Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
-Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
+Ses gousses sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris parce que vous couvrez l'agriculture. La question qui compte pour les producteurs n'a pas changé depuis l'effondrement de la filière en 2018 : est-ce qu'il y a un acheteur stable au bout du champ. On achète encore la récolte de producteurs d'ici et on la transforme nous-mêmes.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -5185,7 +5185,7 @@
       <c r="M69" s="11" t="inlineStr"/>
       <c r="N69" s="11" t="inlineStr"/>
     </row>
-    <row r="70" ht="250" customHeight="1">
+    <row r="70" ht="240" customHeight="1">
       <c r="A70" s="6" t="inlineStr">
         <is>
           <t>froide A</t>
@@ -5240,7 +5240,7 @@
         <is>
           <t>Bonjour Bernard Hervieux,
 Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
-Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
+Ses gousses sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris parce que le sujet se raconte bien en ondes : une entreprise de Québec qui va expliquer à un auditoire pancanadien pourquoi la mauvaise herbe des champs de maïs peut isoler un manteau.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -5253,7 +5253,7 @@
       <c r="M70" s="11" t="inlineStr"/>
       <c r="N70" s="11" t="inlineStr"/>
     </row>
-    <row r="71" ht="250" customHeight="1">
+    <row r="71" ht="240" customHeight="1">
       <c r="A71" s="6" t="inlineStr">
         <is>
           <t>froide A</t>
@@ -5308,7 +5308,7 @@
         <is>
           <t>Bonjour Leïla Jolin-Dahel,
 Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
-Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
+Ses gousses sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris parce que vous couvrez l'agriculture. La question qui compte pour les producteurs n'a pas changé depuis l'effondrement de la filière en 2018 : est-ce qu'il y a un acheteur stable au bout du champ. On achète encore la récolte de producteurs d'ici et on la transforme nous-mêmes.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -5321,7 +5321,7 @@
       <c r="M71" s="11" t="inlineStr"/>
       <c r="N71" s="11" t="inlineStr"/>
     </row>
-    <row r="72" ht="250" customHeight="1">
+    <row r="72" ht="240" customHeight="1">
       <c r="A72" s="6" t="inlineStr">
         <is>
           <t>froide A</t>
@@ -5376,7 +5376,7 @@
         <is>
           <t>Bonjour Kodjo Edjinam Nulagnon LOGO,
 Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
-Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
+Ses gousses sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris parce que vous couvrez l'environnement. Notre pari est économique avant d'être militant : si l'asclépiade devient payante, les agriculteurs la gardent dans leurs champs, et les monarques retrouvent de l'habitat de reproduction.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -5389,7 +5389,7 @@
       <c r="M72" s="11" t="inlineStr"/>
       <c r="N72" s="11" t="inlineStr"/>
     </row>
-    <row r="73" ht="250" customHeight="1">
+    <row r="73" ht="240" customHeight="1">
       <c r="A73" s="6" t="inlineStr">
         <is>
           <t>froide A</t>
@@ -5444,7 +5444,7 @@
         <is>
           <t>Bonjour Annie Labrecque,
 Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
-Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
+Ses gousses sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris parce que vous couvrez l'agriculture. La question qui compte pour les producteurs n'a pas changé depuis l'effondrement de la filière en 2018 : est-ce qu'il y a un acheteur stable au bout du champ. On achète encore la récolte de producteurs d'ici et on la transforme nous-mêmes.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -5457,7 +5457,7 @@
       <c r="M73" s="11" t="inlineStr"/>
       <c r="N73" s="11" t="inlineStr"/>
     </row>
-    <row r="74" ht="250" customHeight="1">
+    <row r="74" ht="240" customHeight="1">
       <c r="A74" s="6" t="inlineStr">
         <is>
           <t>froide A</t>
@@ -5512,7 +5512,7 @@
         <is>
           <t>Bonjour Marianne Lachapelle,
 Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
-Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
+Ses gousses sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris entre autres parce qu'une des premières usines de transformation de la fibre était à Granby, et que l'Estrie compte encore des producteurs d'asclépiade.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -5525,7 +5525,7 @@
       <c r="M74" s="11" t="inlineStr"/>
       <c r="N74" s="11" t="inlineStr"/>
     </row>
-    <row r="75" ht="250" customHeight="1">
+    <row r="75" ht="240" customHeight="1">
       <c r="A75" s="6" t="inlineStr">
         <is>
           <t>froide A</t>
@@ -5580,7 +5580,7 @@
         <is>
           <t>Bonjour Sophie Lachapelle,
 Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
-Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
+Ses gousses sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris parce que vous couvrez l'agriculture. La question qui compte pour les producteurs n'a pas changé depuis l'effondrement de la filière en 2018 : est-ce qu'il y a un acheteur stable au bout du champ. On achète encore la récolte de producteurs d'ici et on la transforme nous-mêmes.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -5593,7 +5593,7 @@
       <c r="M75" s="11" t="inlineStr"/>
       <c r="N75" s="11" t="inlineStr"/>
     </row>
-    <row r="76" ht="250" customHeight="1">
+    <row r="76" ht="240" customHeight="1">
       <c r="A76" s="6" t="inlineStr">
         <is>
           <t>froide A</t>
@@ -5648,7 +5648,7 @@
         <is>
           <t>Bonjour Alain Laforest,
 Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
-Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
+Ses gousses sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris parce que le sujet se raconte bien en ondes : une entreprise de Québec qui va expliquer à un auditoire pancanadien pourquoi la mauvaise herbe des champs de maïs peut isoler un manteau.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -5661,7 +5661,7 @@
       <c r="M76" s="11" t="inlineStr"/>
       <c r="N76" s="11" t="inlineStr"/>
     </row>
-    <row r="77" ht="250" customHeight="1">
+    <row r="77" ht="240" customHeight="1">
       <c r="A77" s="6" t="inlineStr">
         <is>
           <t>froide A</t>
@@ -5716,7 +5716,7 @@
         <is>
           <t>Bonjour Mikaël Lalancette,
 Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
-Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
+Ses gousses sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris parce que c'est une nouvelle de chez nous qui passe au national.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -5729,7 +5729,7 @@
       <c r="M77" s="11" t="inlineStr"/>
       <c r="N77" s="11" t="inlineStr"/>
     </row>
-    <row r="78" ht="250" customHeight="1">
+    <row r="78" ht="240" customHeight="1">
       <c r="A78" s="6" t="inlineStr">
         <is>
           <t>froide A</t>
@@ -5784,7 +5784,7 @@
         <is>
           <t>Bonjour Jean-Luc Lavallée,
 Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
-Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
+Ses gousses sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris parce que vous couvrez l'économie. On a bâti nos propres procédés de transformation parce qu'aucun sous-traitant ne voulait toucher à l'asclépiade, puis on a changé de modèle manufacturier l'an dernier pour rendre un manteau accessible à 300 $. J'en ai fait une vidéo ici : https://www.youtube.com/watch?v=GKyHh-Ok9JU.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -5797,7 +5797,7 @@
       <c r="M78" s="11" t="inlineStr"/>
       <c r="N78" s="11" t="inlineStr"/>
     </row>
-    <row r="79" ht="250" customHeight="1">
+    <row r="79" ht="240" customHeight="1">
       <c r="A79" s="6" t="inlineStr">
         <is>
           <t>froide A</t>
@@ -5852,7 +5852,7 @@
         <is>
           <t>Bonjour Jean-Francois Leblanc,
 Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
-Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
+Ses gousses sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris parce que vous couvrez le plein air. À poids égal, la littérature donne la soie d'asclépiade pour environ 10 % plus isolante que le duvet. C'est un repère de laboratoire, pas une promesse de manteau, et c'est exactement pour ça que je préfère qu'on la teste.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -5865,7 +5865,7 @@
       <c r="M79" s="11" t="inlineStr"/>
       <c r="N79" s="11" t="inlineStr"/>
     </row>
-    <row r="80" ht="250" customHeight="1">
+    <row r="80" ht="240" customHeight="1">
       <c r="A80" s="6" t="inlineStr">
         <is>
           <t>froide A</t>
@@ -5920,7 +5920,7 @@
         <is>
           <t>Bonjour Julie Leduc,
 Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
-Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
+Ses gousses sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris parce que vous couvrez le plein air. À poids égal, la littérature donne la soie d'asclépiade pour environ 10 % plus isolante que le duvet. C'est un repère de laboratoire, pas une promesse de manteau, et c'est exactement pour ça que je préfère qu'on la teste.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -5933,7 +5933,7 @@
       <c r="M80" s="11" t="inlineStr"/>
       <c r="N80" s="11" t="inlineStr"/>
     </row>
-    <row r="81" ht="250" customHeight="1">
+    <row r="81" ht="240" customHeight="1">
       <c r="A81" s="6" t="inlineStr">
         <is>
           <t>froide A</t>
@@ -5988,7 +5988,7 @@
         <is>
           <t>Bonjour Annie Martin,
 Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
-Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
+Ses gousses sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris parce que vous couvrez l'agriculture. La question qui compte pour les producteurs n'a pas changé depuis l'effondrement de la filière en 2018 : est-ce qu'il y a un acheteur stable au bout du champ. On achète encore la récolte de producteurs d'ici et on la transforme nous-mêmes.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -6001,7 +6001,7 @@
       <c r="M81" s="11" t="inlineStr"/>
       <c r="N81" s="11" t="inlineStr"/>
     </row>
-    <row r="82" ht="250" customHeight="1">
+    <row r="82" ht="240" customHeight="1">
       <c r="A82" s="6" t="inlineStr">
         <is>
           <t>froide A</t>
@@ -6076,7 +6076,7 @@
       <c r="M82" s="11" t="inlineStr"/>
       <c r="N82" s="11" t="inlineStr"/>
     </row>
-    <row r="83" ht="250" customHeight="1">
+    <row r="83" ht="240" customHeight="1">
       <c r="A83" s="6" t="inlineStr">
         <is>
           <t>froide A</t>
@@ -6131,7 +6131,7 @@
         <is>
           <t>Bonjour Charles Mathieu,
 Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
-Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
+Ses gousses sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris parce que vous couvrez l'environnement. Notre pari est économique avant d'être militant : si l'asclépiade devient payante, les agriculteurs la gardent dans leurs champs, et les monarques retrouvent de l'habitat de reproduction.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -6144,7 +6144,7 @@
       <c r="M83" s="11" t="inlineStr"/>
       <c r="N83" s="11" t="inlineStr"/>
     </row>
-    <row r="84" ht="250" customHeight="1">
+    <row r="84" ht="240" customHeight="1">
       <c r="A84" s="6" t="inlineStr">
         <is>
           <t>froide A</t>
@@ -6199,7 +6199,7 @@
         <is>
           <t>Bonjour Clara Matthey-Jonais,
 Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
-Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
+Ses gousses sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris parce que vous couvrez l'agriculture. La question qui compte pour les producteurs n'a pas changé depuis l'effondrement de la filière en 2018 : est-ce qu'il y a un acheteur stable au bout du champ. On achète encore la récolte de producteurs d'ici et on la transforme nous-mêmes.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -6212,7 +6212,7 @@
       <c r="M84" s="11" t="inlineStr"/>
       <c r="N84" s="11" t="inlineStr"/>
     </row>
-    <row r="85" ht="250" customHeight="1">
+    <row r="85" ht="240" customHeight="1">
       <c r="A85" s="6" t="inlineStr">
         <is>
           <t>froide A</t>
@@ -6267,7 +6267,7 @@
         <is>
           <t>Bonjour Valérian Mazataud,
 Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
-Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
+Ses gousses sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris parce que vous couvrez l'agriculture. La question qui compte pour les producteurs n'a pas changé depuis l'effondrement de la filière en 2018 : est-ce qu'il y a un acheteur stable au bout du champ. On achète encore la récolte de producteurs d'ici et on la transforme nous-mêmes.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -6280,7 +6280,7 @@
       <c r="M85" s="11" t="inlineStr"/>
       <c r="N85" s="11" t="inlineStr"/>
     </row>
-    <row r="86" ht="250" customHeight="1">
+    <row r="86" ht="240" customHeight="1">
       <c r="A86" s="6" t="inlineStr">
         <is>
           <t>froide A</t>
@@ -6335,7 +6335,7 @@
         <is>
           <t>Bonjour Lili Mercure,
 Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
-Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
+Ses gousses sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris parce que le sujet se raconte bien en ondes : une entreprise de Québec qui va expliquer à un auditoire pancanadien pourquoi la mauvaise herbe des champs de maïs peut isoler un manteau.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -6348,7 +6348,7 @@
       <c r="M86" s="11" t="inlineStr"/>
       <c r="N86" s="11" t="inlineStr"/>
     </row>
-    <row r="87" ht="250" customHeight="1">
+    <row r="87" ht="240" customHeight="1">
       <c r="A87" s="6" t="inlineStr">
         <is>
           <t>froide A</t>
@@ -6403,7 +6403,7 @@
         <is>
           <t>Bonjour Nicolas Mesly,
 Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
-Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
+Ses gousses sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris parce que vous couvrez l'agriculture. La question qui compte pour les producteurs n'a pas changé depuis l'effondrement de la filière en 2018 : est-ce qu'il y a un acheteur stable au bout du champ. On achète encore la récolte de producteurs d'ici et on la transforme nous-mêmes.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -6416,7 +6416,7 @@
       <c r="M87" s="11" t="inlineStr"/>
       <c r="N87" s="11" t="inlineStr"/>
     </row>
-    <row r="88" ht="250" customHeight="1">
+    <row r="88" ht="240" customHeight="1">
       <c r="A88" s="6" t="inlineStr">
         <is>
           <t>froide A</t>
@@ -6471,7 +6471,7 @@
         <is>
           <t>Bonjour Nicolas Michaud,
 Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
-Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
+Ses gousses sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris parce que vous couvrez l'agriculture. La question qui compte pour les producteurs n'a pas changé depuis l'effondrement de la filière en 2018 : est-ce qu'il y a un acheteur stable au bout du champ. On achète encore la récolte de producteurs d'ici et on la transforme nous-mêmes.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -6484,7 +6484,7 @@
       <c r="M88" s="11" t="inlineStr"/>
       <c r="N88" s="11" t="inlineStr"/>
     </row>
-    <row r="89" ht="250" customHeight="1">
+    <row r="89" ht="240" customHeight="1">
       <c r="A89" s="6" t="inlineStr">
         <is>
           <t>froide A</t>
@@ -6539,7 +6539,7 @@
         <is>
           <t>Bonjour Véronique Morin,
 Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
-Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
+Ses gousses sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris parce que vous couvrez l'agriculture. La question qui compte pour les producteurs n'a pas changé depuis l'effondrement de la filière en 2018 : est-ce qu'il y a un acheteur stable au bout du champ. On achète encore la récolte de producteurs d'ici et on la transforme nous-mêmes.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -6552,7 +6552,7 @@
       <c r="M89" s="11" t="inlineStr"/>
       <c r="N89" s="11" t="inlineStr"/>
     </row>
-    <row r="90" ht="250" customHeight="1">
+    <row r="90" ht="240" customHeight="1">
       <c r="A90" s="6" t="inlineStr">
         <is>
           <t>froide A</t>
@@ -6607,7 +6607,7 @@
         <is>
           <t>Bonjour Lila Mouch,
 Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
-Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
+Ses gousses sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris parce que le sujet se raconte bien en ondes : une entreprise de Québec qui va expliquer à un auditoire pancanadien pourquoi la mauvaise herbe des champs de maïs peut isoler un manteau.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -6620,7 +6620,7 @@
       <c r="M90" s="11" t="inlineStr"/>
       <c r="N90" s="11" t="inlineStr"/>
     </row>
-    <row r="91" ht="250" customHeight="1">
+    <row r="91" ht="240" customHeight="1">
       <c r="A91" s="6" t="inlineStr">
         <is>
           <t>froide A</t>
@@ -6675,7 +6675,7 @@
         <is>
           <t>Bonjour Olivier Mougeot,
 Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
-Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
+Ses gousses sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris parce que c'est une nouvelle de chez nous qui passe au national.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -6688,7 +6688,7 @@
       <c r="M91" s="11" t="inlineStr"/>
       <c r="N91" s="11" t="inlineStr"/>
     </row>
-    <row r="92" ht="250" customHeight="1">
+    <row r="92" ht="240" customHeight="1">
       <c r="A92" s="6" t="inlineStr">
         <is>
           <t>froide A</t>
@@ -6743,7 +6743,7 @@
         <is>
           <t>Bonjour Emmanuelle Mozayan-Verschaeve,
 Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
-Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
+Ses gousses sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris parce que vous couvrez le plein air. À poids égal, la littérature donne la soie d'asclépiade pour environ 10 % plus isolante que le duvet. C'est un repère de laboratoire, pas une promesse de manteau, et c'est exactement pour ça que je préfère qu'on la teste.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -6756,7 +6756,7 @@
       <c r="M92" s="11" t="inlineStr"/>
       <c r="N92" s="11" t="inlineStr"/>
     </row>
-    <row r="93" ht="250" customHeight="1">
+    <row r="93" ht="240" customHeight="1">
       <c r="A93" s="6" t="inlineStr">
         <is>
           <t>froide A</t>
@@ -6811,7 +6811,7 @@
         <is>
           <t>Bonjour Jean-Benoît Nadeau,
 Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
-Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
+Ses gousses sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris parce que vous couvrez le plein air. À poids égal, la littérature donne la soie d'asclépiade pour environ 10 % plus isolante que le duvet. C'est un repère de laboratoire, pas une promesse de manteau, et c'est exactement pour ça que je préfère qu'on la teste.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -6824,7 +6824,7 @@
       <c r="M93" s="11" t="inlineStr"/>
       <c r="N93" s="11" t="inlineStr"/>
     </row>
-    <row r="94" ht="250" customHeight="1">
+    <row r="94" ht="240" customHeight="1">
       <c r="A94" s="6" t="inlineStr">
         <is>
           <t>froide A</t>
@@ -6879,7 +6879,7 @@
         <is>
           <t>Bonjour Yves Ouellet,
 Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
-Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
+Ses gousses sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris parce que vous couvrez le plein air. À poids égal, la littérature donne la soie d'asclépiade pour environ 10 % plus isolante que le duvet. C'est un repère de laboratoire, pas une promesse de manteau, et c'est exactement pour ça que je préfère qu'on la teste.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -6892,7 +6892,7 @@
       <c r="M94" s="11" t="inlineStr"/>
       <c r="N94" s="11" t="inlineStr"/>
     </row>
-    <row r="95" ht="250" customHeight="1">
+    <row r="95" ht="240" customHeight="1">
       <c r="A95" s="6" t="inlineStr">
         <is>
           <t>froide A</t>
@@ -6947,7 +6947,7 @@
         <is>
           <t>Bonjour Josée Panet-Raymond,
 Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
-Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
+Ses gousses sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris parce que vous couvrez l'agriculture. La question qui compte pour les producteurs n'a pas changé depuis l'effondrement de la filière en 2018 : est-ce qu'il y a un acheteur stable au bout du champ. On achète encore la récolte de producteurs d'ici et on la transforme nous-mêmes.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -6960,7 +6960,7 @@
       <c r="M95" s="11" t="inlineStr"/>
       <c r="N95" s="11" t="inlineStr"/>
     </row>
-    <row r="96" ht="250" customHeight="1">
+    <row r="96" ht="240" customHeight="1">
       <c r="A96" s="6" t="inlineStr">
         <is>
           <t>froide A</t>
@@ -7015,7 +7015,7 @@
         <is>
           <t>Bonjour Yannick Patelli,
 Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
-Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
+Ses gousses sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris parce que vous couvrez l'agriculture. La question qui compte pour les producteurs n'a pas changé depuis l'effondrement de la filière en 2018 : est-ce qu'il y a un acheteur stable au bout du champ. On achète encore la récolte de producteurs d'ici et on la transforme nous-mêmes.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -7028,7 +7028,7 @@
       <c r="M96" s="11" t="inlineStr"/>
       <c r="N96" s="11" t="inlineStr"/>
     </row>
-    <row r="97" ht="250" customHeight="1">
+    <row r="97" ht="240" customHeight="1">
       <c r="A97" s="6" t="inlineStr">
         <is>
           <t>froide A</t>
@@ -7083,7 +7083,7 @@
         <is>
           <t>Bonjour Félix Pedneault,
 Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
-Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
+Ses gousses sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris parce que vous couvrez l'environnement. Notre pari est économique avant d'être militant : si l'asclépiade devient payante, les agriculteurs la gardent dans leurs champs, et les monarques retrouvent de l'habitat de reproduction.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -7096,7 +7096,7 @@
       <c r="M97" s="11" t="inlineStr"/>
       <c r="N97" s="11" t="inlineStr"/>
     </row>
-    <row r="98" ht="250" customHeight="1">
+    <row r="98" ht="240" customHeight="1">
       <c r="A98" s="6" t="inlineStr">
         <is>
           <t>froide A</t>
@@ -7151,7 +7151,7 @@
         <is>
           <t>Bonjour Marie-Eve Poulin,
 Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
-Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
+Ses gousses sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris parce que vous couvrez le plein air. À poids égal, la littérature donne la soie d'asclépiade pour environ 10 % plus isolante que le duvet. C'est un repère de laboratoire, pas une promesse de manteau, et c'est exactement pour ça que je préfère qu'on la teste.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -7164,7 +7164,7 @@
       <c r="M98" s="11" t="inlineStr"/>
       <c r="N98" s="11" t="inlineStr"/>
     </row>
-    <row r="99" ht="250" customHeight="1">
+    <row r="99" ht="240" customHeight="1">
       <c r="A99" s="6" t="inlineStr">
         <is>
           <t>froide A</t>
@@ -7219,7 +7219,7 @@
         <is>
           <t>Bonjour Marie-Hélène Proulx,
 Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
-Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
+Ses gousses sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris parce que vous couvrez l'agriculture. La question qui compte pour les producteurs n'a pas changé depuis l'effondrement de la filière en 2018 : est-ce qu'il y a un acheteur stable au bout du champ. On achète encore la récolte de producteurs d'ici et on la transforme nous-mêmes.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -7232,7 +7232,7 @@
       <c r="M99" s="11" t="inlineStr"/>
       <c r="N99" s="11" t="inlineStr"/>
     </row>
-    <row r="100" ht="250" customHeight="1">
+    <row r="100" ht="240" customHeight="1">
       <c r="A100" s="6" t="inlineStr">
         <is>
           <t>froide A</t>
@@ -7287,7 +7287,7 @@
         <is>
           <t>Bonjour Jean-Hugues Roy,
 Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
-Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
+Ses gousses sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris parce que c'est une nouvelle de chez nous qui passe au national.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -7300,7 +7300,7 @@
       <c r="M100" s="11" t="inlineStr"/>
       <c r="N100" s="11" t="inlineStr"/>
     </row>
-    <row r="101" ht="250" customHeight="1">
+    <row r="101" ht="240" customHeight="1">
       <c r="A101" s="6" t="inlineStr">
         <is>
           <t>froide A</t>
@@ -7355,7 +7355,7 @@
         <is>
           <t>Bonjour Martin Roy,
 Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
-Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
+Ses gousses sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris parce que c'est une nouvelle de chez nous qui passe au national.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -7368,7 +7368,7 @@
       <c r="M101" s="11" t="inlineStr"/>
       <c r="N101" s="11" t="inlineStr"/>
     </row>
-    <row r="102" ht="250" customHeight="1">
+    <row r="102" ht="240" customHeight="1">
       <c r="A102" s="6" t="inlineStr">
         <is>
           <t>froide A</t>
@@ -7423,7 +7423,7 @@
         <is>
           <t>Bonjour Sylvain Sarrazin,
 Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
-Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
+Ses gousses sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris parce que vous couvrez le plein air. À poids égal, la littérature donne la soie d'asclépiade pour environ 10 % plus isolante que le duvet. C'est un repère de laboratoire, pas une promesse de manteau, et c'est exactement pour ça que je préfère qu'on la teste.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -7436,7 +7436,7 @@
       <c r="M102" s="11" t="inlineStr"/>
       <c r="N102" s="11" t="inlineStr"/>
     </row>
-    <row r="103" ht="250" customHeight="1">
+    <row r="103" ht="240" customHeight="1">
       <c r="A103" s="6" t="inlineStr">
         <is>
           <t>froide A</t>
@@ -7491,7 +7491,7 @@
         <is>
           <t>Bonjour Pierre Sormany,
 Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
-Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
+Ses gousses sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris parce que vous couvrez le plein air. À poids égal, la littérature donne la soie d'asclépiade pour environ 10 % plus isolante que le duvet. C'est un repère de laboratoire, pas une promesse de manteau, et c'est exactement pour ça que je préfère qu'on la teste.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -7504,7 +7504,7 @@
       <c r="M103" s="11" t="inlineStr"/>
       <c r="N103" s="11" t="inlineStr"/>
     </row>
-    <row r="104" ht="250" customHeight="1">
+    <row r="104" ht="240" customHeight="1">
       <c r="A104" s="6" t="inlineStr">
         <is>
           <t>froide A</t>
@@ -7559,7 +7559,7 @@
         <is>
           <t>Bonjour Scott Stevenson,
 Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
-Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
+Ses gousses sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris entre autres parce qu'une des premières usines de transformation de la fibre était à Granby, et que l'Estrie compte encore des producteurs d'asclépiade.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -7572,7 +7572,7 @@
       <c r="M104" s="11" t="inlineStr"/>
       <c r="N104" s="11" t="inlineStr"/>
     </row>
-    <row r="105" ht="250" customHeight="1">
+    <row r="105" ht="240" customHeight="1">
       <c r="A105" s="6" t="inlineStr">
         <is>
           <t>froide A</t>
@@ -7627,7 +7627,7 @@
         <is>
           <t>Bonjour Michèle Tanganika,
 Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
-Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
+Ses gousses sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris parce que vous couvrez l'agriculture. La question qui compte pour les producteurs n'a pas changé depuis l'effondrement de la filière en 2018 : est-ce qu'il y a un acheteur stable au bout du champ. On achète encore la récolte de producteurs d'ici et on la transforme nous-mêmes.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -7640,7 +7640,7 @@
       <c r="M105" s="11" t="inlineStr"/>
       <c r="N105" s="11" t="inlineStr"/>
     </row>
-    <row r="106" ht="250" customHeight="1">
+    <row r="106" ht="240" customHeight="1">
       <c r="A106" s="6" t="inlineStr">
         <is>
           <t>froide A</t>
@@ -7695,7 +7695,7 @@
         <is>
           <t>Bonjour Stephane Tellier,
 Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
-Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
+Ses gousses sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris parce que le sujet se raconte bien en ondes : une entreprise de Québec qui va expliquer à un auditoire pancanadien pourquoi la mauvaise herbe des champs de maïs peut isoler un manteau.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -7708,7 +7708,7 @@
       <c r="M106" s="11" t="inlineStr"/>
       <c r="N106" s="11" t="inlineStr"/>
     </row>
-    <row r="107" ht="250" customHeight="1">
+    <row r="107" ht="240" customHeight="1">
       <c r="A107" s="6" t="inlineStr">
         <is>
           <t>froide A</t>
@@ -7763,7 +7763,7 @@
         <is>
           <t>Bonjour Karine Tremblay,
 Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
-Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
+Ses gousses sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris entre autres parce qu'une des premières usines de transformation de la fibre était à Granby, et que l'Estrie compte encore des producteurs d'asclépiade.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -7776,7 +7776,7 @@
       <c r="M107" s="11" t="inlineStr"/>
       <c r="N107" s="11" t="inlineStr"/>
     </row>
-    <row r="108" ht="250" customHeight="1">
+    <row r="108" ht="240" customHeight="1">
       <c r="A108" s="6" t="inlineStr">
         <is>
           <t>froide A</t>
@@ -7831,7 +7831,7 @@
         <is>
           <t>Bonjour Jean-Francois Venne,
 Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
-Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
+Ses gousses sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris parce que vous couvrez l'environnement. Notre pari est économique avant d'être militant : si l'asclépiade devient payante, les agriculteurs la gardent dans leurs champs, et les monarques retrouvent de l'habitat de reproduction.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -7844,7 +7844,7 @@
       <c r="M108" s="11" t="inlineStr"/>
       <c r="N108" s="11" t="inlineStr"/>
     </row>
-    <row r="109" ht="250" customHeight="1">
+    <row r="109" ht="240" customHeight="1">
       <c r="A109" s="6" t="inlineStr">
         <is>
           <t>froide A</t>
@@ -7899,7 +7899,7 @@
         <is>
           <t>Bonjour Shahram Yazdanpanah,
 Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
-Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
+Ses gousses sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris parce que vous couvrez le plein air. À poids égal, la littérature donne la soie d'asclépiade pour environ 10 % plus isolante que le duvet. C'est un repère de laboratoire, pas une promesse de manteau, et c'est exactement pour ça que je préfère qu'on la teste.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -7912,7 +7912,7 @@
       <c r="M109" s="11" t="inlineStr"/>
       <c r="N109" s="11" t="inlineStr"/>
     </row>
-    <row r="110" ht="250" customHeight="1">
+    <row r="110" ht="240" customHeight="1">
       <c r="A110" s="6" t="inlineStr">
         <is>
           <t>froide B</t>
@@ -7967,7 +7967,7 @@
         <is>
           <t>Bonjour Malika Alaoui,
 Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
-Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
+Ses gousses sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris parce que vous couvrez l'art de vivre et la consommation. Le contraste se photographie bien : la gousse dans le champ, la soie blanche dans la main, le manteau porté en ville.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -7980,7 +7980,7 @@
       <c r="M110" s="11" t="inlineStr"/>
       <c r="N110" s="11" t="inlineStr"/>
     </row>
-    <row r="111" ht="250" customHeight="1">
+    <row r="111" ht="240" customHeight="1">
       <c r="A111" s="6" t="inlineStr">
         <is>
           <t>froide B</t>
@@ -8035,7 +8035,7 @@
         <is>
           <t>Bonjour Yahia Arkat,
 Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
-Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
+Ses gousses sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris parce que vous couvrez l'environnement. Notre pari est économique avant d'être militant : si l'asclépiade devient payante, les agriculteurs la gardent dans leurs champs, et les monarques retrouvent de l'habitat de reproduction.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -8048,7 +8048,7 @@
       <c r="M111" s="11" t="inlineStr"/>
       <c r="N111" s="11" t="inlineStr"/>
     </row>
-    <row r="112" ht="250" customHeight="1">
+    <row r="112" ht="240" customHeight="1">
       <c r="A112" s="6" t="inlineStr">
         <is>
           <t>froide B</t>
@@ -8103,7 +8103,7 @@
         <is>
           <t>Bonjour MARC-OLIVIER BISSON,
 Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
-Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
+Ses gousses sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris parce que vous couvrez l'agriculture. La question qui compte pour les producteurs n'a pas changé depuis l'effondrement de la filière en 2018 : est-ce qu'il y a un acheteur stable au bout du champ. On achète encore la récolte de producteurs d'ici et on la transforme nous-mêmes.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -8116,7 +8116,7 @@
       <c r="M112" s="11" t="inlineStr"/>
       <c r="N112" s="11" t="inlineStr"/>
     </row>
-    <row r="113" ht="250" customHeight="1">
+    <row r="113" ht="240" customHeight="1">
       <c r="A113" s="6" t="inlineStr">
         <is>
           <t>froide B</t>
@@ -8171,7 +8171,7 @@
         <is>
           <t>Bonjour Maïté Belmir,
 Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
-Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
+Ses gousses sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris parce que vous couvrez l'environnement. Notre pari est économique avant d'être militant : si l'asclépiade devient payante, les agriculteurs la gardent dans leurs champs, et les monarques retrouvent de l'habitat de reproduction.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -8184,7 +8184,7 @@
       <c r="M113" s="11" t="inlineStr"/>
       <c r="N113" s="11" t="inlineStr"/>
     </row>
-    <row r="114" ht="250" customHeight="1">
+    <row r="114" ht="240" customHeight="1">
       <c r="A114" s="6" t="inlineStr">
         <is>
           <t>froide B</t>
@@ -8239,7 +8239,7 @@
         <is>
           <t>Bonjour André Bernard,
 Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
-Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
+Ses gousses sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris parce que vous couvrez l'environnement. Notre pari est économique avant d'être militant : si l'asclépiade devient payante, les agriculteurs la gardent dans leurs champs, et les monarques retrouvent de l'habitat de reproduction.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -8252,7 +8252,7 @@
       <c r="M114" s="11" t="inlineStr"/>
       <c r="N114" s="11" t="inlineStr"/>
     </row>
-    <row r="115" ht="250" customHeight="1">
+    <row r="115" ht="240" customHeight="1">
       <c r="A115" s="6" t="inlineStr">
         <is>
           <t>froide B</t>
@@ -8307,7 +8307,7 @@
         <is>
           <t>Bonjour Didier Bert,
 Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
-Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
+Ses gousses sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris parce que vous couvrez l'environnement. Notre pari est économique avant d'être militant : si l'asclépiade devient payante, les agriculteurs la gardent dans leurs champs, et les monarques retrouvent de l'habitat de reproduction.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -8320,7 +8320,7 @@
       <c r="M115" s="11" t="inlineStr"/>
       <c r="N115" s="11" t="inlineStr"/>
     </row>
-    <row r="116" ht="250" customHeight="1">
+    <row r="116" ht="240" customHeight="1">
       <c r="A116" s="6" t="inlineStr">
         <is>
           <t>froide B</t>
@@ -8375,7 +8375,7 @@
         <is>
           <t>Bonjour Sophie-Andrée Blondin,
 Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
-Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
+Ses gousses sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris parce que le sujet se raconte bien en ondes : une entreprise de Québec qui va expliquer à un auditoire pancanadien pourquoi la mauvaise herbe des champs de maïs peut isoler un manteau.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -8388,7 +8388,7 @@
       <c r="M116" s="11" t="inlineStr"/>
       <c r="N116" s="11" t="inlineStr"/>
     </row>
-    <row r="117" ht="250" customHeight="1">
+    <row r="117" ht="240" customHeight="1">
       <c r="A117" s="6" t="inlineStr">
         <is>
           <t>froide B</t>
@@ -8443,7 +8443,7 @@
         <is>
           <t>Bonjour Pierre Brochu,
 Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
-Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
+Ses gousses sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris entre autres parce qu'une des premières usines de transformation de la fibre était à Granby, et que l'Estrie compte encore des producteurs d'asclépiade.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -8456,7 +8456,7 @@
       <c r="M117" s="11" t="inlineStr"/>
       <c r="N117" s="11" t="inlineStr"/>
     </row>
-    <row r="118" ht="250" customHeight="1">
+    <row r="118" ht="240" customHeight="1">
       <c r="A118" s="6" t="inlineStr">
         <is>
           <t>froide B</t>
@@ -8511,7 +8511,7 @@
         <is>
           <t>Bonjour Gilles Bérubé,
 Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
-Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
+Ses gousses sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris entre autres parce que la Montérégie est une des régions où l'asclépiade se cultive encore, et que c'est de champs comme ceux-là que vient la fibre qu'on transforme.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -8524,7 +8524,7 @@
       <c r="M118" s="11" t="inlineStr"/>
       <c r="N118" s="11" t="inlineStr"/>
     </row>
-    <row r="119" ht="250" customHeight="1">
+    <row r="119" ht="240" customHeight="1">
       <c r="A119" s="6" t="inlineStr">
         <is>
           <t>froide B</t>
@@ -8579,7 +8579,7 @@
         <is>
           <t>Bonjour Daphné Cameron,
 Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
-Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
+Ses gousses sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris parce que vous couvrez l'agriculture. La question qui compte pour les producteurs n'a pas changé depuis l'effondrement de la filière en 2018 : est-ce qu'il y a un acheteur stable au bout du champ. On achète encore la récolte de producteurs d'ici et on la transforme nous-mêmes.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -8592,7 +8592,7 @@
       <c r="M119" s="11" t="inlineStr"/>
       <c r="N119" s="11" t="inlineStr"/>
     </row>
-    <row r="120" ht="250" customHeight="1">
+    <row r="120" ht="240" customHeight="1">
       <c r="A120" s="6" t="inlineStr">
         <is>
           <t>froide B</t>
@@ -8647,7 +8647,7 @@
         <is>
           <t>Bonjour Godefroy Macaire Chabi,
 Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
-Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
+Ses gousses sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris parce que c'est une nouvelle de chez nous qui passe au national.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -8660,7 +8660,7 @@
       <c r="M120" s="11" t="inlineStr"/>
       <c r="N120" s="11" t="inlineStr"/>
     </row>
-    <row r="121" ht="250" customHeight="1">
+    <row r="121" ht="240" customHeight="1">
       <c r="A121" s="6" t="inlineStr">
         <is>
           <t>froide B</t>
@@ -8715,7 +8715,7 @@
         <is>
           <t>Bonjour Sara Champagne,
 Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
-Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
+Ses gousses sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris parce que vous couvrez l'environnement. Notre pari est économique avant d'être militant : si l'asclépiade devient payante, les agriculteurs la gardent dans leurs champs, et les monarques retrouvent de l'habitat de reproduction.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -8728,7 +8728,7 @@
       <c r="M121" s="11" t="inlineStr"/>
       <c r="N121" s="11" t="inlineStr"/>
     </row>
-    <row r="122" ht="250" customHeight="1">
+    <row r="122" ht="240" customHeight="1">
       <c r="A122" s="6" t="inlineStr">
         <is>
           <t>froide B</t>
@@ -8783,7 +8783,7 @@
         <is>
           <t>Bonjour Sarah Champagne,
 Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
-Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
+Ses gousses sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris parce que vous couvrez l'agriculture. La question qui compte pour les producteurs n'a pas changé depuis l'effondrement de la filière en 2018 : est-ce qu'il y a un acheteur stable au bout du champ. On achète encore la récolte de producteurs d'ici et on la transforme nous-mêmes.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -8796,7 +8796,7 @@
       <c r="M122" s="11" t="inlineStr"/>
       <c r="N122" s="11" t="inlineStr"/>
     </row>
-    <row r="123" ht="250" customHeight="1">
+    <row r="123" ht="240" customHeight="1">
       <c r="A123" s="6" t="inlineStr">
         <is>
           <t>froide B</t>
@@ -8851,7 +8851,7 @@
         <is>
           <t>Bonjour Éric-Pierre Champagne,
 Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
-Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
+Ses gousses sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris parce que vous couvrez l'environnement. Notre pari est économique avant d'être militant : si l'asclépiade devient payante, les agriculteurs la gardent dans leurs champs, et les monarques retrouvent de l'habitat de reproduction.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -8864,7 +8864,7 @@
       <c r="M123" s="11" t="inlineStr"/>
       <c r="N123" s="11" t="inlineStr"/>
     </row>
-    <row r="124" ht="250" customHeight="1">
+    <row r="124" ht="240" customHeight="1">
       <c r="A124" s="6" t="inlineStr">
         <is>
           <t>froide B</t>
@@ -8919,7 +8919,7 @@
         <is>
           <t>Bonjour Marine Corniou,
 Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
-Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
+Ses gousses sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris parce que vous couvrez l'environnement. Notre pari est économique avant d'être militant : si l'asclépiade devient payante, les agriculteurs la gardent dans leurs champs, et les monarques retrouvent de l'habitat de reproduction.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -8932,7 +8932,7 @@
       <c r="M124" s="11" t="inlineStr"/>
       <c r="N124" s="11" t="inlineStr"/>
     </row>
-    <row r="125" ht="250" customHeight="1">
+    <row r="125" ht="240" customHeight="1">
       <c r="A125" s="6" t="inlineStr">
         <is>
           <t>froide B</t>
@@ -8987,7 +8987,7 @@
         <is>
           <t>Bonjour Catherine Crépeau,
 Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
-Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
+Ses gousses sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris parce que vous couvrez l'environnement. Notre pari est économique avant d'être militant : si l'asclépiade devient payante, les agriculteurs la gardent dans leurs champs, et les monarques retrouvent de l'habitat de reproduction.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -9000,7 +9000,7 @@
       <c r="M125" s="11" t="inlineStr"/>
       <c r="N125" s="11" t="inlineStr"/>
     </row>
-    <row r="126" ht="250" customHeight="1">
+    <row r="126" ht="240" customHeight="1">
       <c r="A126" s="6" t="inlineStr">
         <is>
           <t>froide B</t>
@@ -9055,7 +9055,7 @@
         <is>
           <t>Bonjour Laurence Dami-Houle,
 Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
-Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
+Ses gousses sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris parce que c'est une nouvelle de chez nous qui passe au national.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -9068,7 +9068,7 @@
       <c r="M126" s="11" t="inlineStr"/>
       <c r="N126" s="11" t="inlineStr"/>
     </row>
-    <row r="127" ht="250" customHeight="1">
+    <row r="127" ht="240" customHeight="1">
       <c r="A127" s="6" t="inlineStr">
         <is>
           <t>froide B</t>
@@ -9123,7 +9123,7 @@
         <is>
           <t>Bonjour Amélie Daoust-Boisvert,
 Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
-Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
+Ses gousses sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris entre autres parce que la Montérégie est une des régions où l'asclépiade se cultive encore, et que c'est de champs comme ceux-là que vient la fibre qu'on transforme.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -9136,7 +9136,7 @@
       <c r="M127" s="11" t="inlineStr"/>
       <c r="N127" s="11" t="inlineStr"/>
     </row>
-    <row r="128" ht="250" customHeight="1">
+    <row r="128" ht="240" customHeight="1">
       <c r="A128" s="6" t="inlineStr">
         <is>
           <t>froide B</t>
@@ -9191,7 +9191,7 @@
         <is>
           <t>Bonjour Dominique Degré,
 Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
-Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
+Ses gousses sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris entre autres parce que la Montérégie est une des régions où l'asclépiade se cultive encore, et que c'est de champs comme ceux-là que vient la fibre qu'on transforme.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -9204,7 +9204,7 @@
       <c r="M128" s="11" t="inlineStr"/>
       <c r="N128" s="11" t="inlineStr"/>
     </row>
-    <row r="129" ht="250" customHeight="1">
+    <row r="129" ht="240" customHeight="1">
       <c r="A129" s="6" t="inlineStr">
         <is>
           <t>froide B</t>
@@ -9259,7 +9259,7 @@
         <is>
           <t>Bonjour Quentin Dufranne,
 Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
-Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
+Ses gousses sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris parce que vous couvrez l'environnement. Notre pari est économique avant d'être militant : si l'asclépiade devient payante, les agriculteurs la gardent dans leurs champs, et les monarques retrouvent de l'habitat de reproduction.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -9272,7 +9272,7 @@
       <c r="M129" s="11" t="inlineStr"/>
       <c r="N129" s="11" t="inlineStr"/>
     </row>
-    <row r="130" ht="250" customHeight="1">
+    <row r="130" ht="240" customHeight="1">
       <c r="A130" s="6" t="inlineStr">
         <is>
           <t>froide B</t>
@@ -9327,7 +9327,7 @@
         <is>
           <t>Bonjour Ève Dumas,
 Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
-Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
+Ses gousses sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris parce que vous couvrez l'agriculture. La question qui compte pour les producteurs n'a pas changé depuis l'effondrement de la filière en 2018 : est-ce qu'il y a un acheteur stable au bout du champ. On achète encore la récolte de producteurs d'ici et on la transforme nous-mêmes.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -9340,7 +9340,7 @@
       <c r="M130" s="11" t="inlineStr"/>
       <c r="N130" s="11" t="inlineStr"/>
     </row>
-    <row r="131" ht="250" customHeight="1">
+    <row r="131" ht="240" customHeight="1">
       <c r="A131" s="6" t="inlineStr">
         <is>
           <t>froide B</t>
@@ -9395,7 +9395,7 @@
         <is>
           <t>Bonjour Michel Fortier,
 Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
-Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
+Ses gousses sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris parce que c'est une nouvelle de chez nous qui passe au national.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -9408,7 +9408,7 @@
       <c r="M131" s="11" t="inlineStr"/>
       <c r="N131" s="11" t="inlineStr"/>
     </row>
-    <row r="132" ht="250" customHeight="1">
+    <row r="132" ht="240" customHeight="1">
       <c r="A132" s="6" t="inlineStr">
         <is>
           <t>froide B</t>
@@ -9463,7 +9463,7 @@
         <is>
           <t>Bonjour Marie-Eve Fournier,
 Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
-Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
+Ses gousses sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris parce que vous couvrez l'économie. On a bâti nos propres procédés de transformation parce qu'aucun sous-traitant ne voulait toucher à l'asclépiade, puis on a changé de modèle manufacturier l'an dernier pour rendre un manteau accessible à 300 $. J'en ai fait une vidéo ici : https://www.youtube.com/watch?v=GKyHh-Ok9JU.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -9476,7 +9476,7 @@
       <c r="M132" s="11" t="inlineStr"/>
       <c r="N132" s="11" t="inlineStr"/>
     </row>
-    <row r="133" ht="250" customHeight="1">
+    <row r="133" ht="240" customHeight="1">
       <c r="A133" s="6" t="inlineStr">
         <is>
           <t>froide B</t>
@@ -9531,7 +9531,7 @@
         <is>
           <t>Bonjour Raymond Fournier,
 Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
-Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
+Ses gousses sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris entre autres parce que la Montérégie est une des régions où l'asclépiade se cultive encore, et que c'est de champs comme ceux-là que vient la fibre qu'on transforme.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -9544,7 +9544,7 @@
       <c r="M133" s="11" t="inlineStr"/>
       <c r="N133" s="11" t="inlineStr"/>
     </row>
-    <row r="134" ht="250" customHeight="1">
+    <row r="134" ht="240" customHeight="1">
       <c r="A134" s="6" t="inlineStr">
         <is>
           <t>froide B</t>
@@ -9599,7 +9599,7 @@
         <is>
           <t>Bonjour Marie-Pier Frappier,
 Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
-Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
+Ses gousses sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris parce que vous couvrez l'économie. On a bâti nos propres procédés de transformation parce qu'aucun sous-traitant ne voulait toucher à l'asclépiade, puis on a changé de modèle manufacturier l'an dernier pour rendre un manteau accessible à 300 $. J'en ai fait une vidéo ici : https://www.youtube.com/watch?v=GKyHh-Ok9JU.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -9612,7 +9612,7 @@
       <c r="M134" s="11" t="inlineStr"/>
       <c r="N134" s="11" t="inlineStr"/>
     </row>
-    <row r="135" ht="250" customHeight="1">
+    <row r="135" ht="240" customHeight="1">
       <c r="A135" s="6" t="inlineStr">
         <is>
           <t>froide B</t>
@@ -9667,7 +9667,7 @@
         <is>
           <t>Bonjour Marie-Julie Gagnon,
 Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
-Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
+Ses gousses sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris entre autres parce que la Montérégie est une des régions où l'asclépiade se cultive encore, et que c'est de champs comme ceux-là que vient la fibre qu'on transforme.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -9680,7 +9680,7 @@
       <c r="M135" s="11" t="inlineStr"/>
       <c r="N135" s="11" t="inlineStr"/>
     </row>
-    <row r="136" ht="250" customHeight="1">
+    <row r="136" ht="240" customHeight="1">
       <c r="A136" s="6" t="inlineStr">
         <is>
           <t>froide B</t>
@@ -9735,7 +9735,7 @@
         <is>
           <t>Bonjour Chloé Germain-Thérien,
 Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
-Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
+Ses gousses sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris entre autres parce que l'asclépiade a eu son grand moment industriel chez vous : l'usine de Saint-Tite achetait 90 % des récoltes du Québec avant que la filière se casse en 2018. Des producteurs de la Mauricie cultivent encore, et on continue d'acheter leur récolte.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -9748,7 +9748,7 @@
       <c r="M136" s="11" t="inlineStr"/>
       <c r="N136" s="11" t="inlineStr"/>
     </row>
-    <row r="137" ht="250" customHeight="1">
+    <row r="137" ht="240" customHeight="1">
       <c r="A137" s="6" t="inlineStr">
         <is>
           <t>froide B</t>
@@ -9803,7 +9803,7 @@
         <is>
           <t>Bonjour Charlotte Glorieux,
 Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
-Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
+Ses gousses sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris parce que vous couvrez le plein air. À poids égal, la littérature donne la soie d'asclépiade pour environ 10 % plus isolante que le duvet. C'est un repère de laboratoire, pas une promesse de manteau, et c'est exactement pour ça que je préfère qu'on la teste.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -9816,7 +9816,7 @@
       <c r="M137" s="11" t="inlineStr"/>
       <c r="N137" s="11" t="inlineStr"/>
     </row>
-    <row r="138" ht="250" customHeight="1">
+    <row r="138" ht="240" customHeight="1">
       <c r="A138" s="6" t="inlineStr">
         <is>
           <t>froide B</t>
@@ -9871,7 +9871,7 @@
         <is>
           <t>Bonjour Annie Hudon,
 Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
-Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
+Ses gousses sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris parce que vous couvrez l'économie. On a bâti nos propres procédés de transformation parce qu'aucun sous-traitant ne voulait toucher à l'asclépiade, puis on a changé de modèle manufacturier l'an dernier pour rendre un manteau accessible à 300 $. J'en ai fait une vidéo ici : https://www.youtube.com/watch?v=GKyHh-Ok9JU.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -9884,7 +9884,7 @@
       <c r="M138" s="11" t="inlineStr"/>
       <c r="N138" s="11" t="inlineStr"/>
     </row>
-    <row r="139" ht="250" customHeight="1">
+    <row r="139" ht="240" customHeight="1">
       <c r="A139" s="6" t="inlineStr">
         <is>
           <t>froide B</t>
@@ -9939,7 +9939,7 @@
         <is>
           <t>Bonjour Ahmed Kouaou,
 Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
-Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
+Ses gousses sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris parce que vous couvrez l'environnement. Notre pari est économique avant d'être militant : si l'asclépiade devient payante, les agriculteurs la gardent dans leurs champs, et les monarques retrouvent de l'habitat de reproduction.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -9952,7 +9952,7 @@
       <c r="M139" s="11" t="inlineStr"/>
       <c r="N139" s="11" t="inlineStr"/>
     </row>
-    <row r="140" ht="250" customHeight="1">
+    <row r="140" ht="240" customHeight="1">
       <c r="A140" s="6" t="inlineStr">
         <is>
           <t>froide B</t>
@@ -10007,7 +10007,7 @@
         <is>
           <t>Bonjour Tania Krywiak,
 Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
-Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
+Ses gousses sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris parce que vous couvrez l'environnement. Notre pari est économique avant d'être militant : si l'asclépiade devient payante, les agriculteurs la gardent dans leurs champs, et les monarques retrouvent de l'habitat de reproduction.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -10020,7 +10020,7 @@
       <c r="M140" s="11" t="inlineStr"/>
       <c r="N140" s="11" t="inlineStr"/>
     </row>
-    <row r="141" ht="250" customHeight="1">
+    <row r="141" ht="240" customHeight="1">
       <c r="A141" s="6" t="inlineStr">
         <is>
           <t>froide B</t>
@@ -10075,7 +10075,7 @@
         <is>
           <t>Bonjour Jacinthe Lafrance,
 Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
-Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
+Ses gousses sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris entre autres parce que l'asclépiade a eu son grand moment industriel chez vous : l'usine de Saint-Tite achetait 90 % des récoltes du Québec avant que la filière se casse en 2018. Des producteurs de la Mauricie cultivent encore, et on continue d'acheter leur récolte.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -10088,7 +10088,7 @@
       <c r="M141" s="11" t="inlineStr"/>
       <c r="N141" s="11" t="inlineStr"/>
     </row>
-    <row r="142" ht="250" customHeight="1">
+    <row r="142" ht="240" customHeight="1">
       <c r="A142" s="6" t="inlineStr">
         <is>
           <t>froide B</t>
@@ -10143,7 +10143,7 @@
         <is>
           <t>Bonjour Bruno Lamolet,
 Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
-Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
+Ses gousses sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris entre autres parce que la Montérégie est une des régions où l'asclépiade se cultive encore, et que c'est de champs comme ceux-là que vient la fibre qu'on transforme.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -10156,7 +10156,7 @@
       <c r="M142" s="11" t="inlineStr"/>
       <c r="N142" s="11" t="inlineStr"/>
     </row>
-    <row r="143" ht="250" customHeight="1">
+    <row r="143" ht="240" customHeight="1">
       <c r="A143" s="6" t="inlineStr">
         <is>
           <t>froide B</t>
@@ -10211,7 +10211,7 @@
         <is>
           <t>Bonjour Yvan Lamontagne,
 Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
-Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
+Ses gousses sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris entre autres parce qu'une des premières usines de transformation de la fibre était à Granby, et que l'Estrie compte encore des producteurs d'asclépiade.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -10224,7 +10224,7 @@
       <c r="M143" s="11" t="inlineStr"/>
       <c r="N143" s="11" t="inlineStr"/>
     </row>
-    <row r="144" ht="250" customHeight="1">
+    <row r="144" ht="240" customHeight="1">
       <c r="A144" s="6" t="inlineStr">
         <is>
           <t>froide B</t>
@@ -10279,7 +10279,7 @@
         <is>
           <t>Bonjour Yves Langlois,
 Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
-Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
+Ses gousses sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris entre autres parce qu'une des premières usines de transformation de la fibre était à Granby, et que l'Estrie compte encore des producteurs d'asclépiade.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -10292,7 +10292,7 @@
       <c r="M144" s="11" t="inlineStr"/>
       <c r="N144" s="11" t="inlineStr"/>
     </row>
-    <row r="145" ht="250" customHeight="1">
+    <row r="145" ht="240" customHeight="1">
       <c r="A145" s="6" t="inlineStr">
         <is>
           <t>froide B</t>
@@ -10347,7 +10347,7 @@
         <is>
           <t>Bonjour Anne Marie Lecomte,
 Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
-Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
+Ses gousses sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris parce que vous couvrez l'économie. On a bâti nos propres procédés de transformation parce qu'aucun sous-traitant ne voulait toucher à l'asclépiade, puis on a changé de modèle manufacturier l'an dernier pour rendre un manteau accessible à 300 $. J'en ai fait une vidéo ici : https://www.youtube.com/watch?v=GKyHh-Ok9JU.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -10360,7 +10360,7 @@
       <c r="M145" s="11" t="inlineStr"/>
       <c r="N145" s="11" t="inlineStr"/>
     </row>
-    <row r="146" ht="250" customHeight="1">
+    <row r="146" ht="240" customHeight="1">
       <c r="A146" s="6" t="inlineStr">
         <is>
           <t>froide B</t>
@@ -10415,7 +10415,7 @@
         <is>
           <t>Bonjour Stéphanie Mac Farlane,
 Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
-Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
+Ses gousses sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris entre autres parce que la Montérégie est une des régions où l'asclépiade se cultive encore, et que c'est de champs comme ceux-là que vient la fibre qu'on transforme.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -10428,7 +10428,7 @@
       <c r="M146" s="11" t="inlineStr"/>
       <c r="N146" s="11" t="inlineStr"/>
     </row>
-    <row r="147" ht="250" customHeight="1">
+    <row r="147" ht="240" customHeight="1">
       <c r="A147" s="6" t="inlineStr">
         <is>
           <t>froide B</t>
@@ -10483,7 +10483,7 @@
         <is>
           <t>Bonjour Philippe Marois,
 Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
-Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
+Ses gousses sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris entre autres parce que la Montérégie est une des régions où l'asclépiade se cultive encore, et que c'est de champs comme ceux-là que vient la fibre qu'on transforme.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -10496,7 +10496,7 @@
       <c r="M147" s="11" t="inlineStr"/>
       <c r="N147" s="11" t="inlineStr"/>
     </row>
-    <row r="148" ht="250" customHeight="1">
+    <row r="148" ht="240" customHeight="1">
       <c r="A148" s="6" t="inlineStr">
         <is>
           <t>froide B</t>
@@ -10551,7 +10551,7 @@
         <is>
           <t>Bonjour Gildas Meneu,
 Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
-Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
+Ses gousses sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris parce que vous couvrez l'agriculture. La question qui compte pour les producteurs n'a pas changé depuis l'effondrement de la filière en 2018 : est-ce qu'il y a un acheteur stable au bout du champ. On achète encore la récolte de producteurs d'ici et on la transforme nous-mêmes.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -10564,7 +10564,7 @@
       <c r="M148" s="11" t="inlineStr"/>
       <c r="N148" s="11" t="inlineStr"/>
     </row>
-    <row r="149" ht="250" customHeight="1">
+    <row r="149" ht="240" customHeight="1">
       <c r="A149" s="6" t="inlineStr">
         <is>
           <t>froide B</t>
@@ -10619,7 +10619,7 @@
         <is>
           <t>Bonjour Louis-Xavier Michaud,
 Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
-Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
+Ses gousses sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris parce que c'est une nouvelle de chez nous qui passe au national.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -10632,7 +10632,7 @@
       <c r="M149" s="11" t="inlineStr"/>
       <c r="N149" s="11" t="inlineStr"/>
     </row>
-    <row r="150" ht="250" customHeight="1">
+    <row r="150" ht="240" customHeight="1">
       <c r="A150" s="6" t="inlineStr">
         <is>
           <t>froide B</t>
@@ -10687,7 +10687,7 @@
         <is>
           <t>Bonjour Anne Montplaisir,
 Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
-Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
+Ses gousses sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris parce que vous couvrez le plein air. À poids égal, la littérature donne la soie d'asclépiade pour environ 10 % plus isolante que le duvet. C'est un repère de laboratoire, pas une promesse de manteau, et c'est exactement pour ça que je préfère qu'on la teste.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -10700,7 +10700,7 @@
       <c r="M150" s="11" t="inlineStr"/>
       <c r="N150" s="11" t="inlineStr"/>
     </row>
-    <row r="151" ht="250" customHeight="1">
+    <row r="151" ht="240" customHeight="1">
       <c r="A151" s="6" t="inlineStr">
         <is>
           <t>froide B</t>
@@ -10755,7 +10755,7 @@
         <is>
           <t>Bonjour Karianne Nepton-Philippe,
 Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
-Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
+Ses gousses sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris parce que c'est une nouvelle de chez nous qui passe au national.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -10768,7 +10768,7 @@
       <c r="M151" s="11" t="inlineStr"/>
       <c r="N151" s="11" t="inlineStr"/>
     </row>
-    <row r="152" ht="250" customHeight="1">
+    <row r="152" ht="240" customHeight="1">
       <c r="A152" s="6" t="inlineStr">
         <is>
           <t>froide B</t>
@@ -10823,7 +10823,7 @@
         <is>
           <t>Bonjour Geneviève Normand,
 Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
-Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
+Ses gousses sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris entre autres parce que la Montérégie est une des régions où l'asclépiade se cultive encore, et que c'est de champs comme ceux-là que vient la fibre qu'on transforme.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -10836,7 +10836,7 @@
       <c r="M152" s="11" t="inlineStr"/>
       <c r="N152" s="11" t="inlineStr"/>
     </row>
-    <row r="153" ht="250" customHeight="1">
+    <row r="153" ht="240" customHeight="1">
       <c r="A153" s="6" t="inlineStr">
         <is>
           <t>froide B</t>
@@ -10891,7 +10891,7 @@
         <is>
           <t>Bonjour Carole Payer,
 Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
-Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
+Ses gousses sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris entre autres parce que l'asclépiade se cultive dans votre région depuis la première vague de 2013, et que plusieurs des producteurs qui ont tenu bon nous vendent encore leur récolte.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -10904,7 +10904,7 @@
       <c r="M153" s="11" t="inlineStr"/>
       <c r="N153" s="11" t="inlineStr"/>
     </row>
-    <row r="154" ht="250" customHeight="1">
+    <row r="154" ht="240" customHeight="1">
       <c r="A154" s="6" t="inlineStr">
         <is>
           <t>froide B</t>
@@ -10959,7 +10959,7 @@
         <is>
           <t>Bonjour Boris Proulx,
 Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
-Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
+Ses gousses sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris parce que vous couvrez l'environnement. Notre pari est économique avant d'être militant : si l'asclépiade devient payante, les agriculteurs la gardent dans leurs champs, et les monarques retrouvent de l'habitat de reproduction.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -10972,7 +10972,7 @@
       <c r="M154" s="11" t="inlineStr"/>
       <c r="N154" s="11" t="inlineStr"/>
     </row>
-    <row r="155" ht="250" customHeight="1">
+    <row r="155" ht="240" customHeight="1">
       <c r="A155" s="6" t="inlineStr">
         <is>
           <t>froide B</t>
@@ -11027,7 +11027,7 @@
         <is>
           <t>Bonjour Philippe Robitaille-Grou,
 Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
-Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
+Ses gousses sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris parce que vous couvrez l'environnement. Notre pari est économique avant d'être militant : si l'asclépiade devient payante, les agriculteurs la gardent dans leurs champs, et les monarques retrouvent de l'habitat de reproduction.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -11040,7 +11040,7 @@
       <c r="M155" s="11" t="inlineStr"/>
       <c r="N155" s="11" t="inlineStr"/>
     </row>
-    <row r="156" ht="250" customHeight="1">
+    <row r="156" ht="240" customHeight="1">
       <c r="A156" s="6" t="inlineStr">
         <is>
           <t>froide B</t>
@@ -11095,7 +11095,7 @@
         <is>
           <t>Bonjour Gwen Roley,
 Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
-Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
+Ses gousses sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris parce que vous couvrez l'environnement. Notre pari est économique avant d'être militant : si l'asclépiade devient payante, les agriculteurs la gardent dans leurs champs, et les monarques retrouvent de l'habitat de reproduction.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -11108,7 +11108,7 @@
       <c r="M156" s="11" t="inlineStr"/>
       <c r="N156" s="11" t="inlineStr"/>
     </row>
-    <row r="157" ht="250" customHeight="1">
+    <row r="157" ht="240" customHeight="1">
       <c r="A157" s="6" t="inlineStr">
         <is>
           <t>froide B</t>
@@ -11163,7 +11163,7 @@
         <is>
           <t>Bonjour Mathieu-Robert Sauvé,
 Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
-Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
+Ses gousses sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris parce que vous couvrez l'environnement. Notre pari est économique avant d'être militant : si l'asclépiade devient payante, les agriculteurs la gardent dans leurs champs, et les monarques retrouvent de l'habitat de reproduction.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -11176,7 +11176,7 @@
       <c r="M157" s="11" t="inlineStr"/>
       <c r="N157" s="11" t="inlineStr"/>
     </row>
-    <row r="158" ht="250" customHeight="1">
+    <row r="158" ht="240" customHeight="1">
       <c r="A158" s="6" t="inlineStr">
         <is>
           <t>froide B</t>
@@ -11231,7 +11231,7 @@
         <is>
           <t>Bonjour Pierre St-Arnaud,
 Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
-Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
+Ses gousses sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris parce que vous couvrez l'agriculture. La question qui compte pour les producteurs n'a pas changé depuis l'effondrement de la filière en 2018 : est-ce qu'il y a un acheteur stable au bout du champ. On achète encore la récolte de producteurs d'ici et on la transforme nous-mêmes.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -11244,7 +11244,7 @@
       <c r="M158" s="11" t="inlineStr"/>
       <c r="N158" s="11" t="inlineStr"/>
     </row>
-    <row r="159" ht="250" customHeight="1">
+    <row r="159" ht="240" customHeight="1">
       <c r="A159" s="6" t="inlineStr">
         <is>
           <t>froide B</t>
@@ -11299,7 +11299,7 @@
         <is>
           <t>Bonjour Katherine Tremblay,
 Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
-Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
+Ses gousses sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris entre autres parce que la Montérégie est une des régions où l'asclépiade se cultive encore, et que c'est de champs comme ceux-là que vient la fibre qu'on transforme.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -11312,7 +11312,7 @@
       <c r="M159" s="11" t="inlineStr"/>
       <c r="N159" s="11" t="inlineStr"/>
     </row>
-    <row r="160" ht="250" customHeight="1">
+    <row r="160" ht="240" customHeight="1">
       <c r="A160" s="6" t="inlineStr">
         <is>
           <t>froide B</t>
@@ -11367,7 +11367,7 @@
         <is>
           <t>Bonjour Michel Tremblay,
 Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
-Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
+Ses gousses sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris entre autres parce que l'asclépiade se cultive dans votre région depuis la première vague de 2013, et que plusieurs des producteurs qui ont tenu bon nous vendent encore leur récolte.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -11380,7 +11380,7 @@
       <c r="M160" s="11" t="inlineStr"/>
       <c r="N160" s="11" t="inlineStr"/>
     </row>
-    <row r="161" ht="250" customHeight="1">
+    <row r="161" ht="240" customHeight="1">
       <c r="A161" s="6" t="inlineStr">
         <is>
           <t>froide B</t>
@@ -11435,7 +11435,7 @@
         <is>
           <t>Bonjour Martin Vallières,
 Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
-Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
+Ses gousses sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris parce que vous couvrez l'économie. On a bâti nos propres procédés de transformation parce qu'aucun sous-traitant ne voulait toucher à l'asclépiade, puis on a changé de modèle manufacturier l'an dernier pour rendre un manteau accessible à 300 $. J'en ai fait une vidéo ici : https://www.youtube.com/watch?v=GKyHh-Ok9JU.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -11448,7 +11448,7 @@
       <c r="M161" s="11" t="inlineStr"/>
       <c r="N161" s="11" t="inlineStr"/>
     </row>
-    <row r="162" ht="250" customHeight="1">
+    <row r="162" ht="240" customHeight="1">
       <c r="A162" s="6" t="inlineStr">
         <is>
           <t>froide B</t>
@@ -11503,7 +11503,7 @@
         <is>
           <t>Bonjour Yanick Villedieu,
 Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
-Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
+Ses gousses sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris parce que vous couvrez l'environnement. Notre pari est économique avant d'être militant : si l'asclépiade devient payante, les agriculteurs la gardent dans leurs champs, et les monarques retrouvent de l'habitat de reproduction.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -11516,7 +11516,7 @@
       <c r="M162" s="11" t="inlineStr"/>
       <c r="N162" s="11" t="inlineStr"/>
     </row>
-    <row r="163" ht="250" customHeight="1">
+    <row r="163" ht="240" customHeight="1">
       <c r="A163" s="6" t="inlineStr">
         <is>
           <t>froide C</t>
@@ -11571,7 +11571,7 @@
         <is>
           <t>Bonjour Jonathan Allard,
 Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
-Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
+Ses gousses sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris parce que vous couvrez l'environnement. Notre pari est économique avant d'être militant : si l'asclépiade devient payante, les agriculteurs la gardent dans leurs champs, et les monarques retrouvent de l'habitat de reproduction.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -11584,7 +11584,7 @@
       <c r="M163" s="11" t="inlineStr"/>
       <c r="N163" s="11" t="inlineStr"/>
     </row>
-    <row r="164" ht="250" customHeight="1">
+    <row r="164" ht="240" customHeight="1">
       <c r="A164" s="6" t="inlineStr">
         <is>
           <t>froide C</t>
@@ -11639,7 +11639,7 @@
         <is>
           <t>Bonjour Anick Baribeau,
 Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
-Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
+Ses gousses sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris entre autres parce que l'asclépiade a eu son grand moment industriel chez vous : l'usine de Saint-Tite achetait 90 % des récoltes du Québec avant que la filière se casse en 2018. Des producteurs de la Mauricie cultivent encore, et on continue d'acheter leur récolte.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -11652,7 +11652,7 @@
       <c r="M164" s="11" t="inlineStr"/>
       <c r="N164" s="11" t="inlineStr"/>
     </row>
-    <row r="165" ht="250" customHeight="1">
+    <row r="165" ht="240" customHeight="1">
       <c r="A165" s="6" t="inlineStr">
         <is>
           <t>froide C</t>
@@ -11707,7 +11707,7 @@
         <is>
           <t>Bonjour Félix-Antoine Beauchemin,
 Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
-Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
+Ses gousses sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris entre autres parce que la Montérégie est une des régions où l'asclépiade se cultive encore, et que c'est de champs comme ceux-là que vient la fibre qu'on transforme.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -11720,7 +11720,7 @@
       <c r="M165" s="11" t="inlineStr"/>
       <c r="N165" s="11" t="inlineStr"/>
     </row>
-    <row r="166" ht="250" customHeight="1">
+    <row r="166" ht="240" customHeight="1">
       <c r="A166" s="6" t="inlineStr">
         <is>
           <t>froide C</t>
@@ -11775,7 +11775,7 @@
         <is>
           <t>Bonjour Karim Benessaieh,
 Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
-Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
+Ses gousses sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris parce que vous couvrez l'environnement. Notre pari est économique avant d'être militant : si l'asclépiade devient payante, les agriculteurs la gardent dans leurs champs, et les monarques retrouvent de l'habitat de reproduction.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -11788,7 +11788,7 @@
       <c r="M166" s="11" t="inlineStr"/>
       <c r="N166" s="11" t="inlineStr"/>
     </row>
-    <row r="167" ht="250" customHeight="1">
+    <row r="167" ht="240" customHeight="1">
       <c r="A167" s="6" t="inlineStr">
         <is>
           <t>froide C</t>
@@ -11843,7 +11843,7 @@
         <is>
           <t>Bonjour Julia Bernier,
 Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
-Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
+Ses gousses sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris entre autres parce que l'asclépiade se cultive dans votre région depuis la première vague de 2013, et que plusieurs des producteurs qui ont tenu bon nous vendent encore leur récolte.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -11856,7 +11856,7 @@
       <c r="M167" s="11" t="inlineStr"/>
       <c r="N167" s="11" t="inlineStr"/>
     </row>
-    <row r="168" ht="250" customHeight="1">
+    <row r="168" ht="240" customHeight="1">
       <c r="A168" s="6" t="inlineStr">
         <is>
           <t>froide C</t>
@@ -11911,7 +11911,7 @@
         <is>
           <t>Bonjour Karine Boivin Forcier,
 Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
-Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
+Ses gousses sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris entre autres parce qu'un de nos fournisseurs d'asclépiade cultive au Lac-Saint-Jean depuis nos tout débuts, et qu'il l'est encore aujourd'hui. La fibre de chez vous se retrouve dans nos produits.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -11924,7 +11924,7 @@
       <c r="M168" s="11" t="inlineStr"/>
       <c r="N168" s="11" t="inlineStr"/>
     </row>
-    <row r="169" ht="250" customHeight="1">
+    <row r="169" ht="240" customHeight="1">
       <c r="A169" s="6" t="inlineStr">
         <is>
           <t>froide C</t>
@@ -11979,7 +11979,7 @@
         <is>
           <t>Bonjour Audrey Bonaque,
 Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
-Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
+Ses gousses sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris parce que le sujet se raconte bien en ondes : une entreprise de Québec qui va expliquer à un auditoire pancanadien pourquoi la mauvaise herbe des champs de maïs peut isoler un manteau.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -11992,7 +11992,7 @@
       <c r="M169" s="11" t="inlineStr"/>
       <c r="N169" s="11" t="inlineStr"/>
     </row>
-    <row r="170" ht="250" customHeight="1">
+    <row r="170" ht="240" customHeight="1">
       <c r="A170" s="6" t="inlineStr">
         <is>
           <t>froide C</t>
@@ -12047,7 +12047,7 @@
         <is>
           <t>Bonjour Luc Boulanger,
 Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
-Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
+Ses gousses sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris parce que vous couvrez l'art de vivre et la consommation. Le contraste se photographie bien : la gousse dans le champ, la soie blanche dans la main, le manteau porté en ville.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -12060,7 +12060,7 @@
       <c r="M170" s="11" t="inlineStr"/>
       <c r="N170" s="11" t="inlineStr"/>
     </row>
-    <row r="171" ht="250" customHeight="1">
+    <row r="171" ht="240" customHeight="1">
       <c r="A171" s="6" t="inlineStr">
         <is>
           <t>froide C</t>
@@ -12115,7 +12115,7 @@
         <is>
           <t>Bonjour Mario Boulianne,
 Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
-Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
+Ses gousses sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris parce que c'est une nouvelle de chez nous qui passe au national.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -12128,7 +12128,7 @@
       <c r="M171" s="11" t="inlineStr"/>
       <c r="N171" s="11" t="inlineStr"/>
     </row>
-    <row r="172" ht="250" customHeight="1">
+    <row r="172" ht="240" customHeight="1">
       <c r="A172" s="6" t="inlineStr">
         <is>
           <t>froide C</t>
@@ -12183,7 +12183,7 @@
         <is>
           <t>Bonjour Bernard Brault,
 Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
-Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
+Ses gousses sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris entre autres parce que la Montérégie est une des régions où l'asclépiade se cultive encore, et que c'est de champs comme ceux-là que vient la fibre qu'on transforme.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -12196,7 +12196,7 @@
       <c r="M172" s="11" t="inlineStr"/>
       <c r="N172" s="11" t="inlineStr"/>
     </row>
-    <row r="173" ht="250" customHeight="1">
+    <row r="173" ht="240" customHeight="1">
       <c r="A173" s="6" t="inlineStr">
         <is>
           <t>froide C</t>
@@ -12251,7 +12251,7 @@
         <is>
           <t>Bonjour Pierre Brisson,
 Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
-Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
+Ses gousses sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris parce que vous couvrez l'économie. On a bâti nos propres procédés de transformation parce qu'aucun sous-traitant ne voulait toucher à l'asclépiade, puis on a changé de modèle manufacturier l'an dernier pour rendre un manteau accessible à 300 $. J'en ai fait une vidéo ici : https://www.youtube.com/watch?v=GKyHh-Ok9JU.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -12264,7 +12264,7 @@
       <c r="M173" s="11" t="inlineStr"/>
       <c r="N173" s="11" t="inlineStr"/>
     </row>
-    <row r="174" ht="250" customHeight="1">
+    <row r="174" ht="240" customHeight="1">
       <c r="A174" s="6" t="inlineStr">
         <is>
           <t>froide C</t>
@@ -12319,7 +12319,7 @@
         <is>
           <t>Bonjour Laurence Brisson Dubreuil,
 Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
-Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
+Ses gousses sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris parce que le sujet se raconte bien en ondes : une entreprise de Québec qui va expliquer à un auditoire pancanadien pourquoi la mauvaise herbe des champs de maïs peut isoler un manteau.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -12332,7 +12332,7 @@
       <c r="M174" s="11" t="inlineStr"/>
       <c r="N174" s="11" t="inlineStr"/>
     </row>
-    <row r="175" ht="250" customHeight="1">
+    <row r="175" ht="240" customHeight="1">
       <c r="A175" s="6" t="inlineStr">
         <is>
           <t>froide C</t>
@@ -12387,7 +12387,7 @@
         <is>
           <t>Bonjour Nathaniel Bronner,
 Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
-Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
+Ses gousses sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris parce que le sujet se raconte bien en ondes : une entreprise de Québec qui va expliquer à un auditoire pancanadien pourquoi la mauvaise herbe des champs de maïs peut isoler un manteau.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -12400,7 +12400,7 @@
       <c r="M175" s="11" t="inlineStr"/>
       <c r="N175" s="11" t="inlineStr"/>
     </row>
-    <row r="176" ht="250" customHeight="1">
+    <row r="176" ht="240" customHeight="1">
       <c r="A176" s="6" t="inlineStr">
         <is>
           <t>froide C</t>
@@ -12455,7 +12455,7 @@
         <is>
           <t>Bonjour Marie-France Bélanger,
 Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
-Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
+Ses gousses sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris parce que vous couvrez l'art de vivre et la consommation. Le contraste se photographie bien : la gousse dans le champ, la soie blanche dans la main, le manteau porté en ville.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -12468,7 +12468,7 @@
       <c r="M176" s="11" t="inlineStr"/>
       <c r="N176" s="11" t="inlineStr"/>
     </row>
-    <row r="177" ht="250" customHeight="1">
+    <row r="177" ht="240" customHeight="1">
       <c r="A177" s="6" t="inlineStr">
         <is>
           <t>froide C</t>
@@ -12523,7 +12523,7 @@
         <is>
           <t>Bonjour Diane Bérard,
 Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
-Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
+Ses gousses sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris parce que vous couvrez l'économie. On a bâti nos propres procédés de transformation parce qu'aucun sous-traitant ne voulait toucher à l'asclépiade, puis on a changé de modèle manufacturier l'an dernier pour rendre un manteau accessible à 300 $. J'en ai fait une vidéo ici : https://www.youtube.com/watch?v=GKyHh-Ok9JU.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -12536,7 +12536,7 @@
       <c r="M177" s="11" t="inlineStr"/>
       <c r="N177" s="11" t="inlineStr"/>
     </row>
-    <row r="178" ht="250" customHeight="1">
+    <row r="178" ht="240" customHeight="1">
       <c r="A178" s="6" t="inlineStr">
         <is>
           <t>froide C</t>
@@ -12591,7 +12591,7 @@
         <is>
           <t>Bonjour Julien Cayouette,
 Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
-Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
+Ses gousses sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris parce que vous couvrez l'environnement. Notre pari est économique avant d'être militant : si l'asclépiade devient payante, les agriculteurs la gardent dans leurs champs, et les monarques retrouvent de l'habitat de reproduction.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -12604,7 +12604,7 @@
       <c r="M178" s="11" t="inlineStr"/>
       <c r="N178" s="11" t="inlineStr"/>
     </row>
-    <row r="179" ht="250" customHeight="1">
+    <row r="179" ht="240" customHeight="1">
       <c r="A179" s="6" t="inlineStr">
         <is>
           <t>froide C</t>
@@ -12659,7 +12659,7 @@
         <is>
           <t>Bonjour Rudy Chabannes,
 Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
-Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
+Ses gousses sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris parce que le sujet se raconte bien en ondes : une entreprise de Québec qui va expliquer à un auditoire pancanadien pourquoi la mauvaise herbe des champs de maïs peut isoler un manteau.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -12672,7 +12672,7 @@
       <c r="M179" s="11" t="inlineStr"/>
       <c r="N179" s="11" t="inlineStr"/>
     </row>
-    <row r="180" ht="250" customHeight="1">
+    <row r="180" ht="240" customHeight="1">
       <c r="A180" s="6" t="inlineStr">
         <is>
           <t>froide C</t>
@@ -12727,7 +12727,7 @@
         <is>
           <t>Bonjour Denis-Martin Chabot,
 Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
-Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
+Ses gousses sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris parce que le sujet se raconte bien en ondes : une entreprise de Québec qui va expliquer à un auditoire pancanadien pourquoi la mauvaise herbe des champs de maïs peut isoler un manteau.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -12740,7 +12740,7 @@
       <c r="M180" s="11" t="inlineStr"/>
       <c r="N180" s="11" t="inlineStr"/>
     </row>
-    <row r="181" ht="250" customHeight="1">
+    <row r="181" ht="240" customHeight="1">
       <c r="A181" s="6" t="inlineStr">
         <is>
           <t>froide C</t>
@@ -12795,7 +12795,7 @@
         <is>
           <t>Bonjour Loubna Majda Chourouk,
 Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
-Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
+Ses gousses sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris parce que le sujet se raconte bien en ondes : une entreprise de Québec qui va expliquer à un auditoire pancanadien pourquoi la mauvaise herbe des champs de maïs peut isoler un manteau.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -12808,7 +12808,7 @@
       <c r="M181" s="11" t="inlineStr"/>
       <c r="N181" s="11" t="inlineStr"/>
     </row>
-    <row r="182" ht="250" customHeight="1">
+    <row r="182" ht="240" customHeight="1">
       <c r="A182" s="6" t="inlineStr">
         <is>
           <t>froide C</t>
@@ -12863,7 +12863,7 @@
         <is>
           <t>Bonjour Sarah Collardey,
 Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
-Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
+Ses gousses sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris parce que vous couvrez l'environnement. Notre pari est économique avant d'être militant : si l'asclépiade devient payante, les agriculteurs la gardent dans leurs champs, et les monarques retrouvent de l'habitat de reproduction.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -12876,7 +12876,7 @@
       <c r="M182" s="11" t="inlineStr"/>
       <c r="N182" s="11" t="inlineStr"/>
     </row>
-    <row r="183" ht="250" customHeight="1">
+    <row r="183" ht="240" customHeight="1">
       <c r="A183" s="6" t="inlineStr">
         <is>
           <t>froide C</t>
@@ -12931,7 +12931,7 @@
         <is>
           <t>Bonjour Kathleen Couillard,
 Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
-Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
+Ses gousses sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris entre autres parce que la Montérégie est une des régions où l'asclépiade se cultive encore, et que c'est de champs comme ceux-là que vient la fibre qu'on transforme.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -12944,7 +12944,7 @@
       <c r="M183" s="11" t="inlineStr"/>
       <c r="N183" s="11" t="inlineStr"/>
     </row>
-    <row r="184" ht="250" customHeight="1">
+    <row r="184" ht="240" customHeight="1">
       <c r="A184" s="6" t="inlineStr">
         <is>
           <t>froide C</t>
@@ -12999,7 +12999,7 @@
         <is>
           <t>Bonjour Oumou DIAKITÉ,
 Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
-Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
+Ses gousses sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris parce que vous couvrez l'art de vivre et la consommation. Le contraste se photographie bien : la gousse dans le champ, la soie blanche dans la main, le manteau porté en ville.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -13012,7 +13012,7 @@
       <c r="M184" s="11" t="inlineStr"/>
       <c r="N184" s="11" t="inlineStr"/>
     </row>
-    <row r="185" ht="250" customHeight="1">
+    <row r="185" ht="240" customHeight="1">
       <c r="A185" s="6" t="inlineStr">
         <is>
           <t>froide C</t>
@@ -13067,7 +13067,7 @@
         <is>
           <t>Bonjour Agnès Delavault,
 Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
-Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
+Ses gousses sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris parce que vous couvrez l'art de vivre et la consommation. Le contraste se photographie bien : la gousse dans le champ, la soie blanche dans la main, le manteau porté en ville.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -13080,7 +13080,7 @@
       <c r="M185" s="11" t="inlineStr"/>
       <c r="N185" s="11" t="inlineStr"/>
     </row>
-    <row r="186" ht="250" customHeight="1">
+    <row r="186" ht="240" customHeight="1">
       <c r="A186" s="6" t="inlineStr">
         <is>
           <t>froide C</t>
@@ -13135,7 +13135,7 @@
         <is>
           <t>Bonjour Marcelin Delice,
 Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
-Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
+Ses gousses sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris parce que vous couvrez l'environnement. Notre pari est économique avant d'être militant : si l'asclépiade devient payante, les agriculteurs la gardent dans leurs champs, et les monarques retrouvent de l'habitat de reproduction.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -13148,7 +13148,7 @@
       <c r="M186" s="11" t="inlineStr"/>
       <c r="N186" s="11" t="inlineStr"/>
     </row>
-    <row r="187" ht="250" customHeight="1">
+    <row r="187" ht="240" customHeight="1">
       <c r="A187" s="6" t="inlineStr">
         <is>
           <t>froide C</t>
@@ -13203,7 +13203,7 @@
         <is>
           <t>Bonjour Alain Demers,
 Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
-Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
+Ses gousses sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris parce que vous couvrez le plein air. À poids égal, la littérature donne la soie d'asclépiade pour environ 10 % plus isolante que le duvet. C'est un repère de laboratoire, pas une promesse de manteau, et c'est exactement pour ça que je préfère qu'on la teste.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -13216,7 +13216,7 @@
       <c r="M187" s="11" t="inlineStr"/>
       <c r="N187" s="11" t="inlineStr"/>
     </row>
-    <row r="188" ht="250" customHeight="1">
+    <row r="188" ht="240" customHeight="1">
       <c r="A188" s="6" t="inlineStr">
         <is>
           <t>froide C</t>
@@ -13271,7 +13271,7 @@
         <is>
           <t>Bonjour Ivanoh Demers,
 Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
-Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
+Ses gousses sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris parce que vous couvrez l'économie. On a bâti nos propres procédés de transformation parce qu'aucun sous-traitant ne voulait toucher à l'asclépiade, puis on a changé de modèle manufacturier l'an dernier pour rendre un manteau accessible à 300 $. J'en ai fait une vidéo ici : https://www.youtube.com/watch?v=GKyHh-Ok9JU.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -13284,7 +13284,7 @@
       <c r="M188" s="11" t="inlineStr"/>
       <c r="N188" s="11" t="inlineStr"/>
     </row>
-    <row r="189" ht="250" customHeight="1">
+    <row r="189" ht="240" customHeight="1">
       <c r="A189" s="6" t="inlineStr">
         <is>
           <t>froide C</t>
@@ -13339,7 +13339,7 @@
         <is>
           <t>Bonjour Claude Deschênes,
 Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
-Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
+Ses gousses sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris parce que vous couvrez l'art de vivre et la consommation. Le contraste se photographie bien : la gousse dans le champ, la soie blanche dans la main, le manteau porté en ville.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -13352,7 +13352,7 @@
       <c r="M189" s="11" t="inlineStr"/>
       <c r="N189" s="11" t="inlineStr"/>
     </row>
-    <row r="190" ht="250" customHeight="1">
+    <row r="190" ht="240" customHeight="1">
       <c r="A190" s="6" t="inlineStr">
         <is>
           <t>froide C</t>
@@ -13407,7 +13407,7 @@
         <is>
           <t>Bonjour Thomas Deshaies,
 Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
-Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
+Ses gousses sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris entre autres parce qu'une des premières usines de transformation de la fibre était à Granby, et que l'Estrie compte encore des producteurs d'asclépiade.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -13420,7 +13420,7 @@
       <c r="M190" s="11" t="inlineStr"/>
       <c r="N190" s="11" t="inlineStr"/>
     </row>
-    <row r="191" ht="250" customHeight="1">
+    <row r="191" ht="240" customHeight="1">
       <c r="A191" s="6" t="inlineStr">
         <is>
           <t>froide C</t>
@@ -13475,7 +13475,7 @@
         <is>
           <t>Bonjour Claude Desjardins,
 Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
-Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
+Ses gousses sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris parce que vous couvrez l'économie. On a bâti nos propres procédés de transformation parce qu'aucun sous-traitant ne voulait toucher à l'asclépiade, puis on a changé de modèle manufacturier l'an dernier pour rendre un manteau accessible à 300 $. J'en ai fait une vidéo ici : https://www.youtube.com/watch?v=GKyHh-Ok9JU.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -13488,7 +13488,7 @@
       <c r="M191" s="11" t="inlineStr"/>
       <c r="N191" s="11" t="inlineStr"/>
     </row>
-    <row r="192" ht="250" customHeight="1">
+    <row r="192" ht="240" customHeight="1">
       <c r="A192" s="6" t="inlineStr">
         <is>
           <t>froide C</t>
@@ -13543,7 +13543,7 @@
         <is>
           <t>Bonjour Martine Deslauriers,
 Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
-Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
+Ses gousses sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris parce que vous couvrez l'environnement. Notre pari est économique avant d'être militant : si l'asclépiade devient payante, les agriculteurs la gardent dans leurs champs, et les monarques retrouvent de l'habitat de reproduction.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -13556,7 +13556,7 @@
       <c r="M192" s="11" t="inlineStr"/>
       <c r="N192" s="11" t="inlineStr"/>
     </row>
-    <row r="193" ht="250" customHeight="1">
+    <row r="193" ht="240" customHeight="1">
       <c r="A193" s="6" t="inlineStr">
         <is>
           <t>froide C</t>
@@ -13611,7 +13611,7 @@
         <is>
           <t>Bonjour Marie-Claude Di Lillo,
 Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
-Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
+Ses gousses sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris parce que c'est une nouvelle de chez nous qui passe au national.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -13624,7 +13624,7 @@
       <c r="M193" s="11" t="inlineStr"/>
       <c r="N193" s="11" t="inlineStr"/>
     </row>
-    <row r="194" ht="250" customHeight="1">
+    <row r="194" ht="240" customHeight="1">
       <c r="A194" s="6" t="inlineStr">
         <is>
           <t>froide C</t>
@@ -13679,7 +13679,7 @@
         <is>
           <t>Bonjour Jean-René Dufort,
 Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
-Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
+Ses gousses sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris parce que le sujet se raconte bien en ondes : une entreprise de Québec qui va expliquer à un auditoire pancanadien pourquoi la mauvaise herbe des champs de maïs peut isoler un manteau.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -13692,7 +13692,7 @@
       <c r="M194" s="11" t="inlineStr"/>
       <c r="N194" s="11" t="inlineStr"/>
     </row>
-    <row r="195" ht="250" customHeight="1">
+    <row r="195" ht="240" customHeight="1">
       <c r="A195" s="6" t="inlineStr">
         <is>
           <t>froide C</t>
@@ -13747,7 +13747,7 @@
         <is>
           <t>Bonjour Richard Dupaul,
 Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
-Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
+Ses gousses sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris parce que vous couvrez l'économie. On a bâti nos propres procédés de transformation parce qu'aucun sous-traitant ne voulait toucher à l'asclépiade, puis on a changé de modèle manufacturier l'an dernier pour rendre un manteau accessible à 300 $. J'en ai fait une vidéo ici : https://www.youtube.com/watch?v=GKyHh-Ok9JU.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -13760,7 +13760,7 @@
       <c r="M195" s="11" t="inlineStr"/>
       <c r="N195" s="11" t="inlineStr"/>
     </row>
-    <row r="196" ht="250" customHeight="1">
+    <row r="196" ht="240" customHeight="1">
       <c r="A196" s="6" t="inlineStr">
         <is>
           <t>froide C</t>
@@ -13815,7 +13815,7 @@
         <is>
           <t>Bonjour Stéphanie Dupuis,
 Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
-Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
+Ses gousses sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris parce que vous couvrez l'art de vivre et la consommation. Le contraste se photographie bien : la gousse dans le champ, la soie blanche dans la main, le manteau porté en ville.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -13828,7 +13828,7 @@
       <c r="M196" s="11" t="inlineStr"/>
       <c r="N196" s="11" t="inlineStr"/>
     </row>
-    <row r="197" ht="250" customHeight="1">
+    <row r="197" ht="240" customHeight="1">
       <c r="A197" s="6" t="inlineStr">
         <is>
           <t>froide C</t>
@@ -13883,7 +13883,7 @@
         <is>
           <t>Bonjour Maxim Fauteux,
 Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
-Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
+Ses gousses sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris entre autres parce qu'un de nos fournisseurs d'asclépiade cultive au Lac-Saint-Jean depuis nos tout débuts, et qu'il l'est encore aujourd'hui. La fibre de chez vous se retrouve dans nos produits.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -13896,7 +13896,7 @@
       <c r="M197" s="11" t="inlineStr"/>
       <c r="N197" s="11" t="inlineStr"/>
     </row>
-    <row r="198" ht="250" customHeight="1">
+    <row r="198" ht="240" customHeight="1">
       <c r="A198" s="6" t="inlineStr">
         <is>
           <t>froide C</t>
@@ -13951,7 +13951,7 @@
         <is>
           <t>Bonjour Ronald Georges,
 Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
-Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
+Ses gousses sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris parce que le sujet se raconte bien en ondes : une entreprise de Québec qui va expliquer à un auditoire pancanadien pourquoi la mauvaise herbe des champs de maïs peut isoler un manteau.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -13964,7 +13964,7 @@
       <c r="M198" s="11" t="inlineStr"/>
       <c r="N198" s="11" t="inlineStr"/>
     </row>
-    <row r="199" ht="250" customHeight="1">
+    <row r="199" ht="240" customHeight="1">
       <c r="A199" s="6" t="inlineStr">
         <is>
           <t>froide C</t>
@@ -14019,7 +14019,7 @@
         <is>
           <t>Bonjour Stéphane Giroux,
 Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
-Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
+Ses gousses sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris parce que vous couvrez l'économie. On a bâti nos propres procédés de transformation parce qu'aucun sous-traitant ne voulait toucher à l'asclépiade, puis on a changé de modèle manufacturier l'an dernier pour rendre un manteau accessible à 300 $. J'en ai fait une vidéo ici : https://www.youtube.com/watch?v=GKyHh-Ok9JU.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -14032,7 +14032,7 @@
       <c r="M199" s="11" t="inlineStr"/>
       <c r="N199" s="11" t="inlineStr"/>
     </row>
-    <row r="200" ht="250" customHeight="1">
+    <row r="200" ht="240" customHeight="1">
       <c r="A200" s="6" t="inlineStr">
         <is>
           <t>froide C</t>
@@ -14087,7 +14087,7 @@
         <is>
           <t>Bonjour Zacharie Goudreault,
 Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
-Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
+Ses gousses sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris parce que vous couvrez l'environnement. Notre pari est économique avant d'être militant : si l'asclépiade devient payante, les agriculteurs la gardent dans leurs champs, et les monarques retrouvent de l'habitat de reproduction.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -14100,7 +14100,7 @@
       <c r="M200" s="11" t="inlineStr"/>
       <c r="N200" s="11" t="inlineStr"/>
     </row>
-    <row r="201" ht="250" customHeight="1">
+    <row r="201" ht="240" customHeight="1">
       <c r="A201" s="6" t="inlineStr">
         <is>
           <t>froide C</t>
@@ -14155,7 +14155,7 @@
         <is>
           <t>Bonjour Isabelle Grégoire,
 Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
-Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
+Ses gousses sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris parce que vous couvrez l'art de vivre et la consommation. Le contraste se photographie bien : la gousse dans le champ, la soie blanche dans la main, le manteau porté en ville.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -14168,7 +14168,7 @@
       <c r="M201" s="11" t="inlineStr"/>
       <c r="N201" s="11" t="inlineStr"/>
     </row>
-    <row r="202" ht="250" customHeight="1">
+    <row r="202" ht="240" customHeight="1">
       <c r="A202" s="6" t="inlineStr">
         <is>
           <t>froide C</t>
@@ -14223,7 +14223,7 @@
         <is>
           <t>Bonjour Chantal Guy,
 Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
-Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
+Ses gousses sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris parce que vous couvrez l'art de vivre et la consommation. Le contraste se photographie bien : la gousse dans le champ, la soie blanche dans la main, le manteau porté en ville.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -14236,7 +14236,7 @@
       <c r="M202" s="11" t="inlineStr"/>
       <c r="N202" s="11" t="inlineStr"/>
     </row>
-    <row r="203" ht="250" customHeight="1">
+    <row r="203" ht="240" customHeight="1">
       <c r="A203" s="6" t="inlineStr">
         <is>
           <t>froide C</t>
@@ -14291,7 +14291,7 @@
         <is>
           <t>Bonjour Matthieu Hains,
 Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
-Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
+Ses gousses sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris parce que vous couvrez l'économie. On a bâti nos propres procédés de transformation parce qu'aucun sous-traitant ne voulait toucher à l'asclépiade, puis on a changé de modèle manufacturier l'an dernier pour rendre un manteau accessible à 300 $. J'en ai fait une vidéo ici : https://www.youtube.com/watch?v=GKyHh-Ok9JU.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -14304,7 +14304,7 @@
       <c r="M203" s="11" t="inlineStr"/>
       <c r="N203" s="11" t="inlineStr"/>
     </row>
-    <row r="204" ht="250" customHeight="1">
+    <row r="204" ht="240" customHeight="1">
       <c r="A204" s="6" t="inlineStr">
         <is>
           <t>froide C</t>
@@ -14360,7 +14360,7 @@
       <c r="M204" s="11" t="inlineStr"/>
       <c r="N204" s="11" t="inlineStr"/>
     </row>
-    <row r="205" ht="250" customHeight="1">
+    <row r="205" ht="240" customHeight="1">
       <c r="A205" s="6" t="inlineStr">
         <is>
           <t>froide C</t>
@@ -14415,7 +14415,7 @@
         <is>
           <t>Bonjour ANGELO JEAN-BAPTISTE,
 Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
-Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
+Ses gousses sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris parce que vous couvrez l'environnement. Notre pari est économique avant d'être militant : si l'asclépiade devient payante, les agriculteurs la gardent dans leurs champs, et les monarques retrouvent de l'habitat de reproduction.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -14428,7 +14428,7 @@
       <c r="M205" s="11" t="inlineStr"/>
       <c r="N205" s="11" t="inlineStr"/>
     </row>
-    <row r="206" ht="250" customHeight="1">
+    <row r="206" ht="240" customHeight="1">
       <c r="A206" s="6" t="inlineStr">
         <is>
           <t>froide C</t>
@@ -14483,7 +14483,7 @@
         <is>
           <t>Bonjour Andréanne Joly,
 Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
-Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
+Ses gousses sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris parce que vous couvrez l'art de vivre et la consommation. Le contraste se photographie bien : la gousse dans le champ, la soie blanche dans la main, le manteau porté en ville.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -14496,7 +14496,7 @@
       <c r="M206" s="11" t="inlineStr"/>
       <c r="N206" s="11" t="inlineStr"/>
     </row>
-    <row r="207" ht="250" customHeight="1">
+    <row r="207" ht="240" customHeight="1">
       <c r="A207" s="6" t="inlineStr">
         <is>
           <t>froide C</t>
@@ -14551,7 +14551,7 @@
         <is>
           <t>Bonjour Hugo Joncas,
 Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
-Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
+Ses gousses sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris parce que vous couvrez l'économie. On a bâti nos propres procédés de transformation parce qu'aucun sous-traitant ne voulait toucher à l'asclépiade, puis on a changé de modèle manufacturier l'an dernier pour rendre un manteau accessible à 300 $. J'en ai fait une vidéo ici : https://www.youtube.com/watch?v=GKyHh-Ok9JU.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -14564,7 +14564,7 @@
       <c r="M207" s="11" t="inlineStr"/>
       <c r="N207" s="11" t="inlineStr"/>
     </row>
-    <row r="208" ht="250" customHeight="1">
+    <row r="208" ht="240" customHeight="1">
       <c r="A208" s="6" t="inlineStr">
         <is>
           <t>froide C</t>
@@ -14619,7 +14619,7 @@
         <is>
           <t>Bonjour Philémon La Frenière-Prémont,
 Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
-Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
+Ses gousses sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris parce que le sujet se raconte bien en ondes : une entreprise de Québec qui va expliquer à un auditoire pancanadien pourquoi la mauvaise herbe des champs de maïs peut isoler un manteau.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -14632,7 +14632,7 @@
       <c r="M208" s="11" t="inlineStr"/>
       <c r="N208" s="11" t="inlineStr"/>
     </row>
-    <row r="209" ht="250" customHeight="1">
+    <row r="209" ht="240" customHeight="1">
       <c r="A209" s="6" t="inlineStr">
         <is>
           <t>froide C</t>
@@ -14687,7 +14687,7 @@
         <is>
           <t>Bonjour Henri Laban,
 Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
-Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
+Ses gousses sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris parce que le sujet se raconte bien en ondes : une entreprise de Québec qui va expliquer à un auditoire pancanadien pourquoi la mauvaise herbe des champs de maïs peut isoler un manteau.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -14700,7 +14700,7 @@
       <c r="M209" s="11" t="inlineStr"/>
       <c r="N209" s="11" t="inlineStr"/>
     </row>
-    <row r="210" ht="250" customHeight="1">
+    <row r="210" ht="240" customHeight="1">
       <c r="A210" s="6" t="inlineStr">
         <is>
           <t>froide C</t>
@@ -14756,7 +14756,7 @@
       <c r="M210" s="11" t="inlineStr"/>
       <c r="N210" s="11" t="inlineStr"/>
     </row>
-    <row r="211" ht="250" customHeight="1">
+    <row r="211" ht="240" customHeight="1">
       <c r="A211" s="6" t="inlineStr">
         <is>
           <t>froide C</t>
@@ -14811,7 +14811,7 @@
         <is>
           <t>Bonjour Joannie Lafrenière,
 Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
-Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
+Ses gousses sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris parce que vous couvrez l'art de vivre et la consommation. Le contraste se photographie bien : la gousse dans le champ, la soie blanche dans la main, le manteau porté en ville.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -14824,7 +14824,7 @@
       <c r="M211" s="11" t="inlineStr"/>
       <c r="N211" s="11" t="inlineStr"/>
     </row>
-    <row r="212" ht="250" customHeight="1">
+    <row r="212" ht="240" customHeight="1">
       <c r="A212" s="6" t="inlineStr">
         <is>
           <t>froide C</t>
@@ -14879,7 +14879,7 @@
         <is>
           <t>Bonjour Angie Landry,
 Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
-Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
+Ses gousses sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris parce que vous couvrez l'environnement. Notre pari est économique avant d'être militant : si l'asclépiade devient payante, les agriculteurs la gardent dans leurs champs, et les monarques retrouvent de l'habitat de reproduction.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -14892,7 +14892,7 @@
       <c r="M212" s="11" t="inlineStr"/>
       <c r="N212" s="11" t="inlineStr"/>
     </row>
-    <row r="213" ht="250" customHeight="1">
+    <row r="213" ht="240" customHeight="1">
       <c r="A213" s="6" t="inlineStr">
         <is>
           <t>froide C</t>
@@ -14947,7 +14947,7 @@
         <is>
           <t>Bonjour Camille Langlade,
 Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
-Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
+Ses gousses sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris parce que vous couvrez l'environnement. Notre pari est économique avant d'être militant : si l'asclépiade devient payante, les agriculteurs la gardent dans leurs champs, et les monarques retrouvent de l'habitat de reproduction.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -14960,7 +14960,7 @@
       <c r="M213" s="11" t="inlineStr"/>
       <c r="N213" s="11" t="inlineStr"/>
     </row>
-    <row r="214" ht="250" customHeight="1">
+    <row r="214" ht="240" customHeight="1">
       <c r="A214" s="6" t="inlineStr">
         <is>
           <t>froide C</t>
@@ -15015,7 +15015,7 @@
         <is>
           <t>Bonjour Claudia Larochelle,
 Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
-Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
+Ses gousses sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris parce que le sujet se raconte bien en ondes : une entreprise de Québec qui va expliquer à un auditoire pancanadien pourquoi la mauvaise herbe des champs de maïs peut isoler un manteau.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -15028,7 +15028,7 @@
       <c r="M214" s="11" t="inlineStr"/>
       <c r="N214" s="11" t="inlineStr"/>
     </row>
-    <row r="215" ht="250" customHeight="1">
+    <row r="215" ht="240" customHeight="1">
       <c r="A215" s="6" t="inlineStr">
         <is>
           <t>froide C</t>
@@ -15083,7 +15083,7 @@
         <is>
           <t>Bonjour Étienne Leblanc,
 Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
-Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
+Ses gousses sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris parce que vous couvrez l'environnement. Notre pari est économique avant d'être militant : si l'asclépiade devient payante, les agriculteurs la gardent dans leurs champs, et les monarques retrouvent de l'habitat de reproduction.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -15096,7 +15096,7 @@
       <c r="M215" s="11" t="inlineStr"/>
       <c r="N215" s="11" t="inlineStr"/>
     </row>
-    <row r="216" ht="250" customHeight="1">
+    <row r="216" ht="240" customHeight="1">
       <c r="A216" s="6" t="inlineStr">
         <is>
           <t>froide C</t>
@@ -15151,7 +15151,7 @@
         <is>
           <t>Bonjour Louise Leduc,
 Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
-Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
+Ses gousses sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris parce que vous couvrez l'art de vivre et la consommation. Le contraste se photographie bien : la gousse dans le champ, la soie blanche dans la main, le manteau porté en ville.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -15164,7 +15164,7 @@
       <c r="M216" s="11" t="inlineStr"/>
       <c r="N216" s="11" t="inlineStr"/>
     </row>
-    <row r="217" ht="250" customHeight="1">
+    <row r="217" ht="240" customHeight="1">
       <c r="A217" s="6" t="inlineStr">
         <is>
           <t>froide C</t>
@@ -15219,7 +15219,7 @@
         <is>
           <t>Bonjour Guillaume Longuépée,
 Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
-Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
+Ses gousses sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris parce que vous couvrez l'économie. On a bâti nos propres procédés de transformation parce qu'aucun sous-traitant ne voulait toucher à l'asclépiade, puis on a changé de modèle manufacturier l'an dernier pour rendre un manteau accessible à 300 $. J'en ai fait une vidéo ici : https://www.youtube.com/watch?v=GKyHh-Ok9JU.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -15232,7 +15232,7 @@
       <c r="M217" s="11" t="inlineStr"/>
       <c r="N217" s="11" t="inlineStr"/>
     </row>
-    <row r="218" ht="250" customHeight="1">
+    <row r="218" ht="240" customHeight="1">
       <c r="A218" s="6" t="inlineStr">
         <is>
           <t>froide C</t>
@@ -15287,7 +15287,7 @@
         <is>
           <t>Bonjour Roxane Léouzon,
 Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
-Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
+Ses gousses sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris parce que vous couvrez l'économie. On a bâti nos propres procédés de transformation parce qu'aucun sous-traitant ne voulait toucher à l'asclépiade, puis on a changé de modèle manufacturier l'an dernier pour rendre un manteau accessible à 300 $. J'en ai fait une vidéo ici : https://www.youtube.com/watch?v=GKyHh-Ok9JU.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -15300,7 +15300,7 @@
       <c r="M218" s="11" t="inlineStr"/>
       <c r="N218" s="11" t="inlineStr"/>
     </row>
-    <row r="219" ht="250" customHeight="1">
+    <row r="219" ht="240" customHeight="1">
       <c r="A219" s="6" t="inlineStr">
         <is>
           <t>froide C</t>
@@ -15355,7 +15355,7 @@
         <is>
           <t>Bonjour Ève Lévesque,
 Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
-Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
+Ses gousses sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris parce que le sujet se raconte bien en ondes : une entreprise de Québec qui va expliquer à un auditoire pancanadien pourquoi la mauvaise herbe des champs de maïs peut isoler un manteau.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -15368,7 +15368,7 @@
       <c r="M219" s="11" t="inlineStr"/>
       <c r="N219" s="11" t="inlineStr"/>
     </row>
-    <row r="220" ht="250" customHeight="1">
+    <row r="220" ht="240" customHeight="1">
       <c r="A220" s="6" t="inlineStr">
         <is>
           <t>froide C</t>
@@ -15423,7 +15423,7 @@
         <is>
           <t>Bonjour Sophie Mangado,
 Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
-Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
+Ses gousses sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris parce que le sujet se raconte bien en ondes : une entreprise de Québec qui va expliquer à un auditoire pancanadien pourquoi la mauvaise herbe des champs de maïs peut isoler un manteau.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -15436,7 +15436,7 @@
       <c r="M220" s="11" t="inlineStr"/>
       <c r="N220" s="11" t="inlineStr"/>
     </row>
-    <row r="221" ht="250" customHeight="1">
+    <row r="221" ht="240" customHeight="1">
       <c r="A221" s="6" t="inlineStr">
         <is>
           <t>froide C</t>
@@ -15491,7 +15491,7 @@
         <is>
           <t>Bonjour Colin McGregor,
 Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
-Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
+Ses gousses sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris parce que vous couvrez l'environnement. Notre pari est économique avant d'être militant : si l'asclépiade devient payante, les agriculteurs la gardent dans leurs champs, et les monarques retrouvent de l'habitat de reproduction.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -15504,7 +15504,7 @@
       <c r="M221" s="11" t="inlineStr"/>
       <c r="N221" s="11" t="inlineStr"/>
     </row>
-    <row r="222" ht="250" customHeight="1">
+    <row r="222" ht="240" customHeight="1">
       <c r="A222" s="6" t="inlineStr">
         <is>
           <t>froide C</t>
@@ -15559,7 +15559,7 @@
         <is>
           <t>Bonjour Isabelle Morin,
 Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
-Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
+Ses gousses sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris parce que vous couvrez l'art de vivre et la consommation. Le contraste se photographie bien : la gousse dans le champ, la soie blanche dans la main, le manteau porté en ville.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -15572,7 +15572,7 @@
       <c r="M222" s="11" t="inlineStr"/>
       <c r="N222" s="11" t="inlineStr"/>
     </row>
-    <row r="223" ht="250" customHeight="1">
+    <row r="223" ht="240" customHeight="1">
       <c r="A223" s="6" t="inlineStr">
         <is>
           <t>froide C</t>
@@ -15627,7 +15627,7 @@
         <is>
           <t>Bonjour Timothy Morson,
 Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
-Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
+Ses gousses sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris entre autres parce que l'asclépiade se cultive dans votre région depuis la première vague de 2013, et que plusieurs des producteurs qui ont tenu bon nous vendent encore leur récolte.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -15640,7 +15640,7 @@
       <c r="M223" s="11" t="inlineStr"/>
       <c r="N223" s="11" t="inlineStr"/>
     </row>
-    <row r="224" ht="250" customHeight="1">
+    <row r="224" ht="240" customHeight="1">
       <c r="A224" s="6" t="inlineStr">
         <is>
           <t>froide C</t>
@@ -15695,7 +15695,7 @@
         <is>
           <t>Bonjour Rachid Najahi,
 Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
-Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
+Ses gousses sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris parce que vous couvrez l'art de vivre et la consommation. Le contraste se photographie bien : la gousse dans le champ, la soie blanche dans la main, le manteau porté en ville.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -15708,7 +15708,7 @@
       <c r="M224" s="11" t="inlineStr"/>
       <c r="N224" s="11" t="inlineStr"/>
     </row>
-    <row r="225" ht="250" customHeight="1">
+    <row r="225" ht="240" customHeight="1">
       <c r="A225" s="6" t="inlineStr">
         <is>
           <t>froide C</t>
@@ -15763,7 +15763,7 @@
         <is>
           <t>Bonjour Richard Olivier,
 Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
-Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
+Ses gousses sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris parce que le sujet se raconte bien en ondes : une entreprise de Québec qui va expliquer à un auditoire pancanadien pourquoi la mauvaise herbe des champs de maïs peut isoler un manteau.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -15776,7 +15776,7 @@
       <c r="M225" s="11" t="inlineStr"/>
       <c r="N225" s="11" t="inlineStr"/>
     </row>
-    <row r="226" ht="250" customHeight="1">
+    <row r="226" ht="240" customHeight="1">
       <c r="A226" s="6" t="inlineStr">
         <is>
           <t>froide C</t>
@@ -15831,7 +15831,7 @@
         <is>
           <t>Bonjour MELISSA PELLETIER,
 Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
-Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
+Ses gousses sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris entre autres parce que la Montérégie est une des régions où l'asclépiade se cultive encore, et que c'est de champs comme ceux-là que vient la fibre qu'on transforme.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -15844,7 +15844,7 @@
       <c r="M226" s="11" t="inlineStr"/>
       <c r="N226" s="11" t="inlineStr"/>
     </row>
-    <row r="227" ht="250" customHeight="1">
+    <row r="227" ht="240" customHeight="1">
       <c r="A227" s="6" t="inlineStr">
         <is>
           <t>froide C</t>
@@ -15899,7 +15899,7 @@
         <is>
           <t>Bonjour Isaac Peltz,
 Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
-Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
+Ses gousses sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris entre autres parce que l'asclépiade se cultive dans votre région depuis la première vague de 2013, et que plusieurs des producteurs qui ont tenu bon nous vendent encore leur récolte.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -15912,7 +15912,7 @@
       <c r="M227" s="11" t="inlineStr"/>
       <c r="N227" s="11" t="inlineStr"/>
     </row>
-    <row r="228" ht="250" customHeight="1">
+    <row r="228" ht="240" customHeight="1">
       <c r="A228" s="6" t="inlineStr">
         <is>
           <t>froide C</t>
@@ -15967,7 +15967,7 @@
         <is>
           <t>Bonjour Frédéric Perron,
 Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
-Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
+Ses gousses sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris parce que vous couvrez l'art de vivre et la consommation. Le contraste se photographie bien : la gousse dans le champ, la soie blanche dans la main, le manteau porté en ville.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -15980,7 +15980,7 @@
       <c r="M228" s="11" t="inlineStr"/>
       <c r="N228" s="11" t="inlineStr"/>
     </row>
-    <row r="229" ht="250" customHeight="1">
+    <row r="229" ht="240" customHeight="1">
       <c r="A229" s="6" t="inlineStr">
         <is>
           <t>froide C</t>
@@ -16035,7 +16035,7 @@
         <is>
           <t>Bonjour Nathalie Petrowski,
 Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
-Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
+Ses gousses sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris parce que le sujet se raconte bien en ondes : une entreprise de Québec qui va expliquer à un auditoire pancanadien pourquoi la mauvaise herbe des champs de maïs peut isoler un manteau.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -16048,7 +16048,7 @@
       <c r="M229" s="11" t="inlineStr"/>
       <c r="N229" s="11" t="inlineStr"/>
     </row>
-    <row r="230" ht="250" customHeight="1">
+    <row r="230" ht="240" customHeight="1">
       <c r="A230" s="6" t="inlineStr">
         <is>
           <t>froide C</t>
@@ -16103,7 +16103,7 @@
         <is>
           <t>Bonjour Francis Plourde,
 Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
-Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
+Ses gousses sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris parce que c'est une nouvelle de chez nous qui passe au national.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -16116,7 +16116,7 @@
       <c r="M230" s="11" t="inlineStr"/>
       <c r="N230" s="11" t="inlineStr"/>
     </row>
-    <row r="231" ht="250" customHeight="1">
+    <row r="231" ht="240" customHeight="1">
       <c r="A231" s="6" t="inlineStr">
         <is>
           <t>froide C</t>
@@ -16171,7 +16171,7 @@
         <is>
           <t>Bonjour Raymonde Provencher,
 Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
-Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
+Ses gousses sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris parce que le sujet se raconte bien en ondes : une entreprise de Québec qui va expliquer à un auditoire pancanadien pourquoi la mauvaise herbe des champs de maïs peut isoler un manteau.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -16184,7 +16184,7 @@
       <c r="M231" s="11" t="inlineStr"/>
       <c r="N231" s="11" t="inlineStr"/>
     </row>
-    <row r="232" ht="250" customHeight="1">
+    <row r="232" ht="240" customHeight="1">
       <c r="A232" s="6" t="inlineStr">
         <is>
           <t>froide C</t>
@@ -16239,7 +16239,7 @@
         <is>
           <t>Bonjour Richard Prudhomme,
 Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
-Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
+Ses gousses sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris parce que vous couvrez l'art de vivre et la consommation. Le contraste se photographie bien : la gousse dans le champ, la soie blanche dans la main, le manteau porté en ville.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -16252,7 +16252,7 @@
       <c r="M232" s="11" t="inlineStr"/>
       <c r="N232" s="11" t="inlineStr"/>
     </row>
-    <row r="233" ht="250" customHeight="1">
+    <row r="233" ht="240" customHeight="1">
       <c r="A233" s="6" t="inlineStr">
         <is>
           <t>froide C</t>
@@ -16307,7 +16307,7 @@
         <is>
           <t>Bonjour Pascale Renaud,
 Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
-Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
+Ses gousses sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris parce que vous couvrez l'art de vivre et la consommation. Le contraste se photographie bien : la gousse dans le champ, la soie blanche dans la main, le manteau porté en ville.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -16320,7 +16320,7 @@
       <c r="M233" s="11" t="inlineStr"/>
       <c r="N233" s="11" t="inlineStr"/>
     </row>
-    <row r="234" ht="250" customHeight="1">
+    <row r="234" ht="240" customHeight="1">
       <c r="A234" s="6" t="inlineStr">
         <is>
           <t>froide C</t>
@@ -16375,7 +16375,7 @@
         <is>
           <t>Bonjour Marc Sony Ricot,
 Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
-Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
+Ses gousses sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris parce que vous couvrez l'art de vivre et la consommation. Le contraste se photographie bien : la gousse dans le champ, la soie blanche dans la main, le manteau porté en ville.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -16388,7 +16388,7 @@
       <c r="M234" s="11" t="inlineStr"/>
       <c r="N234" s="11" t="inlineStr"/>
     </row>
-    <row r="235" ht="250" customHeight="1">
+    <row r="235" ht="240" customHeight="1">
       <c r="A235" s="6" t="inlineStr">
         <is>
           <t>froide C</t>
@@ -16443,7 +16443,7 @@
         <is>
           <t>Bonjour Marie-Paul Rouleau,
 Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
-Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
+Ses gousses sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris parce que vous couvrez l'environnement. Notre pari est économique avant d'être militant : si l'asclépiade devient payante, les agriculteurs la gardent dans leurs champs, et les monarques retrouvent de l'habitat de reproduction.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -16456,7 +16456,7 @@
       <c r="M235" s="11" t="inlineStr"/>
       <c r="N235" s="11" t="inlineStr"/>
     </row>
-    <row r="236" ht="250" customHeight="1">
+    <row r="236" ht="240" customHeight="1">
       <c r="A236" s="6" t="inlineStr">
         <is>
           <t>froide C</t>
@@ -16511,7 +16511,7 @@
         <is>
           <t>Bonjour Emmalie Ruest,
 Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
-Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
+Ses gousses sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris parce que le sujet se raconte bien en ondes : une entreprise de Québec qui va expliquer à un auditoire pancanadien pourquoi la mauvaise herbe des champs de maïs peut isoler un manteau.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -16524,7 +16524,7 @@
       <c r="M236" s="11" t="inlineStr"/>
       <c r="N236" s="11" t="inlineStr"/>
     </row>
-    <row r="237" ht="250" customHeight="1">
+    <row r="237" ht="240" customHeight="1">
       <c r="A237" s="6" t="inlineStr">
         <is>
           <t>froide C</t>
@@ -16579,7 +16579,7 @@
         <is>
           <t>Bonjour Louis-Philippe Samson,
 Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
-Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
+Ses gousses sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris entre autres parce que l'asclépiade se cultive dans votre région depuis la première vague de 2013, et que plusieurs des producteurs qui ont tenu bon nous vendent encore leur récolte.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -16592,7 +16592,7 @@
       <c r="M237" s="11" t="inlineStr"/>
       <c r="N237" s="11" t="inlineStr"/>
     </row>
-    <row r="238" ht="250" customHeight="1">
+    <row r="238" ht="240" customHeight="1">
       <c r="A238" s="6" t="inlineStr">
         <is>
           <t>froide C</t>
@@ -16647,7 +16647,7 @@
         <is>
           <t>Bonjour Catherine Schlager,
 Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
-Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
+Ses gousses sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris parce que vous couvrez l'art de vivre et la consommation. Le contraste se photographie bien : la gousse dans le champ, la soie blanche dans la main, le manteau porté en ville.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -16660,7 +16660,7 @@
       <c r="M238" s="11" t="inlineStr"/>
       <c r="N238" s="11" t="inlineStr"/>
     </row>
-    <row r="239" ht="250" customHeight="1">
+    <row r="239" ht="240" customHeight="1">
       <c r="A239" s="6" t="inlineStr">
         <is>
           <t>froide C</t>
@@ -16715,7 +16715,7 @@
         <is>
           <t>Bonjour Olivier Schmouker,
 Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
-Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
+Ses gousses sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris parce que vous couvrez l'économie. On a bâti nos propres procédés de transformation parce qu'aucun sous-traitant ne voulait toucher à l'asclépiade, puis on a changé de modèle manufacturier l'an dernier pour rendre un manteau accessible à 300 $. J'en ai fait une vidéo ici : https://www.youtube.com/watch?v=GKyHh-Ok9JU.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -16728,7 +16728,7 @@
       <c r="M239" s="11" t="inlineStr"/>
       <c r="N239" s="11" t="inlineStr"/>
     </row>
-    <row r="240" ht="250" customHeight="1">
+    <row r="240" ht="240" customHeight="1">
       <c r="A240" s="6" t="inlineStr">
         <is>
           <t>froide C</t>
@@ -16783,7 +16783,7 @@
         <is>
           <t>Bonjour Jacques Sennechael,
 Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
-Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
+Ses gousses sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris parce que c'est une nouvelle de chez nous qui passe au national.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -16796,7 +16796,7 @@
       <c r="M240" s="11" t="inlineStr"/>
       <c r="N240" s="11" t="inlineStr"/>
     </row>
-    <row r="241" ht="250" customHeight="1">
+    <row r="241" ht="240" customHeight="1">
       <c r="A241" s="6" t="inlineStr">
         <is>
           <t>froide C</t>
@@ -16851,7 +16851,7 @@
         <is>
           <t>Bonjour Alexandre Shields,
 Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
-Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
+Ses gousses sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris parce que vous couvrez l'environnement. Notre pari est économique avant d'être militant : si l'asclépiade devient payante, les agriculteurs la gardent dans leurs champs, et les monarques retrouvent de l'habitat de reproduction.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -16864,7 +16864,7 @@
       <c r="M241" s="11" t="inlineStr"/>
       <c r="N241" s="11" t="inlineStr"/>
     </row>
-    <row r="242" ht="250" customHeight="1">
+    <row r="242" ht="240" customHeight="1">
       <c r="A242" s="6" t="inlineStr">
         <is>
           <t>froide C</t>
@@ -16919,7 +16919,7 @@
         <is>
           <t>Bonjour Chloé Sondervorst,
 Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
-Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
+Ses gousses sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris parce que vous couvrez l'environnement. Notre pari est économique avant d'être militant : si l'asclépiade devient payante, les agriculteurs la gardent dans leurs champs, et les monarques retrouvent de l'habitat de reproduction.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -16932,7 +16932,7 @@
       <c r="M242" s="11" t="inlineStr"/>
       <c r="N242" s="11" t="inlineStr"/>
     </row>
-    <row r="243" ht="250" customHeight="1">
+    <row r="243" ht="240" customHeight="1">
       <c r="A243" s="6" t="inlineStr">
         <is>
           <t>froide C</t>
@@ -16987,7 +16987,7 @@
         <is>
           <t>Bonjour Kimberley Sullivan,
 Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
-Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
+Ses gousses sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris entre autres parce que la Montérégie est une des régions où l'asclépiade se cultive encore, et que c'est de champs comme ceux-là que vient la fibre qu'on transforme.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -17000,7 +17000,7 @@
       <c r="M243" s="11" t="inlineStr"/>
       <c r="N243" s="11" t="inlineStr"/>
     </row>
-    <row r="244" ht="250" customHeight="1">
+    <row r="244" ht="240" customHeight="1">
       <c r="A244" s="6" t="inlineStr">
         <is>
           <t>froide C</t>
@@ -17055,7 +17055,7 @@
         <is>
           <t>Bonjour William Thériault,
 Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
-Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
+Ses gousses sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris entre autres parce que la Montérégie est une des régions où l'asclépiade se cultive encore, et que c'est de champs comme ceux-là que vient la fibre qu'on transforme.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -17068,7 +17068,7 @@
       <c r="M244" s="11" t="inlineStr"/>
       <c r="N244" s="11" t="inlineStr"/>
     </row>
-    <row r="245" ht="250" customHeight="1">
+    <row r="245" ht="240" customHeight="1">
       <c r="A245" s="6" t="inlineStr">
         <is>
           <t>froide C</t>
@@ -17123,7 +17123,7 @@
         <is>
           <t>Bonjour Katia Tobar,
 Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
-Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
+Ses gousses sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris parce que vous couvrez l'économie. On a bâti nos propres procédés de transformation parce qu'aucun sous-traitant ne voulait toucher à l'asclépiade, puis on a changé de modèle manufacturier l'an dernier pour rendre un manteau accessible à 300 $. J'en ai fait une vidéo ici : https://www.youtube.com/watch?v=GKyHh-Ok9JU.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -17136,7 +17136,7 @@
       <c r="M245" s="11" t="inlineStr"/>
       <c r="N245" s="11" t="inlineStr"/>
     </row>
-    <row r="246" ht="250" customHeight="1">
+    <row r="246" ht="240" customHeight="1">
       <c r="A246" s="6" t="inlineStr">
         <is>
           <t>froide C</t>
@@ -17191,7 +17191,7 @@
         <is>
           <t>Bonjour Martin Tremblay,
 Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
-Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
+Ses gousses sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris parce que vous couvrez l'environnement. Notre pari est économique avant d'être militant : si l'asclépiade devient payante, les agriculteurs la gardent dans leurs champs, et les monarques retrouvent de l'habitat de reproduction.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -17204,7 +17204,7 @@
       <c r="M246" s="11" t="inlineStr"/>
       <c r="N246" s="11" t="inlineStr"/>
     </row>
-    <row r="247" ht="250" customHeight="1">
+    <row r="247" ht="240" customHeight="1">
       <c r="A247" s="6" t="inlineStr">
         <is>
           <t>froide C</t>
@@ -17259,7 +17259,7 @@
         <is>
           <t>Bonjour Marie-Christine Trottier,
 Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
-Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
+Ses gousses sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris parce que le sujet se raconte bien en ondes : une entreprise de Québec qui va expliquer à un auditoire pancanadien pourquoi la mauvaise herbe des champs de maïs peut isoler un manteau.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -17272,7 +17272,7 @@
       <c r="M247" s="11" t="inlineStr"/>
       <c r="N247" s="11" t="inlineStr"/>
     </row>
-    <row r="248" ht="250" customHeight="1">
+    <row r="248" ht="240" customHeight="1">
       <c r="A248" s="6" t="inlineStr">
         <is>
           <t>froide C</t>
@@ -17327,7 +17327,7 @@
         <is>
           <t>Bonjour Pierre-Luc Trudel,
 Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
-Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
+Ses gousses sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris parce que vous couvrez l'économie. On a bâti nos propres procédés de transformation parce qu'aucun sous-traitant ne voulait toucher à l'asclépiade, puis on a changé de modèle manufacturier l'an dernier pour rendre un manteau accessible à 300 $. J'en ai fait une vidéo ici : https://www.youtube.com/watch?v=GKyHh-Ok9JU.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -17340,7 +17340,7 @@
       <c r="M248" s="11" t="inlineStr"/>
       <c r="N248" s="11" t="inlineStr"/>
     </row>
-    <row r="249" ht="250" customHeight="1">
+    <row r="249" ht="240" customHeight="1">
       <c r="A249" s="6" t="inlineStr">
         <is>
           <t>froide C</t>
@@ -17395,7 +17395,7 @@
         <is>
           <t>Bonjour David Turbis,
 Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
-Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
+Ses gousses sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris parce que le sujet se raconte bien en ondes : une entreprise de Québec qui va expliquer à un auditoire pancanadien pourquoi la mauvaise herbe des champs de maïs peut isoler un manteau.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -17408,7 +17408,7 @@
       <c r="M249" s="11" t="inlineStr"/>
       <c r="N249" s="11" t="inlineStr"/>
     </row>
-    <row r="250" ht="250" customHeight="1">
+    <row r="250" ht="240" customHeight="1">
       <c r="A250" s="6" t="inlineStr">
         <is>
           <t>froide C</t>
@@ -17463,7 +17463,7 @@
         <is>
           <t>Bonjour Paule Vermot-Desroches,
 Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
-Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
+Ses gousses sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris entre autres parce que l'asclépiade a eu son grand moment industriel chez vous : l'usine de Saint-Tite achetait 90 % des récoltes du Québec avant que la filière se casse en 2018. Des producteurs de la Mauricie cultivent encore, et on continue d'acheter leur récolte.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -17476,7 +17476,7 @@
       <c r="M250" s="11" t="inlineStr"/>
       <c r="N250" s="11" t="inlineStr"/>
     </row>
-    <row r="251" ht="250" customHeight="1">
+    <row r="251" ht="240" customHeight="1">
       <c r="A251" s="6" t="inlineStr">
         <is>
           <t>froide C</t>
@@ -17531,7 +17531,7 @@
         <is>
           <t>Bonjour Alexandra Viau,
 Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
-Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
+Ses gousses sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris parce que le sujet se raconte bien en ondes : une entreprise de Québec qui va expliquer à un auditoire pancanadien pourquoi la mauvaise herbe des champs de maïs peut isoler un manteau.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -17544,7 +17544,7 @@
       <c r="M251" s="11" t="inlineStr"/>
       <c r="N251" s="11" t="inlineStr"/>
     </row>
-    <row r="252" ht="250" customHeight="1">
+    <row r="252" ht="240" customHeight="1">
       <c r="A252" s="6" t="inlineStr">
         <is>
           <t>froide C</t>
@@ -17599,7 +17599,7 @@
         <is>
           <t>Bonjour Raymond Viger,
 Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
-Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
+Ses gousses sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris parce que vous couvrez l'environnement. Notre pari est économique avant d'être militant : si l'asclépiade devient payante, les agriculteurs la gardent dans leurs champs, et les monarques retrouvent de l'habitat de reproduction.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -17612,7 +17612,7 @@
       <c r="M252" s="11" t="inlineStr"/>
       <c r="N252" s="11" t="inlineStr"/>
     </row>
-    <row r="253" ht="250" customHeight="1">
+    <row r="253" ht="240" customHeight="1">
       <c r="A253" s="6" t="inlineStr">
         <is>
           <t>froide C</t>
@@ -17667,7 +17667,7 @@
         <is>
           <t>Bonjour Paul Émile d'Entremont,
 Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
-Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
+Ses gousses sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris parce que c'est une nouvelle de chez nous qui passe au national.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -17680,7 +17680,7 @@
       <c r="M253" s="11" t="inlineStr"/>
       <c r="N253" s="11" t="inlineStr"/>
     </row>
-    <row r="254" ht="250" customHeight="1">
+    <row r="254" ht="240" customHeight="1">
       <c r="A254" s="6" t="inlineStr">
         <is>
           <t>froide C</t>
@@ -17735,7 +17735,7 @@
         <is>
           <t>Bonjour Augustin de Baudinière,
 Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
-Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
+Ses gousses sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris parce que vous couvrez l'environnement. Notre pari est économique avant d'être militant : si l'asclépiade devient payante, les agriculteurs la gardent dans leurs champs, et les monarques retrouvent de l'habitat de reproduction.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -17748,7 +17748,7 @@
       <c r="M254" s="11" t="inlineStr"/>
       <c r="N254" s="11" t="inlineStr"/>
     </row>
-    <row r="255" ht="250" customHeight="1">
+    <row r="255" ht="240" customHeight="1">
       <c r="A255" s="6" t="inlineStr">
         <is>
           <t>froide C</t>
@@ -17803,7 +17803,7 @@
         <is>
           <t>Bonjour Ivan de Jacquelin-Dulphe,
 Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
-Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
+Ses gousses sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris parce que vous couvrez l'environnement. Notre pari est économique avant d'être militant : si l'asclépiade devient payante, les agriculteurs la gardent dans leurs champs, et les monarques retrouvent de l'habitat de reproduction.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -17816,7 +17816,7 @@
       <c r="M255" s="11" t="inlineStr"/>
       <c r="N255" s="11" t="inlineStr"/>
     </row>
-    <row r="256" ht="250" customHeight="1">
+    <row r="256" ht="240" customHeight="1">
       <c r="A256" s="6" t="inlineStr">
         <is>
           <t>froide A</t>
@@ -17892,7 +17892,7 @@
       <c r="M256" s="11" t="inlineStr"/>
       <c r="N256" s="11" t="inlineStr"/>
     </row>
-    <row r="257" ht="250" customHeight="1">
+    <row r="257" ht="240" customHeight="1">
       <c r="A257" s="6" t="inlineStr">
         <is>
           <t>froide B</t>

</xml_diff>

<commit_message>
Sort Antoine Stab: plus aucune ligne sans adresse
La règle est générale plutôt que nominative: une ligne sans courriel ne sert à
rien dans un chiffrier d'envoi, donc elle sort. Antoine Stab était le dernier
cas.

250 contacts, 32 en liste chaude et 218 en liste froide, toutes adresses
remplies.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015pjLsGPzf1MX1JC7QiKGGk
</commit_message>
<xml_diff>
--- a/communique-dragons/Lasclay_brouillons_a_editer.xlsx
+++ b/communique-dragons/Lasclay_brouillons_a_editer.xlsx
@@ -11,7 +11,7 @@
     <sheet name="Brouillons à éditer" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Brouillons à éditer'!$A$1:$N$252</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Brouillons à éditer'!$A$1:$N$251</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -498,7 +498,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B23"/>
+  <dimension ref="A1:B17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -508,7 +508,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Version 10</t>
+          <t>Version 11 — prête à envoyer</t>
         </is>
       </c>
       <c r="B1" s="2" t="inlineStr"/>
@@ -520,212 +520,140 @@
     <row r="3" ht="58" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>Retirés de la liste chaude</t>
+          <t>Toutes les adresses sont là</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Sophie Poisson, Caroline Bertrand et Karine Benoist, faute d'adresse. Leurs brouillons restent dans le code si leurs adresses refont surface. Julia Haurio et Protégez-Vous étaient déjà partis.</t>
+          <t>250 contacts : 32 en liste chaude, 218 en liste froide. Plus une seule ligne sans courriel.</t>
         </is>
       </c>
     </row>
     <row r="4" ht="58" customHeight="1">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>Madeleine Goubau</t>
+          <t>Sortis</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Son courriel reconnaît maintenant qu'elle connaît la plante : elle en avait parlé à Moteur de recherche le 9 février 2023. Il enchaîne sur ce qu'elle n'a peut-être pas vu, la fibre une fois transformée en isolant.</t>
+          <t>Antoine Stab (liste froide), Sophie Poisson, Caroline Bertrand et Karine Benoist (liste chaude), tous faute d'adresse. Julia Haurio et Protégez-Vous, sur ta demande. Leurs brouillons restent dans le code si les adresses refont surface.</t>
         </is>
       </c>
     </row>
     <row r="5" ht="58" customHeight="1">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t>Nouveau total</t>
+          <t>Madeleine Goubau</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>251 contacts : 32 en liste chaude, 219 en liste froide. Toutes les adresses de la liste chaude sont remplies.</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="58" customHeight="1">
-      <c r="A6" s="3" t="inlineStr">
-        <is>
-          <t>Reste sans adresse</t>
-        </is>
-      </c>
-      <c r="B6" s="2" t="inlineStr">
-        <is>
-          <t>Antoine Stab, en liste froide.</t>
-        </is>
-      </c>
+          <t>Relancée sur son propre segment de Moteur de recherche, février 2023.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr"/>
+      <c r="B6" s="2" t="inlineStr"/>
     </row>
     <row r="7">
-      <c r="A7" s="2" t="inlineStr"/>
+      <c r="A7" s="1" t="inlineStr">
+        <is>
+          <t>Ce qui reste à vérifier</t>
+        </is>
+      </c>
       <c r="B7" s="2" t="inlineStr"/>
     </row>
     <row r="8">
-      <c r="A8" s="1" t="inlineStr">
-        <is>
-          <t>Les versions précédentes</t>
-        </is>
-      </c>
+      <c r="A8" s="2" t="inlineStr"/>
       <c r="B8" s="2" t="inlineStr"/>
     </row>
-    <row r="9">
-      <c r="A9" s="2" t="inlineStr"/>
-      <c r="B9" s="2" t="inlineStr"/>
+    <row r="9" ht="58" customHeight="1">
+      <c r="A9" s="3" t="inlineStr">
+        <is>
+          <t>Ne pas envoyer</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>Anne-Sophie Roy à l'adresse Québecor, doublon de sa ligne Radio-Canada. Annie Lafrance et Francis Higgins en liste froide, doublons de la liste chaude.</t>
+        </is>
+      </c>
     </row>
     <row r="10" ht="58" customHeight="1">
       <c r="A10" s="3" t="inlineStr">
         <is>
-          <t>v9</t>
+          <t>Six salutations</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>Julia Haurio et Protégez-Vous retirés.</t>
+          <t>Fiches FPJQ mal formées, signalées dans la colonne Précaution.</t>
         </is>
       </c>
     </row>
     <row r="11" ht="58" customHeight="1">
       <c r="A11" s="3" t="inlineStr">
         <is>
-          <t>v8</t>
+          <t>Registre</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>« Petits cochons » retirés.</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="58" customHeight="1">
-      <c r="A12" s="3" t="inlineStr">
-        <is>
-          <t>v7</t>
-        </is>
-      </c>
-      <c r="B12" s="2" t="inlineStr">
-        <is>
-          <t>Ton ouverture adoptée, paragraphe des missions retiré.</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="58" customHeight="1">
-      <c r="A13" s="3" t="inlineStr">
-        <is>
-          <t>v6</t>
-        </is>
-      </c>
-      <c r="B13" s="2" t="inlineStr">
-        <is>
-          <t>Limoilou sorti de la présentation.</t>
-        </is>
-      </c>
-    </row>
-    <row r="14" ht="58" customHeight="1">
-      <c r="A14" s="3" t="inlineStr">
-        <is>
-          <t>v5</t>
-        </is>
-      </c>
-      <c r="B14" s="2" t="inlineStr">
-        <is>
-          <t>« Invité disponible » retiré, l'asclépiade en tête des objets.</t>
-        </is>
-      </c>
+          <t>Chloé Pouliot au « tu », tout le reste au « vous ». Bascule la colonne et je relance.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr"/>
+      <c r="B12" s="2" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="1" t="inlineStr">
+        <is>
+          <t>Rappels</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr"/>
+      <c r="B14" s="2" t="inlineStr"/>
     </row>
     <row r="15" ht="58" customHeight="1">
       <c r="A15" s="3" t="inlineStr">
         <is>
-          <t>v4</t>
+          <t>Diffusion</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>Objets refaits : de titre d'essai à annonce datée.</t>
+          <t>Jeudi 17 septembre 2026, 20 h (20 h 30 NT), CBC et CBC Gem. Prévente le samedi 12 septembre à 9 h.</t>
         </is>
       </c>
     </row>
     <row r="16" ht="58" customHeight="1">
       <c r="A16" s="3" t="inlineStr">
         <is>
-          <t>v3</t>
+          <t>Envoi</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>Présentation et « pourquoi vous » dans les courriels froids.</t>
+          <t>Missive depuis media@lasclay.com, un appel par journaliste, suivi des ouvertures et des clics désactivé, environ 60 par jour. Le mode par défaut dépose un brouillon.</t>
         </is>
       </c>
     </row>
     <row r="17" ht="58" customHeight="1">
       <c r="A17" s="3" t="inlineStr">
         <is>
-          <t>v2</t>
+          <t>Interdits CBC</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>Registre de Gabriel : plus d'excuses, plus de mise en garde, plus de confidentialité.</t>
-        </is>
-      </c>
-    </row>
-    <row r="18" ht="58" customHeight="1">
-      <c r="A18" s="3" t="inlineStr">
-        <is>
-          <t>Repris mot pour mot</t>
-        </is>
-      </c>
-      <c r="B18" s="2" t="inlineStr">
-        <is>
-          <t>Larocque et Pouliot.</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="2" t="inlineStr"/>
-      <c r="B19" s="2" t="inlineStr"/>
-    </row>
-    <row r="20">
-      <c r="A20" s="1" t="inlineStr">
-        <is>
-          <t>Rappels</t>
-        </is>
-      </c>
-      <c r="B20" s="2" t="inlineStr"/>
-    </row>
-    <row r="21">
-      <c r="A21" s="2" t="inlineStr"/>
-      <c r="B21" s="2" t="inlineStr"/>
-    </row>
-    <row r="22" ht="58" customHeight="1">
-      <c r="A22" s="3" t="inlineStr">
-        <is>
-          <t>Diffusion</t>
-        </is>
-      </c>
-      <c r="B22" s="2" t="inlineStr">
-        <is>
-          <t>Jeudi 17 septembre 2026, 20 h (20 h 30 NT), CBC et CBC Gem. Prévente le samedi 12 septembre à 9 h.</t>
-        </is>
-      </c>
-    </row>
-    <row r="23" ht="58" customHeight="1">
-      <c r="A23" s="3" t="inlineStr">
-        <is>
-          <t>Ne pas envoyer</t>
-        </is>
-      </c>
-      <c r="B23" s="2" t="inlineStr">
-        <is>
-          <t>Anne-Sophie Roy à l'adresse Québecor. Annie Lafrance et Francis Higgins en liste froide.</t>
+          <t>Rien sur l'issue avant le 17. Aucun logo ni « vu à Dragons' Den ».</t>
         </is>
       </c>
     </row>
@@ -740,7 +668,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N252"/>
+  <dimension ref="A1:N251"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -812,7 +740,7 @@
       </c>
       <c r="K1" s="4" t="inlineStr">
         <is>
-          <t>Brouillon v10</t>
+          <t>Brouillon v11</t>
         </is>
       </c>
       <c r="L1" s="4" t="inlineStr">
@@ -17626,82 +17554,13 @@
       <c r="M251" s="11" t="inlineStr"/>
       <c r="N251" s="11" t="inlineStr"/>
     </row>
-    <row r="252" ht="240" customHeight="1">
-      <c r="A252" s="6" t="inlineStr">
-        <is>
-          <t>froide B</t>
-        </is>
-      </c>
-      <c r="B252" s="6" t="inlineStr">
-        <is>
-          <t>Antoine Stab</t>
-        </is>
-      </c>
-      <c r="C252" s="6" t="inlineStr">
-        <is>
-          <t>Espaces</t>
-        </is>
-      </c>
-      <c r="D252" s="6" t="inlineStr"/>
-      <c r="E252" s="6" t="inlineStr">
-        <is>
-          <t>Montreal</t>
-        </is>
-      </c>
-      <c r="F252" s="6" t="inlineStr">
-        <is>
-          <t>Journaliste</t>
-        </is>
-      </c>
-      <c r="G252" s="7" t="inlineStr">
-        <is>
-          <t>Environnement; Plein air</t>
-        </is>
-      </c>
-      <c r="H252" s="7" t="inlineStr">
-        <is>
-          <t>J</t>
-        </is>
-      </c>
-      <c r="I252" s="8" t="inlineStr">
-        <is>
-          <t>vous</t>
-        </is>
-      </c>
-      <c r="J252" s="9" t="inlineStr">
-        <is>
-          <t>L'asclépiade s'en va à Dragons' Den le 17 septembre!</t>
-        </is>
-      </c>
-      <c r="K252" s="10" t="inlineStr">
-        <is>
-          <t>Bonjour Antoine Stab,
-Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une
-mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et
-menacé : le papillon monarque.
-Vous aviez écrit sur le soyer du Québec dans Espaces en février 2015, à l'époque où la fibre
-devait remplacer le duvet.
-On a démarré après la chute de cette première filière. Six ans plus tard, on achète encore de l'asclépiade québécoise, on transforme l'isolant nous-mêmes, et il
-existe maintenant un manteau à inserts d'asclépiade amovibles autour de 300 $.
-Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
-Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
-Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Et si vous
-voulez tester le manteau plutôt que me croire sur parole, je vous en envoie un avec plaisir.
-J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
-Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
-        </is>
-      </c>
-      <c r="L252" s="11" t="inlineStr"/>
-      <c r="M252" s="11" t="inlineStr"/>
-      <c r="N252" s="11" t="inlineStr"/>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:N252"/>
+  <autoFilter ref="A1:N251"/>
   <dataValidations count="2">
-    <dataValidation sqref="N2:N252" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="N2:N251" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"à réécrire au complet,à corriger,bon,ne pas envoyer"</formula1>
     </dataValidation>
-    <dataValidation sqref="I2:I252" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="I2:I251" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"tu,vous,—"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Rend le navigateur de brouillons lisible sans JavaScript
L'aperçu de fichier des applications mobiles n'exécute pas les scripts : la
page, qui construisait sa liste au chargement, s'y ouvrait vide sous l'entête.
Les 250 fiches sont maintenant écrites en dur et les filtres sont des boutons
radio cachés que le CSS lit. Vérifié dans un Chromium sans interface, script
désactivé, à 390 pixels de large.

Les six courriels écrits ou collés à la main étaient coupés vers 95 caractères.
Un client de messagerie replie déjà les paragraphes : sur un téléphone la
coupure se voyait deux fois et le texte tombait en escalier. Les retours à la
ligne posés à la main sautent, les paragraphes restent.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015pjLsGPzf1MX1JC7QiKGGk
</commit_message>
<xml_diff>
--- a/communique-dragons/Lasclay_brouillons_a_editer.xlsx
+++ b/communique-dragons/Lasclay_brouillons_a_editer.xlsx
@@ -760,22 +760,12 @@
       <c r="K2" s="2" t="inlineStr">
         <is>
           <t>Bonjour M. Larocque,
-En mai dernier, nous avons discuté au téléphone suite à quoi, votre article sur le
-déménagement de notre production textile en Tunisie a été publié et TRÈS relayé.
-Parmi mes projets avec tout le temps que j'allais sauver, il y avait de me concentrer sur
-« faire connaître l'asclépiade » au plus grand nombre de gens possible. Eh bien, le
-17 septembre prochain on va faire un énorme pas dans la bonne direction :
-Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC
-et CBC Gem.
-Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité
-qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer
-une suite au dernier article.
-Notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise :
-https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
-J'espère vraiment un boom des ventes avec cette visibilité, ce
-qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec
-chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se
-reproduire dans leurs plantations.
+En mai dernier, nous avons discuté au téléphone suite à quoi, votre article sur le déménagement de notre production textile en Tunisie a été publié et TRÈS relayé.
+Parmi mes projets avec tout le temps que j'allais sauver, il y avait de me concentrer sur « faire connaître l'asclépiade » au plus grand nombre de gens possible. Eh bien, le 17 septembre prochain on va faire un énorme pas dans la bonne direction :
+Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
+Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer une suite au dernier article.
+Notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
+J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
       </c>
@@ -895,28 +885,14 @@
       <c r="K4" s="2" t="inlineStr">
         <is>
           <t>Bonjour Chloé,
-J'espère que tu vas bien. Tu as peut-être vu passer mon vidéo portant sur notre changement
-de modèle manufacturier (https://www.youtube.com/watch?v=GKyHh-Ok9JU) ou l'article de
-Sylvain Larocque en mai dernier sur ce sujet. C'est en quelque sorte une suite logique à
-l'article « Lasclay devant le dilemme de fabriquer au Québec » que tu avais publié en
-décembre dernier.
-Neuf mois plus tard, le dilemme est tranché et il tient : l'asclépiade et l'isolant restent
-à Limoilou, la coquille se fait en Tunisie, et le manteau se vend autour de 300 $.
-Parmi les raisons de ce changement, il y avait clairement que j'avais besoin de temps pour
-me recentrer sur mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les
-monarques par la culture de l'asclépiade.
+J'espère que tu vas bien. Tu as peut-être vu passer mon vidéo portant sur notre changement de modèle manufacturier (https://www.youtube.com/watch?v=GKyHh-Ok9JU) ou l'article de Sylvain Larocque en mai dernier sur ce sujet. C'est en quelque sorte une suite logique à l'article « Lasclay devant le dilemme de fabriquer au Québec » que tu avais publié en décembre dernier.
+Neuf mois plus tard, le dilemme est tranché et il tient : l'asclépiade et l'isolant restent à Limoilou, la coquille se fait en Tunisie, et le manteau se vend autour de 300 $.
+Parmi les raisons de ce changement, il y avait clairement que j'avais besoin de temps pour me recentrer sur mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
 Eh bien, le 17 septembre prochain on va faire un énorme pas dans la bonne direction :
-Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC
-et CBC Gem.
-Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité
-qui arrive bien rarement. Je voulais t'en faire part et qui sait, peut-être t'inspirer une
-suite à ton dernier article.
-Notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise :
-https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
-J'espère vraiment un boom des ventes avec cette visibilité, ce
-qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec
-chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se
-reproduire dans leurs plantations.
+Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
+Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais t'en faire part et qui sait, peut-être t'inspirer une suite à ton dernier article.
+Notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
+J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésite pas à me contacter si tu as des questions.</t>
         </is>
       </c>
@@ -2729,19 +2705,12 @@
       <c r="K34" s="2" t="inlineStr">
         <is>
           <t>Bonjour Marie Allard,
-Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une
-mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et
-menacé : le papillon monarque.
-Il y a une belle histoire de sciences dans l'asclépiade. La soie attachée à ses graines n'est
-pas un poil : c'est un tube creux enduit d'une cire hydrophobe, et les fibres portent une
-charge qui les fait se repousser. C'est ce qui forme le parachute autour de la graine, et
-c'est ce qui emprisonne l'air. Chaque follicule en produit plus de 200.
-On en fait de l'isolant pour des manteaux et des mitaines. Et c'est la seule plante que les
-chenilles du monarque peuvent manger, ce qui est toute la raison d'être de l'entreprise.
-Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
-Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
-Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. L'atelier de
-Limoilou est ouvert si vos lecteurs aimeraient voir comment une gousse devient un manteau.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
+Il y a une belle histoire de sciences dans l'asclépiade. La soie attachée à ses graines n'est pas un poil : c'est un tube creux enduit d'une cire hydrophobe, et les fibres portent une charge qui les fait se repousser. C'est ce qui forme le parachute autour de la graine, et c'est ce qui emprisonne l'air. Chaque follicule en produit plus de 200.
+On en fait de l'isolant pour des manteaux et des mitaines. Et c'est la seule plante que les chenilles du monarque peuvent manger, ce qui est toute la raison d'être de l'entreprise.
+Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
+Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
+Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. L'atelier de Limoilou est ouvert si vos lecteurs aimeraient voir comment une gousse devient un manteau.
 Notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
@@ -3978,17 +3947,11 @@
       <c r="K52" s="2" t="inlineStr">
         <is>
           <t>Bonjour Gabriel Delisle,
-Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une
-mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et
-menacé : le papillon monarque.
-L'asclépiade a été une histoire mauricienne avant d'être la nôtre : l'usine de Saint-Tite
-achetait 90 % des récoltes du Québec. On a démarré après la chute de cette filière, et six ans
-plus tard on achète encore de l'asclépiade québécoise et on la
-transforme nous-mêmes à Québec.
-Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
-Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
-Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet : huit ans après
-Saint-Tite, il reste quelque chose de cette promesse-là, et ça se raconte.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
+L'asclépiade a été une histoire mauricienne avant d'être la nôtre : l'usine de Saint-Tite achetait 90 % des récoltes du Québec. On a démarré après la chute de cette filière, et six ans plus tard on achète encore de l'asclépiade québécoise et on la transforme nous-mêmes à Québec.
+Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
+Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
+Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet : huit ans après Saint-Tite, il reste quelque chose de cette promesse-là, et ça se raconte.
 Notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
@@ -5708,19 +5671,12 @@
       <c r="K77" s="2" t="inlineStr">
         <is>
           <t>Bonjour Réjean Martin,
-Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une
-mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et
-menacé : le papillon monarque.
-Vous couvrez Mékinac, donc Saint-Tite, donc l'endroit où l'asclépiade a eu son grand moment
-industriel au Québec. L'usine achetait 90 % des récoltes de la province avant que la filière
-se casse en 2018.
-On a démarré après. Six ans plus tard, on achète encore de l'asclépiade québécoise et on la
-transforme nous-mêmes à Québec.
-Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
-Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
-Je voulais vous en faire part parce que vos lecteurs ont vu la promesse de l'asclépiade de
-plus près que n'importe qui. Qui sait, peut-être vous inspirer un sujet sur ce que la plante
-est devenue depuis. Je peux parler des volumes, de la récolte, et de ce qui reste à régler.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
+Vous couvrez Mékinac, donc Saint-Tite, donc l'endroit où l'asclépiade a eu son grand moment industriel au Québec. L'usine achetait 90 % des récoltes de la province avant que la filière se casse en 2018.
+On a démarré après. Six ans plus tard, on achète encore de l'asclépiade québécoise et on la transforme nous-mêmes à Québec.
+Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
+Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
+Je voulais vous en faire part parce que vos lecteurs ont vu la promesse de l'asclépiade de plus près que n'importe qui. Qui sait, peut-être vous inspirer un sujet sur ce que la plante est devenue depuis. Je peux parler des volumes, de la récolte, et de ce qui reste à régler.
 Notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
@@ -17695,20 +17651,12 @@
       <c r="K251" s="2" t="inlineStr">
         <is>
           <t>Bonjour Jean-Michel Leprince,
-Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une
-mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et
-menacé : le papillon monarque.
-Vous couvrez l'asclépiade depuis au moins 2014 : le Téléjournal, la soie d'Amérique partie
-sur l'Everest, le pouvoir absorbant de la fibre sur les hydrocarbures, le lien avec le
-monarque. Vous avez suivi cette histoire plus longtemps que la plupart des entreprises qui
-s'y sont essayées.
-On a démarré après la chute de la première filière. Six ans plus tard, on achète encore de l'asclépiade québécoise et on transforme l'isolant nous-mêmes à
-Limoilou.
-Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
-Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
-Vous êtes probablement la personne au Québec qui a le plus longtemps suivi cette plante-là.
-Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet : ce serait la
-première fois qu'on raconte ce que la filière est devenue après la chute.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
+Vous couvrez l'asclépiade depuis au moins 2014 : le Téléjournal, la soie d'Amérique partie sur l'Everest, le pouvoir absorbant de la fibre sur les hydrocarbures, le lien avec le monarque. Vous avez suivi cette histoire plus longtemps que la plupart des entreprises qui s'y sont essayées.
+On a démarré après la chute de la première filière. Six ans plus tard, on achète encore de l'asclépiade québécoise et on transforme l'isolant nous-mêmes à Limoilou.
+Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
+Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
+Vous êtes probablement la personne au Québec qui a le plus longtemps suivi cette plante-là. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet : ce serait la première fois qu'on raconte ce que la filière est devenue après la chute.
 Notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>

</xml_diff>

<commit_message>
Remercie chaque contact de la liste chaude pour son travail
Le rappel de l'article énonçait un fait — « publié et TRÈS relayé » — sans
dire ce qu'on en pense. Les 28 contacts dont on connaît la publication ou
l'échange reçoivent maintenant un remerciement qui nomme ce que leur texte a
fait de bien : avoir pris la filière au complet, avoir écrit quand il n'y
avait rien à montrer, avoir signalé un retard plutôt que de laisser passer.

Larocque reçoit l'avis positif demandé : le sujet était délicat, il a été
traité avec justesse, et le bilan de l'article est bon pour nous.

Trois contacts n'ont aucun historique connu et ne sont donc pas remerciés :
on ne remercie pas pour un article hypothétique.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015pjLsGPzf1MX1JC7QiKGGk
</commit_message>
<xml_diff>
--- a/communique-dragons/Lasclay_brouillons_a_editer.xlsx
+++ b/communique-dragons/Lasclay_brouillons_a_editer.xlsx
@@ -450,7 +450,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B17"/>
+  <dimension ref="A1:B18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -460,7 +460,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Version 12 — média kit</t>
+          <t>Version 12 — média kit et remerciements</t>
         </is>
       </c>
       <c r="B1" s="2" t="n"/>
@@ -496,114 +496,126 @@
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
         <is>
+          <t>Remerciements</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>Les 28 contacts de la liste chaude dont on connaît l'article ou l'échange sont remerciés, chacun pour ce que son texte a fait de bien. Mireille Roberge, Sophie Laforest et Jessica Dostie n'ont aucun historique connu : on ne les remercie pas pour un article hypothétique. Si tu sais ce qu'elles ont publié, dis-le et j'ajoute.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="3" t="inlineStr">
+        <is>
           <t>Rappel CBC</t>
         </is>
       </c>
-      <c r="B5" s="2" t="inlineStr">
+      <c r="B6" s="2" t="inlineStr">
         <is>
           <t>Les images du plateau servent à annoncer la diffusion, pas à illustrer une promotion de produits, et aucun logo ni marque Dragons' Den n'est autorisé. À vérifier avant de déposer les fichiers dans le dossier.</t>
         </is>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" s="3" t="n"/>
-      <c r="B6" s="2" t="n"/>
-    </row>
     <row r="7">
-      <c r="A7" s="1" t="inlineStr">
+      <c r="A7" s="3" t="n"/>
+      <c r="B7" s="2" t="n"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="1" t="inlineStr">
         <is>
           <t>Ce qui reste à vérifier</t>
         </is>
       </c>
-      <c r="B7" s="2" t="n"/>
-    </row>
-    <row r="8">
-      <c r="A8" s="3" t="n"/>
       <c r="B8" s="2" t="n"/>
     </row>
     <row r="9">
-      <c r="A9" s="3" t="inlineStr">
-        <is>
-          <t>Ne pas envoyer</t>
-        </is>
-      </c>
-      <c r="B9" s="2" t="inlineStr">
-        <is>
-          <t>Anne-Sophie Roy à l'adresse Québecor, doublon de sa ligne Radio-Canada. Annie Lafrance et Francis Higgins en liste froide, doublons de la liste chaude.</t>
-        </is>
-      </c>
+      <c r="A9" s="3" t="n"/>
+      <c r="B9" s="2" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="3" t="inlineStr">
         <is>
-          <t>Six salutations</t>
+          <t>Ne pas envoyer</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>Fiches FPJQ mal formées, signalées dans la colonne Précaution.</t>
+          <t>Anne-Sophie Roy à l'adresse Québecor, doublon de sa ligne Radio-Canada. Annie Lafrance et Francis Higgins en liste froide, doublons de la liste chaude.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
         <is>
+          <t>Six salutations</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>Fiches FPJQ mal formées, signalées dans la colonne Précaution.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="3" t="inlineStr">
+        <is>
           <t>Registre</t>
         </is>
       </c>
-      <c r="B11" s="2" t="inlineStr">
+      <c r="B12" s="2" t="inlineStr">
         <is>
           <t>Chloé Pouliot au « tu », tout le reste au « vous ». Bascule la colonne et je relance.</t>
         </is>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" s="3" t="n"/>
-      <c r="B12" s="2" t="n"/>
-    </row>
     <row r="13">
-      <c r="A13" s="1" t="inlineStr">
+      <c r="A13" s="3" t="n"/>
+      <c r="B13" s="2" t="n"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="1" t="inlineStr">
         <is>
           <t>Rappels</t>
         </is>
       </c>
-      <c r="B13" s="2" t="n"/>
-    </row>
-    <row r="14">
-      <c r="A14" s="3" t="n"/>
       <c r="B14" s="2" t="n"/>
     </row>
     <row r="15">
-      <c r="A15" s="3" t="inlineStr">
-        <is>
-          <t>Diffusion</t>
-        </is>
-      </c>
-      <c r="B15" s="2" t="inlineStr">
-        <is>
-          <t>Jeudi 17 septembre 2026, 20 h (20 h 30 NT), CBC et CBC Gem. Prévente le samedi 12 septembre à 9 h.</t>
-        </is>
-      </c>
+      <c r="A15" s="3" t="n"/>
+      <c r="B15" s="2" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="3" t="inlineStr">
         <is>
-          <t>Envoi</t>
+          <t>Diffusion</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>Missive depuis media@lasclay.com, un appel par journaliste, suivi des ouvertures et des clics désactivé, environ 60 par jour. Le mode par défaut dépose un brouillon.</t>
+          <t>Jeudi 17 septembre 2026, 20 h (20 h 30 NT), CBC et CBC Gem. Prévente le samedi 12 septembre à 9 h.</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="3" t="inlineStr">
         <is>
+          <t>Envoi</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>Missive depuis media@lasclay.com, un appel par journaliste, suivi des ouvertures et des clics désactivé, environ 60 par jour. Le mode par défaut dépose un brouillon.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="3" t="inlineStr">
+        <is>
           <t>Interdits CBC</t>
         </is>
       </c>
-      <c r="B17" s="2" t="inlineStr">
+      <c r="B18" s="2" t="inlineStr">
         <is>
           <t>Rien sur l'issue avant le 17. Aucun logo ni « vu à Dragons' Den ».</t>
         </is>
@@ -761,6 +773,7 @@
         <is>
           <t>Bonjour M. Larocque,
 En mai dernier, nous avons discuté au téléphone suite à quoi, votre article sur le déménagement de notre production textile en Tunisie a été publié et TRÈS relayé.
+Je vous en remercie sincèrement. Le sujet était délicat et vous l'avez traité avec justesse : de notre côté, le bilan de cet article est très positif.
 Parmi mes projets avec tout le temps que j'allais sauver, il y avait de me concentrer sur « faire connaître l'asclépiade » au plus grand nombre de gens possible. Eh bien, le 17 septembre prochain on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer une suite au dernier article.
@@ -823,6 +836,7 @@
         <is>
           <t>Bonjour Mme Bérubé,
 En février, vous avez signé « La sinueuse route de la soie du Nord ». C'est un des rares textes à avoir pris la filière au complet, et pas juste une entreprise.
+Merci d'avoir pris cette peine-là. La filière a plus besoin d'être racontée en entier qu'entreprise par entreprise, et presque personne ne le fait.
 Depuis, tout mon temps va à mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
 Eh bien, le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -886,6 +900,7 @@
         <is>
           <t>Bonjour Chloé,
 J'espère que tu vas bien. Tu as peut-être vu passer mon vidéo portant sur notre changement de modèle manufacturier (https://www.youtube.com/watch?v=GKyHh-Ok9JU) ou l'article de Sylvain Larocque en mai dernier sur ce sujet. C'est en quelque sorte une suite logique à l'article « Lasclay devant le dilemme de fabriquer au Québec » que tu avais publié en décembre dernier.
+Merci encore pour ce texte, d'ailleurs. Tu avais posé le dilemme sans le trancher à ma place, et c'est exactement comme ça qu'il fallait le poser.
 Neuf mois plus tard, le dilemme est tranché et il tient : l'asclépiade et l'isolant restent à Limoilou, la coquille se fait en Tunisie, et le manteau se vend autour de 300 $.
 Parmi les raisons de ce changement, il y avait clairement que j'avais besoin de temps pour me recentrer sur mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
 Eh bien, le 17 septembre prochain on va faire un énorme pas dans la bonne direction :
@@ -950,6 +965,7 @@
         <is>
           <t>Bonjour Mme Paquet,
 On s'était parlé en septembre dernier pour Pleins feux sur Québec. Cette année, la date tombe presque au même endroit.
+Merci pour la tribune de l'an dernier. Ce genre de rendez-vous local vaut cher pour une entreprise de notre taille.
 Eh bien, le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part : je suis disponible pour une entrevue la semaine du 14 septembre et le vendredi 18 au matin.
@@ -1012,6 +1028,7 @@
         <is>
           <t>Bonjour Mme Roy,
 Vous nous aviez appelés en mars 2025 pour votre reportage sur le dropshipping, comme exemple d'une entreprise qui fabrique vraiment. Et en décembre 2020, vous aviez signé un des tout premiers articles sur nos mitaines.
+Merci pour les deux. Être cité comme l'exemple d'une entreprise qui fabrique vraiment, dans un reportage sur le dropshipping, c'est exactement la distinction qu'on essaie de faire comprendre.
 Depuis, tout mon temps va à mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
 Eh bien, le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -1075,6 +1092,7 @@
         <is>
           <t>Bonjour Mme Lafrance,
 En avril 2024, vous aviez signé « L'asclépiade : plus que la fibre de demain » dans Le Soleil Affaires, où vous m'aviez cité disant qu'on croyait à cette matière depuis les débuts. On y croit encore.
+Merci d'avoir gardé cette citation-là : elle a bien vieilli.
 Parmi les raisons de ce changement, il y avait clairement que j'avais besoin de temps pour me recentrer sur mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
 Eh bien, le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -1138,6 +1156,7 @@
         <is>
           <t>Bonjour Mme Tison,
 En novembre 2021, vous aviez écrit « Le timide retour de l'asclépiade ». Le retour est pas mal moins timide qu'à l'époque : il y a maintenant un manteau et une veste à inserts d'asclépiade amovibles, autour de 300 $.
+Merci d'avoir écrit sur la plante à une époque où il n'y avait presque rien à montrer. C'est le genre de texte qui aide une filière avant qu'elle existe.
 Depuis, tout mon temps va à mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
 Eh bien, le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -1201,6 +1220,7 @@
         <is>
           <t>Bonjour Mme Lacombe,
 En novembre 2023, vous nous aviez contactés pour le suivi d'une précommande qui traînait. Vous aviez raison de le faire. Depuis, on sort graduellement de la précommande pour vendre du déjà produit, et les délais n'ont plus rien à voir.
+Merci de nous l'avoir signalé plutôt que de laisser passer : c'est comme ça qu'on a corrigé le tir.
 Depuis, tout mon temps va à mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
 Eh bien, le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -1264,6 +1284,7 @@
         <is>
           <t>Bonjour Mme Roulot-Ganzmann,
 On s'était parlé en novembre 2023 pour du matériel sur nos produits d'asclépiade.
+Merci de vous être intéressée à la matière elle-même. C'est rarement le premier angle qu'on nous propose.
 Depuis, tout mon temps va à mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
 Eh bien, le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -1327,6 +1348,7 @@
         <is>
           <t>Bonjour Mme Brault,
 On s'était parlé en janvier 2023 pour Le Soleil. L'atelier est toujours dans Limoilou, et c'est encore là que la soie d'asclépiade devient de l'isolant.
+Merci pour l'attention que vous nous aviez portée à l'époque : Le Soleil a été un des premiers à nous suivre sérieusement.
 Depuis, tout mon temps va à mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
 Eh bien, le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -1390,6 +1412,7 @@
         <is>
           <t>Bonjour Mme Fillion,
 On s'était parlé d'asclépiade en janvier 2023. Depuis, le statut du monarque comme espèce en voie de disparition a été confirmé au Canada, et les États-Unis ont proposé de l'inscrire comme menacée. La plante n'a jamais été aussi pertinente.
+Merci d'avoir pris l'asclépiade au sérieux à un moment où bien peu de monde le faisait.
 Depuis, tout mon temps va à mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
 Eh bien, le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -1453,6 +1476,7 @@
         <is>
           <t>Bonjour Mme Aubert Bonn,
 En novembre 2022, vous aviez couvert nos nouveaux produits d'asclépiade. Le catalogue compte maintenant plus de 40 produits, et La Tribune a repris en décembre dernier l'article de Chloé Pouliot sur notre changement de modèle manufacturier.
+Merci de l'avoir fait quand le catalogue tenait encore sur une main. L'Estrie nous suit depuis, et ça part de là.
 Parmi les raisons de ce changement, il y avait clairement que j'avais besoin de temps pour me recentrer sur mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
 Eh bien, le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -1516,6 +1540,7 @@
         <is>
           <t>Bonjour Mme Émond,
 En septembre 2022, on s'était parlé de notre glacière d'asclépiade imprimée en 3D. On a continué à inventer nos propres procédés depuis, parce que personne d'autre ne les fait.
+Merci de vous être arrêtée sur un détail technique. C'est rare, et c'est pourtant là que se joue la différence entre une vraie matière et un argument de vente.
 Depuis, tout mon temps va à mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
 Eh bien, le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -1579,6 +1604,7 @@
         <is>
           <t>Bonjour Mme Portelance,
 On avait échangé en juillet 2022 pour le cahier Action climatique. L'asclépiade est une vivace indigène qui se cultive avec peu d'intrants et qui stocke du carbone dans un système racinaire pérenne.
+Merci d'avoir ouvert le cahier climatique à une plante : les solutions agricoles y passent moins souvent que les technologies.
 Depuis, tout mon temps va à mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
 Eh bien, le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -1642,6 +1668,7 @@
         <is>
           <t>Bonjour Mme Elboujdaini,
 On s'était parlé du programme de semences en mai 2022. La Campagne nationale de plantation en est à sa 5e édition, et on a distribué environ 10 millions de graines d'asclépiade en Amérique du Nord.
+Merci d'avoir parlé du programme de semences. C'est la partie la moins spectaculaire de ce qu'on fait, et la plus utile aux monarques.
 Eh bien, le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part : je suis disponible pour une entrevue la semaine du 14 septembre et le vendredi 18 au matin.
@@ -1704,6 +1731,7 @@
         <is>
           <t>Bonjour M. Tison,
 On s'était parlé pour la section Affaires en septembre 2021, à l'époque où on venait de rapatrier notre production faute de sous-traitant prêt à toucher à la fibre. Le modèle a changé depuis : la vidéo est ici, https://www.youtube.com/watch?v=GKyHh-Ok9JU, et Sylvain Larocque en a parlé en mai.
+Merci d'avoir raconté ce rapatriement au moment où c'était encore un pari. Le texte a beaucoup circulé chez nos clients.
 Parmi les raisons de ce changement, il y avait clairement que j'avais besoin de temps pour me recentrer sur mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
 Eh bien, le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -1767,6 +1795,7 @@
         <is>
           <t>Bonjour Mme Simard,
 Vous aviez présenté nos moufles isolées à l'asclépiade le 17 septembre 2021. Drôle de coïncidence : la diffusion tombe cinq ans jour pour jour après votre article.
+Merci pour ce coup de pouce de la première heure : à l'époque, une mention dans La Presse changeait notre semaine.
 Depuis, tout mon temps va à mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
 Eh bien, le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -1830,6 +1859,7 @@
         <is>
           <t>Bonjour Mme Friis,
 Vous aviez travaillé sur l'impact climatique de l'asclépiade en septembre 2021.
+Merci de vous être penchée sur l'impact réel plutôt que sur l'intention. C'est ce qui sépare une plante utile d'un argument vert.
 Depuis, tout mon temps va à mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
 Eh bien, le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -1893,6 +1923,7 @@
         <is>
           <t>Bonjour M. Perreault,
 On s'était parlé en juillet 2021.
+Merci de l'intérêt que vous nous aviez porté à l'époque : on partait de zéro.
 Depuis, tout mon temps va à mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
 Eh bien, le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -1956,6 +1987,7 @@
         <is>
           <t>Bonjour M. Higgins,
 On s'était parlé pour Le Soleil en juillet 2021. L'atelier est toujours dans Limoilou.
+Merci d'avoir couvert l'atelier quand il n'était qu'un local et deux machines.
 Depuis, tout mon temps va à mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
 Eh bien, le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -2019,6 +2051,7 @@
         <is>
           <t>Bonjour Mme Samson,
 En mars 2021, vous aviez signé « Les grandes promesses de l'asclépiade, la soie d'Amérique ». Cinq ans plus tard, je peux vous dire lesquelles ont été tenues : il y a des produits finis, l'isolant se transforme toujours au Québec, on achète encore de l'asclépiade québécoise, et un manteau se vend autour de 300 $.
+Merci d'avoir écrit « promesses » plutôt qu'autre chose. Le mot était juste, et il l'est resté le temps qu'on les tienne.
 Depuis, tout mon temps va à mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
 Eh bien, le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -2082,6 +2115,7 @@
         <is>
           <t>Bonjour M. Ménard,
 On s'était parlé à La Terre en janvier 2021. Cinq ans plus tard, on achète encore de l'asclépiade québécoise et on la transforme nous-mêmes à Québec.
+Merci d'avoir porté le sujet auprès des producteurs. C'est le lectorat qui compte le plus pour nous : sans champs, il n'y a pas de fibre.
 Depuis, tout mon temps va à mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
 Eh bien, le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -2200,6 +2234,7 @@
         <is>
           <t>Bonjour Mme Drouin,
 En janvier 2021, vous aviez écrit « Devenir viral avant même de se lancer en affaires ». Six ans plus tard, l'entreprise existe pour vrai, avec plus de 40 produits.
+Merci d'avoir écrit sur nous quand il n'y avait littéralement rien à acheter. Vous nous avez pris au sérieux avant tout le monde.
 Depuis, tout mon temps va à mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
 Eh bien, le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -2254,6 +2289,7 @@
         <is>
           <t>Bonjour M. Roy,
 En octobre 2020, vous avez écrit « La deuxième vie de l'asclépiade ». Vous avez été le tout premier journaliste à parler de nous. Et l'agriculteur du Lac-Saint-Jean qui vous avait donné envie du sujet est encore notre fournisseur aujourd'hui : six ans plus tard, l'asclépiade de chez vous se retrouve toujours dans nos produits.
+Merci, sincèrement. On n'oublie pas qui a écrit le premier article, et le vôtre nous a servi de carte de visite pendant des années.
 Depuis, tout mon temps va à mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
 Eh bien, le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -2423,6 +2459,7 @@
         <is>
           <t>Bonjour M. McKenna,
 En décembre 2021, vous aviez écrit « Des écouteurs de Québec pour oublier les AirPods », sur Sounds Good. J'étais un des trois. J'ai vendu mes parts en 2022 pour me consacrer entièrement à Lasclay, l'autre entreprise que j'avais démarrée entretemps, qui transforme la soie d'asclépiade en isolant textile.
+Merci pour ce texte-là : il a compté pour Sounds Good, et j'en garde un bon souvenir.
 Depuis, tout mon temps va à mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
 Eh bien, le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -2477,6 +2514,7 @@
         <is>
           <t>Bonjour Mme Lemieux,
 En décembre 2021, vous aviez écrit « Les deux mains dans l'écoresponsabilité » pour le Journal de Montréal. Notre modèle manufacturier a changé depuis, et j'en ai fait une vidéo ici : https://www.youtube.com/watch?v=GKyHh-Ok9JU.
+Merci d'avoir mis l'écoresponsabilité au cœur du texte plutôt qu'en décoration.
 Parmi les raisons de ce changement, il y avait clairement que j'avais besoin de temps pour me recentrer sur mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
 Eh bien, le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -2531,6 +2569,7 @@
         <is>
           <t>Bonjour Mme Grenier-Héroux,
 En janvier 2021, vous aviez écrit « La soie d'Amérique, le pari de deux ambitieux » dans Le Devoir. Le pari a six ans, et il tient : plus de 40 produits, environ 10 millions de graines distribuées, et un isolant toujours transformé à Limoilou.
+Merci d'avoir appelé ça un pari. C'en était un, et le mot était plus honnête que tous les superlatifs qu'on nous colle habituellement.
 Depuis, tout mon temps va à mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
 Eh bien, le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -2586,6 +2625,7 @@
           <t>Bonjour Mme Goubau,
 Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe : l'asclépiade, que vous connaissez bien, puisque vous en aviez parlé à Moteur de recherche en février 2023. On la cultive pour sauvegarder un pollinisateur emblématique et menacé, le papillon monarque.
 Ce que vous n'avez peut-être pas vu de près, c'est ce que la fibre donne une fois transformée. Ses gousses sont remplies d'une soie creuse, très légère et naturellement hydrophobe, qu'on transforme en isolant à Québec, et qui se retrouve dans des manteaux, des mitaines et des tuques.
+Merci d'en avoir parlé en ondes, d'ailleurs : c'est rare qu'on explique la plante avant de vendre quoi que ce soit.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet.

</xml_diff>

<commit_message>
Passe Stéphanie Bérubé au squelette de Chloé, au tutoiement
Le remerciement entre dans le corps du texte plutôt que dans son paragraphe
séparé : « merci pour ce bel article, qui a fait une place de choix à Lasclay
et à ses défis ». C'est le jugement de Gabriel sur son texte, pas le mien.

Elle et Chloé Pouliot sont les deux seuls contacts au « tu ».

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015pjLsGPzf1MX1JC7QiKGGk
</commit_message>
<xml_diff>
--- a/communique-dragons/Lasclay_brouillons_a_editer.xlsx
+++ b/communique-dragons/Lasclay_brouillons_a_editer.xlsx
@@ -450,7 +450,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B20"/>
+  <dimension ref="A1:B21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -508,138 +508,150 @@
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
         <is>
-          <t>Goubau, ta version</t>
+          <t>Stéphanie Bérubé</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Ton texte est repris mot pour mot. La leçon vaut plus large : sans historique, la présentation tient en une phrase, pas deux paragraphes, et « depuis 5 ans, on travaille fort à la faire connaître » remplace le paragraphe des deux missions. Sophie Laforest, le dernier contact sans historique, est réécrite sur ce squelette.</t>
+          <t>Réécrite sur le squelette de Chloé, au « tu ». Le remerciement dit ce que tu voulais qu'il dise : un bel article, qui a fait une place de choix à Lasclay et à ses défis. Deux contacts sont maintenant au tutoiement, elle et Chloé.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
         <is>
-          <t>Remerciements</t>
+          <t>Goubau, ta version</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>26 des 28 brouillons chauds remercient le contact, chacun pour ce que son texte a fait de bien. Les deux exceptions sont Sophie Laforest, dont on ne connaît aucune publication, et Madeleine Goubau, dont tu as retiré le remerciement toi-même en réécrivant son courriel.</t>
+          <t>Ton texte est repris mot pour mot. La leçon vaut plus large : sans historique, la présentation tient en une phrase, pas deux paragraphes, et « depuis 5 ans, on travaille fort à la faire connaître » remplace le paragraphe des deux missions. Sophie Laforest, le dernier contact sans historique, est réécrite sur ce squelette.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
         <is>
+          <t>Remerciements</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>26 des 28 brouillons chauds remercient le contact, chacun pour ce que son texte a fait de bien. Les deux exceptions sont Sophie Laforest, dont on ne connaît aucune publication, et Madeleine Goubau, dont tu as retiré le remerciement toi-même en réécrivant son courriel.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="3" t="inlineStr">
+        <is>
           <t>Rappel CBC</t>
         </is>
       </c>
-      <c r="B8" s="2" t="inlineStr">
+      <c r="B9" s="2" t="inlineStr">
         <is>
           <t>Les images du plateau servent à annoncer la diffusion, pas à illustrer une promotion de produits, et aucun logo ni marque Dragons' Den n'est autorisé. À vérifier avant de déposer les fichiers dans le dossier.</t>
         </is>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" s="3" t="n"/>
-      <c r="B9" s="2" t="n"/>
-    </row>
     <row r="10">
-      <c r="A10" s="1" t="inlineStr">
+      <c r="A10" s="3" t="n"/>
+      <c r="B10" s="2" t="n"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="1" t="inlineStr">
         <is>
           <t>Ce qui reste à vérifier</t>
         </is>
       </c>
-      <c r="B10" s="2" t="n"/>
-    </row>
-    <row r="11">
-      <c r="A11" s="3" t="n"/>
       <c r="B11" s="2" t="n"/>
     </row>
     <row r="12">
-      <c r="A12" s="3" t="inlineStr">
-        <is>
-          <t>Ne pas envoyer</t>
-        </is>
-      </c>
-      <c r="B12" s="2" t="inlineStr">
-        <is>
-          <t>Anne-Sophie Roy à l'adresse Québecor, doublon de sa ligne Radio-Canada. Annie Lafrance et Francis Higgins en liste froide, doublons de la liste chaude.</t>
-        </is>
-      </c>
+      <c r="A12" s="3" t="n"/>
+      <c r="B12" s="2" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
         <is>
-          <t>Six salutations</t>
+          <t>Ne pas envoyer</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>Fiches FPJQ mal formées, signalées dans la colonne Précaution.</t>
+          <t>Anne-Sophie Roy à l'adresse Québecor, doublon de sa ligne Radio-Canada. Annie Lafrance et Francis Higgins en liste froide, doublons de la liste chaude.</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
         <is>
+          <t>Six salutations</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>Fiches FPJQ mal formées, signalées dans la colonne Précaution.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="3" t="inlineStr">
+        <is>
           <t>Registre</t>
         </is>
       </c>
-      <c r="B14" s="2" t="inlineStr">
-        <is>
-          <t>Chloé Pouliot au « tu », tout le reste au « vous ». Bascule la colonne et je relance.</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="3" t="n"/>
-      <c r="B15" s="2" t="n"/>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>Chloé Pouliot et Stéphanie Bérubé au « tu », tout le reste au « vous ». Bascule la colonne et je relance.</t>
+        </is>
+      </c>
     </row>
     <row r="16">
-      <c r="A16" s="1" t="inlineStr">
+      <c r="A16" s="3" t="n"/>
+      <c r="B16" s="2" t="n"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="1" t="inlineStr">
         <is>
           <t>Rappels</t>
         </is>
       </c>
-      <c r="B16" s="2" t="n"/>
-    </row>
-    <row r="17">
-      <c r="A17" s="3" t="n"/>
       <c r="B17" s="2" t="n"/>
     </row>
     <row r="18">
-      <c r="A18" s="3" t="inlineStr">
-        <is>
-          <t>Diffusion</t>
-        </is>
-      </c>
-      <c r="B18" s="2" t="inlineStr">
-        <is>
-          <t>Jeudi 17 septembre 2026, 20 h (20 h 30 NT), CBC et CBC Gem. Prévente le samedi 12 septembre à 9 h.</t>
-        </is>
-      </c>
+      <c r="A18" s="3" t="n"/>
+      <c r="B18" s="2" t="n"/>
     </row>
     <row r="19">
       <c r="A19" s="3" t="inlineStr">
         <is>
-          <t>Envoi</t>
+          <t>Diffusion</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>Missive depuis media@lasclay.com, un appel par journaliste, suivi des ouvertures et des clics désactivé, environ 60 par jour. Le mode par défaut dépose un brouillon.</t>
+          <t>Jeudi 17 septembre 2026, 20 h (20 h 30 NT), CBC et CBC Gem. Prévente le samedi 12 septembre à 9 h.</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="3" t="inlineStr">
         <is>
+          <t>Envoi</t>
+        </is>
+      </c>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>Missive depuis media@lasclay.com, un appel par journaliste, suivi des ouvertures et des clics désactivé, environ 60 par jour. Le mode par défaut dépose un brouillon.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="3" t="inlineStr">
+        <is>
           <t>Interdits CBC</t>
         </is>
       </c>
-      <c r="B20" s="2" t="inlineStr">
+      <c r="B21" s="2" t="inlineStr">
         <is>
           <t>Rien sur l'issue avant le 17. Aucun logo ni « vu à Dragons' Den ».</t>
         </is>
@@ -848,7 +860,7 @@
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>vous</t>
+          <t>tu</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
@@ -858,16 +870,15 @@
       </c>
       <c r="K3" s="2" t="inlineStr">
         <is>
-          <t>Bonjour Mme Bérubé,
-En février, vous avez signé « La sinueuse route de la soie du Nord ». C'est un des rares textes à avoir pris la filière au complet, et pas juste une entreprise.
-Merci d'avoir pris cette peine-là. La filière a plus besoin d'être racontée en entier qu'entreprise par entreprise, et presque personne ne le fait.
+          <t>Bonjour Stéphanie,
+J'espère que tu vas bien. En février dernier, tu as signé « La sinueuse route de la soie du Nord », un des rares textes à avoir pris la filière au complet plutôt qu'une entreprise à la fois. Merci pour ce bel article, qui a fait une place de choix à Lasclay et à ses défis.
 Depuis, tout mon temps va à mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
 Eh bien, le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
-Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer une suite à votre dernier article.
-Notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
-J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
-Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
+Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais t'en faire part et qui sait, peut-être t'inspirer une suite à ton dernier article.
+Notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
+J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
+Au plaisir et n'hésite pas à me contacter si tu as des questions.</t>
         </is>
       </c>
       <c r="L3" s="5" t="n"/>

</xml_diff>